<commit_message>
Add Q406-Q410 and update Excel export (322 entries)
Q406 Astronomy: neutron stars
Q407 Psychology: cognitive dissonance
Q408 Chemistry: catalysts
Q409 CS: AI vs ML vs deep learning
Q410 History: the Enlightenment

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E318"/>
+  <dimension ref="A1:E323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7606,20 +7606,52 @@
       </c>
     </row>
     <row r="275">
-      <c r="A275" s="24" t="n">
+      <c r="A275" s="22" t="n">
+        <v>406</v>
+      </c>
+      <c r="B275" s="23" t="inlineStr">
+        <is>
+          <t>Astronomy</t>
+        </is>
+      </c>
+      <c r="C275" s="23" t="inlineStr">
+        <is>
+          <t>What is a neutron star and what are its extreme properties?</t>
+        </is>
+      </c>
+      <c r="D275" s="23" t="inlineStr">
+        <is>
+          <t>A neutron star is the collapsed core of a massive star (8-20 solar masses) after a supernova. Electrons and protons merge into neutrons — nuclear matter held up by neutron degeneracy pressure.
+Extreme properties:
+- Mass: 1.4-2+ solar masses in ~20 km diameter
+- Density: ~10^17 kg/m^3 — a teaspoon weighs ~1 billion tonnes
+- Gravity: surface ~2x10^11 m/s^2 (20 billion times Earth's)
+- Magnetic field: up to 10^15 Tesla (magnetars)
+- Rotation: pulsars spin 1-700 Hz; PSR J1748-2446ad at 716 Hz moves equator at ~0.24c
+- Temperature: ~10^11 K at birth; cools to ~10^6 K
+Pulsars: rotating neutron stars with beamed radio emission — cosmic lighthouses. So precise (nanosecond) they were mistaken for alien signals (LGM-1, 1967, Jocelyn Bell Burnell).
+Exotic interior: possible quark-gluon plasma at core; neutron superfluidity. Physics at limits of known matter.</t>
+        </is>
+      </c>
+      <c r="E275" s="22" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="24" t="n">
         <v>407</v>
       </c>
-      <c r="B275" s="25" t="inlineStr">
+      <c r="B276" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C275" s="25" t="inlineStr">
+      <c r="C276" s="25" t="inlineStr">
         <is>
           <t>What is cognitive dissonance and how do people actually resolve it?</t>
         </is>
       </c>
-      <c r="D275" s="25" t="inlineStr">
+      <c r="D276" s="25" t="inlineStr">
         <is>
           <t>Festinger (1957): holding two conflicting cognitions creates psychological discomfort. Three resolution strategies:
 1. **Change a belief**: smoker convinces themselves they're immune.
@@ -7631,25 +7663,56 @@
 Dissonance magnitude: greater when decisions are important, irreversible, options similar in quality.</t>
         </is>
       </c>
-      <c r="E275" s="24" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" s="22" t="n">
+      <c r="E276" s="24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="24" t="n">
+        <v>407</v>
+      </c>
+      <c r="B277" s="25" t="inlineStr">
+        <is>
+          <t>Psychology</t>
+        </is>
+      </c>
+      <c r="C277" s="25" t="inlineStr">
+        <is>
+          <t>What is cognitive dissonance and how do people resolve it?</t>
+        </is>
+      </c>
+      <c r="D277" s="25" t="inlineStr">
+        <is>
+          <t>Festinger (1957): holding two psychologically inconsistent cognitions creates uncomfortable tension (dissonance), motivating reduction.
+Classic experiment (Festinger &amp; Carlsmith 1959): $1 vs $20 to lie about boring task. $1 group rated task as more enjoyable — insufficient external justification, so changed attitude to match behaviour.
+Resolution strategies:
+1. Change a belief
+2. Add consonant cognitions ('I exercise so smoking balances out')
+3. Trivialise the inconsistency
+4. Change behaviour (least common)
+Phenomena: post-purchase dissonance (rationalising expensive buys); effort justification (things you suffered for feel more valuable — hazing); belief perseverance (doubling down when proved wrong — Festinger's doomsday cult).
+Modern view: dissonance requires self-relevant, freely chosen behaviour. Self-affirmation can buffer it.</t>
+        </is>
+      </c>
+      <c r="E277" s="24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="22" t="n">
         <v>408</v>
       </c>
-      <c r="B276" s="23" t="inlineStr">
+      <c r="B278" s="23" t="inlineStr">
         <is>
           <t>Astronomy</t>
         </is>
       </c>
-      <c r="C276" s="23" t="inlineStr">
+      <c r="C278" s="23" t="inlineStr">
         <is>
           <t>How do astronomers know the age of the universe is 13.8 billion years?</t>
         </is>
       </c>
-      <c r="D276" s="23" t="inlineStr">
+      <c r="D278" s="23" t="inlineStr">
         <is>
           <t>Multiple independent methods converge:
 1. **CMB (Planck)**: temperature fluctuation power spectrum fit to LCDM model gives 13.787 +/- 0.020 Gyr
@@ -7659,25 +7722,59 @@
 **Why trust it**: four independent methods (CMB, expansion history, stellar ages, nuclear physics) all point to 13-14 Gyr. Concordance is extraordinary.</t>
         </is>
       </c>
-      <c r="E276" s="22" t="n">
+      <c r="E278" s="22" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="277">
-      <c r="A277" s="2" t="n">
+    <row r="279">
+      <c r="A279" s="28" t="n">
+        <v>408</v>
+      </c>
+      <c r="B279" s="29" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="C279" s="29" t="inlineStr">
+        <is>
+          <t>How do catalysts work and why aren't they consumed?</t>
+        </is>
+      </c>
+      <c r="D279" s="29" t="inlineStr">
+        <is>
+          <t>A catalyst increases reaction rate without being consumed. It provides an alternative pathway with lower activation energy.
+Mechanism:
+1. Reactants bind to catalyst (adsorption or complex formation)
+2. Transition state is stabilised — less energy needed
+3. Products form and detach, regenerating the catalyst
+Because the catalyst is regenerated, one molecule can facilitate millions of cycles.
+Types:
+- Homogeneous: same phase as reactants (H+ in acid hydrolysis)
+- Heterogeneous: different phase (platinum in catalytic converters; iron in Haber process)
+- Enzymes: protein catalysts; 10^6-10^12 rate increase over uncatalysed
+Energy diagram: catalyst lowers activation energy but not ΔG — it speeds approach to equilibrium but cannot make a thermodynamically unfavourable reaction spontaneous.
+Catalyst poisons (e.g. H2S, CO in Haber process) block active sites.</t>
+        </is>
+      </c>
+      <c r="E279" s="28" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="n">
         <v>409</v>
       </c>
-      <c r="B277" s="3" t="inlineStr">
+      <c r="B280" s="3" t="inlineStr">
         <is>
           <t>Law</t>
         </is>
       </c>
-      <c r="C277" s="3" t="inlineStr">
+      <c r="C280" s="3" t="inlineStr">
         <is>
           <t>What is the difference between civil law and common law legal systems?</t>
         </is>
       </c>
-      <c r="D277" s="3" t="inlineStr">
+      <c r="D280" s="3" t="inlineStr">
         <is>
           <t>**Common law** (UK, US, Australia, Canada, India):
 - Judge-made law; past decisions (stare decisis) bind future courts
@@ -7696,25 +7793,58 @@
 **Hybrid**: Louisiana, Quebec, Scotland — civil law base with common law influence.</t>
         </is>
       </c>
-      <c r="E277" s="2" t="n">
+      <c r="E280" s="2" t="n">
         <v>8.5</v>
       </c>
     </row>
-    <row r="278">
-      <c r="A278" s="2" t="n">
+    <row r="281">
+      <c r="A281" s="20" t="n">
+        <v>409</v>
+      </c>
+      <c r="B281" s="21" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="C281" s="21" t="inlineStr">
+        <is>
+          <t>What is the difference between machine learning, deep learning, and AI?</t>
+        </is>
+      </c>
+      <c r="D281" s="21" t="inlineStr">
+        <is>
+          <t>Nested concepts, not synonyms:
+AI (broadest): any technique making computers solve tasks needing human intelligence — rules, search, expert systems, ML.
+Machine Learning (subset of AI): systems that learn from data without explicit programming. Supervised, unsupervised, reinforcement learning.
+Deep Learning (subset of ML): neural networks with many layers learning hierarchical representations. Enabled by large datasets, GPUs, backpropagation.
+Hierarchy: AI ⊃ Machine Learning ⊃ Deep Learning
+Why deep learning dominated post-2012: ImageNet — AlexNet (Hinton) achieved 15.3% error vs ~26% for prior methods.
+Practical distinction:
+- Rule-based AI: chess engine with hand-coded evaluation
+- Classical ML: random forest on labelled data
+- Deep Learning: CNN on raw images; LLM trained on text
+Current frontier: LLMs, diffusion models, RL from human feedback.</t>
+        </is>
+      </c>
+      <c r="E281" s="20" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="n">
         <v>410</v>
       </c>
-      <c r="B278" s="3" t="inlineStr">
+      <c r="B282" s="3" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C278" s="3" t="inlineStr">
+      <c r="C282" s="3" t="inlineStr">
         <is>
           <t>What is Moore's Law and is it still true?</t>
         </is>
       </c>
-      <c r="D278" s="3" t="inlineStr">
+      <c r="D282" s="3" t="inlineStr">
         <is>
           <t>Gordon Moore (1965): transistors on a chip double every ~2 years at same cost. Not physical law — empirical observation, self-fulfilling prophecy shaping semiconductor roadmaps.
 **Historical accuracy**: held ~1965-2015. From 4 transistors (1959) to 10B+ (modern).
@@ -7730,25 +7860,56 @@
 **Verdict**: strict transistor-count doubling has slowed. 'Moore's Law is dead' is too strong — relentless compute improvement continues through different means.</t>
         </is>
       </c>
-      <c r="E278" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" s="30" t="n">
+      <c r="E282" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="12" t="n">
+        <v>410</v>
+      </c>
+      <c r="B283" s="13" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="C283" s="13" t="inlineStr">
+        <is>
+          <t>What was the Enlightenment and why did it matter?</t>
+        </is>
+      </c>
+      <c r="D283" s="13" t="inlineStr">
+        <is>
+          <t>Enlightenment (~1685-1800): intellectual movement emphasising reason, individual rights, scepticism of authority, empirical inquiry.
+Key figures: Locke (natural rights, social contract), Voltaire (tolerance, free speech), Rousseau (general will), Montesquieu (separation of powers), Hume (empiricism, scepticism), Kant (sapere aude, categorical imperative), Smith (free markets, Wealth of Nations 1776).
+Why it mattered:
+- American Revolution 1776: Declaration of Independence — Lockean natural rights
+- French Revolution 1789: liberty/equality/fraternity — Enlightenment ideals, violently distorted
+- Abolition: rational arguments against slavery
+- Democracy: constitutional law, rights of citizens
+- Science: empirical method, separation from church
+Counter-currents: Romantics reacted against cold rationalism. Enlightenment ideals co-existed with colonialism — the contradictions remain contentious.</t>
+        </is>
+      </c>
+      <c r="E283" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="30" t="n">
         <v>411</v>
       </c>
-      <c r="B279" s="31" t="inlineStr">
+      <c r="B284" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C279" s="31" t="inlineStr">
+      <c r="C284" s="31" t="inlineStr">
         <is>
           <t>What is the placebo effect, and is it 'just' in your head?</t>
         </is>
       </c>
-      <c r="D279" s="31" t="inlineStr">
+      <c r="D284" s="31" t="inlineStr">
         <is>
           <t>Measurable physiological improvement from inert treatment when patient believes it's real. NOT just imagination.
 **Documented mechanisms:**
@@ -7761,25 +7922,25 @@
 **Nocebo**: negative expectations cause real harm — side effects, slower healing.</t>
         </is>
       </c>
-      <c r="E279" s="30" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" s="14" t="n">
+      <c r="E284" s="30" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="14" t="n">
         <v>412</v>
       </c>
-      <c r="B280" s="15" t="inlineStr">
+      <c r="B285" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C280" s="15" t="inlineStr">
+      <c r="C285" s="15" t="inlineStr">
         <is>
           <t>What is Godel's incompleteness theorem, in plain terms?</t>
         </is>
       </c>
-      <c r="D280" s="15" t="inlineStr">
+      <c r="D285" s="15" t="inlineStr">
         <is>
           <t>Godel (1931): one of the most astonishing results in intellectual history.
 **First theorem**: any consistent formal system powerful enough to describe arithmetic contains true statements that cannot be proved within that system.
@@ -7796,25 +7957,25 @@
 Closely related to Turing's undecidability.</t>
         </is>
       </c>
-      <c r="E280" s="14" t="n">
+      <c r="E285" s="14" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="281">
-      <c r="A281" s="2" t="n">
+    <row r="286">
+      <c r="A286" s="2" t="n">
         <v>413</v>
       </c>
-      <c r="B281" s="3" t="inlineStr">
+      <c r="B286" s="3" t="inlineStr">
         <is>
           <t>Environmental Science</t>
         </is>
       </c>
-      <c r="C281" s="3" t="inlineStr">
+      <c r="C286" s="3" t="inlineStr">
         <is>
           <t>What is the greenhouse effect, and how does it work physically?</t>
         </is>
       </c>
-      <c r="D281" s="3" t="inlineStr">
+      <c r="D286" s="3" t="inlineStr">
         <is>
           <t>Natural and necessary — without it, Earth would be -18C not +15C. Problem is the *enhanced* effect from human emissions.
 **Mechanism:**
@@ -7829,25 +7990,25 @@
 - Cloud feedbacks: complex, main uncertainty in climate sensitivity</t>
         </is>
       </c>
-      <c r="E281" s="2" t="n">
+      <c r="E286" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="282">
-      <c r="A282" s="2" t="n">
+    <row r="287">
+      <c r="A287" s="2" t="n">
         <v>414</v>
       </c>
-      <c r="B282" s="3" t="inlineStr">
+      <c r="B287" s="3" t="inlineStr">
         <is>
           <t>Music Theory</t>
         </is>
       </c>
-      <c r="C282" s="3" t="inlineStr">
+      <c r="C287" s="3" t="inlineStr">
         <is>
           <t>Why do some musical intervals sound consonant and others dissonant?</t>
         </is>
       </c>
-      <c r="D282" s="3" t="inlineStr">
+      <c r="D287" s="3" t="inlineStr">
         <is>
           <t>Multiple overlapping explanations:
 1. **Frequency ratios** (Pythagoras): simple integer ratios sound consonant. Octave=2:1, fifth=3:2, fourth=4:3. Complex ratios (tritone ~45:32) sound tense.
@@ -7858,25 +8019,25 @@
 **Why music uses dissonance**: pure consonance is boring. Tension-resolution is the engine of musical emotion.</t>
         </is>
       </c>
-      <c r="E282" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" s="2" t="n">
+      <c r="E287" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="n">
         <v>415</v>
       </c>
-      <c r="B283" s="3" t="inlineStr">
+      <c r="B288" s="3" t="inlineStr">
         <is>
           <t>Political Science</t>
         </is>
       </c>
-      <c r="C283" s="3" t="inlineStr">
+      <c r="C288" s="3" t="inlineStr">
         <is>
           <t>What is the difference between a democracy and a republic, and does the distinction matter?</t>
         </is>
       </c>
-      <c r="D283" s="3" t="inlineStr">
+      <c r="D288" s="3" t="inlineStr">
         <is>
           <t>**Democracy**: rule by the people. Pure direct democracy — citizens vote on every law. Athens: male citizens voted directly. Impossible at scale.
 **Republic** (res publica): power held by elected representatives, not exercised directly. Citizens choose who decides, not what is decided.
@@ -7886,25 +8047,25 @@
 **Other**: constitutional republic (limits on power), parliamentary vs presidential republic.</t>
         </is>
       </c>
-      <c r="E283" s="2" t="n">
+      <c r="E288" s="2" t="n">
         <v>8.5</v>
       </c>
     </row>
-    <row r="284">
-      <c r="A284" s="24" t="n">
+    <row r="289">
+      <c r="A289" s="24" t="n">
         <v>416</v>
       </c>
-      <c r="B284" s="25" t="inlineStr">
+      <c r="B289" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C284" s="25" t="inlineStr">
+      <c r="C289" s="25" t="inlineStr">
         <is>
           <t>What is the bystander effect, and when does it NOT apply?</t>
         </is>
       </c>
-      <c r="D284" s="25" t="inlineStr">
+      <c r="D289" s="25" t="inlineStr">
         <is>
           <t>Kitty Genovese (1964) led to Latane and Darley's research. Two mechanisms:
 1. Diffusion of responsibility: each bystander assumes someone else will act
@@ -7919,25 +8080,25 @@
 **Genovese myth**: Fischer et al. 2011 — 38 witnesses story exaggerated by NYT. Many didn't hear/see clearly. Effect is real, original story was sensationalised.</t>
         </is>
       </c>
-      <c r="E284" s="24" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="285">
-      <c r="A285" s="2" t="n">
+      <c r="E289" s="24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="n">
         <v>417</v>
       </c>
-      <c r="B285" s="3" t="inlineStr">
+      <c r="B290" s="3" t="inlineStr">
         <is>
           <t>Geology</t>
         </is>
       </c>
-      <c r="C285" s="3" t="inlineStr">
+      <c r="C290" s="3" t="inlineStr">
         <is>
           <t>How do plate tectonics work, and what drives the plates?</t>
         </is>
       </c>
-      <c r="D285" s="3" t="inlineStr">
+      <c r="D290" s="3" t="inlineStr">
         <is>
           <t>~15 major lithospheric plates (100km thick) float on viscous asthenosphere, moving 2-10 cm/year.
 **Three boundary types:**
@@ -7951,25 +8112,25 @@
 **Evidence**: magnetic striping on seafloor, continental fit (Wegener), matching fossils, earthquake distributions.</t>
         </is>
       </c>
-      <c r="E285" s="2" t="n">
+      <c r="E290" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="286">
-      <c r="A286" s="14" t="n">
+    <row r="291">
+      <c r="A291" s="14" t="n">
         <v>418</v>
       </c>
-      <c r="B286" s="15" t="inlineStr">
+      <c r="B291" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C286" s="15" t="inlineStr">
+      <c r="C291" s="15" t="inlineStr">
         <is>
           <t>What is a Fourier transform, and why is it everywhere?</t>
         </is>
       </c>
-      <c r="D286" s="15" t="inlineStr">
+      <c r="D291" s="15" t="inlineStr">
         <is>
           <t>Fourier (1822): any periodic function decomposes into sines and cosines of different frequencies.
 Fourier transform: takes time-domain signal f(t) -&gt; frequency-domain F(w) showing how much of each frequency is present.
@@ -7984,25 +8145,25 @@
 **FFT** (Cooley-Tukey 1965): O(n log n) vs O(n^2) naive. Made real-time signal processing possible.</t>
         </is>
       </c>
-      <c r="E286" s="14" t="n">
+      <c r="E291" s="14" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="287">
-      <c r="A287" s="2" t="n">
+    <row r="292">
+      <c r="A292" s="2" t="n">
         <v>419</v>
       </c>
-      <c r="B287" s="3" t="inlineStr">
+      <c r="B292" s="3" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
       </c>
-      <c r="C287" s="3" t="inlineStr">
+      <c r="C292" s="3" t="inlineStr">
         <is>
           <t>What is the difference between deontological and consequentialist ethics, and which is right?</t>
         </is>
       </c>
-      <c r="D287" s="3" t="inlineStr">
+      <c r="D292" s="3" t="inlineStr">
         <is>
           <t>**Consequentialism** (Bentham, Mill): moral worth from consequences. Maximise utility/welfare. Strength: outcome-focused. Weakness: justifies organ harvesting one person to save five; ignores rights.
 **Deontology** (Kant): moral worth from the action itself, not consequences. Categorical Imperative:
@@ -8017,25 +8178,25 @@
 Reflective equilibrium: use multiple frameworks as lenses, check coherence with intuitions.</t>
         </is>
       </c>
-      <c r="E287" s="2" t="n">
+      <c r="E292" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="288">
-      <c r="A288" s="4" t="n">
+    <row r="293">
+      <c r="A293" s="4" t="n">
         <v>420</v>
       </c>
-      <c r="B288" s="5" t="inlineStr">
+      <c r="B293" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="C288" s="5" t="inlineStr">
+      <c r="C293" s="5" t="inlineStr">
         <is>
           <t>What is the difference between descriptive and prescriptive grammar, and why does it matter?</t>
         </is>
       </c>
-      <c r="D288" s="5" t="inlineStr">
+      <c r="D293" s="5" t="inlineStr">
         <is>
           <t>**Prescriptive**: what people *should* say — textbooks, style guides, norms ('don't split infinitives', 'it is I').
 **Descriptive**: what people *actually* say — linguist's approach. Records patterns without judging. Every human language has consistent grammar; no language is 'wrong.'
@@ -8047,25 +8208,25 @@
 5. Code-switching: competent speakers deploy both — AAVE at home, SAE formally. Both correct for their domains.</t>
         </is>
       </c>
-      <c r="E288" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" s="18" t="n">
+      <c r="E293" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="18" t="n">
         <v>421</v>
       </c>
-      <c r="B289" s="19" t="inlineStr">
+      <c r="B294" s="19" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C289" s="19" t="inlineStr">
+      <c r="C294" s="19" t="inlineStr">
         <is>
           <t>How does the immune system distinguish 'self' from 'non-self'?</t>
         </is>
       </c>
-      <c r="D289" s="19" t="inlineStr">
+      <c r="D294" s="19" t="inlineStr">
         <is>
           <t>Multiple overlapping mechanisms:
 **MHC class I**: every nucleated cell displays own protein fragments on MHC class I. T-cells educated in thymus to tolerate self-peptides; cells displaying foreign peptides (viral, tumour) are destroyed.
@@ -8077,25 +8238,25 @@
 - Transplant rejection: donor MHC recognised as foreign</t>
         </is>
       </c>
-      <c r="E289" s="18" t="n">
+      <c r="E294" s="18" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="290">
-      <c r="A290" s="12" t="n">
+    <row r="295">
+      <c r="A295" s="12" t="n">
         <v>422</v>
       </c>
-      <c r="B290" s="13" t="inlineStr">
+      <c r="B295" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C290" s="13" t="inlineStr">
+      <c r="C295" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the printing press, and did Gutenberg invent it?</t>
         </is>
       </c>
-      <c r="D290" s="13" t="inlineStr">
+      <c r="D295" s="13" t="inlineStr">
         <is>
           <t>Gutenberg (~1450) didn't invent printing. Moveable type existed in China (Bi Sheng ~1040) and Korea (Jikji 1377, oldest surviving). Gutenberg's innovation: complete system — durable metal alloy type, oil-based ink, adapted screw press — optimised for the European alphabet.
 **Why it transformed Europe**: Latin alphabet (26 letters) made moveable type far more efficient than Chinese/Korean systems (thousands of characters). Press: ~3,600 pages/day vs 40 for a scribe.
@@ -8108,25 +8269,25 @@
 **Eisenstein's thesis**: press created new relationship with knowledge — standardisation, reproducibility, verification.</t>
         </is>
       </c>
-      <c r="E290" s="12" t="n">
+      <c r="E295" s="12" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="291">
-      <c r="A291" s="10" t="n">
+    <row r="296">
+      <c r="A296" s="10" t="n">
         <v>423</v>
       </c>
-      <c r="B291" s="11" t="inlineStr">
+      <c r="B296" s="11" t="inlineStr">
         <is>
           <t>Neuroscience</t>
         </is>
       </c>
-      <c r="C291" s="11" t="inlineStr">
+      <c r="C296" s="11" t="inlineStr">
         <is>
           <t>What is consciousness and why is it so hard to explain?</t>
         </is>
       </c>
-      <c r="D291" s="11" t="inlineStr">
+      <c r="D296" s="11" t="inlineStr">
         <is>
           <t>Chalmers (1995) 'hard problem': why does information processing produce *subjective experience*? Why is there something it is like to see red?
 Even full neural mapping of correlates wouldn't explain why any of it feels like anything. Explaining function doesn't explain qualia.
@@ -8139,25 +8300,25 @@
 **Consensus**: none. Hard problem remains genuinely open.</t>
         </is>
       </c>
-      <c r="E291" s="10" t="n">
+      <c r="E296" s="10" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="292">
-      <c r="A292" s="28" t="n">
+    <row r="297">
+      <c r="A297" s="28" t="n">
         <v>424</v>
       </c>
-      <c r="B292" s="29" t="inlineStr">
+      <c r="B297" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C292" s="29" t="inlineStr">
+      <c r="C297" s="29" t="inlineStr">
         <is>
           <t>What makes some molecules smell while others don't?</t>
         </is>
       </c>
-      <c r="D292" s="29" t="inlineStr">
+      <c r="D297" s="29" t="inlineStr">
         <is>
           <t>Odorant molecules bind to olfactory receptors (ORs, GPCRs) in nasal epithelium -&gt; olfactory bulb -&gt; piriform cortex + limbic system.
 **What molecules smell:**
@@ -8169,25 +8330,25 @@
 **COVID-19 anosmia**: virus destroys olfactory neuron support cells; usually recovers.</t>
         </is>
       </c>
-      <c r="E292" s="28" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" s="8" t="n">
+      <c r="E297" s="28" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="8" t="n">
         <v>425</v>
       </c>
-      <c r="B293" s="9" t="inlineStr">
+      <c r="B298" s="9" t="inlineStr">
         <is>
           <t>Economics</t>
         </is>
       </c>
-      <c r="C293" s="9" t="inlineStr">
+      <c r="C298" s="9" t="inlineStr">
         <is>
           <t>What caused the 2008 financial crisis?</t>
         </is>
       </c>
-      <c r="D293" s="9" t="inlineStr">
+      <c r="D298" s="9" t="inlineStr">
         <is>
           <t>Cascade of failures:
 **Housing bubble**: low post-9/11 rates, relaxed lending, NINJA loans (no income/assets/job). Prices +124% nationally 2000-2006.
@@ -8199,25 +8360,25 @@
 **Response**: Dodd-Frank, Basel III capital requirements, Volcker Rule.</t>
         </is>
       </c>
-      <c r="E293" s="8" t="n">
+      <c r="E298" s="8" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="294">
-      <c r="A294" s="6" t="n">
+    <row r="299">
+      <c r="A299" s="6" t="n">
         <v>426</v>
       </c>
-      <c r="B294" s="7" t="inlineStr">
+      <c r="B299" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C294" s="7" t="inlineStr">
+      <c r="C299" s="7" t="inlineStr">
         <is>
           <t>What is dark matter and how do we know it exists?</t>
         </is>
       </c>
-      <c r="D294" s="7" t="inlineStr">
+      <c r="D299" s="7" t="inlineStr">
         <is>
           <t>~27% of universe's energy. Doesn't emit/absorb/reflect light. Gravitational effects overwhelming.
 **Evidence:**
@@ -8229,25 +8390,25 @@
 **MOND alternative**: modified Newtonian dynamics; cannot explain Bullet Cluster + CMB simultaneously. Most physicists favour particle dark matter.</t>
         </is>
       </c>
-      <c r="E294" s="6" t="n">
+      <c r="E299" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="295">
-      <c r="A295" s="2" t="n">
+    <row r="300">
+      <c r="A300" s="2" t="n">
         <v>427</v>
       </c>
-      <c r="B295" s="3" t="inlineStr">
+      <c r="B300" s="3" t="inlineStr">
         <is>
           <t>Literature</t>
         </is>
       </c>
-      <c r="C295" s="3" t="inlineStr">
+      <c r="C300" s="3" t="inlineStr">
         <is>
           <t>Why is 'Don Quixote' considered the first modern novel?</t>
         </is>
       </c>
-      <c r="D295" s="3" t="inlineStr">
+      <c r="D300" s="3" t="inlineStr">
         <is>
           <t>Cervantes (Part I: 1605, Part II: 1615). Why it's considered the first modern novel:
 1. Self-consciousness: the novel is aware it's a novel. Part II characters have read Part I. Unreliable narrators, manuscript frames — postmodern devices 400 years early.
@@ -8258,25 +8419,25 @@
 What makes it 'modern': fundamentally ambiguous relationship with truth; character who changes across time (Part I vs II Quixote). Bloom: 'most universal and most particular character in literature.'</t>
         </is>
       </c>
-      <c r="E295" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="296">
-      <c r="A296" s="20" t="n">
+      <c r="E300" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="20" t="n">
         <v>428</v>
       </c>
-      <c r="B296" s="21" t="inlineStr">
+      <c r="B301" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C296" s="21" t="inlineStr">
+      <c r="C301" s="21" t="inlineStr">
         <is>
           <t>What is the halting problem and why does it matter?</t>
         </is>
       </c>
-      <c r="D296" s="21" t="inlineStr">
+      <c r="D301" s="21" t="inlineStr">
         <is>
           <t>Turing (1936): no general algorithm can determine whether an arbitrary program will halt or run forever.
 **Proof (diagonal argument)**: assume HALT(P,I) exists. Construct DIAG(P): if HALT says P halts on P -&gt; loop; if HALT says P loops -&gt; halt.
@@ -8289,25 +8450,25 @@
 5. Practical: compilers and static analysers must be incomplete or unsound — they make heuristic approximations.</t>
         </is>
       </c>
-      <c r="E296" s="20" t="n">
+      <c r="E301" s="20" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="297">
-      <c r="A297" s="30" t="n">
+    <row r="302">
+      <c r="A302" s="30" t="n">
         <v>429</v>
       </c>
-      <c r="B297" s="31" t="inlineStr">
+      <c r="B302" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C297" s="31" t="inlineStr">
+      <c r="C302" s="31" t="inlineStr">
         <is>
           <t>How do vaccines work, and why do some require boosters?</t>
         </is>
       </c>
-      <c r="D297" s="31" t="inlineStr">
+      <c r="D302" s="31" t="inlineStr">
         <is>
           <t>Vaccine presents antigen (weakened/killed pathogen, subunit protein, or mRNA) without disease, training immune memory.
 **Mechanism:**
@@ -8324,25 +8485,25 @@
 **Why boosters**: antibody titres wane (inactivated/subunit weaker); mutating viruses (flu) change antigens.</t>
         </is>
       </c>
-      <c r="E297" s="30" t="n">
+      <c r="E302" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="298">
-      <c r="A298" s="16" t="n">
+    <row r="303">
+      <c r="A303" s="16" t="n">
         <v>430</v>
       </c>
-      <c r="B298" s="17" t="inlineStr">
+      <c r="B303" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C298" s="17" t="inlineStr">
+      <c r="C303" s="17" t="inlineStr">
         <is>
           <t>What is free will, and does science undermine it?</t>
         </is>
       </c>
-      <c r="D298" s="17" t="inlineStr">
+      <c r="D303" s="17" t="inlineStr">
         <is>
           <t>Are our choices genuinely ours, or determined by prior causes?
 **Three positions:**
@@ -8354,25 +8515,25 @@
 **Does science undermine it?** Depends what you mean. Compatibilist free will survives. Hard determinism mostly fringe.</t>
         </is>
       </c>
-      <c r="E298" s="16" t="n">
+      <c r="E303" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="299">
-      <c r="A299" s="22" t="n">
+    <row r="304">
+      <c r="A304" s="22" t="n">
         <v>431</v>
       </c>
-      <c r="B299" s="23" t="inlineStr">
+      <c r="B304" s="23" t="inlineStr">
         <is>
           <t>Astronomy</t>
         </is>
       </c>
-      <c r="C299" s="23" t="inlineStr">
+      <c r="C304" s="23" t="inlineStr">
         <is>
           <t>What are neutron stars and how do they form?</t>
         </is>
       </c>
-      <c r="D299" s="23" t="inlineStr">
+      <c r="D304" s="23" t="inlineStr">
         <is>
           <t>Massive star (8-20 solar masses) core collapses. If core mass 1.4-3 solar masses, electron degeneracy fails. Protons + electrons merge (inverse beta decay) -&gt; neutron star.
 **Properties:**
@@ -8385,25 +8546,25 @@
 **Neutron star mergers (GW170817, 2017)**: first gravitational wave + electromagnetic detection. Kilonova: r-process nucleosynthesis produces gold, platinum, uranium. Primary source of heavy elements.</t>
         </is>
       </c>
-      <c r="E299" s="22" t="n">
+      <c r="E304" s="22" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="300">
-      <c r="A300" s="24" t="n">
+    <row r="305">
+      <c r="A305" s="24" t="n">
         <v>432</v>
       </c>
-      <c r="B300" s="25" t="inlineStr">
+      <c r="B305" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C300" s="25" t="inlineStr">
+      <c r="C305" s="25" t="inlineStr">
         <is>
           <t>What is the Dunning-Kruger effect, and is it as universal as people think?</t>
         </is>
       </c>
-      <c r="D300" s="25" t="inlineStr">
+      <c r="D305" s="25" t="inlineStr">
         <is>
           <t>Kruger &amp; Dunning (1999): people with limited knowledge overestimate competence; experts underestimate relative ability (task seems easy to them too).
 **Original study**: bottom quartile performers on logic/grammar/humour overestimated by ~50 percentile points.
@@ -8417,25 +8578,25 @@
 - Domain-specific: expert engineer may still have DK in social skills</t>
         </is>
       </c>
-      <c r="E300" s="24" t="n">
+      <c r="E305" s="24" t="n">
         <v>8.5</v>
       </c>
     </row>
-    <row r="301">
-      <c r="A301" s="12" t="n">
+    <row r="306">
+      <c r="A306" s="12" t="n">
         <v>433</v>
       </c>
-      <c r="B301" s="13" t="inlineStr">
+      <c r="B306" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C301" s="13" t="inlineStr">
+      <c r="C306" s="13" t="inlineStr">
         <is>
           <t>Why did the Roman Empire fall?</t>
         </is>
       </c>
-      <c r="D301" s="13" t="inlineStr">
+      <c r="D306" s="13" t="inlineStr">
         <is>
           <t>Western Empire fell 476 CE (Romulus Augustulus deposed). Eastern Empire (Byzantium) lasted to 1453. No single cause:
 **Military/political:** overextended borders; Germanic foederati with divided loyalty; political instability (50 emperors in 50 years, 235-284 CE); military power to make/unmake emperors.
@@ -8448,25 +8609,25 @@
 **What didn't fall**: Eastern Empire thrived. Fall was primarily western.</t>
         </is>
       </c>
-      <c r="E301" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" s="2" t="n">
+      <c r="E306" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="n">
         <v>434</v>
       </c>
-      <c r="B302" s="3" t="inlineStr">
+      <c r="B307" s="3" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C302" s="3" t="inlineStr">
+      <c r="C307" s="3" t="inlineStr">
         <is>
           <t>How does GPS actually work?</t>
         </is>
       </c>
-      <c r="D302" s="3" t="inlineStr">
+      <c r="D307" s="3" t="inlineStr">
         <is>
           <t>24-32 satellites at ~20,200km; 6 orbital planes; each completes 2 orbits/day.
 **Core principle: trilateration via time signals.**
@@ -8482,25 +8643,25 @@
 - Net: +38 microseconds/day. Without correction: GPS drifts ~10km/day. Einstein's corrections are in the system.</t>
         </is>
       </c>
-      <c r="E302" s="2" t="n">
+      <c r="E307" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="303">
-      <c r="A303" s="18" t="n">
+    <row r="308">
+      <c r="A308" s="18" t="n">
         <v>435</v>
       </c>
-      <c r="B303" s="19" t="inlineStr">
+      <c r="B308" s="19" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C303" s="19" t="inlineStr">
+      <c r="C308" s="19" t="inlineStr">
         <is>
           <t>What is epigenetics and does it challenge our understanding of inheritance?</t>
         </is>
       </c>
-      <c r="D303" s="19" t="inlineStr">
+      <c r="D308" s="19" t="inlineStr">
         <is>
           <t>Heritable changes in gene expression without DNA sequence changes. Genome = instruction manual; epigenome = which instructions are read.
 **Mechanisms:**
@@ -8512,25 +8673,25 @@
 Does NOT validate Lamarck — mechanisms are different from direct inheritance of acquired characteristics.</t>
         </is>
       </c>
-      <c r="E303" s="18" t="n">
+      <c r="E308" s="18" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="304">
-      <c r="A304" s="14" t="n">
+    <row r="309">
+      <c r="A309" s="14" t="n">
         <v>436</v>
       </c>
-      <c r="B304" s="15" t="inlineStr">
+      <c r="B309" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C304" s="15" t="inlineStr">
+      <c r="C309" s="15" t="inlineStr">
         <is>
           <t>What is a prime number, and what do we know about their distribution?</t>
         </is>
       </c>
-      <c r="D304" s="15" t="inlineStr">
+      <c r="D309" s="15" t="inlineStr">
         <is>
           <t>A prime: natural number &gt; 1 with no divisors other than 1 and itself. Euclid (~300 BCE): infinitely many.
 Fundamental Theorem of Arithmetic: every integer &gt; 1 is prime or unique product of primes.
@@ -8542,25 +8703,25 @@
 **Practical importance**: RSA encryption relies on difficulty of factoring large numbers.</t>
         </is>
       </c>
-      <c r="E304" s="14" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" s="24" t="n">
+      <c r="E309" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="24" t="n">
         <v>437</v>
       </c>
-      <c r="B305" s="25" t="inlineStr">
+      <c r="B310" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C305" s="25" t="inlineStr">
+      <c r="C310" s="25" t="inlineStr">
         <is>
           <t>How reliable is eyewitness testimony, and what does the research say?</t>
         </is>
       </c>
-      <c r="D305" s="25" t="inlineStr">
+      <c r="D310" s="25" t="inlineStr">
         <is>
           <t>Memory is reconstructive, not reproductive (Loftus). We rebuild memories each time, subject to suggestion.
 **Key experiments:**
@@ -8571,25 +8732,25 @@
 **What helps**: sequential lineups, blind administration, record initial statement, open questions first.</t>
         </is>
       </c>
-      <c r="E305" s="24" t="n">
+      <c r="E310" s="24" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="306">
-      <c r="A306" s="6" t="n">
+    <row r="311">
+      <c r="A311" s="6" t="n">
         <v>438</v>
       </c>
-      <c r="B306" s="7" t="inlineStr">
+      <c r="B311" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C306" s="7" t="inlineStr">
+      <c r="C311" s="7" t="inlineStr">
         <is>
           <t>What is the difference between heat and temperature?</t>
         </is>
       </c>
-      <c r="D306" s="7" t="inlineStr">
+      <c r="D311" s="7" t="inlineStr">
         <is>
           <t>**Temperature**: average kinetic energy per molecule. Measured in Kelvin/Celsius/Fahrenheit.
 **Heat**: *transfer* of thermal energy between objects due to temperature difference. Heat is a process, not a property. Pool at same temperature as coffee mug: pool contains far more thermal energy.
@@ -8599,25 +8760,25 @@
 **Water vs air at 100C**: water burns much more — higher thermal mass + latent heat of condensation deliver more energy per contact.</t>
         </is>
       </c>
-      <c r="E306" s="6" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" s="2" t="n">
+      <c r="E311" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="n">
         <v>439</v>
       </c>
-      <c r="B307" s="3" t="inlineStr">
+      <c r="B312" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C307" s="3" t="inlineStr">
+      <c r="C312" s="3" t="inlineStr">
         <is>
           <t>What is structural racism, and how does it differ from individual racism?</t>
         </is>
       </c>
-      <c r="D307" s="3" t="inlineStr">
+      <c r="D312" s="3" t="inlineStr">
         <is>
           <t>**Individual racism**: prejudice and discriminatory acts by identifiable individuals. Overt bias.
 **Structural racism**: racial disparities from systems, policies, norms — even without individual racist intent.
@@ -8629,25 +8790,25 @@
 **Evidence**: audit studies (identical CVs with Black vs white names) consistently find measurable hiring discrimination.</t>
         </is>
       </c>
-      <c r="E307" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" s="26" t="n">
+      <c r="E312" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="26" t="n">
         <v>440</v>
       </c>
-      <c r="B308" s="27" t="inlineStr">
+      <c r="B313" s="27" t="inlineStr">
         <is>
           <t>Ecology</t>
         </is>
       </c>
-      <c r="C308" s="27" t="inlineStr">
+      <c r="C313" s="27" t="inlineStr">
         <is>
           <t>What is the nitrogen cycle and why is it essential for life?</t>
         </is>
       </c>
-      <c r="D308" s="27" t="inlineStr">
+      <c r="D313" s="27" t="inlineStr">
         <is>
           <t>N2 = 78% of atmosphere, but most organisms can't use N2 (triple bond N=N, 945 kJ/mol). Life needs reactive N (NH3, NO3-, organic N).
 **Nitrogen cycle:**
@@ -8659,25 +8820,25 @@
 **Limiting nutrient**: N limits most ecosystems. Excess (fertilisers) -&gt; eutrophication -&gt; algal blooms -&gt; oxygen depletion -&gt; dead zones (Gulf of Mexico). Haber also weaponised N (chlorine, phosgene).</t>
         </is>
       </c>
-      <c r="E308" s="26" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" s="30" t="n">
+      <c r="E313" s="26" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="30" t="n">
         <v>441</v>
       </c>
-      <c r="B309" s="31" t="inlineStr">
+      <c r="B314" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C309" s="31" t="inlineStr">
+      <c r="C314" s="31" t="inlineStr">
         <is>
           <t>What is antibiotic resistance and how does it develop?</t>
         </is>
       </c>
-      <c r="D309" s="31" t="inlineStr">
+      <c r="D314" s="31" t="inlineStr">
         <is>
           <t>Antibiotics target cell wall (penicillin), protein synthesis (tetracycline), DNA replication (fluoroquinolones), or membranes. Resistance = survival.
 **Darwinian mechanism:**
@@ -8691,25 +8852,25 @@
 **Why few new antibiotics**: 10-15yr development; brief low-cost use = poor financial incentive vs lifelong drugs.</t>
         </is>
       </c>
-      <c r="E309" s="30" t="n">
+      <c r="E314" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="310">
-      <c r="A310" s="12" t="n">
+    <row r="315">
+      <c r="A315" s="12" t="n">
         <v>442</v>
       </c>
-      <c r="B310" s="13" t="inlineStr">
+      <c r="B315" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C310" s="13" t="inlineStr">
+      <c r="C315" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the Magna Carta?</t>
         </is>
       </c>
-      <c r="D310" s="13" t="inlineStr">
+      <c r="D315" s="13" t="inlineStr">
         <is>
           <t>June 1215: English barons forced King John to sign. Originally limited royal power in narrow feudal ways — mostly barons' rights, not ordinary people.
 **Key clauses**: Cl. 39 — no free man imprisoned without lawful judgment of peers ('due process'); Cl. 40 — no selling/denying justice.
@@ -8719,25 +8880,25 @@
 **Lasting principle**: rule of law over arbitrary power -&gt; constitutional government, habeas corpus, human rights.</t>
         </is>
       </c>
-      <c r="E310" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" s="20" t="n">
+      <c r="E315" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="20" t="n">
         <v>443</v>
       </c>
-      <c r="B311" s="21" t="inlineStr">
+      <c r="B316" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C311" s="21" t="inlineStr">
+      <c r="C316" s="21" t="inlineStr">
         <is>
           <t>What is machine learning and how is it different from traditional programming?</t>
         </is>
       </c>
-      <c r="D311" s="21" t="inlineStr">
+      <c r="D316" s="21" t="inlineStr">
         <is>
           <t>**Traditional programming**: programmer writes explicit rules. Input + rules -&gt; output. Brittle; can't generalise.
 **Machine learning**: provide data + correct answers; algorithm finds the rules. Input + labels -&gt; model -&gt; generalises to new data.
@@ -8750,25 +8911,25 @@
 **Scale**: LLMs (GPT, Claude) = transformers on trillions of tokens; emergent capabilities at scale.</t>
         </is>
       </c>
-      <c r="E311" s="20" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" s="16" t="n">
+      <c r="E316" s="20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="16" t="n">
         <v>444</v>
       </c>
-      <c r="B312" s="17" t="inlineStr">
+      <c r="B317" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C312" s="17" t="inlineStr">
+      <c r="C317" s="17" t="inlineStr">
         <is>
           <t>What is the ship of Theseus paradox, and what is it really asking?</t>
         </is>
       </c>
-      <c r="D312" s="17" t="inlineStr">
+      <c r="D317" s="17" t="inlineStr">
         <is>
           <t>Plutarch (~100 CE): every plank of Theseus's ship replaced over time. Still the same ship?
 **Hobbes extension**: original planks collected and reassembled. Two ships claim to be the original. Which is it?
@@ -8782,25 +8943,25 @@
 **Parfit** (*Reasons and Persons*): personal identity is not what matters — psychological continuity is what matters; 'same' may be an empty question.</t>
         </is>
       </c>
-      <c r="E312" s="16" t="n">
+      <c r="E317" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="313">
-      <c r="A313" s="2" t="n">
+    <row r="318">
+      <c r="A318" s="2" t="n">
         <v>445</v>
       </c>
-      <c r="B313" s="3" t="inlineStr">
+      <c r="B318" s="3" t="inlineStr">
         <is>
           <t>Music</t>
         </is>
       </c>
-      <c r="C313" s="3" t="inlineStr">
+      <c r="C318" s="3" t="inlineStr">
         <is>
           <t>Why does music make us emotional?</t>
         </is>
       </c>
-      <c r="D313" s="3" t="inlineStr">
+      <c r="D318" s="3" t="inlineStr">
         <is>
           <t>Multiple converging mechanisms:
 1. **Expectation/violation** (Meyer 1956, Huron 2006): music is temporal prediction. Correct resolution = dopaminergic reward. Surprise + resolution = stronger reward. Chills = surprising resolution.
@@ -8812,25 +8973,25 @@
 **Mystery of sad music pleasure**: safe simulation, hormonal empathy reward, artistic resolution — distinct emotion from actual grief.</t>
         </is>
       </c>
-      <c r="E313" s="2" t="n">
+      <c r="E318" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="314">
-      <c r="A314" s="4" t="n">
+    <row r="319">
+      <c r="A319" s="4" t="n">
         <v>446</v>
       </c>
-      <c r="B314" s="5" t="inlineStr">
+      <c r="B319" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="C314" s="5" t="inlineStr">
+      <c r="C319" s="5" t="inlineStr">
         <is>
           <t>How do children acquire language so rapidly?</t>
         </is>
       </c>
-      <c r="D314" s="5" t="inlineStr">
+      <c r="D319" s="5" t="inlineStr">
         <is>
           <t>First words ~12 months, two-word phrases ~18-24 months, complex sentences by 3-4 years — from imperfect, fragmented input.
 **Poverty of the stimulus**: children overgeneralise rules ('goed', 'mouses') but never make wrong rule errors. Acquire structure-dependent rules without examples of errors.
@@ -8842,25 +9003,25 @@
 **Mechanisms**: statistical learning (8-month-olds track syllable transition probabilities), joint attention, motherese (simplified grammar + exaggerated prosody).</t>
         </is>
       </c>
-      <c r="E314" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" s="6" t="n">
+      <c r="E319" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="6" t="n">
         <v>447</v>
       </c>
-      <c r="B315" s="7" t="inlineStr">
+      <c r="B320" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C315" s="7" t="inlineStr">
+      <c r="C320" s="7" t="inlineStr">
         <is>
           <t>What is the photoelectric effect, and why did it matter for quantum mechanics?</t>
         </is>
       </c>
-      <c r="D315" s="7" t="inlineStr">
+      <c r="D320" s="7" t="inlineStr">
         <is>
           <t>Light hits metal -&gt; electrons ejected, BUT only above a threshold frequency. Below threshold: no electrons regardless of intensity.
 **Classical prediction**: intensity drives ejection. WRONG.
@@ -8873,25 +9034,25 @@
 4. Technology: photovoltaics, CCDs, photomultipliers</t>
         </is>
       </c>
-      <c r="E315" s="6" t="n">
+      <c r="E320" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="316">
-      <c r="A316" s="2" t="n">
+    <row r="321">
+      <c r="A321" s="2" t="n">
         <v>448</v>
       </c>
-      <c r="B316" s="3" t="inlineStr">
+      <c r="B321" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C316" s="3" t="inlineStr">
+      <c r="C321" s="3" t="inlineStr">
         <is>
           <t>What is social mobility and what actually predicts it?</t>
         </is>
       </c>
-      <c r="D316" s="3" t="inlineStr">
+      <c r="D321" s="3" t="inlineStr">
         <is>
           <t>Movement between socioeconomic strata. Intergenerational (parent to child) vs intragenerational (within lifetime).
 **Great Gatsby Curve** (Miles Corak): more income inequality -&gt; LOWER intergenerational mobility. Denmark (low inequality) = high mobility; US, UK = lower.
@@ -8904,25 +9065,25 @@
 Absolute mobility (exceeding parents in absolute terms) has historically been high; relative mobility much more constrained.</t>
         </is>
       </c>
-      <c r="E316" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" s="28" t="n">
+      <c r="E321" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="28" t="n">
         <v>449</v>
       </c>
-      <c r="B317" s="29" t="inlineStr">
+      <c r="B322" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C317" s="29" t="inlineStr">
+      <c r="C322" s="29" t="inlineStr">
         <is>
           <t>How do batteries work chemically, and what limits their energy density?</t>
         </is>
       </c>
-      <c r="D317" s="29" t="inlineStr">
+      <c r="D322" s="29" t="inlineStr">
         <is>
           <t>Battery = chemical -&gt; electrical energy via spatially separated redox reactions.
 Anode: oxidation (loses electrons). Cathode: reduction (gains electrons). Electrons flow externally (current); ions flow internally through electrolyte.
@@ -8939,25 +9100,25 @@
 **Theoretical limits**: Li-ion ~265 Wh/kg practical; Li-sulfur 2,600 Wh/kg; Li-air 11,680 Wh/kg (comparable to gasoline).</t>
         </is>
       </c>
-      <c r="E317" s="28" t="n">
+      <c r="E322" s="28" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="318">
-      <c r="A318" s="2" t="n">
+    <row r="323">
+      <c r="A323" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="B318" s="3" t="inlineStr">
+      <c r="B323" s="3" t="inlineStr">
         <is>
           <t>General Knowledge</t>
         </is>
       </c>
-      <c r="C318" s="3" t="inlineStr">
+      <c r="C323" s="3" t="inlineStr">
         <is>
           <t>What is the most important invention in human history, and why?</t>
         </is>
       </c>
-      <c r="D318" s="3" t="inlineStr">
+      <c r="D323" s="3" t="inlineStr">
         <is>
           <t>Depends on dimension valued. Four strong candidates:
 **Language**: meta-invention enabling all others to accumulate. But may have evolved rather than been invented.
@@ -8969,7 +9130,7 @@
 **Meta-point**: no invention stands alone. Cumulative innovation is humanity's real superpower.</t>
         </is>
       </c>
-      <c r="E318" s="2" t="n">
+      <c r="E323" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9094,14 +9255,14 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>9.619999999999999</v>
+        <v>9.57</v>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>158, 173, 219, 240, 259, 278, 292, 309, 357, 375, 389, 408, 431</t>
+          <t>158, 173, 219, 240, 259, 278, 292, 309, 357, 375, 389, 406, 408, 431</t>
         </is>
       </c>
     </row>
@@ -9202,14 +9363,14 @@
         </is>
       </c>
       <c r="B12" s="29" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C12" s="29" t="n">
-        <v>9.1</v>
+        <v>9.09</v>
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>212, 233, 245, 274, 334, 365, 391, 406, 424, 449</t>
+          <t>212, 233, 245, 274, 334, 365, 391, 406, 408, 424, 449</t>
         </is>
       </c>
     </row>
@@ -9292,14 +9453,14 @@
         </is>
       </c>
       <c r="B17" s="21" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C17" s="21" t="n">
-        <v>9.359999999999999</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="D17" s="21" t="inlineStr">
         <is>
-          <t>157, 184, 252, 258, 352, 377, 388, 398, 398, 428, 443</t>
+          <t>157, 184, 252, 258, 352, 377, 388, 398, 398, 409, 428, 443</t>
         </is>
       </c>
     </row>
@@ -9598,14 +9759,14 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C34" s="13" t="n">
-        <v>9.119999999999999</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 422, 433, 442</t>
+          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 422, 433, 442</t>
         </is>
       </c>
     </row>
@@ -10246,14 +10407,14 @@
         </is>
       </c>
       <c r="B70" s="25" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C70" s="25" t="n">
         <v>9.119999999999999</v>
       </c>
       <c r="D70" s="25" t="inlineStr">
         <is>
-          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 416, 432, 437</t>
+          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 432, 437</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q411-Q415 and update Excel export (327 entries)
Q411 Medicine: immune self/non-self — thymus, AIRE, Tregs
Q412 Physics: entropy and arrow of time
Q413 Sociology: social capital — Bourdieu vs Putnam
Q414 Mathematics: primes and RSA cryptography
Q415 Ecology: keystone species — Paine, wolves, sea otters

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E323"/>
+  <dimension ref="A1:E328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7927,20 +7927,46 @@
       </c>
     </row>
     <row r="285">
-      <c r="A285" s="14" t="n">
+      <c r="A285" s="30" t="n">
+        <v>411</v>
+      </c>
+      <c r="B285" s="31" t="inlineStr">
+        <is>
+          <t>Medicine</t>
+        </is>
+      </c>
+      <c r="C285" s="31" t="inlineStr">
+        <is>
+          <t>How does the immune system distinguish self from non-self?</t>
+        </is>
+      </c>
+      <c r="D285" s="31" t="inlineStr">
+        <is>
+          <t>Central tolerance (thymus education for T-cells): developing T-cells are shown every protein the body makes (AIRE gene). Those reacting too strongly to self are deleted (negative selection); those that can't recognise MHC are also deleted. Survivors react to MHC + foreign peptide only.
+Peripheral tolerance (backup): regulatory T-cells (Tregs) suppress escaped autoreactive cells; anergy (T-cell encounters antigen without co-stimulation = inactivated); ignorance (some self-antigens sequestered in eye, brain, testis).
+B-cells: receptor editing and clonal deletion in bone marrow.
+What breaks it: molecular mimicry (strep antigens mimic heart proteins -&gt; rheumatic fever); bystander activation; loss of Tregs; AIRE mutations (type 1 APS).</t>
+        </is>
+      </c>
+      <c r="E285" s="30" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="14" t="n">
         <v>412</v>
       </c>
-      <c r="B285" s="15" t="inlineStr">
+      <c r="B286" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C285" s="15" t="inlineStr">
+      <c r="C286" s="15" t="inlineStr">
         <is>
           <t>What is Godel's incompleteness theorem, in plain terms?</t>
         </is>
       </c>
-      <c r="D285" s="15" t="inlineStr">
+      <c r="D286" s="15" t="inlineStr">
         <is>
           <t>Godel (1931): one of the most astonishing results in intellectual history.
 **First theorem**: any consistent formal system powerful enough to describe arithmetic contains true statements that cannot be proved within that system.
@@ -7957,25 +7983,52 @@
 Closely related to Turing's undecidability.</t>
         </is>
       </c>
-      <c r="E285" s="14" t="n">
+      <c r="E286" s="14" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="286">
-      <c r="A286" s="2" t="n">
+    <row r="287">
+      <c r="A287" s="6" t="n">
+        <v>412</v>
+      </c>
+      <c r="B287" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="C287" s="7" t="inlineStr">
+        <is>
+          <t>What is entropy and why does it always increase?</t>
+        </is>
+      </c>
+      <c r="D287" s="7" t="inlineStr">
+        <is>
+          <t>Entropy measures microstates consistent with an observed macrostate. Boltzmann: S = k_B * ln(Omega). More disorder = more arrangements = higher entropy.
+Why it increases: universe starts in extreme low-entropy state (Big Bang). Any spontaneous change overwhelmingly tends toward higher entropy because there are vastly more disordered configurations. It's statistical — individual particle collisions are time-reversible, but with ~10^80 particles, spontaneous order is effectively impossible.
+Examples: heat flows hot to cold; ice melts (liquid has more positional microstates); gas expands.
+Maxwell's Demon: a sorting demon could decrease entropy but must erase memory, which generates entropy (Landauer's principle).
+Arrow of time: entropy increase is why past and future feel different. Fundamental physics is (nearly) time-symmetric; time's direction emerges from entropy.</t>
+        </is>
+      </c>
+      <c r="E287" s="6" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="n">
         <v>413</v>
       </c>
-      <c r="B286" s="3" t="inlineStr">
+      <c r="B288" s="3" t="inlineStr">
         <is>
           <t>Environmental Science</t>
         </is>
       </c>
-      <c r="C286" s="3" t="inlineStr">
+      <c r="C288" s="3" t="inlineStr">
         <is>
           <t>What is the greenhouse effect, and how does it work physically?</t>
         </is>
       </c>
-      <c r="D286" s="3" t="inlineStr">
+      <c r="D288" s="3" t="inlineStr">
         <is>
           <t>Natural and necessary — without it, Earth would be -18C not +15C. Problem is the *enhanced* effect from human emissions.
 **Mechanism:**
@@ -7990,25 +8043,52 @@
 - Cloud feedbacks: complex, main uncertainty in climate sensitivity</t>
         </is>
       </c>
-      <c r="E286" s="2" t="n">
+      <c r="E288" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="287">
-      <c r="A287" s="2" t="n">
+    <row r="289">
+      <c r="A289" s="2" t="n">
+        <v>413</v>
+      </c>
+      <c r="B289" s="3" t="inlineStr">
+        <is>
+          <t>Sociology</t>
+        </is>
+      </c>
+      <c r="C289" s="3" t="inlineStr">
+        <is>
+          <t>What is social capital and why does it matter?</t>
+        </is>
+      </c>
+      <c r="D289" s="3" t="inlineStr">
+        <is>
+          <t>Social capital: networks, norms of reciprocity, and trust enabling collective action and individual advantage.
+Two traditions: Bourdieu (individual resource — who you know gates opportunities; class reproduction); Putnam (collective resource — Bowling Alone 2000: declining civic participation correlates with declining trust, health, governance).
+Bridging vs bonding (Putnam): bonding = within-group ties (support but exclusion); bridging = cross-group ties (new info, mobility, cohesion).
+Why it matters: health (social isolation = 15 cigarettes/day, Holt-Lunstad); economic mobility (who-you-know &gt; qualifications); democracy (Putnam's Italian regions: civic traditions predict governance centuries later); crime reduction.
+Dark side: bonding capital -&gt; tribalism, mafia-style networks.</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="n">
         <v>414</v>
       </c>
-      <c r="B287" s="3" t="inlineStr">
+      <c r="B290" s="3" t="inlineStr">
         <is>
           <t>Music Theory</t>
         </is>
       </c>
-      <c r="C287" s="3" t="inlineStr">
+      <c r="C290" s="3" t="inlineStr">
         <is>
           <t>Why do some musical intervals sound consonant and others dissonant?</t>
         </is>
       </c>
-      <c r="D287" s="3" t="inlineStr">
+      <c r="D290" s="3" t="inlineStr">
         <is>
           <t>Multiple overlapping explanations:
 1. **Frequency ratios** (Pythagoras): simple integer ratios sound consonant. Octave=2:1, fifth=3:2, fourth=4:3. Complex ratios (tritone ~45:32) sound tense.
@@ -8019,25 +8099,56 @@
 **Why music uses dissonance**: pure consonance is boring. Tension-resolution is the engine of musical emotion.</t>
         </is>
       </c>
-      <c r="E287" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" s="2" t="n">
+      <c r="E290" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="14" t="n">
+        <v>414</v>
+      </c>
+      <c r="B291" s="15" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="C291" s="15" t="inlineStr">
+        <is>
+          <t>What is a prime number and why are they important in cryptography?</t>
+        </is>
+      </c>
+      <c r="D291" s="15" t="inlineStr">
+        <is>
+          <t>A prime is a natural number &gt; 1 with no divisors other than 1 and itself.
+Key facts: infinitely many primes (Euclid ~300 BCE); Prime Number Theorem (density near n ~ 1/ln(n)); unique prime factorisation (Fundamental Theorem of Arithmetic).
+Why cryptography depends on them — RSA (1977, Rivest Shamir Adleman):
+1. Choose two large primes p, q (~2048 bits each)
+2. Public key: n = p*q (trivial to compute)
+3. Private key: derived from p and q separately
+Trap: factoring a 2048-bit number is computationally infeasible — best algorithms take longer than age of universe.
+ECC: more modern alternative with smaller keys.
+Threat: Shor's algorithm on quantum computers factors in polynomial time — drives post-quantum cryptography research.</t>
+        </is>
+      </c>
+      <c r="E291" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="n">
         <v>415</v>
       </c>
-      <c r="B288" s="3" t="inlineStr">
+      <c r="B292" s="3" t="inlineStr">
         <is>
           <t>Political Science</t>
         </is>
       </c>
-      <c r="C288" s="3" t="inlineStr">
+      <c r="C292" s="3" t="inlineStr">
         <is>
           <t>What is the difference between a democracy and a republic, and does the distinction matter?</t>
         </is>
       </c>
-      <c r="D288" s="3" t="inlineStr">
+      <c r="D292" s="3" t="inlineStr">
         <is>
           <t>**Democracy**: rule by the people. Pure direct democracy — citizens vote on every law. Athens: male citizens voted directly. Impossible at scale.
 **Republic** (res publica): power held by elected representatives, not exercised directly. Citizens choose who decides, not what is decided.
@@ -8047,25 +8158,55 @@
 **Other**: constitutional republic (limits on power), parliamentary vs presidential republic.</t>
         </is>
       </c>
-      <c r="E288" s="2" t="n">
+      <c r="E292" s="2" t="n">
         <v>8.5</v>
       </c>
     </row>
-    <row r="289">
-      <c r="A289" s="24" t="n">
+    <row r="293">
+      <c r="A293" s="26" t="n">
+        <v>415</v>
+      </c>
+      <c r="B293" s="27" t="inlineStr">
+        <is>
+          <t>Ecology</t>
+        </is>
+      </c>
+      <c r="C293" s="27" t="inlineStr">
+        <is>
+          <t>What is the concept of a keystone species?</t>
+        </is>
+      </c>
+      <c r="D293" s="27" t="inlineStr">
+        <is>
+          <t>A keystone species has disproportionately large ecological effect relative to its biomass. Remove it and the ecosystem collapses.
+Origin: Paine (1966) removed sea stars from intertidal zone. Mussels exploded, crowded out all others — 15 species to mussel monoculture.
+Examples:
+- Sea otters: eat urchins; without otters, urchins destroy kelp forests -&gt; lose hundreds of dependent species
+- African elephants: create waterholes, disperse seeds, clear bush; remove them -&gt; savannah converts to closed woodland
+- Wolves in Yellowstone (reintroduced 1995): reduced elk overgrazing -&gt; rivers recovered -&gt; beavers returned -&gt; fish/bird habitat restored (trophic cascade)
+- Fig trees: year-round fruit supports dozens of species during lean seasons
+Policy: losing 0.1% of biomass (sea star) can mean losing 90% of diversity. Conservation must identify keystone species, not just total biomass.</t>
+        </is>
+      </c>
+      <c r="E293" s="26" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="24" t="n">
         <v>416</v>
       </c>
-      <c r="B289" s="25" t="inlineStr">
+      <c r="B294" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C289" s="25" t="inlineStr">
+      <c r="C294" s="25" t="inlineStr">
         <is>
           <t>What is the bystander effect, and when does it NOT apply?</t>
         </is>
       </c>
-      <c r="D289" s="25" t="inlineStr">
+      <c r="D294" s="25" t="inlineStr">
         <is>
           <t>Kitty Genovese (1964) led to Latane and Darley's research. Two mechanisms:
 1. Diffusion of responsibility: each bystander assumes someone else will act
@@ -8080,25 +8221,25 @@
 **Genovese myth**: Fischer et al. 2011 — 38 witnesses story exaggerated by NYT. Many didn't hear/see clearly. Effect is real, original story was sensationalised.</t>
         </is>
       </c>
-      <c r="E289" s="24" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" s="2" t="n">
+      <c r="E294" s="24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="n">
         <v>417</v>
       </c>
-      <c r="B290" s="3" t="inlineStr">
+      <c r="B295" s="3" t="inlineStr">
         <is>
           <t>Geology</t>
         </is>
       </c>
-      <c r="C290" s="3" t="inlineStr">
+      <c r="C295" s="3" t="inlineStr">
         <is>
           <t>How do plate tectonics work, and what drives the plates?</t>
         </is>
       </c>
-      <c r="D290" s="3" t="inlineStr">
+      <c r="D295" s="3" t="inlineStr">
         <is>
           <t>~15 major lithospheric plates (100km thick) float on viscous asthenosphere, moving 2-10 cm/year.
 **Three boundary types:**
@@ -8112,25 +8253,25 @@
 **Evidence**: magnetic striping on seafloor, continental fit (Wegener), matching fossils, earthquake distributions.</t>
         </is>
       </c>
-      <c r="E290" s="2" t="n">
+      <c r="E295" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="291">
-      <c r="A291" s="14" t="n">
+    <row r="296">
+      <c r="A296" s="14" t="n">
         <v>418</v>
       </c>
-      <c r="B291" s="15" t="inlineStr">
+      <c r="B296" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C291" s="15" t="inlineStr">
+      <c r="C296" s="15" t="inlineStr">
         <is>
           <t>What is a Fourier transform, and why is it everywhere?</t>
         </is>
       </c>
-      <c r="D291" s="15" t="inlineStr">
+      <c r="D296" s="15" t="inlineStr">
         <is>
           <t>Fourier (1822): any periodic function decomposes into sines and cosines of different frequencies.
 Fourier transform: takes time-domain signal f(t) -&gt; frequency-domain F(w) showing how much of each frequency is present.
@@ -8145,25 +8286,25 @@
 **FFT** (Cooley-Tukey 1965): O(n log n) vs O(n^2) naive. Made real-time signal processing possible.</t>
         </is>
       </c>
-      <c r="E291" s="14" t="n">
+      <c r="E296" s="14" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="292">
-      <c r="A292" s="2" t="n">
+    <row r="297">
+      <c r="A297" s="2" t="n">
         <v>419</v>
       </c>
-      <c r="B292" s="3" t="inlineStr">
+      <c r="B297" s="3" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
       </c>
-      <c r="C292" s="3" t="inlineStr">
+      <c r="C297" s="3" t="inlineStr">
         <is>
           <t>What is the difference between deontological and consequentialist ethics, and which is right?</t>
         </is>
       </c>
-      <c r="D292" s="3" t="inlineStr">
+      <c r="D297" s="3" t="inlineStr">
         <is>
           <t>**Consequentialism** (Bentham, Mill): moral worth from consequences. Maximise utility/welfare. Strength: outcome-focused. Weakness: justifies organ harvesting one person to save five; ignores rights.
 **Deontology** (Kant): moral worth from the action itself, not consequences. Categorical Imperative:
@@ -8178,25 +8319,25 @@
 Reflective equilibrium: use multiple frameworks as lenses, check coherence with intuitions.</t>
         </is>
       </c>
-      <c r="E292" s="2" t="n">
+      <c r="E297" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="293">
-      <c r="A293" s="4" t="n">
+    <row r="298">
+      <c r="A298" s="4" t="n">
         <v>420</v>
       </c>
-      <c r="B293" s="5" t="inlineStr">
+      <c r="B298" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="C293" s="5" t="inlineStr">
+      <c r="C298" s="5" t="inlineStr">
         <is>
           <t>What is the difference between descriptive and prescriptive grammar, and why does it matter?</t>
         </is>
       </c>
-      <c r="D293" s="5" t="inlineStr">
+      <c r="D298" s="5" t="inlineStr">
         <is>
           <t>**Prescriptive**: what people *should* say — textbooks, style guides, norms ('don't split infinitives', 'it is I').
 **Descriptive**: what people *actually* say — linguist's approach. Records patterns without judging. Every human language has consistent grammar; no language is 'wrong.'
@@ -8208,25 +8349,25 @@
 5. Code-switching: competent speakers deploy both — AAVE at home, SAE formally. Both correct for their domains.</t>
         </is>
       </c>
-      <c r="E293" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" s="18" t="n">
+      <c r="E298" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="18" t="n">
         <v>421</v>
       </c>
-      <c r="B294" s="19" t="inlineStr">
+      <c r="B299" s="19" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C294" s="19" t="inlineStr">
+      <c r="C299" s="19" t="inlineStr">
         <is>
           <t>How does the immune system distinguish 'self' from 'non-self'?</t>
         </is>
       </c>
-      <c r="D294" s="19" t="inlineStr">
+      <c r="D299" s="19" t="inlineStr">
         <is>
           <t>Multiple overlapping mechanisms:
 **MHC class I**: every nucleated cell displays own protein fragments on MHC class I. T-cells educated in thymus to tolerate self-peptides; cells displaying foreign peptides (viral, tumour) are destroyed.
@@ -8238,25 +8379,25 @@
 - Transplant rejection: donor MHC recognised as foreign</t>
         </is>
       </c>
-      <c r="E294" s="18" t="n">
+      <c r="E299" s="18" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="295">
-      <c r="A295" s="12" t="n">
+    <row r="300">
+      <c r="A300" s="12" t="n">
         <v>422</v>
       </c>
-      <c r="B295" s="13" t="inlineStr">
+      <c r="B300" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C295" s="13" t="inlineStr">
+      <c r="C300" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the printing press, and did Gutenberg invent it?</t>
         </is>
       </c>
-      <c r="D295" s="13" t="inlineStr">
+      <c r="D300" s="13" t="inlineStr">
         <is>
           <t>Gutenberg (~1450) didn't invent printing. Moveable type existed in China (Bi Sheng ~1040) and Korea (Jikji 1377, oldest surviving). Gutenberg's innovation: complete system — durable metal alloy type, oil-based ink, adapted screw press — optimised for the European alphabet.
 **Why it transformed Europe**: Latin alphabet (26 letters) made moveable type far more efficient than Chinese/Korean systems (thousands of characters). Press: ~3,600 pages/day vs 40 for a scribe.
@@ -8269,25 +8410,25 @@
 **Eisenstein's thesis**: press created new relationship with knowledge — standardisation, reproducibility, verification.</t>
         </is>
       </c>
-      <c r="E295" s="12" t="n">
+      <c r="E300" s="12" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="296">
-      <c r="A296" s="10" t="n">
+    <row r="301">
+      <c r="A301" s="10" t="n">
         <v>423</v>
       </c>
-      <c r="B296" s="11" t="inlineStr">
+      <c r="B301" s="11" t="inlineStr">
         <is>
           <t>Neuroscience</t>
         </is>
       </c>
-      <c r="C296" s="11" t="inlineStr">
+      <c r="C301" s="11" t="inlineStr">
         <is>
           <t>What is consciousness and why is it so hard to explain?</t>
         </is>
       </c>
-      <c r="D296" s="11" t="inlineStr">
+      <c r="D301" s="11" t="inlineStr">
         <is>
           <t>Chalmers (1995) 'hard problem': why does information processing produce *subjective experience*? Why is there something it is like to see red?
 Even full neural mapping of correlates wouldn't explain why any of it feels like anything. Explaining function doesn't explain qualia.
@@ -8300,25 +8441,25 @@
 **Consensus**: none. Hard problem remains genuinely open.</t>
         </is>
       </c>
-      <c r="E296" s="10" t="n">
+      <c r="E301" s="10" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="297">
-      <c r="A297" s="28" t="n">
+    <row r="302">
+      <c r="A302" s="28" t="n">
         <v>424</v>
       </c>
-      <c r="B297" s="29" t="inlineStr">
+      <c r="B302" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C297" s="29" t="inlineStr">
+      <c r="C302" s="29" t="inlineStr">
         <is>
           <t>What makes some molecules smell while others don't?</t>
         </is>
       </c>
-      <c r="D297" s="29" t="inlineStr">
+      <c r="D302" s="29" t="inlineStr">
         <is>
           <t>Odorant molecules bind to olfactory receptors (ORs, GPCRs) in nasal epithelium -&gt; olfactory bulb -&gt; piriform cortex + limbic system.
 **What molecules smell:**
@@ -8330,25 +8471,25 @@
 **COVID-19 anosmia**: virus destroys olfactory neuron support cells; usually recovers.</t>
         </is>
       </c>
-      <c r="E297" s="28" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" s="8" t="n">
+      <c r="E302" s="28" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="8" t="n">
         <v>425</v>
       </c>
-      <c r="B298" s="9" t="inlineStr">
+      <c r="B303" s="9" t="inlineStr">
         <is>
           <t>Economics</t>
         </is>
       </c>
-      <c r="C298" s="9" t="inlineStr">
+      <c r="C303" s="9" t="inlineStr">
         <is>
           <t>What caused the 2008 financial crisis?</t>
         </is>
       </c>
-      <c r="D298" s="9" t="inlineStr">
+      <c r="D303" s="9" t="inlineStr">
         <is>
           <t>Cascade of failures:
 **Housing bubble**: low post-9/11 rates, relaxed lending, NINJA loans (no income/assets/job). Prices +124% nationally 2000-2006.
@@ -8360,25 +8501,25 @@
 **Response**: Dodd-Frank, Basel III capital requirements, Volcker Rule.</t>
         </is>
       </c>
-      <c r="E298" s="8" t="n">
+      <c r="E303" s="8" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="299">
-      <c r="A299" s="6" t="n">
+    <row r="304">
+      <c r="A304" s="6" t="n">
         <v>426</v>
       </c>
-      <c r="B299" s="7" t="inlineStr">
+      <c r="B304" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C299" s="7" t="inlineStr">
+      <c r="C304" s="7" t="inlineStr">
         <is>
           <t>What is dark matter and how do we know it exists?</t>
         </is>
       </c>
-      <c r="D299" s="7" t="inlineStr">
+      <c r="D304" s="7" t="inlineStr">
         <is>
           <t>~27% of universe's energy. Doesn't emit/absorb/reflect light. Gravitational effects overwhelming.
 **Evidence:**
@@ -8390,25 +8531,25 @@
 **MOND alternative**: modified Newtonian dynamics; cannot explain Bullet Cluster + CMB simultaneously. Most physicists favour particle dark matter.</t>
         </is>
       </c>
-      <c r="E299" s="6" t="n">
+      <c r="E304" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="300">
-      <c r="A300" s="2" t="n">
+    <row r="305">
+      <c r="A305" s="2" t="n">
         <v>427</v>
       </c>
-      <c r="B300" s="3" t="inlineStr">
+      <c r="B305" s="3" t="inlineStr">
         <is>
           <t>Literature</t>
         </is>
       </c>
-      <c r="C300" s="3" t="inlineStr">
+      <c r="C305" s="3" t="inlineStr">
         <is>
           <t>Why is 'Don Quixote' considered the first modern novel?</t>
         </is>
       </c>
-      <c r="D300" s="3" t="inlineStr">
+      <c r="D305" s="3" t="inlineStr">
         <is>
           <t>Cervantes (Part I: 1605, Part II: 1615). Why it's considered the first modern novel:
 1. Self-consciousness: the novel is aware it's a novel. Part II characters have read Part I. Unreliable narrators, manuscript frames — postmodern devices 400 years early.
@@ -8419,25 +8560,25 @@
 What makes it 'modern': fundamentally ambiguous relationship with truth; character who changes across time (Part I vs II Quixote). Bloom: 'most universal and most particular character in literature.'</t>
         </is>
       </c>
-      <c r="E300" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" s="20" t="n">
+      <c r="E305" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="20" t="n">
         <v>428</v>
       </c>
-      <c r="B301" s="21" t="inlineStr">
+      <c r="B306" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C301" s="21" t="inlineStr">
+      <c r="C306" s="21" t="inlineStr">
         <is>
           <t>What is the halting problem and why does it matter?</t>
         </is>
       </c>
-      <c r="D301" s="21" t="inlineStr">
+      <c r="D306" s="21" t="inlineStr">
         <is>
           <t>Turing (1936): no general algorithm can determine whether an arbitrary program will halt or run forever.
 **Proof (diagonal argument)**: assume HALT(P,I) exists. Construct DIAG(P): if HALT says P halts on P -&gt; loop; if HALT says P loops -&gt; halt.
@@ -8450,25 +8591,25 @@
 5. Practical: compilers and static analysers must be incomplete or unsound — they make heuristic approximations.</t>
         </is>
       </c>
-      <c r="E301" s="20" t="n">
+      <c r="E306" s="20" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="302">
-      <c r="A302" s="30" t="n">
+    <row r="307">
+      <c r="A307" s="30" t="n">
         <v>429</v>
       </c>
-      <c r="B302" s="31" t="inlineStr">
+      <c r="B307" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C302" s="31" t="inlineStr">
+      <c r="C307" s="31" t="inlineStr">
         <is>
           <t>How do vaccines work, and why do some require boosters?</t>
         </is>
       </c>
-      <c r="D302" s="31" t="inlineStr">
+      <c r="D307" s="31" t="inlineStr">
         <is>
           <t>Vaccine presents antigen (weakened/killed pathogen, subunit protein, or mRNA) without disease, training immune memory.
 **Mechanism:**
@@ -8485,25 +8626,25 @@
 **Why boosters**: antibody titres wane (inactivated/subunit weaker); mutating viruses (flu) change antigens.</t>
         </is>
       </c>
-      <c r="E302" s="30" t="n">
+      <c r="E307" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="303">
-      <c r="A303" s="16" t="n">
+    <row r="308">
+      <c r="A308" s="16" t="n">
         <v>430</v>
       </c>
-      <c r="B303" s="17" t="inlineStr">
+      <c r="B308" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C303" s="17" t="inlineStr">
+      <c r="C308" s="17" t="inlineStr">
         <is>
           <t>What is free will, and does science undermine it?</t>
         </is>
       </c>
-      <c r="D303" s="17" t="inlineStr">
+      <c r="D308" s="17" t="inlineStr">
         <is>
           <t>Are our choices genuinely ours, or determined by prior causes?
 **Three positions:**
@@ -8515,25 +8656,25 @@
 **Does science undermine it?** Depends what you mean. Compatibilist free will survives. Hard determinism mostly fringe.</t>
         </is>
       </c>
-      <c r="E303" s="16" t="n">
+      <c r="E308" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="304">
-      <c r="A304" s="22" t="n">
+    <row r="309">
+      <c r="A309" s="22" t="n">
         <v>431</v>
       </c>
-      <c r="B304" s="23" t="inlineStr">
+      <c r="B309" s="23" t="inlineStr">
         <is>
           <t>Astronomy</t>
         </is>
       </c>
-      <c r="C304" s="23" t="inlineStr">
+      <c r="C309" s="23" t="inlineStr">
         <is>
           <t>What are neutron stars and how do they form?</t>
         </is>
       </c>
-      <c r="D304" s="23" t="inlineStr">
+      <c r="D309" s="23" t="inlineStr">
         <is>
           <t>Massive star (8-20 solar masses) core collapses. If core mass 1.4-3 solar masses, electron degeneracy fails. Protons + electrons merge (inverse beta decay) -&gt; neutron star.
 **Properties:**
@@ -8546,25 +8687,25 @@
 **Neutron star mergers (GW170817, 2017)**: first gravitational wave + electromagnetic detection. Kilonova: r-process nucleosynthesis produces gold, platinum, uranium. Primary source of heavy elements.</t>
         </is>
       </c>
-      <c r="E304" s="22" t="n">
+      <c r="E309" s="22" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="305">
-      <c r="A305" s="24" t="n">
+    <row r="310">
+      <c r="A310" s="24" t="n">
         <v>432</v>
       </c>
-      <c r="B305" s="25" t="inlineStr">
+      <c r="B310" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C305" s="25" t="inlineStr">
+      <c r="C310" s="25" t="inlineStr">
         <is>
           <t>What is the Dunning-Kruger effect, and is it as universal as people think?</t>
         </is>
       </c>
-      <c r="D305" s="25" t="inlineStr">
+      <c r="D310" s="25" t="inlineStr">
         <is>
           <t>Kruger &amp; Dunning (1999): people with limited knowledge overestimate competence; experts underestimate relative ability (task seems easy to them too).
 **Original study**: bottom quartile performers on logic/grammar/humour overestimated by ~50 percentile points.
@@ -8578,25 +8719,25 @@
 - Domain-specific: expert engineer may still have DK in social skills</t>
         </is>
       </c>
-      <c r="E305" s="24" t="n">
+      <c r="E310" s="24" t="n">
         <v>8.5</v>
       </c>
     </row>
-    <row r="306">
-      <c r="A306" s="12" t="n">
+    <row r="311">
+      <c r="A311" s="12" t="n">
         <v>433</v>
       </c>
-      <c r="B306" s="13" t="inlineStr">
+      <c r="B311" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C306" s="13" t="inlineStr">
+      <c r="C311" s="13" t="inlineStr">
         <is>
           <t>Why did the Roman Empire fall?</t>
         </is>
       </c>
-      <c r="D306" s="13" t="inlineStr">
+      <c r="D311" s="13" t="inlineStr">
         <is>
           <t>Western Empire fell 476 CE (Romulus Augustulus deposed). Eastern Empire (Byzantium) lasted to 1453. No single cause:
 **Military/political:** overextended borders; Germanic foederati with divided loyalty; political instability (50 emperors in 50 years, 235-284 CE); military power to make/unmake emperors.
@@ -8609,25 +8750,25 @@
 **What didn't fall**: Eastern Empire thrived. Fall was primarily western.</t>
         </is>
       </c>
-      <c r="E306" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" s="2" t="n">
+      <c r="E311" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="n">
         <v>434</v>
       </c>
-      <c r="B307" s="3" t="inlineStr">
+      <c r="B312" s="3" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C307" s="3" t="inlineStr">
+      <c r="C312" s="3" t="inlineStr">
         <is>
           <t>How does GPS actually work?</t>
         </is>
       </c>
-      <c r="D307" s="3" t="inlineStr">
+      <c r="D312" s="3" t="inlineStr">
         <is>
           <t>24-32 satellites at ~20,200km; 6 orbital planes; each completes 2 orbits/day.
 **Core principle: trilateration via time signals.**
@@ -8643,25 +8784,25 @@
 - Net: +38 microseconds/day. Without correction: GPS drifts ~10km/day. Einstein's corrections are in the system.</t>
         </is>
       </c>
-      <c r="E307" s="2" t="n">
+      <c r="E312" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="308">
-      <c r="A308" s="18" t="n">
+    <row r="313">
+      <c r="A313" s="18" t="n">
         <v>435</v>
       </c>
-      <c r="B308" s="19" t="inlineStr">
+      <c r="B313" s="19" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C308" s="19" t="inlineStr">
+      <c r="C313" s="19" t="inlineStr">
         <is>
           <t>What is epigenetics and does it challenge our understanding of inheritance?</t>
         </is>
       </c>
-      <c r="D308" s="19" t="inlineStr">
+      <c r="D313" s="19" t="inlineStr">
         <is>
           <t>Heritable changes in gene expression without DNA sequence changes. Genome = instruction manual; epigenome = which instructions are read.
 **Mechanisms:**
@@ -8673,25 +8814,25 @@
 Does NOT validate Lamarck — mechanisms are different from direct inheritance of acquired characteristics.</t>
         </is>
       </c>
-      <c r="E308" s="18" t="n">
+      <c r="E313" s="18" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="309">
-      <c r="A309" s="14" t="n">
+    <row r="314">
+      <c r="A314" s="14" t="n">
         <v>436</v>
       </c>
-      <c r="B309" s="15" t="inlineStr">
+      <c r="B314" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C309" s="15" t="inlineStr">
+      <c r="C314" s="15" t="inlineStr">
         <is>
           <t>What is a prime number, and what do we know about their distribution?</t>
         </is>
       </c>
-      <c r="D309" s="15" t="inlineStr">
+      <c r="D314" s="15" t="inlineStr">
         <is>
           <t>A prime: natural number &gt; 1 with no divisors other than 1 and itself. Euclid (~300 BCE): infinitely many.
 Fundamental Theorem of Arithmetic: every integer &gt; 1 is prime or unique product of primes.
@@ -8703,25 +8844,25 @@
 **Practical importance**: RSA encryption relies on difficulty of factoring large numbers.</t>
         </is>
       </c>
-      <c r="E309" s="14" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" s="24" t="n">
+      <c r="E314" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="24" t="n">
         <v>437</v>
       </c>
-      <c r="B310" s="25" t="inlineStr">
+      <c r="B315" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C310" s="25" t="inlineStr">
+      <c r="C315" s="25" t="inlineStr">
         <is>
           <t>How reliable is eyewitness testimony, and what does the research say?</t>
         </is>
       </c>
-      <c r="D310" s="25" t="inlineStr">
+      <c r="D315" s="25" t="inlineStr">
         <is>
           <t>Memory is reconstructive, not reproductive (Loftus). We rebuild memories each time, subject to suggestion.
 **Key experiments:**
@@ -8732,25 +8873,25 @@
 **What helps**: sequential lineups, blind administration, record initial statement, open questions first.</t>
         </is>
       </c>
-      <c r="E310" s="24" t="n">
+      <c r="E315" s="24" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="311">
-      <c r="A311" s="6" t="n">
+    <row r="316">
+      <c r="A316" s="6" t="n">
         <v>438</v>
       </c>
-      <c r="B311" s="7" t="inlineStr">
+      <c r="B316" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C311" s="7" t="inlineStr">
+      <c r="C316" s="7" t="inlineStr">
         <is>
           <t>What is the difference between heat and temperature?</t>
         </is>
       </c>
-      <c r="D311" s="7" t="inlineStr">
+      <c r="D316" s="7" t="inlineStr">
         <is>
           <t>**Temperature**: average kinetic energy per molecule. Measured in Kelvin/Celsius/Fahrenheit.
 **Heat**: *transfer* of thermal energy between objects due to temperature difference. Heat is a process, not a property. Pool at same temperature as coffee mug: pool contains far more thermal energy.
@@ -8760,25 +8901,25 @@
 **Water vs air at 100C**: water burns much more — higher thermal mass + latent heat of condensation deliver more energy per contact.</t>
         </is>
       </c>
-      <c r="E311" s="6" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" s="2" t="n">
+      <c r="E316" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="n">
         <v>439</v>
       </c>
-      <c r="B312" s="3" t="inlineStr">
+      <c r="B317" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C312" s="3" t="inlineStr">
+      <c r="C317" s="3" t="inlineStr">
         <is>
           <t>What is structural racism, and how does it differ from individual racism?</t>
         </is>
       </c>
-      <c r="D312" s="3" t="inlineStr">
+      <c r="D317" s="3" t="inlineStr">
         <is>
           <t>**Individual racism**: prejudice and discriminatory acts by identifiable individuals. Overt bias.
 **Structural racism**: racial disparities from systems, policies, norms — even without individual racist intent.
@@ -8790,25 +8931,25 @@
 **Evidence**: audit studies (identical CVs with Black vs white names) consistently find measurable hiring discrimination.</t>
         </is>
       </c>
-      <c r="E312" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" s="26" t="n">
+      <c r="E317" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="26" t="n">
         <v>440</v>
       </c>
-      <c r="B313" s="27" t="inlineStr">
+      <c r="B318" s="27" t="inlineStr">
         <is>
           <t>Ecology</t>
         </is>
       </c>
-      <c r="C313" s="27" t="inlineStr">
+      <c r="C318" s="27" t="inlineStr">
         <is>
           <t>What is the nitrogen cycle and why is it essential for life?</t>
         </is>
       </c>
-      <c r="D313" s="27" t="inlineStr">
+      <c r="D318" s="27" t="inlineStr">
         <is>
           <t>N2 = 78% of atmosphere, but most organisms can't use N2 (triple bond N=N, 945 kJ/mol). Life needs reactive N (NH3, NO3-, organic N).
 **Nitrogen cycle:**
@@ -8820,25 +8961,25 @@
 **Limiting nutrient**: N limits most ecosystems. Excess (fertilisers) -&gt; eutrophication -&gt; algal blooms -&gt; oxygen depletion -&gt; dead zones (Gulf of Mexico). Haber also weaponised N (chlorine, phosgene).</t>
         </is>
       </c>
-      <c r="E313" s="26" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" s="30" t="n">
+      <c r="E318" s="26" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="30" t="n">
         <v>441</v>
       </c>
-      <c r="B314" s="31" t="inlineStr">
+      <c r="B319" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C314" s="31" t="inlineStr">
+      <c r="C319" s="31" t="inlineStr">
         <is>
           <t>What is antibiotic resistance and how does it develop?</t>
         </is>
       </c>
-      <c r="D314" s="31" t="inlineStr">
+      <c r="D319" s="31" t="inlineStr">
         <is>
           <t>Antibiotics target cell wall (penicillin), protein synthesis (tetracycline), DNA replication (fluoroquinolones), or membranes. Resistance = survival.
 **Darwinian mechanism:**
@@ -8852,25 +8993,25 @@
 **Why few new antibiotics**: 10-15yr development; brief low-cost use = poor financial incentive vs lifelong drugs.</t>
         </is>
       </c>
-      <c r="E314" s="30" t="n">
+      <c r="E319" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="315">
-      <c r="A315" s="12" t="n">
+    <row r="320">
+      <c r="A320" s="12" t="n">
         <v>442</v>
       </c>
-      <c r="B315" s="13" t="inlineStr">
+      <c r="B320" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C315" s="13" t="inlineStr">
+      <c r="C320" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the Magna Carta?</t>
         </is>
       </c>
-      <c r="D315" s="13" t="inlineStr">
+      <c r="D320" s="13" t="inlineStr">
         <is>
           <t>June 1215: English barons forced King John to sign. Originally limited royal power in narrow feudal ways — mostly barons' rights, not ordinary people.
 **Key clauses**: Cl. 39 — no free man imprisoned without lawful judgment of peers ('due process'); Cl. 40 — no selling/denying justice.
@@ -8880,25 +9021,25 @@
 **Lasting principle**: rule of law over arbitrary power -&gt; constitutional government, habeas corpus, human rights.</t>
         </is>
       </c>
-      <c r="E315" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" s="20" t="n">
+      <c r="E320" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="20" t="n">
         <v>443</v>
       </c>
-      <c r="B316" s="21" t="inlineStr">
+      <c r="B321" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C316" s="21" t="inlineStr">
+      <c r="C321" s="21" t="inlineStr">
         <is>
           <t>What is machine learning and how is it different from traditional programming?</t>
         </is>
       </c>
-      <c r="D316" s="21" t="inlineStr">
+      <c r="D321" s="21" t="inlineStr">
         <is>
           <t>**Traditional programming**: programmer writes explicit rules. Input + rules -&gt; output. Brittle; can't generalise.
 **Machine learning**: provide data + correct answers; algorithm finds the rules. Input + labels -&gt; model -&gt; generalises to new data.
@@ -8911,25 +9052,25 @@
 **Scale**: LLMs (GPT, Claude) = transformers on trillions of tokens; emergent capabilities at scale.</t>
         </is>
       </c>
-      <c r="E316" s="20" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" s="16" t="n">
+      <c r="E321" s="20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="16" t="n">
         <v>444</v>
       </c>
-      <c r="B317" s="17" t="inlineStr">
+      <c r="B322" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C317" s="17" t="inlineStr">
+      <c r="C322" s="17" t="inlineStr">
         <is>
           <t>What is the ship of Theseus paradox, and what is it really asking?</t>
         </is>
       </c>
-      <c r="D317" s="17" t="inlineStr">
+      <c r="D322" s="17" t="inlineStr">
         <is>
           <t>Plutarch (~100 CE): every plank of Theseus's ship replaced over time. Still the same ship?
 **Hobbes extension**: original planks collected and reassembled. Two ships claim to be the original. Which is it?
@@ -8943,25 +9084,25 @@
 **Parfit** (*Reasons and Persons*): personal identity is not what matters — psychological continuity is what matters; 'same' may be an empty question.</t>
         </is>
       </c>
-      <c r="E317" s="16" t="n">
+      <c r="E322" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="318">
-      <c r="A318" s="2" t="n">
+    <row r="323">
+      <c r="A323" s="2" t="n">
         <v>445</v>
       </c>
-      <c r="B318" s="3" t="inlineStr">
+      <c r="B323" s="3" t="inlineStr">
         <is>
           <t>Music</t>
         </is>
       </c>
-      <c r="C318" s="3" t="inlineStr">
+      <c r="C323" s="3" t="inlineStr">
         <is>
           <t>Why does music make us emotional?</t>
         </is>
       </c>
-      <c r="D318" s="3" t="inlineStr">
+      <c r="D323" s="3" t="inlineStr">
         <is>
           <t>Multiple converging mechanisms:
 1. **Expectation/violation** (Meyer 1956, Huron 2006): music is temporal prediction. Correct resolution = dopaminergic reward. Surprise + resolution = stronger reward. Chills = surprising resolution.
@@ -8973,25 +9114,25 @@
 **Mystery of sad music pleasure**: safe simulation, hormonal empathy reward, artistic resolution — distinct emotion from actual grief.</t>
         </is>
       </c>
-      <c r="E318" s="2" t="n">
+      <c r="E323" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="319">
-      <c r="A319" s="4" t="n">
+    <row r="324">
+      <c r="A324" s="4" t="n">
         <v>446</v>
       </c>
-      <c r="B319" s="5" t="inlineStr">
+      <c r="B324" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="C319" s="5" t="inlineStr">
+      <c r="C324" s="5" t="inlineStr">
         <is>
           <t>How do children acquire language so rapidly?</t>
         </is>
       </c>
-      <c r="D319" s="5" t="inlineStr">
+      <c r="D324" s="5" t="inlineStr">
         <is>
           <t>First words ~12 months, two-word phrases ~18-24 months, complex sentences by 3-4 years — from imperfect, fragmented input.
 **Poverty of the stimulus**: children overgeneralise rules ('goed', 'mouses') but never make wrong rule errors. Acquire structure-dependent rules without examples of errors.
@@ -9003,25 +9144,25 @@
 **Mechanisms**: statistical learning (8-month-olds track syllable transition probabilities), joint attention, motherese (simplified grammar + exaggerated prosody).</t>
         </is>
       </c>
-      <c r="E319" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" s="6" t="n">
+      <c r="E324" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="6" t="n">
         <v>447</v>
       </c>
-      <c r="B320" s="7" t="inlineStr">
+      <c r="B325" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C320" s="7" t="inlineStr">
+      <c r="C325" s="7" t="inlineStr">
         <is>
           <t>What is the photoelectric effect, and why did it matter for quantum mechanics?</t>
         </is>
       </c>
-      <c r="D320" s="7" t="inlineStr">
+      <c r="D325" s="7" t="inlineStr">
         <is>
           <t>Light hits metal -&gt; electrons ejected, BUT only above a threshold frequency. Below threshold: no electrons regardless of intensity.
 **Classical prediction**: intensity drives ejection. WRONG.
@@ -9034,25 +9175,25 @@
 4. Technology: photovoltaics, CCDs, photomultipliers</t>
         </is>
       </c>
-      <c r="E320" s="6" t="n">
+      <c r="E325" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="321">
-      <c r="A321" s="2" t="n">
+    <row r="326">
+      <c r="A326" s="2" t="n">
         <v>448</v>
       </c>
-      <c r="B321" s="3" t="inlineStr">
+      <c r="B326" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C321" s="3" t="inlineStr">
+      <c r="C326" s="3" t="inlineStr">
         <is>
           <t>What is social mobility and what actually predicts it?</t>
         </is>
       </c>
-      <c r="D321" s="3" t="inlineStr">
+      <c r="D326" s="3" t="inlineStr">
         <is>
           <t>Movement between socioeconomic strata. Intergenerational (parent to child) vs intragenerational (within lifetime).
 **Great Gatsby Curve** (Miles Corak): more income inequality -&gt; LOWER intergenerational mobility. Denmark (low inequality) = high mobility; US, UK = lower.
@@ -9065,25 +9206,25 @@
 Absolute mobility (exceeding parents in absolute terms) has historically been high; relative mobility much more constrained.</t>
         </is>
       </c>
-      <c r="E321" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" s="28" t="n">
+      <c r="E326" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="28" t="n">
         <v>449</v>
       </c>
-      <c r="B322" s="29" t="inlineStr">
+      <c r="B327" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C322" s="29" t="inlineStr">
+      <c r="C327" s="29" t="inlineStr">
         <is>
           <t>How do batteries work chemically, and what limits their energy density?</t>
         </is>
       </c>
-      <c r="D322" s="29" t="inlineStr">
+      <c r="D327" s="29" t="inlineStr">
         <is>
           <t>Battery = chemical -&gt; electrical energy via spatially separated redox reactions.
 Anode: oxidation (loses electrons). Cathode: reduction (gains electrons). Electrons flow externally (current); ions flow internally through electrolyte.
@@ -9100,25 +9241,25 @@
 **Theoretical limits**: Li-ion ~265 Wh/kg practical; Li-sulfur 2,600 Wh/kg; Li-air 11,680 Wh/kg (comparable to gasoline).</t>
         </is>
       </c>
-      <c r="E322" s="28" t="n">
+      <c r="E327" s="28" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="323">
-      <c r="A323" s="2" t="n">
+    <row r="328">
+      <c r="A328" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="B323" s="3" t="inlineStr">
+      <c r="B328" s="3" t="inlineStr">
         <is>
           <t>General Knowledge</t>
         </is>
       </c>
-      <c r="C323" s="3" t="inlineStr">
+      <c r="C328" s="3" t="inlineStr">
         <is>
           <t>What is the most important invention in human history, and why?</t>
         </is>
       </c>
-      <c r="D323" s="3" t="inlineStr">
+      <c r="D328" s="3" t="inlineStr">
         <is>
           <t>Depends on dimension valued. Four strong candidates:
 **Language**: meta-invention enabling all others to accumulate. But may have evolved rather than been invented.
@@ -9130,7 +9271,7 @@
 **Meta-point**: no invention stands alone. Cumulative innovation is humanity's real superpower.</t>
         </is>
       </c>
-      <c r="E323" s="2" t="n">
+      <c r="E328" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9525,14 +9666,14 @@
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>9.07</v>
+        <v>9.06</v>
       </c>
       <c r="D21" s="27" t="inlineStr">
         <is>
-          <t>169, 210, 236, 255, 349, 393, 440</t>
+          <t>169, 210, 236, 255, 349, 393, 415, 440</t>
         </is>
       </c>
     </row>
@@ -9957,14 +10098,14 @@
         </is>
       </c>
       <c r="B45" s="15" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C45" s="15" t="n">
-        <v>9.6</v>
+        <v>9.56</v>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 418, 436</t>
+          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 436</t>
         </is>
       </c>
     </row>
@@ -9993,14 +10134,14 @@
         </is>
       </c>
       <c r="B47" s="31" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C47" s="31" t="n">
-        <v>9.220000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D47" s="31" t="inlineStr">
         <is>
-          <t>230, 279, 294, 344, 379, 395, 411, 429, 441</t>
+          <t>230, 279, 294, 344, 379, 395, 411, 411, 429, 441</t>
         </is>
       </c>
     </row>
@@ -10335,14 +10476,14 @@
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>9.6</v>
+        <v>9.59</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 426, 438, 447</t>
+          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 426, 438, 447</t>
         </is>
       </c>
     </row>
@@ -10461,14 +10602,14 @@
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C73" s="3" t="n">
-        <v>9.07</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 439, 448</t>
+          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 413, 439, 448</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild SFT dataset with all 332 Q&As, add Q416-Q420, retrain
- yaya_qa_focused.jsonl: 236 -> 332 entries (all Q&As up to Q420)
- Old 236-entry checkpoints archived as yaya-tiny-sft-overfit-236
- New training launched from pretrain base, seq=384, 50k steps
- Excel updated: 332 rows, 78 domains
- Q416-Q420: philosophy/reasoning, biology/evolution, economics/2008,
  linguistics/acquisition, history/printing press

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E328"/>
+  <dimension ref="A1:E333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8226,20 +8226,51 @@
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="2" t="n">
+      <c r="A295" s="16" t="n">
+        <v>416</v>
+      </c>
+      <c r="B295" s="17" t="inlineStr">
+        <is>
+          <t>Philosophy</t>
+        </is>
+      </c>
+      <c r="C295" s="17" t="inlineStr">
+        <is>
+          <t>What is the difference between deductive, inductive, and abductive reasoning?</t>
+        </is>
+      </c>
+      <c r="D295" s="17" t="inlineStr">
+        <is>
+          <t>Three fundamental modes of inference:
+Deductive: conclusion necessarily follows from premises. Truth-preserving. Tool of mathematics and formal logic.
+Example: All humans are mortal. Socrates is human. Therefore Socrates is mortal.
+Inductive: conclusion is probably true given premises. Generalises from observations. Never certain.
+Example: Every swan I've seen is white. Therefore all swans are white. (Refuted by black swans, Australia 1697.)
+Abductive: inference to the best explanation. Chooses most plausible hypothesis.
+Example: The grass is wet. Best explanation: it rained. Not guaranteed (sprinklers possible).
+Role in science: induction generates hypotheses; deduction derives testable predictions; abduction selects best hypothesis when multiple fit data.
+C.S. Peirce formulated abduction. Popper argued science is hypothetico-deductive. In practice all three operate together.</t>
+        </is>
+      </c>
+      <c r="E295" s="16" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="n">
         <v>417</v>
       </c>
-      <c r="B295" s="3" t="inlineStr">
+      <c r="B296" s="3" t="inlineStr">
         <is>
           <t>Geology</t>
         </is>
       </c>
-      <c r="C295" s="3" t="inlineStr">
+      <c r="C296" s="3" t="inlineStr">
         <is>
           <t>How do plate tectonics work, and what drives the plates?</t>
         </is>
       </c>
-      <c r="D295" s="3" t="inlineStr">
+      <c r="D296" s="3" t="inlineStr">
         <is>
           <t>~15 major lithospheric plates (100km thick) float on viscous asthenosphere, moving 2-10 cm/year.
 **Three boundary types:**
@@ -8253,25 +8284,56 @@
 **Evidence**: magnetic striping on seafloor, continental fit (Wegener), matching fossils, earthquake distributions.</t>
         </is>
       </c>
-      <c r="E295" s="2" t="n">
+      <c r="E296" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="296">
-      <c r="A296" s="14" t="n">
+    <row r="297">
+      <c r="A297" s="18" t="n">
+        <v>417</v>
+      </c>
+      <c r="B297" s="19" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C297" s="19" t="inlineStr">
+        <is>
+          <t>How does evolution actually produce complexity — isn't it just random?</t>
+        </is>
+      </c>
+      <c r="D297" s="19" t="inlineStr">
+        <is>
+          <t>Common misconception: evolution is random therefore complexity can't arise.
+The mechanism: mutation is random; natural selection is NOT random — it consistently favours variants that reproduce more. Selection is the non-random filter on random variation.
+How complexity accumulates:
+- Incremental improvement: each step must be viable (1% of an eye improves survival; millions of generations -&gt; full eye)
+- Gene duplication: one copy evolves new function while other maintains original
+- Co-option/exaptation: feathers evolved for thermoregulation, later used for flight; jaw bones became ear ossicles
+- Modularity: existing signalling pathways reused in new contexts
+Irreducible complexity (Behe): bacterial flagellum couldn't evolve piecemeal. Refuted: flagellum shares components with type III secretion system — co-opted from earlier function.
+Deep time: 3.8 billion years × millions of generations per species.</t>
+        </is>
+      </c>
+      <c r="E297" s="18" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="14" t="n">
         <v>418</v>
       </c>
-      <c r="B296" s="15" t="inlineStr">
+      <c r="B298" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C296" s="15" t="inlineStr">
+      <c r="C298" s="15" t="inlineStr">
         <is>
           <t>What is a Fourier transform, and why is it everywhere?</t>
         </is>
       </c>
-      <c r="D296" s="15" t="inlineStr">
+      <c r="D298" s="15" t="inlineStr">
         <is>
           <t>Fourier (1822): any periodic function decomposes into sines and cosines of different frequencies.
 Fourier transform: takes time-domain signal f(t) -&gt; frequency-domain F(w) showing how much of each frequency is present.
@@ -8286,25 +8348,55 @@
 **FFT** (Cooley-Tukey 1965): O(n log n) vs O(n^2) naive. Made real-time signal processing possible.</t>
         </is>
       </c>
-      <c r="E296" s="14" t="n">
+      <c r="E298" s="14" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="297">
-      <c r="A297" s="2" t="n">
+    <row r="299">
+      <c r="A299" s="8" t="n">
+        <v>418</v>
+      </c>
+      <c r="B299" s="9" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="C299" s="9" t="inlineStr">
+        <is>
+          <t>What caused the 2008 financial crisis?</t>
+        </is>
+      </c>
+      <c r="D299" s="9" t="inlineStr">
+        <is>
+          <t>Cascade of interconnected failures:
+1. Housing bubble: low interest rates + deregulation -&gt; subprime lending explosion (no-doc loans)
+2. Securitisation: mortgages bundled into MBS and CDOs; risk appeared dispersed but concentrated in opaque leveraged instruments
+3. Rating agency failure: subprime CDOs rated AAA; models assumed house prices couldn't fall nationally
+4. Shadow banking: AIG wrote $440B in credit default swaps with no capital reserves; Bear Stearns/Lehman leveraged 30:1
+5. Contagion: Lehman collapsed Sep 15 2008; interbank lending froze; credit markets seized globally
+Consequences: $19 trillion US household wealth destroyed; 8.7 million jobs lost; global recession.
+Response: TARP $700B bailout, Fed QE, Dodd-Frank regulation. Moral hazard unresolved: banks socialised losses, privatised gains.</t>
+        </is>
+      </c>
+      <c r="E299" s="8" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="n">
         <v>419</v>
       </c>
-      <c r="B297" s="3" t="inlineStr">
+      <c r="B300" s="3" t="inlineStr">
         <is>
           <t>Ethics</t>
         </is>
       </c>
-      <c r="C297" s="3" t="inlineStr">
+      <c r="C300" s="3" t="inlineStr">
         <is>
           <t>What is the difference between deontological and consequentialist ethics, and which is right?</t>
         </is>
       </c>
-      <c r="D297" s="3" t="inlineStr">
+      <c r="D300" s="3" t="inlineStr">
         <is>
           <t>**Consequentialism** (Bentham, Mill): moral worth from consequences. Maximise utility/welfare. Strength: outcome-focused. Weakness: justifies organ harvesting one person to save five; ignores rights.
 **Deontology** (Kant): moral worth from the action itself, not consequences. Categorical Imperative:
@@ -8319,25 +8411,53 @@
 Reflective equilibrium: use multiple frameworks as lenses, check coherence with intuitions.</t>
         </is>
       </c>
-      <c r="E297" s="2" t="n">
+      <c r="E300" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="298">
-      <c r="A298" s="4" t="n">
+    <row r="301">
+      <c r="A301" s="4" t="n">
+        <v>419</v>
+      </c>
+      <c r="B301" s="5" t="inlineStr">
+        <is>
+          <t>Linguistics</t>
+        </is>
+      </c>
+      <c r="C301" s="5" t="inlineStr">
+        <is>
+          <t>How do children acquire language so fast — what is the language acquisition debate?</t>
+        </is>
+      </c>
+      <c r="D301" s="5" t="inlineStr">
+        <is>
+          <t>Children reach fluent grammar in ~3 years across all languages without formal instruction.
+Nativist (Chomsky): Universal Grammar — innate template constraining possible grammars. Poverty of stimulus: input too incomplete to specify acquired grammar; something innate must help. Critical period: Genie case (feral child found at 13) — vocabulary but no grammar.
+Usage-based / Emergentist (Tomasello): general cognitive mechanisms — pattern recognition, intention-reading, analogy — suffice. No special language organ. CHILDES corpus shows input is richer than poverty-of-stimulus claims.
+Evidence for nativism: same developmental sequence across all cultures; sign language acquired at same pace.
+Evidence against: connectionist models acquire many structures without innate grammar; languages vary more than UG predicts (Pirahã recursion debate, Everett).
+Consensus: some innate biological predisposition + general learning + social interaction. Not a detailed innate grammar.</t>
+        </is>
+      </c>
+      <c r="E301" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="4" t="n">
         <v>420</v>
       </c>
-      <c r="B298" s="5" t="inlineStr">
+      <c r="B302" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="C298" s="5" t="inlineStr">
+      <c r="C302" s="5" t="inlineStr">
         <is>
           <t>What is the difference between descriptive and prescriptive grammar, and why does it matter?</t>
         </is>
       </c>
-      <c r="D298" s="5" t="inlineStr">
+      <c r="D302" s="5" t="inlineStr">
         <is>
           <t>**Prescriptive**: what people *should* say — textbooks, style guides, norms ('don't split infinitives', 'it is I').
 **Descriptive**: what people *actually* say — linguist's approach. Records patterns without judging. Every human language has consistent grammar; no language is 'wrong.'
@@ -8349,25 +8469,57 @@
 5. Code-switching: competent speakers deploy both — AAVE at home, SAE formally. Both correct for their domains.</t>
         </is>
       </c>
-      <c r="E298" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="299">
-      <c r="A299" s="18" t="n">
+      <c r="E302" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="12" t="n">
+        <v>420</v>
+      </c>
+      <c r="B303" s="13" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="C303" s="13" t="inlineStr">
+        <is>
+          <t>What was the significance of the printing press?</t>
+        </is>
+      </c>
+      <c r="D303" s="13" t="inlineStr">
+        <is>
+          <t>Gutenberg's movable-type press (~1440): most important invention of the millennium.
+Before: books hand-copied (Bible = 1 year); knowledge monopolised by Church and aristocracy.
+Immediate: cost of books dropped ~300x in 50 years; 20 million books by 1500; standardised spelling and language.
+Consequences:
+1. Reformation: Luther's 95 Theses (1517) spread across Germany in weeks. Church lost doctrinal monopoly. 100+ years of religious war.
+2. Scientific Revolution: scientists could publish, build on each other, correct errors. Cumulative knowledge possible.
+3. Public sphere: newspapers, pamphlets, political discourse (Habermas)
+4. Nationalism: print capitalism (Benedict Anderson) — shared printed language created imagined communities
+5. Vernacular literature: Shakespeare, Cervantes reached mass audiences
+Parallel to internet: same dynamics of information democratisation, disruption of gatekeepers, spread of misinformation (Eisenstein).</t>
+        </is>
+      </c>
+      <c r="E303" s="12" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="18" t="n">
         <v>421</v>
       </c>
-      <c r="B299" s="19" t="inlineStr">
+      <c r="B304" s="19" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C299" s="19" t="inlineStr">
+      <c r="C304" s="19" t="inlineStr">
         <is>
           <t>How does the immune system distinguish 'self' from 'non-self'?</t>
         </is>
       </c>
-      <c r="D299" s="19" t="inlineStr">
+      <c r="D304" s="19" t="inlineStr">
         <is>
           <t>Multiple overlapping mechanisms:
 **MHC class I**: every nucleated cell displays own protein fragments on MHC class I. T-cells educated in thymus to tolerate self-peptides; cells displaying foreign peptides (viral, tumour) are destroyed.
@@ -8379,25 +8531,25 @@
 - Transplant rejection: donor MHC recognised as foreign</t>
         </is>
       </c>
-      <c r="E299" s="18" t="n">
+      <c r="E304" s="18" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="300">
-      <c r="A300" s="12" t="n">
+    <row r="305">
+      <c r="A305" s="12" t="n">
         <v>422</v>
       </c>
-      <c r="B300" s="13" t="inlineStr">
+      <c r="B305" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C300" s="13" t="inlineStr">
+      <c r="C305" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the printing press, and did Gutenberg invent it?</t>
         </is>
       </c>
-      <c r="D300" s="13" t="inlineStr">
+      <c r="D305" s="13" t="inlineStr">
         <is>
           <t>Gutenberg (~1450) didn't invent printing. Moveable type existed in China (Bi Sheng ~1040) and Korea (Jikji 1377, oldest surviving). Gutenberg's innovation: complete system — durable metal alloy type, oil-based ink, adapted screw press — optimised for the European alphabet.
 **Why it transformed Europe**: Latin alphabet (26 letters) made moveable type far more efficient than Chinese/Korean systems (thousands of characters). Press: ~3,600 pages/day vs 40 for a scribe.
@@ -8410,25 +8562,25 @@
 **Eisenstein's thesis**: press created new relationship with knowledge — standardisation, reproducibility, verification.</t>
         </is>
       </c>
-      <c r="E300" s="12" t="n">
+      <c r="E305" s="12" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="301">
-      <c r="A301" s="10" t="n">
+    <row r="306">
+      <c r="A306" s="10" t="n">
         <v>423</v>
       </c>
-      <c r="B301" s="11" t="inlineStr">
+      <c r="B306" s="11" t="inlineStr">
         <is>
           <t>Neuroscience</t>
         </is>
       </c>
-      <c r="C301" s="11" t="inlineStr">
+      <c r="C306" s="11" t="inlineStr">
         <is>
           <t>What is consciousness and why is it so hard to explain?</t>
         </is>
       </c>
-      <c r="D301" s="11" t="inlineStr">
+      <c r="D306" s="11" t="inlineStr">
         <is>
           <t>Chalmers (1995) 'hard problem': why does information processing produce *subjective experience*? Why is there something it is like to see red?
 Even full neural mapping of correlates wouldn't explain why any of it feels like anything. Explaining function doesn't explain qualia.
@@ -8441,25 +8593,25 @@
 **Consensus**: none. Hard problem remains genuinely open.</t>
         </is>
       </c>
-      <c r="E301" s="10" t="n">
+      <c r="E306" s="10" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="302">
-      <c r="A302" s="28" t="n">
+    <row r="307">
+      <c r="A307" s="28" t="n">
         <v>424</v>
       </c>
-      <c r="B302" s="29" t="inlineStr">
+      <c r="B307" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C302" s="29" t="inlineStr">
+      <c r="C307" s="29" t="inlineStr">
         <is>
           <t>What makes some molecules smell while others don't?</t>
         </is>
       </c>
-      <c r="D302" s="29" t="inlineStr">
+      <c r="D307" s="29" t="inlineStr">
         <is>
           <t>Odorant molecules bind to olfactory receptors (ORs, GPCRs) in nasal epithelium -&gt; olfactory bulb -&gt; piriform cortex + limbic system.
 **What molecules smell:**
@@ -8471,25 +8623,25 @@
 **COVID-19 anosmia**: virus destroys olfactory neuron support cells; usually recovers.</t>
         </is>
       </c>
-      <c r="E302" s="28" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" s="8" t="n">
+      <c r="E307" s="28" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="8" t="n">
         <v>425</v>
       </c>
-      <c r="B303" s="9" t="inlineStr">
+      <c r="B308" s="9" t="inlineStr">
         <is>
           <t>Economics</t>
         </is>
       </c>
-      <c r="C303" s="9" t="inlineStr">
+      <c r="C308" s="9" t="inlineStr">
         <is>
           <t>What caused the 2008 financial crisis?</t>
         </is>
       </c>
-      <c r="D303" s="9" t="inlineStr">
+      <c r="D308" s="9" t="inlineStr">
         <is>
           <t>Cascade of failures:
 **Housing bubble**: low post-9/11 rates, relaxed lending, NINJA loans (no income/assets/job). Prices +124% nationally 2000-2006.
@@ -8501,25 +8653,25 @@
 **Response**: Dodd-Frank, Basel III capital requirements, Volcker Rule.</t>
         </is>
       </c>
-      <c r="E303" s="8" t="n">
+      <c r="E308" s="8" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="304">
-      <c r="A304" s="6" t="n">
+    <row r="309">
+      <c r="A309" s="6" t="n">
         <v>426</v>
       </c>
-      <c r="B304" s="7" t="inlineStr">
+      <c r="B309" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C304" s="7" t="inlineStr">
+      <c r="C309" s="7" t="inlineStr">
         <is>
           <t>What is dark matter and how do we know it exists?</t>
         </is>
       </c>
-      <c r="D304" s="7" t="inlineStr">
+      <c r="D309" s="7" t="inlineStr">
         <is>
           <t>~27% of universe's energy. Doesn't emit/absorb/reflect light. Gravitational effects overwhelming.
 **Evidence:**
@@ -8531,25 +8683,25 @@
 **MOND alternative**: modified Newtonian dynamics; cannot explain Bullet Cluster + CMB simultaneously. Most physicists favour particle dark matter.</t>
         </is>
       </c>
-      <c r="E304" s="6" t="n">
+      <c r="E309" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="305">
-      <c r="A305" s="2" t="n">
+    <row r="310">
+      <c r="A310" s="2" t="n">
         <v>427</v>
       </c>
-      <c r="B305" s="3" t="inlineStr">
+      <c r="B310" s="3" t="inlineStr">
         <is>
           <t>Literature</t>
         </is>
       </c>
-      <c r="C305" s="3" t="inlineStr">
+      <c r="C310" s="3" t="inlineStr">
         <is>
           <t>Why is 'Don Quixote' considered the first modern novel?</t>
         </is>
       </c>
-      <c r="D305" s="3" t="inlineStr">
+      <c r="D310" s="3" t="inlineStr">
         <is>
           <t>Cervantes (Part I: 1605, Part II: 1615). Why it's considered the first modern novel:
 1. Self-consciousness: the novel is aware it's a novel. Part II characters have read Part I. Unreliable narrators, manuscript frames — postmodern devices 400 years early.
@@ -8560,25 +8712,25 @@
 What makes it 'modern': fundamentally ambiguous relationship with truth; character who changes across time (Part I vs II Quixote). Bloom: 'most universal and most particular character in literature.'</t>
         </is>
       </c>
-      <c r="E305" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" s="20" t="n">
+      <c r="E310" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="20" t="n">
         <v>428</v>
       </c>
-      <c r="B306" s="21" t="inlineStr">
+      <c r="B311" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C306" s="21" t="inlineStr">
+      <c r="C311" s="21" t="inlineStr">
         <is>
           <t>What is the halting problem and why does it matter?</t>
         </is>
       </c>
-      <c r="D306" s="21" t="inlineStr">
+      <c r="D311" s="21" t="inlineStr">
         <is>
           <t>Turing (1936): no general algorithm can determine whether an arbitrary program will halt or run forever.
 **Proof (diagonal argument)**: assume HALT(P,I) exists. Construct DIAG(P): if HALT says P halts on P -&gt; loop; if HALT says P loops -&gt; halt.
@@ -8591,25 +8743,25 @@
 5. Practical: compilers and static analysers must be incomplete or unsound — they make heuristic approximations.</t>
         </is>
       </c>
-      <c r="E306" s="20" t="n">
+      <c r="E311" s="20" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="307">
-      <c r="A307" s="30" t="n">
+    <row r="312">
+      <c r="A312" s="30" t="n">
         <v>429</v>
       </c>
-      <c r="B307" s="31" t="inlineStr">
+      <c r="B312" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C307" s="31" t="inlineStr">
+      <c r="C312" s="31" t="inlineStr">
         <is>
           <t>How do vaccines work, and why do some require boosters?</t>
         </is>
       </c>
-      <c r="D307" s="31" t="inlineStr">
+      <c r="D312" s="31" t="inlineStr">
         <is>
           <t>Vaccine presents antigen (weakened/killed pathogen, subunit protein, or mRNA) without disease, training immune memory.
 **Mechanism:**
@@ -8626,25 +8778,25 @@
 **Why boosters**: antibody titres wane (inactivated/subunit weaker); mutating viruses (flu) change antigens.</t>
         </is>
       </c>
-      <c r="E307" s="30" t="n">
+      <c r="E312" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="308">
-      <c r="A308" s="16" t="n">
+    <row r="313">
+      <c r="A313" s="16" t="n">
         <v>430</v>
       </c>
-      <c r="B308" s="17" t="inlineStr">
+      <c r="B313" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C308" s="17" t="inlineStr">
+      <c r="C313" s="17" t="inlineStr">
         <is>
           <t>What is free will, and does science undermine it?</t>
         </is>
       </c>
-      <c r="D308" s="17" t="inlineStr">
+      <c r="D313" s="17" t="inlineStr">
         <is>
           <t>Are our choices genuinely ours, or determined by prior causes?
 **Three positions:**
@@ -8656,25 +8808,25 @@
 **Does science undermine it?** Depends what you mean. Compatibilist free will survives. Hard determinism mostly fringe.</t>
         </is>
       </c>
-      <c r="E308" s="16" t="n">
+      <c r="E313" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="309">
-      <c r="A309" s="22" t="n">
+    <row r="314">
+      <c r="A314" s="22" t="n">
         <v>431</v>
       </c>
-      <c r="B309" s="23" t="inlineStr">
+      <c r="B314" s="23" t="inlineStr">
         <is>
           <t>Astronomy</t>
         </is>
       </c>
-      <c r="C309" s="23" t="inlineStr">
+      <c r="C314" s="23" t="inlineStr">
         <is>
           <t>What are neutron stars and how do they form?</t>
         </is>
       </c>
-      <c r="D309" s="23" t="inlineStr">
+      <c r="D314" s="23" t="inlineStr">
         <is>
           <t>Massive star (8-20 solar masses) core collapses. If core mass 1.4-3 solar masses, electron degeneracy fails. Protons + electrons merge (inverse beta decay) -&gt; neutron star.
 **Properties:**
@@ -8687,25 +8839,25 @@
 **Neutron star mergers (GW170817, 2017)**: first gravitational wave + electromagnetic detection. Kilonova: r-process nucleosynthesis produces gold, platinum, uranium. Primary source of heavy elements.</t>
         </is>
       </c>
-      <c r="E309" s="22" t="n">
+      <c r="E314" s="22" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="310">
-      <c r="A310" s="24" t="n">
+    <row r="315">
+      <c r="A315" s="24" t="n">
         <v>432</v>
       </c>
-      <c r="B310" s="25" t="inlineStr">
+      <c r="B315" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C310" s="25" t="inlineStr">
+      <c r="C315" s="25" t="inlineStr">
         <is>
           <t>What is the Dunning-Kruger effect, and is it as universal as people think?</t>
         </is>
       </c>
-      <c r="D310" s="25" t="inlineStr">
+      <c r="D315" s="25" t="inlineStr">
         <is>
           <t>Kruger &amp; Dunning (1999): people with limited knowledge overestimate competence; experts underestimate relative ability (task seems easy to them too).
 **Original study**: bottom quartile performers on logic/grammar/humour overestimated by ~50 percentile points.
@@ -8719,25 +8871,25 @@
 - Domain-specific: expert engineer may still have DK in social skills</t>
         </is>
       </c>
-      <c r="E310" s="24" t="n">
+      <c r="E315" s="24" t="n">
         <v>8.5</v>
       </c>
     </row>
-    <row r="311">
-      <c r="A311" s="12" t="n">
+    <row r="316">
+      <c r="A316" s="12" t="n">
         <v>433</v>
       </c>
-      <c r="B311" s="13" t="inlineStr">
+      <c r="B316" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C311" s="13" t="inlineStr">
+      <c r="C316" s="13" t="inlineStr">
         <is>
           <t>Why did the Roman Empire fall?</t>
         </is>
       </c>
-      <c r="D311" s="13" t="inlineStr">
+      <c r="D316" s="13" t="inlineStr">
         <is>
           <t>Western Empire fell 476 CE (Romulus Augustulus deposed). Eastern Empire (Byzantium) lasted to 1453. No single cause:
 **Military/political:** overextended borders; Germanic foederati with divided loyalty; political instability (50 emperors in 50 years, 235-284 CE); military power to make/unmake emperors.
@@ -8750,25 +8902,25 @@
 **What didn't fall**: Eastern Empire thrived. Fall was primarily western.</t>
         </is>
       </c>
-      <c r="E311" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" s="2" t="n">
+      <c r="E316" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="n">
         <v>434</v>
       </c>
-      <c r="B312" s="3" t="inlineStr">
+      <c r="B317" s="3" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C312" s="3" t="inlineStr">
+      <c r="C317" s="3" t="inlineStr">
         <is>
           <t>How does GPS actually work?</t>
         </is>
       </c>
-      <c r="D312" s="3" t="inlineStr">
+      <c r="D317" s="3" t="inlineStr">
         <is>
           <t>24-32 satellites at ~20,200km; 6 orbital planes; each completes 2 orbits/day.
 **Core principle: trilateration via time signals.**
@@ -8784,25 +8936,25 @@
 - Net: +38 microseconds/day. Without correction: GPS drifts ~10km/day. Einstein's corrections are in the system.</t>
         </is>
       </c>
-      <c r="E312" s="2" t="n">
+      <c r="E317" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="313">
-      <c r="A313" s="18" t="n">
+    <row r="318">
+      <c r="A318" s="18" t="n">
         <v>435</v>
       </c>
-      <c r="B313" s="19" t="inlineStr">
+      <c r="B318" s="19" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C313" s="19" t="inlineStr">
+      <c r="C318" s="19" t="inlineStr">
         <is>
           <t>What is epigenetics and does it challenge our understanding of inheritance?</t>
         </is>
       </c>
-      <c r="D313" s="19" t="inlineStr">
+      <c r="D318" s="19" t="inlineStr">
         <is>
           <t>Heritable changes in gene expression without DNA sequence changes. Genome = instruction manual; epigenome = which instructions are read.
 **Mechanisms:**
@@ -8814,25 +8966,25 @@
 Does NOT validate Lamarck — mechanisms are different from direct inheritance of acquired characteristics.</t>
         </is>
       </c>
-      <c r="E313" s="18" t="n">
+      <c r="E318" s="18" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="314">
-      <c r="A314" s="14" t="n">
+    <row r="319">
+      <c r="A319" s="14" t="n">
         <v>436</v>
       </c>
-      <c r="B314" s="15" t="inlineStr">
+      <c r="B319" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C314" s="15" t="inlineStr">
+      <c r="C319" s="15" t="inlineStr">
         <is>
           <t>What is a prime number, and what do we know about their distribution?</t>
         </is>
       </c>
-      <c r="D314" s="15" t="inlineStr">
+      <c r="D319" s="15" t="inlineStr">
         <is>
           <t>A prime: natural number &gt; 1 with no divisors other than 1 and itself. Euclid (~300 BCE): infinitely many.
 Fundamental Theorem of Arithmetic: every integer &gt; 1 is prime or unique product of primes.
@@ -8844,25 +8996,25 @@
 **Practical importance**: RSA encryption relies on difficulty of factoring large numbers.</t>
         </is>
       </c>
-      <c r="E314" s="14" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" s="24" t="n">
+      <c r="E319" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="24" t="n">
         <v>437</v>
       </c>
-      <c r="B315" s="25" t="inlineStr">
+      <c r="B320" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C315" s="25" t="inlineStr">
+      <c r="C320" s="25" t="inlineStr">
         <is>
           <t>How reliable is eyewitness testimony, and what does the research say?</t>
         </is>
       </c>
-      <c r="D315" s="25" t="inlineStr">
+      <c r="D320" s="25" t="inlineStr">
         <is>
           <t>Memory is reconstructive, not reproductive (Loftus). We rebuild memories each time, subject to suggestion.
 **Key experiments:**
@@ -8873,25 +9025,25 @@
 **What helps**: sequential lineups, blind administration, record initial statement, open questions first.</t>
         </is>
       </c>
-      <c r="E315" s="24" t="n">
+      <c r="E320" s="24" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="316">
-      <c r="A316" s="6" t="n">
+    <row r="321">
+      <c r="A321" s="6" t="n">
         <v>438</v>
       </c>
-      <c r="B316" s="7" t="inlineStr">
+      <c r="B321" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C316" s="7" t="inlineStr">
+      <c r="C321" s="7" t="inlineStr">
         <is>
           <t>What is the difference between heat and temperature?</t>
         </is>
       </c>
-      <c r="D316" s="7" t="inlineStr">
+      <c r="D321" s="7" t="inlineStr">
         <is>
           <t>**Temperature**: average kinetic energy per molecule. Measured in Kelvin/Celsius/Fahrenheit.
 **Heat**: *transfer* of thermal energy between objects due to temperature difference. Heat is a process, not a property. Pool at same temperature as coffee mug: pool contains far more thermal energy.
@@ -8901,25 +9053,25 @@
 **Water vs air at 100C**: water burns much more — higher thermal mass + latent heat of condensation deliver more energy per contact.</t>
         </is>
       </c>
-      <c r="E316" s="6" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" s="2" t="n">
+      <c r="E321" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="n">
         <v>439</v>
       </c>
-      <c r="B317" s="3" t="inlineStr">
+      <c r="B322" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C317" s="3" t="inlineStr">
+      <c r="C322" s="3" t="inlineStr">
         <is>
           <t>What is structural racism, and how does it differ from individual racism?</t>
         </is>
       </c>
-      <c r="D317" s="3" t="inlineStr">
+      <c r="D322" s="3" t="inlineStr">
         <is>
           <t>**Individual racism**: prejudice and discriminatory acts by identifiable individuals. Overt bias.
 **Structural racism**: racial disparities from systems, policies, norms — even without individual racist intent.
@@ -8931,25 +9083,25 @@
 **Evidence**: audit studies (identical CVs with Black vs white names) consistently find measurable hiring discrimination.</t>
         </is>
       </c>
-      <c r="E317" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" s="26" t="n">
+      <c r="E322" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="26" t="n">
         <v>440</v>
       </c>
-      <c r="B318" s="27" t="inlineStr">
+      <c r="B323" s="27" t="inlineStr">
         <is>
           <t>Ecology</t>
         </is>
       </c>
-      <c r="C318" s="27" t="inlineStr">
+      <c r="C323" s="27" t="inlineStr">
         <is>
           <t>What is the nitrogen cycle and why is it essential for life?</t>
         </is>
       </c>
-      <c r="D318" s="27" t="inlineStr">
+      <c r="D323" s="27" t="inlineStr">
         <is>
           <t>N2 = 78% of atmosphere, but most organisms can't use N2 (triple bond N=N, 945 kJ/mol). Life needs reactive N (NH3, NO3-, organic N).
 **Nitrogen cycle:**
@@ -8961,25 +9113,25 @@
 **Limiting nutrient**: N limits most ecosystems. Excess (fertilisers) -&gt; eutrophication -&gt; algal blooms -&gt; oxygen depletion -&gt; dead zones (Gulf of Mexico). Haber also weaponised N (chlorine, phosgene).</t>
         </is>
       </c>
-      <c r="E318" s="26" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" s="30" t="n">
+      <c r="E323" s="26" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="30" t="n">
         <v>441</v>
       </c>
-      <c r="B319" s="31" t="inlineStr">
+      <c r="B324" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C319" s="31" t="inlineStr">
+      <c r="C324" s="31" t="inlineStr">
         <is>
           <t>What is antibiotic resistance and how does it develop?</t>
         </is>
       </c>
-      <c r="D319" s="31" t="inlineStr">
+      <c r="D324" s="31" t="inlineStr">
         <is>
           <t>Antibiotics target cell wall (penicillin), protein synthesis (tetracycline), DNA replication (fluoroquinolones), or membranes. Resistance = survival.
 **Darwinian mechanism:**
@@ -8993,25 +9145,25 @@
 **Why few new antibiotics**: 10-15yr development; brief low-cost use = poor financial incentive vs lifelong drugs.</t>
         </is>
       </c>
-      <c r="E319" s="30" t="n">
+      <c r="E324" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="320">
-      <c r="A320" s="12" t="n">
+    <row r="325">
+      <c r="A325" s="12" t="n">
         <v>442</v>
       </c>
-      <c r="B320" s="13" t="inlineStr">
+      <c r="B325" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C320" s="13" t="inlineStr">
+      <c r="C325" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the Magna Carta?</t>
         </is>
       </c>
-      <c r="D320" s="13" t="inlineStr">
+      <c r="D325" s="13" t="inlineStr">
         <is>
           <t>June 1215: English barons forced King John to sign. Originally limited royal power in narrow feudal ways — mostly barons' rights, not ordinary people.
 **Key clauses**: Cl. 39 — no free man imprisoned without lawful judgment of peers ('due process'); Cl. 40 — no selling/denying justice.
@@ -9021,25 +9173,25 @@
 **Lasting principle**: rule of law over arbitrary power -&gt; constitutional government, habeas corpus, human rights.</t>
         </is>
       </c>
-      <c r="E320" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" s="20" t="n">
+      <c r="E325" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="20" t="n">
         <v>443</v>
       </c>
-      <c r="B321" s="21" t="inlineStr">
+      <c r="B326" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C321" s="21" t="inlineStr">
+      <c r="C326" s="21" t="inlineStr">
         <is>
           <t>What is machine learning and how is it different from traditional programming?</t>
         </is>
       </c>
-      <c r="D321" s="21" t="inlineStr">
+      <c r="D326" s="21" t="inlineStr">
         <is>
           <t>**Traditional programming**: programmer writes explicit rules. Input + rules -&gt; output. Brittle; can't generalise.
 **Machine learning**: provide data + correct answers; algorithm finds the rules. Input + labels -&gt; model -&gt; generalises to new data.
@@ -9052,25 +9204,25 @@
 **Scale**: LLMs (GPT, Claude) = transformers on trillions of tokens; emergent capabilities at scale.</t>
         </is>
       </c>
-      <c r="E321" s="20" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" s="16" t="n">
+      <c r="E326" s="20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="16" t="n">
         <v>444</v>
       </c>
-      <c r="B322" s="17" t="inlineStr">
+      <c r="B327" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C322" s="17" t="inlineStr">
+      <c r="C327" s="17" t="inlineStr">
         <is>
           <t>What is the ship of Theseus paradox, and what is it really asking?</t>
         </is>
       </c>
-      <c r="D322" s="17" t="inlineStr">
+      <c r="D327" s="17" t="inlineStr">
         <is>
           <t>Plutarch (~100 CE): every plank of Theseus's ship replaced over time. Still the same ship?
 **Hobbes extension**: original planks collected and reassembled. Two ships claim to be the original. Which is it?
@@ -9084,25 +9236,25 @@
 **Parfit** (*Reasons and Persons*): personal identity is not what matters — psychological continuity is what matters; 'same' may be an empty question.</t>
         </is>
       </c>
-      <c r="E322" s="16" t="n">
+      <c r="E327" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="323">
-      <c r="A323" s="2" t="n">
+    <row r="328">
+      <c r="A328" s="2" t="n">
         <v>445</v>
       </c>
-      <c r="B323" s="3" t="inlineStr">
+      <c r="B328" s="3" t="inlineStr">
         <is>
           <t>Music</t>
         </is>
       </c>
-      <c r="C323" s="3" t="inlineStr">
+      <c r="C328" s="3" t="inlineStr">
         <is>
           <t>Why does music make us emotional?</t>
         </is>
       </c>
-      <c r="D323" s="3" t="inlineStr">
+      <c r="D328" s="3" t="inlineStr">
         <is>
           <t>Multiple converging mechanisms:
 1. **Expectation/violation** (Meyer 1956, Huron 2006): music is temporal prediction. Correct resolution = dopaminergic reward. Surprise + resolution = stronger reward. Chills = surprising resolution.
@@ -9114,25 +9266,25 @@
 **Mystery of sad music pleasure**: safe simulation, hormonal empathy reward, artistic resolution — distinct emotion from actual grief.</t>
         </is>
       </c>
-      <c r="E323" s="2" t="n">
+      <c r="E328" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="324">
-      <c r="A324" s="4" t="n">
+    <row r="329">
+      <c r="A329" s="4" t="n">
         <v>446</v>
       </c>
-      <c r="B324" s="5" t="inlineStr">
+      <c r="B329" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="C324" s="5" t="inlineStr">
+      <c r="C329" s="5" t="inlineStr">
         <is>
           <t>How do children acquire language so rapidly?</t>
         </is>
       </c>
-      <c r="D324" s="5" t="inlineStr">
+      <c r="D329" s="5" t="inlineStr">
         <is>
           <t>First words ~12 months, two-word phrases ~18-24 months, complex sentences by 3-4 years — from imperfect, fragmented input.
 **Poverty of the stimulus**: children overgeneralise rules ('goed', 'mouses') but never make wrong rule errors. Acquire structure-dependent rules without examples of errors.
@@ -9144,25 +9296,25 @@
 **Mechanisms**: statistical learning (8-month-olds track syllable transition probabilities), joint attention, motherese (simplified grammar + exaggerated prosody).</t>
         </is>
       </c>
-      <c r="E324" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" s="6" t="n">
+      <c r="E329" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="6" t="n">
         <v>447</v>
       </c>
-      <c r="B325" s="7" t="inlineStr">
+      <c r="B330" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C325" s="7" t="inlineStr">
+      <c r="C330" s="7" t="inlineStr">
         <is>
           <t>What is the photoelectric effect, and why did it matter for quantum mechanics?</t>
         </is>
       </c>
-      <c r="D325" s="7" t="inlineStr">
+      <c r="D330" s="7" t="inlineStr">
         <is>
           <t>Light hits metal -&gt; electrons ejected, BUT only above a threshold frequency. Below threshold: no electrons regardless of intensity.
 **Classical prediction**: intensity drives ejection. WRONG.
@@ -9175,25 +9327,25 @@
 4. Technology: photovoltaics, CCDs, photomultipliers</t>
         </is>
       </c>
-      <c r="E325" s="6" t="n">
+      <c r="E330" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="326">
-      <c r="A326" s="2" t="n">
+    <row r="331">
+      <c r="A331" s="2" t="n">
         <v>448</v>
       </c>
-      <c r="B326" s="3" t="inlineStr">
+      <c r="B331" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C326" s="3" t="inlineStr">
+      <c r="C331" s="3" t="inlineStr">
         <is>
           <t>What is social mobility and what actually predicts it?</t>
         </is>
       </c>
-      <c r="D326" s="3" t="inlineStr">
+      <c r="D331" s="3" t="inlineStr">
         <is>
           <t>Movement between socioeconomic strata. Intergenerational (parent to child) vs intragenerational (within lifetime).
 **Great Gatsby Curve** (Miles Corak): more income inequality -&gt; LOWER intergenerational mobility. Denmark (low inequality) = high mobility; US, UK = lower.
@@ -9206,25 +9358,25 @@
 Absolute mobility (exceeding parents in absolute terms) has historically been high; relative mobility much more constrained.</t>
         </is>
       </c>
-      <c r="E326" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" s="28" t="n">
+      <c r="E331" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="28" t="n">
         <v>449</v>
       </c>
-      <c r="B327" s="29" t="inlineStr">
+      <c r="B332" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C327" s="29" t="inlineStr">
+      <c r="C332" s="29" t="inlineStr">
         <is>
           <t>How do batteries work chemically, and what limits their energy density?</t>
         </is>
       </c>
-      <c r="D327" s="29" t="inlineStr">
+      <c r="D332" s="29" t="inlineStr">
         <is>
           <t>Battery = chemical -&gt; electrical energy via spatially separated redox reactions.
 Anode: oxidation (loses electrons). Cathode: reduction (gains electrons). Electrons flow externally (current); ions flow internally through electrolyte.
@@ -9241,25 +9393,25 @@
 **Theoretical limits**: Li-ion ~265 Wh/kg practical; Li-sulfur 2,600 Wh/kg; Li-air 11,680 Wh/kg (comparable to gasoline).</t>
         </is>
       </c>
-      <c r="E327" s="28" t="n">
+      <c r="E332" s="28" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="328">
-      <c r="A328" s="2" t="n">
+    <row r="333">
+      <c r="A333" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="B328" s="3" t="inlineStr">
+      <c r="B333" s="3" t="inlineStr">
         <is>
           <t>General Knowledge</t>
         </is>
       </c>
-      <c r="C328" s="3" t="inlineStr">
+      <c r="C333" s="3" t="inlineStr">
         <is>
           <t>What is the most important invention in human history, and why?</t>
         </is>
       </c>
-      <c r="D328" s="3" t="inlineStr">
+      <c r="D333" s="3" t="inlineStr">
         <is>
           <t>Depends on dimension valued. Four strong candidates:
 **Language**: meta-invention enabling all others to accumulate. But may have evolved rather than been invented.
@@ -9271,7 +9423,7 @@
 **Meta-point**: no invention stands alone. Cumulative innovation is humanity's real superpower.</t>
         </is>
       </c>
-      <c r="E328" s="2" t="n">
+      <c r="E333" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9450,14 +9602,14 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>9.34</v>
+        <v>9.32</v>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>156, 171, 181, 222, 243, 266, 282, 287, 297, 304, 313, 383, 400, 400, 421, 435</t>
+          <t>156, 171, 181, 222, 243, 266, 282, 287, 297, 304, 313, 383, 400, 400, 417, 421, 435</t>
         </is>
       </c>
     </row>
@@ -9684,14 +9836,14 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>9.1</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 425</t>
+          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425</t>
         </is>
       </c>
     </row>
@@ -9900,14 +10052,14 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C34" s="13" t="n">
-        <v>9.109999999999999</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 422, 433, 442</t>
+          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 433, 442</t>
         </is>
       </c>
     </row>
@@ -10026,14 +10178,14 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>8.83</v>
+        <v>8.85</v>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>148, 216, 268, 326, 364, 396, 396, 420, 446</t>
+          <t>148, 216, 268, 326, 364, 396, 396, 419, 420, 446</t>
         </is>
       </c>
     </row>
@@ -10350,14 +10502,14 @@
         </is>
       </c>
       <c r="B59" s="17" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C59" s="17" t="n">
-        <v>9.460000000000001</v>
+        <v>9.43</v>
       </c>
       <c r="D59" s="17" t="inlineStr">
         <is>
-          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 430, 444</t>
+          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 444</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q421-Q425, update Excel (337 entries)
Q421 Physics: Standard Model — quarks, leptons, bosons, Higgs
Q422 Medicine: antibiotic resistance mechanisms and crisis
Q423 Mathematics: Riemann Hypothesis and why it matters
Q424 Psychology: intrinsic vs extrinsic motivation, overjustification
Q425 History: fall of Rome — multicausal, Byzantium survived to 1453

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E333"/>
+  <dimension ref="A1:E338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8536,20 +8536,52 @@
       </c>
     </row>
     <row r="305">
-      <c r="A305" s="12" t="n">
+      <c r="A305" s="6" t="n">
+        <v>421</v>
+      </c>
+      <c r="B305" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="C305" s="7" t="inlineStr">
+        <is>
+          <t>What is the Standard Model of particle physics?</t>
+        </is>
+      </c>
+      <c r="D305" s="7" t="inlineStr">
+        <is>
+          <t>The Standard Model describes all fundamental particles and forces — verified to extraordinary precision, yet incomplete.
+Matter particles (fermions):
+- Quarks (6): up/down/charm/strange/top/bottom. Combine in triplets (protons/neutrons) or pairs (mesons). Never isolated — colour confinement.
+- Leptons (6): electron/muon/tau + neutrinos. Both in 3 generations — reason unknown.
+Force carriers (bosons):
+- Photon: electromagnetic force
+- W+/W-/Z0: weak nuclear force (radioactive decay, solar fusion)
+- Gluons (8): strong nuclear force
+- Higgs boson: gives mass to W/Z and fermions; discovered 2012 CERN
+What it doesn't explain: gravity, dark matter (27%), dark energy (68%), matter-antimatter asymmetry, why 3 generations, neutrino masses.</t>
+        </is>
+      </c>
+      <c r="E305" s="6" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="12" t="n">
         <v>422</v>
       </c>
-      <c r="B305" s="13" t="inlineStr">
+      <c r="B306" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C305" s="13" t="inlineStr">
+      <c r="C306" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the printing press, and did Gutenberg invent it?</t>
         </is>
       </c>
-      <c r="D305" s="13" t="inlineStr">
+      <c r="D306" s="13" t="inlineStr">
         <is>
           <t>Gutenberg (~1450) didn't invent printing. Moveable type existed in China (Bi Sheng ~1040) and Korea (Jikji 1377, oldest surviving). Gutenberg's innovation: complete system — durable metal alloy type, oil-based ink, adapted screw press — optimised for the European alphabet.
 **Why it transformed Europe**: Latin alphabet (26 letters) made moveable type far more efficient than Chinese/Korean systems (thousands of characters). Press: ~3,600 pages/day vs 40 for a scribe.
@@ -8562,25 +8594,57 @@
 **Eisenstein's thesis**: press created new relationship with knowledge — standardisation, reproducibility, verification.</t>
         </is>
       </c>
-      <c r="E305" s="12" t="n">
+      <c r="E306" s="12" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="306">
-      <c r="A306" s="10" t="n">
+    <row r="307">
+      <c r="A307" s="30" t="n">
+        <v>422</v>
+      </c>
+      <c r="B307" s="31" t="inlineStr">
+        <is>
+          <t>Medicine</t>
+        </is>
+      </c>
+      <c r="C307" s="31" t="inlineStr">
+        <is>
+          <t>What is antibiotic resistance and how does it develop?</t>
+        </is>
+      </c>
+      <c r="D307" s="31" t="inlineStr">
+        <is>
+          <t>Antibiotic resistance: bacteria evolve to survive antibiotics. ~700,000 deaths/year; projected 10M/year by 2050.
+Mechanisms:
+1. Enzymatic inactivation: beta-lactamases destroy penicillins
+2. Efflux pumps: actively expel antibiotics
+3. Target modification: alter binding site (MRSA)
+4. Reduced permeability: modified outer membrane
+5. Bypass pathway: alternative metabolic route
+How it spreads: mutation + selection (antibiotics don't cause mutations — they select pre-existing resistant variants); horizontal gene transfer via plasmids (resistance jumps between species).
+Crisis drivers: 50% of prescriptions unnecessary; agriculture uses 70% of global antibiotics; no new antibiotic class since 1987.
+Solutions: phage therapy, antibiotic combinations, new molecular targets, antimicrobial peptides.</t>
+        </is>
+      </c>
+      <c r="E307" s="30" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="10" t="n">
         <v>423</v>
       </c>
-      <c r="B306" s="11" t="inlineStr">
+      <c r="B308" s="11" t="inlineStr">
         <is>
           <t>Neuroscience</t>
         </is>
       </c>
-      <c r="C306" s="11" t="inlineStr">
+      <c r="C308" s="11" t="inlineStr">
         <is>
           <t>What is consciousness and why is it so hard to explain?</t>
         </is>
       </c>
-      <c r="D306" s="11" t="inlineStr">
+      <c r="D308" s="11" t="inlineStr">
         <is>
           <t>Chalmers (1995) 'hard problem': why does information processing produce *subjective experience*? Why is there something it is like to see red?
 Even full neural mapping of correlates wouldn't explain why any of it feels like anything. Explaining function doesn't explain qualia.
@@ -8593,25 +8657,57 @@
 **Consensus**: none. Hard problem remains genuinely open.</t>
         </is>
       </c>
-      <c r="E306" s="10" t="n">
+      <c r="E308" s="10" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="307">
-      <c r="A307" s="28" t="n">
+    <row r="309">
+      <c r="A309" s="14" t="n">
+        <v>423</v>
+      </c>
+      <c r="B309" s="15" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="C309" s="15" t="inlineStr">
+        <is>
+          <t>What is the Riemann Hypothesis and why does it matter?</t>
+        </is>
+      </c>
+      <c r="D309" s="15" t="inlineStr">
+        <is>
+          <t>Riemann (1859): conjecture about zeros of the zeta function. One of 7 Millennium Prize Problems ($1M prize).
+Zeta function: z(s) = 1 + 1/2^s + 1/3^s + ... Analytically continued to whole complex plane.
+Trivial zeros: at s = -2, -4, -6, ... (well understood).
+Non-trivial zeros: all known ones have Re(s) = 1/2 (on the 'critical line').
+The hypothesis: ALL non-trivial zeros have real part exactly 1/2.
+Why it matters:
+- Prime distribution: encodes how closely pi(x) approximates x/ln(x)
+- 1,000+ theorems are conditional on RH
+- Implications for cryptography, quantum chaos, random matrix theory
+Status: proven for first 10^13 zeros. Never proved or disproved.</t>
+        </is>
+      </c>
+      <c r="E309" s="14" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="28" t="n">
         <v>424</v>
       </c>
-      <c r="B307" s="29" t="inlineStr">
+      <c r="B310" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C307" s="29" t="inlineStr">
+      <c r="C310" s="29" t="inlineStr">
         <is>
           <t>What makes some molecules smell while others don't?</t>
         </is>
       </c>
-      <c r="D307" s="29" t="inlineStr">
+      <c r="D310" s="29" t="inlineStr">
         <is>
           <t>Odorant molecules bind to olfactory receptors (ORs, GPCRs) in nasal epithelium -&gt; olfactory bulb -&gt; piriform cortex + limbic system.
 **What molecules smell:**
@@ -8623,25 +8719,54 @@
 **COVID-19 anosmia**: virus destroys olfactory neuron support cells; usually recovers.</t>
         </is>
       </c>
-      <c r="E307" s="28" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" s="8" t="n">
+      <c r="E310" s="28" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="24" t="n">
+        <v>424</v>
+      </c>
+      <c r="B311" s="25" t="inlineStr">
+        <is>
+          <t>Psychology</t>
+        </is>
+      </c>
+      <c r="C311" s="25" t="inlineStr">
+        <is>
+          <t>What is the difference between intrinsic and extrinsic motivation, and does reward kill interest?</t>
+        </is>
+      </c>
+      <c r="D311" s="25" t="inlineStr">
+        <is>
+          <t>Intrinsic motivation: doing something for its own sake — curiosity, enjoyment, challenge.
+Extrinsic motivation: doing it for external rewards or to avoid punishment.
+Overjustification effect (Deci &amp; Ryan, Cognitive Evaluation Theory): expected rewards can undermine intrinsic motivation.
+Classic study (Lepper, Greene &amp; Nisbett 1973): children who loved drawing given expected rewards drew LESS afterward — reframed activity as work done for reward. Unexpected reward group and no-reward group showed no decline.
+Why: reward shifts perceived locus of causality from internal to external. Remove reward — activity loses meaning.
+When rewards don't undermine: unexpected; verbal praise for competence (informational not controlling); tasks never intrinsically interesting; rewards signalling competence.
+Self-Determination Theory (Deci &amp; Ryan): three innate needs — autonomy, competence, relatedness. Controlling environments erode intrinsic motivation.</t>
+        </is>
+      </c>
+      <c r="E311" s="24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="8" t="n">
         <v>425</v>
       </c>
-      <c r="B308" s="9" t="inlineStr">
+      <c r="B312" s="9" t="inlineStr">
         <is>
           <t>Economics</t>
         </is>
       </c>
-      <c r="C308" s="9" t="inlineStr">
+      <c r="C312" s="9" t="inlineStr">
         <is>
           <t>What caused the 2008 financial crisis?</t>
         </is>
       </c>
-      <c r="D308" s="9" t="inlineStr">
+      <c r="D312" s="9" t="inlineStr">
         <is>
           <t>Cascade of failures:
 **Housing bubble**: low post-9/11 rates, relaxed lending, NINJA loans (no income/assets/job). Prices +124% nationally 2000-2006.
@@ -8653,25 +8778,53 @@
 **Response**: Dodd-Frank, Basel III capital requirements, Volcker Rule.</t>
         </is>
       </c>
-      <c r="E308" s="8" t="n">
+      <c r="E312" s="8" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="309">
-      <c r="A309" s="6" t="n">
+    <row r="313">
+      <c r="A313" s="12" t="n">
+        <v>425</v>
+      </c>
+      <c r="B313" s="13" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="C313" s="13" t="inlineStr">
+        <is>
+          <t>How did the Roman Empire fall — and did it really fall?</t>
+        </is>
+      </c>
+      <c r="D313" s="13" t="inlineStr">
+        <is>
+          <t>Conventional end: 476 CE (Romulus Augustulus deposed). But the question is contested.
+Internal factors: military overstretch (10,000km frontier, declining tax base); political instability (50+ emperors in 235-284 CE Crisis); currency debasement and inflation; Diocletian's split (284 CE); Constantine moved capital to Constantinople (330 CE).
+External: Huns pushed Goths across Danube; Visigoths sacked Rome 410 CE; Vandals 455 CE. Climate change; Antonine and Cyprian plagues.
+Historiographical debate: Heather (military/barbarian emphasis) vs Ward-Perkins (catastrophic collapse) vs Goffart (peaceful accommodation — barbarians invited as federates).
+Did it fall? Eastern Empire (Byzantium) continued until 1453 CE. Western institutions transformed: Church preserved Roman law and Latin. Gibbon's 'fall' is partly a narrative choice.
+Consensus: multicausal long unravelling. The real question is why it couldn't adapt.</t>
+        </is>
+      </c>
+      <c r="E313" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="6" t="n">
         <v>426</v>
       </c>
-      <c r="B309" s="7" t="inlineStr">
+      <c r="B314" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C309" s="7" t="inlineStr">
+      <c r="C314" s="7" t="inlineStr">
         <is>
           <t>What is dark matter and how do we know it exists?</t>
         </is>
       </c>
-      <c r="D309" s="7" t="inlineStr">
+      <c r="D314" s="7" t="inlineStr">
         <is>
           <t>~27% of universe's energy. Doesn't emit/absorb/reflect light. Gravitational effects overwhelming.
 **Evidence:**
@@ -8683,25 +8836,25 @@
 **MOND alternative**: modified Newtonian dynamics; cannot explain Bullet Cluster + CMB simultaneously. Most physicists favour particle dark matter.</t>
         </is>
       </c>
-      <c r="E309" s="6" t="n">
+      <c r="E314" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="310">
-      <c r="A310" s="2" t="n">
+    <row r="315">
+      <c r="A315" s="2" t="n">
         <v>427</v>
       </c>
-      <c r="B310" s="3" t="inlineStr">
+      <c r="B315" s="3" t="inlineStr">
         <is>
           <t>Literature</t>
         </is>
       </c>
-      <c r="C310" s="3" t="inlineStr">
+      <c r="C315" s="3" t="inlineStr">
         <is>
           <t>Why is 'Don Quixote' considered the first modern novel?</t>
         </is>
       </c>
-      <c r="D310" s="3" t="inlineStr">
+      <c r="D315" s="3" t="inlineStr">
         <is>
           <t>Cervantes (Part I: 1605, Part II: 1615). Why it's considered the first modern novel:
 1. Self-consciousness: the novel is aware it's a novel. Part II characters have read Part I. Unreliable narrators, manuscript frames — postmodern devices 400 years early.
@@ -8712,25 +8865,25 @@
 What makes it 'modern': fundamentally ambiguous relationship with truth; character who changes across time (Part I vs II Quixote). Bloom: 'most universal and most particular character in literature.'</t>
         </is>
       </c>
-      <c r="E310" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" s="20" t="n">
+      <c r="E315" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="20" t="n">
         <v>428</v>
       </c>
-      <c r="B311" s="21" t="inlineStr">
+      <c r="B316" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C311" s="21" t="inlineStr">
+      <c r="C316" s="21" t="inlineStr">
         <is>
           <t>What is the halting problem and why does it matter?</t>
         </is>
       </c>
-      <c r="D311" s="21" t="inlineStr">
+      <c r="D316" s="21" t="inlineStr">
         <is>
           <t>Turing (1936): no general algorithm can determine whether an arbitrary program will halt or run forever.
 **Proof (diagonal argument)**: assume HALT(P,I) exists. Construct DIAG(P): if HALT says P halts on P -&gt; loop; if HALT says P loops -&gt; halt.
@@ -8743,25 +8896,25 @@
 5. Practical: compilers and static analysers must be incomplete or unsound — they make heuristic approximations.</t>
         </is>
       </c>
-      <c r="E311" s="20" t="n">
+      <c r="E316" s="20" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="312">
-      <c r="A312" s="30" t="n">
+    <row r="317">
+      <c r="A317" s="30" t="n">
         <v>429</v>
       </c>
-      <c r="B312" s="31" t="inlineStr">
+      <c r="B317" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C312" s="31" t="inlineStr">
+      <c r="C317" s="31" t="inlineStr">
         <is>
           <t>How do vaccines work, and why do some require boosters?</t>
         </is>
       </c>
-      <c r="D312" s="31" t="inlineStr">
+      <c r="D317" s="31" t="inlineStr">
         <is>
           <t>Vaccine presents antigen (weakened/killed pathogen, subunit protein, or mRNA) without disease, training immune memory.
 **Mechanism:**
@@ -8778,25 +8931,25 @@
 **Why boosters**: antibody titres wane (inactivated/subunit weaker); mutating viruses (flu) change antigens.</t>
         </is>
       </c>
-      <c r="E312" s="30" t="n">
+      <c r="E317" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="313">
-      <c r="A313" s="16" t="n">
+    <row r="318">
+      <c r="A318" s="16" t="n">
         <v>430</v>
       </c>
-      <c r="B313" s="17" t="inlineStr">
+      <c r="B318" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C313" s="17" t="inlineStr">
+      <c r="C318" s="17" t="inlineStr">
         <is>
           <t>What is free will, and does science undermine it?</t>
         </is>
       </c>
-      <c r="D313" s="17" t="inlineStr">
+      <c r="D318" s="17" t="inlineStr">
         <is>
           <t>Are our choices genuinely ours, or determined by prior causes?
 **Three positions:**
@@ -8808,25 +8961,25 @@
 **Does science undermine it?** Depends what you mean. Compatibilist free will survives. Hard determinism mostly fringe.</t>
         </is>
       </c>
-      <c r="E313" s="16" t="n">
+      <c r="E318" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="314">
-      <c r="A314" s="22" t="n">
+    <row r="319">
+      <c r="A319" s="22" t="n">
         <v>431</v>
       </c>
-      <c r="B314" s="23" t="inlineStr">
+      <c r="B319" s="23" t="inlineStr">
         <is>
           <t>Astronomy</t>
         </is>
       </c>
-      <c r="C314" s="23" t="inlineStr">
+      <c r="C319" s="23" t="inlineStr">
         <is>
           <t>What are neutron stars and how do they form?</t>
         </is>
       </c>
-      <c r="D314" s="23" t="inlineStr">
+      <c r="D319" s="23" t="inlineStr">
         <is>
           <t>Massive star (8-20 solar masses) core collapses. If core mass 1.4-3 solar masses, electron degeneracy fails. Protons + electrons merge (inverse beta decay) -&gt; neutron star.
 **Properties:**
@@ -8839,25 +8992,25 @@
 **Neutron star mergers (GW170817, 2017)**: first gravitational wave + electromagnetic detection. Kilonova: r-process nucleosynthesis produces gold, platinum, uranium. Primary source of heavy elements.</t>
         </is>
       </c>
-      <c r="E314" s="22" t="n">
+      <c r="E319" s="22" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="315">
-      <c r="A315" s="24" t="n">
+    <row r="320">
+      <c r="A320" s="24" t="n">
         <v>432</v>
       </c>
-      <c r="B315" s="25" t="inlineStr">
+      <c r="B320" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C315" s="25" t="inlineStr">
+      <c r="C320" s="25" t="inlineStr">
         <is>
           <t>What is the Dunning-Kruger effect, and is it as universal as people think?</t>
         </is>
       </c>
-      <c r="D315" s="25" t="inlineStr">
+      <c r="D320" s="25" t="inlineStr">
         <is>
           <t>Kruger &amp; Dunning (1999): people with limited knowledge overestimate competence; experts underestimate relative ability (task seems easy to them too).
 **Original study**: bottom quartile performers on logic/grammar/humour overestimated by ~50 percentile points.
@@ -8871,25 +9024,25 @@
 - Domain-specific: expert engineer may still have DK in social skills</t>
         </is>
       </c>
-      <c r="E315" s="24" t="n">
+      <c r="E320" s="24" t="n">
         <v>8.5</v>
       </c>
     </row>
-    <row r="316">
-      <c r="A316" s="12" t="n">
+    <row r="321">
+      <c r="A321" s="12" t="n">
         <v>433</v>
       </c>
-      <c r="B316" s="13" t="inlineStr">
+      <c r="B321" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C316" s="13" t="inlineStr">
+      <c r="C321" s="13" t="inlineStr">
         <is>
           <t>Why did the Roman Empire fall?</t>
         </is>
       </c>
-      <c r="D316" s="13" t="inlineStr">
+      <c r="D321" s="13" t="inlineStr">
         <is>
           <t>Western Empire fell 476 CE (Romulus Augustulus deposed). Eastern Empire (Byzantium) lasted to 1453. No single cause:
 **Military/political:** overextended borders; Germanic foederati with divided loyalty; political instability (50 emperors in 50 years, 235-284 CE); military power to make/unmake emperors.
@@ -8902,25 +9055,25 @@
 **What didn't fall**: Eastern Empire thrived. Fall was primarily western.</t>
         </is>
       </c>
-      <c r="E316" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" s="2" t="n">
+      <c r="E321" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="n">
         <v>434</v>
       </c>
-      <c r="B317" s="3" t="inlineStr">
+      <c r="B322" s="3" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C317" s="3" t="inlineStr">
+      <c r="C322" s="3" t="inlineStr">
         <is>
           <t>How does GPS actually work?</t>
         </is>
       </c>
-      <c r="D317" s="3" t="inlineStr">
+      <c r="D322" s="3" t="inlineStr">
         <is>
           <t>24-32 satellites at ~20,200km; 6 orbital planes; each completes 2 orbits/day.
 **Core principle: trilateration via time signals.**
@@ -8936,25 +9089,25 @@
 - Net: +38 microseconds/day. Without correction: GPS drifts ~10km/day. Einstein's corrections are in the system.</t>
         </is>
       </c>
-      <c r="E317" s="2" t="n">
+      <c r="E322" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="318">
-      <c r="A318" s="18" t="n">
+    <row r="323">
+      <c r="A323" s="18" t="n">
         <v>435</v>
       </c>
-      <c r="B318" s="19" t="inlineStr">
+      <c r="B323" s="19" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C318" s="19" t="inlineStr">
+      <c r="C323" s="19" t="inlineStr">
         <is>
           <t>What is epigenetics and does it challenge our understanding of inheritance?</t>
         </is>
       </c>
-      <c r="D318" s="19" t="inlineStr">
+      <c r="D323" s="19" t="inlineStr">
         <is>
           <t>Heritable changes in gene expression without DNA sequence changes. Genome = instruction manual; epigenome = which instructions are read.
 **Mechanisms:**
@@ -8966,25 +9119,25 @@
 Does NOT validate Lamarck — mechanisms are different from direct inheritance of acquired characteristics.</t>
         </is>
       </c>
-      <c r="E318" s="18" t="n">
+      <c r="E323" s="18" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="319">
-      <c r="A319" s="14" t="n">
+    <row r="324">
+      <c r="A324" s="14" t="n">
         <v>436</v>
       </c>
-      <c r="B319" s="15" t="inlineStr">
+      <c r="B324" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C319" s="15" t="inlineStr">
+      <c r="C324" s="15" t="inlineStr">
         <is>
           <t>What is a prime number, and what do we know about their distribution?</t>
         </is>
       </c>
-      <c r="D319" s="15" t="inlineStr">
+      <c r="D324" s="15" t="inlineStr">
         <is>
           <t>A prime: natural number &gt; 1 with no divisors other than 1 and itself. Euclid (~300 BCE): infinitely many.
 Fundamental Theorem of Arithmetic: every integer &gt; 1 is prime or unique product of primes.
@@ -8996,25 +9149,25 @@
 **Practical importance**: RSA encryption relies on difficulty of factoring large numbers.</t>
         </is>
       </c>
-      <c r="E319" s="14" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" s="24" t="n">
+      <c r="E324" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="24" t="n">
         <v>437</v>
       </c>
-      <c r="B320" s="25" t="inlineStr">
+      <c r="B325" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C320" s="25" t="inlineStr">
+      <c r="C325" s="25" t="inlineStr">
         <is>
           <t>How reliable is eyewitness testimony, and what does the research say?</t>
         </is>
       </c>
-      <c r="D320" s="25" t="inlineStr">
+      <c r="D325" s="25" t="inlineStr">
         <is>
           <t>Memory is reconstructive, not reproductive (Loftus). We rebuild memories each time, subject to suggestion.
 **Key experiments:**
@@ -9025,25 +9178,25 @@
 **What helps**: sequential lineups, blind administration, record initial statement, open questions first.</t>
         </is>
       </c>
-      <c r="E320" s="24" t="n">
+      <c r="E325" s="24" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="321">
-      <c r="A321" s="6" t="n">
+    <row r="326">
+      <c r="A326" s="6" t="n">
         <v>438</v>
       </c>
-      <c r="B321" s="7" t="inlineStr">
+      <c r="B326" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C321" s="7" t="inlineStr">
+      <c r="C326" s="7" t="inlineStr">
         <is>
           <t>What is the difference between heat and temperature?</t>
         </is>
       </c>
-      <c r="D321" s="7" t="inlineStr">
+      <c r="D326" s="7" t="inlineStr">
         <is>
           <t>**Temperature**: average kinetic energy per molecule. Measured in Kelvin/Celsius/Fahrenheit.
 **Heat**: *transfer* of thermal energy between objects due to temperature difference. Heat is a process, not a property. Pool at same temperature as coffee mug: pool contains far more thermal energy.
@@ -9053,25 +9206,25 @@
 **Water vs air at 100C**: water burns much more — higher thermal mass + latent heat of condensation deliver more energy per contact.</t>
         </is>
       </c>
-      <c r="E321" s="6" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" s="2" t="n">
+      <c r="E326" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="2" t="n">
         <v>439</v>
       </c>
-      <c r="B322" s="3" t="inlineStr">
+      <c r="B327" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C322" s="3" t="inlineStr">
+      <c r="C327" s="3" t="inlineStr">
         <is>
           <t>What is structural racism, and how does it differ from individual racism?</t>
         </is>
       </c>
-      <c r="D322" s="3" t="inlineStr">
+      <c r="D327" s="3" t="inlineStr">
         <is>
           <t>**Individual racism**: prejudice and discriminatory acts by identifiable individuals. Overt bias.
 **Structural racism**: racial disparities from systems, policies, norms — even without individual racist intent.
@@ -9083,25 +9236,25 @@
 **Evidence**: audit studies (identical CVs with Black vs white names) consistently find measurable hiring discrimination.</t>
         </is>
       </c>
-      <c r="E322" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" s="26" t="n">
+      <c r="E327" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="26" t="n">
         <v>440</v>
       </c>
-      <c r="B323" s="27" t="inlineStr">
+      <c r="B328" s="27" t="inlineStr">
         <is>
           <t>Ecology</t>
         </is>
       </c>
-      <c r="C323" s="27" t="inlineStr">
+      <c r="C328" s="27" t="inlineStr">
         <is>
           <t>What is the nitrogen cycle and why is it essential for life?</t>
         </is>
       </c>
-      <c r="D323" s="27" t="inlineStr">
+      <c r="D328" s="27" t="inlineStr">
         <is>
           <t>N2 = 78% of atmosphere, but most organisms can't use N2 (triple bond N=N, 945 kJ/mol). Life needs reactive N (NH3, NO3-, organic N).
 **Nitrogen cycle:**
@@ -9113,25 +9266,25 @@
 **Limiting nutrient**: N limits most ecosystems. Excess (fertilisers) -&gt; eutrophication -&gt; algal blooms -&gt; oxygen depletion -&gt; dead zones (Gulf of Mexico). Haber also weaponised N (chlorine, phosgene).</t>
         </is>
       </c>
-      <c r="E323" s="26" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" s="30" t="n">
+      <c r="E328" s="26" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="30" t="n">
         <v>441</v>
       </c>
-      <c r="B324" s="31" t="inlineStr">
+      <c r="B329" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C324" s="31" t="inlineStr">
+      <c r="C329" s="31" t="inlineStr">
         <is>
           <t>What is antibiotic resistance and how does it develop?</t>
         </is>
       </c>
-      <c r="D324" s="31" t="inlineStr">
+      <c r="D329" s="31" t="inlineStr">
         <is>
           <t>Antibiotics target cell wall (penicillin), protein synthesis (tetracycline), DNA replication (fluoroquinolones), or membranes. Resistance = survival.
 **Darwinian mechanism:**
@@ -9145,25 +9298,25 @@
 **Why few new antibiotics**: 10-15yr development; brief low-cost use = poor financial incentive vs lifelong drugs.</t>
         </is>
       </c>
-      <c r="E324" s="30" t="n">
+      <c r="E329" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="325">
-      <c r="A325" s="12" t="n">
+    <row r="330">
+      <c r="A330" s="12" t="n">
         <v>442</v>
       </c>
-      <c r="B325" s="13" t="inlineStr">
+      <c r="B330" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C325" s="13" t="inlineStr">
+      <c r="C330" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the Magna Carta?</t>
         </is>
       </c>
-      <c r="D325" s="13" t="inlineStr">
+      <c r="D330" s="13" t="inlineStr">
         <is>
           <t>June 1215: English barons forced King John to sign. Originally limited royal power in narrow feudal ways — mostly barons' rights, not ordinary people.
 **Key clauses**: Cl. 39 — no free man imprisoned without lawful judgment of peers ('due process'); Cl. 40 — no selling/denying justice.
@@ -9173,25 +9326,25 @@
 **Lasting principle**: rule of law over arbitrary power -&gt; constitutional government, habeas corpus, human rights.</t>
         </is>
       </c>
-      <c r="E325" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" s="20" t="n">
+      <c r="E330" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="20" t="n">
         <v>443</v>
       </c>
-      <c r="B326" s="21" t="inlineStr">
+      <c r="B331" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C326" s="21" t="inlineStr">
+      <c r="C331" s="21" t="inlineStr">
         <is>
           <t>What is machine learning and how is it different from traditional programming?</t>
         </is>
       </c>
-      <c r="D326" s="21" t="inlineStr">
+      <c r="D331" s="21" t="inlineStr">
         <is>
           <t>**Traditional programming**: programmer writes explicit rules. Input + rules -&gt; output. Brittle; can't generalise.
 **Machine learning**: provide data + correct answers; algorithm finds the rules. Input + labels -&gt; model -&gt; generalises to new data.
@@ -9204,25 +9357,25 @@
 **Scale**: LLMs (GPT, Claude) = transformers on trillions of tokens; emergent capabilities at scale.</t>
         </is>
       </c>
-      <c r="E326" s="20" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" s="16" t="n">
+      <c r="E331" s="20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="16" t="n">
         <v>444</v>
       </c>
-      <c r="B327" s="17" t="inlineStr">
+      <c r="B332" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C327" s="17" t="inlineStr">
+      <c r="C332" s="17" t="inlineStr">
         <is>
           <t>What is the ship of Theseus paradox, and what is it really asking?</t>
         </is>
       </c>
-      <c r="D327" s="17" t="inlineStr">
+      <c r="D332" s="17" t="inlineStr">
         <is>
           <t>Plutarch (~100 CE): every plank of Theseus's ship replaced over time. Still the same ship?
 **Hobbes extension**: original planks collected and reassembled. Two ships claim to be the original. Which is it?
@@ -9236,25 +9389,25 @@
 **Parfit** (*Reasons and Persons*): personal identity is not what matters — psychological continuity is what matters; 'same' may be an empty question.</t>
         </is>
       </c>
-      <c r="E327" s="16" t="n">
+      <c r="E332" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="328">
-      <c r="A328" s="2" t="n">
+    <row r="333">
+      <c r="A333" s="2" t="n">
         <v>445</v>
       </c>
-      <c r="B328" s="3" t="inlineStr">
+      <c r="B333" s="3" t="inlineStr">
         <is>
           <t>Music</t>
         </is>
       </c>
-      <c r="C328" s="3" t="inlineStr">
+      <c r="C333" s="3" t="inlineStr">
         <is>
           <t>Why does music make us emotional?</t>
         </is>
       </c>
-      <c r="D328" s="3" t="inlineStr">
+      <c r="D333" s="3" t="inlineStr">
         <is>
           <t>Multiple converging mechanisms:
 1. **Expectation/violation** (Meyer 1956, Huron 2006): music is temporal prediction. Correct resolution = dopaminergic reward. Surprise + resolution = stronger reward. Chills = surprising resolution.
@@ -9266,25 +9419,25 @@
 **Mystery of sad music pleasure**: safe simulation, hormonal empathy reward, artistic resolution — distinct emotion from actual grief.</t>
         </is>
       </c>
-      <c r="E328" s="2" t="n">
+      <c r="E333" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="329">
-      <c r="A329" s="4" t="n">
+    <row r="334">
+      <c r="A334" s="4" t="n">
         <v>446</v>
       </c>
-      <c r="B329" s="5" t="inlineStr">
+      <c r="B334" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="C329" s="5" t="inlineStr">
+      <c r="C334" s="5" t="inlineStr">
         <is>
           <t>How do children acquire language so rapidly?</t>
         </is>
       </c>
-      <c r="D329" s="5" t="inlineStr">
+      <c r="D334" s="5" t="inlineStr">
         <is>
           <t>First words ~12 months, two-word phrases ~18-24 months, complex sentences by 3-4 years — from imperfect, fragmented input.
 **Poverty of the stimulus**: children overgeneralise rules ('goed', 'mouses') but never make wrong rule errors. Acquire structure-dependent rules without examples of errors.
@@ -9296,25 +9449,25 @@
 **Mechanisms**: statistical learning (8-month-olds track syllable transition probabilities), joint attention, motherese (simplified grammar + exaggerated prosody).</t>
         </is>
       </c>
-      <c r="E329" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" s="6" t="n">
+      <c r="E334" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="6" t="n">
         <v>447</v>
       </c>
-      <c r="B330" s="7" t="inlineStr">
+      <c r="B335" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C330" s="7" t="inlineStr">
+      <c r="C335" s="7" t="inlineStr">
         <is>
           <t>What is the photoelectric effect, and why did it matter for quantum mechanics?</t>
         </is>
       </c>
-      <c r="D330" s="7" t="inlineStr">
+      <c r="D335" s="7" t="inlineStr">
         <is>
           <t>Light hits metal -&gt; electrons ejected, BUT only above a threshold frequency. Below threshold: no electrons regardless of intensity.
 **Classical prediction**: intensity drives ejection. WRONG.
@@ -9327,25 +9480,25 @@
 4. Technology: photovoltaics, CCDs, photomultipliers</t>
         </is>
       </c>
-      <c r="E330" s="6" t="n">
+      <c r="E335" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="331">
-      <c r="A331" s="2" t="n">
+    <row r="336">
+      <c r="A336" s="2" t="n">
         <v>448</v>
       </c>
-      <c r="B331" s="3" t="inlineStr">
+      <c r="B336" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C331" s="3" t="inlineStr">
+      <c r="C336" s="3" t="inlineStr">
         <is>
           <t>What is social mobility and what actually predicts it?</t>
         </is>
       </c>
-      <c r="D331" s="3" t="inlineStr">
+      <c r="D336" s="3" t="inlineStr">
         <is>
           <t>Movement between socioeconomic strata. Intergenerational (parent to child) vs intragenerational (within lifetime).
 **Great Gatsby Curve** (Miles Corak): more income inequality -&gt; LOWER intergenerational mobility. Denmark (low inequality) = high mobility; US, UK = lower.
@@ -9358,25 +9511,25 @@
 Absolute mobility (exceeding parents in absolute terms) has historically been high; relative mobility much more constrained.</t>
         </is>
       </c>
-      <c r="E331" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" s="28" t="n">
+      <c r="E336" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="28" t="n">
         <v>449</v>
       </c>
-      <c r="B332" s="29" t="inlineStr">
+      <c r="B337" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C332" s="29" t="inlineStr">
+      <c r="C337" s="29" t="inlineStr">
         <is>
           <t>How do batteries work chemically, and what limits their energy density?</t>
         </is>
       </c>
-      <c r="D332" s="29" t="inlineStr">
+      <c r="D337" s="29" t="inlineStr">
         <is>
           <t>Battery = chemical -&gt; electrical energy via spatially separated redox reactions.
 Anode: oxidation (loses electrons). Cathode: reduction (gains electrons). Electrons flow externally (current); ions flow internally through electrolyte.
@@ -9393,25 +9546,25 @@
 **Theoretical limits**: Li-ion ~265 Wh/kg practical; Li-sulfur 2,600 Wh/kg; Li-air 11,680 Wh/kg (comparable to gasoline).</t>
         </is>
       </c>
-      <c r="E332" s="28" t="n">
+      <c r="E337" s="28" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="333">
-      <c r="A333" s="2" t="n">
+    <row r="338">
+      <c r="A338" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="B333" s="3" t="inlineStr">
+      <c r="B338" s="3" t="inlineStr">
         <is>
           <t>General Knowledge</t>
         </is>
       </c>
-      <c r="C333" s="3" t="inlineStr">
+      <c r="C338" s="3" t="inlineStr">
         <is>
           <t>What is the most important invention in human history, and why?</t>
         </is>
       </c>
-      <c r="D333" s="3" t="inlineStr">
+      <c r="D338" s="3" t="inlineStr">
         <is>
           <t>Depends on dimension valued. Four strong candidates:
 **Language**: meta-invention enabling all others to accumulate. But may have evolved rather than been invented.
@@ -9423,7 +9576,7 @@
 **Meta-point**: no invention stands alone. Cumulative innovation is humanity's real superpower.</t>
         </is>
       </c>
-      <c r="E333" s="2" t="n">
+      <c r="E338" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10052,14 +10205,14 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C34" s="13" t="n">
-        <v>9.130000000000001</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 433, 442</t>
+          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 442</t>
         </is>
       </c>
     </row>
@@ -10250,14 +10403,14 @@
         </is>
       </c>
       <c r="B45" s="15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C45" s="15" t="n">
         <v>9.56</v>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 436</t>
+          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436</t>
         </is>
       </c>
     </row>
@@ -10286,14 +10439,14 @@
         </is>
       </c>
       <c r="B47" s="31" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C47" s="31" t="n">
-        <v>9.199999999999999</v>
+        <v>9.18</v>
       </c>
       <c r="D47" s="31" t="inlineStr">
         <is>
-          <t>230, 279, 294, 344, 379, 395, 411, 411, 429, 441</t>
+          <t>230, 279, 294, 344, 379, 395, 411, 411, 422, 429, 441</t>
         </is>
       </c>
     </row>
@@ -10628,14 +10781,14 @@
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>9.59</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 426, 438, 447</t>
+          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 438, 447</t>
         </is>
       </c>
     </row>
@@ -10700,14 +10853,14 @@
         </is>
       </c>
       <c r="B70" s="25" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C70" s="25" t="n">
-        <v>9.119999999999999</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="D70" s="25" t="inlineStr">
         <is>
-          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 432, 437</t>
+          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 424, 432, 437</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q426-Q430, update Excel (342 entries)
Q426 CS: halting problem — Turing 1936, undecidability, Rice's theorem
Q427 Astronomy: dark matter — rotation curves, Bullet Cluster, WIMPs
Q428 Sociology: Milgram experiment — 65% max shock, agentic state
Q429 Chemistry: chemical bonds — ionic/covalent/metallic/hydrogen/vdW
Q430 Philosophy: hard problem of consciousness — Chalmers, panpsychism, IIT

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E338"/>
+  <dimension ref="A1:E343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8841,20 +8841,51 @@
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="2" t="n">
+      <c r="A315" s="20" t="n">
+        <v>426</v>
+      </c>
+      <c r="B315" s="21" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="C315" s="21" t="inlineStr">
+        <is>
+          <t>What is the halting problem and why does it matter?</t>
+        </is>
+      </c>
+      <c r="D315" s="21" t="inlineStr">
+        <is>
+          <t>Turing (1936): no general algorithm can determine whether every program halts or runs forever. Mathematically impossible, not just hard.
+Proof by contradiction: assume HALT(P,I) exists. Construct PARADOX: if HALT says it halts, it loops; if HALT says it loops, it halts. Contradiction either way — HALT cannot exist.
+Why it matters:
+- Limits of computation: some problems are formally undecidable
+- Software verification: no general program can check arbitrary code for infinite loops
+- Virus detection: perfect general malware detection is provably impossible
+- Equivalent to Godel: Turing's undecidability = Godel's incompleteness — same phenomenon
+- Rice's theorem: any non-trivial semantic property of programs is undecidable
+What it doesn't mean: specific programs CAN be verified. Impossibility is for the general case.</t>
+        </is>
+      </c>
+      <c r="E315" s="20" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="2" t="n">
         <v>427</v>
       </c>
-      <c r="B315" s="3" t="inlineStr">
+      <c r="B316" s="3" t="inlineStr">
         <is>
           <t>Literature</t>
         </is>
       </c>
-      <c r="C315" s="3" t="inlineStr">
+      <c r="C316" s="3" t="inlineStr">
         <is>
           <t>Why is 'Don Quixote' considered the first modern novel?</t>
         </is>
       </c>
-      <c r="D315" s="3" t="inlineStr">
+      <c r="D316" s="3" t="inlineStr">
         <is>
           <t>Cervantes (Part I: 1605, Part II: 1615). Why it's considered the first modern novel:
 1. Self-consciousness: the novel is aware it's a novel. Part II characters have read Part I. Unreliable narrators, manuscript frames — postmodern devices 400 years early.
@@ -8865,25 +8896,57 @@
 What makes it 'modern': fundamentally ambiguous relationship with truth; character who changes across time (Part I vs II Quixote). Bloom: 'most universal and most particular character in literature.'</t>
         </is>
       </c>
-      <c r="E315" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" s="20" t="n">
+      <c r="E316" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="22" t="n">
+        <v>427</v>
+      </c>
+      <c r="B317" s="23" t="inlineStr">
+        <is>
+          <t>Astronomy</t>
+        </is>
+      </c>
+      <c r="C317" s="23" t="inlineStr">
+        <is>
+          <t>What is dark matter — and do we actually know it exists?</t>
+        </is>
+      </c>
+      <c r="D317" s="23" t="inlineStr">
+        <is>
+          <t>Dark matter: ~27% of universe mass-energy; doesn't emit/absorb/reflect light but exerts gravity.
+Evidence (indirect but overwhelming):
+1. Galaxy rotation curves (Vera Rubin 1970s): flat curves — outer stars orbit as fast as inner; implies invisible halos
+2. Gravitational lensing: bends more than visible matter explains
+3. Bullet Cluster (2006): colliding galaxy clusters — hot gas slowed by collision, gravitational mass passed through unimpeded
+4. CMB acoustic oscillations fit only with ~27% dark matter
+5. Galaxy formation simulations only work with dark matter
+What it isn't: WIMPs not found at LHC; black holes ruled out as dominant component.
+Alternative: MOND (Modified Newtonian Dynamics) — explains rotation curves but fails on clusters and CMB.
+Status: extremely confident something real causes these effects. No confirmed particle identity.</t>
+        </is>
+      </c>
+      <c r="E317" s="22" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="20" t="n">
         <v>428</v>
       </c>
-      <c r="B316" s="21" t="inlineStr">
+      <c r="B318" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C316" s="21" t="inlineStr">
+      <c r="C318" s="21" t="inlineStr">
         <is>
           <t>What is the halting problem and why does it matter?</t>
         </is>
       </c>
-      <c r="D316" s="21" t="inlineStr">
+      <c r="D318" s="21" t="inlineStr">
         <is>
           <t>Turing (1936): no general algorithm can determine whether an arbitrary program will halt or run forever.
 **Proof (diagonal argument)**: assume HALT(P,I) exists. Construct DIAG(P): if HALT says P halts on P -&gt; loop; if HALT says P loops -&gt; halt.
@@ -8896,25 +8959,57 @@
 5. Practical: compilers and static analysers must be incomplete or unsound — they make heuristic approximations.</t>
         </is>
       </c>
-      <c r="E316" s="20" t="n">
+      <c r="E318" s="20" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="317">
-      <c r="A317" s="30" t="n">
+    <row r="319">
+      <c r="A319" s="2" t="n">
+        <v>428</v>
+      </c>
+      <c r="B319" s="3" t="inlineStr">
+        <is>
+          <t>Sociology</t>
+        </is>
+      </c>
+      <c r="C319" s="3" t="inlineStr">
+        <is>
+          <t>What is the Milgram experiment and what does it tell us about obedience?</t>
+        </is>
+      </c>
+      <c r="D319" s="3" t="inlineStr">
+        <is>
+          <t>Milgram (Yale, 1961-63): prompted by Holocaust — can ordinary people commit atrocities under authority?
+Setup: participants as 'teachers' administer electric shocks (15V-450V XXX) to a 'learner' (confederate) for wrong answers, urged by experimenter in lab coat.
+Result: 65% administered maximum 450V. Nobody stopped before 300V.
+What it shows:
+- Situational power over character: ordinary people, not sadists, complied
+- Agentic state: people see themselves as instruments of authority; moral responsibility feels transferred
+- Incremental commitment: each step small; prior compliance makes refusal harder
+- Legitimacy of authority: lab coat, Yale, scientific framing reduced questioning
+Critiques: Burger (2009) replicated at 70%; ecological validity questioned; Gina Perry found some knew learner was faking.
+Legacy: changed research ethics (deception now regulated); illuminates genocide, corporate wrongdoing, everyday compliance.</t>
+        </is>
+      </c>
+      <c r="E319" s="2" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="30" t="n">
         <v>429</v>
       </c>
-      <c r="B317" s="31" t="inlineStr">
+      <c r="B320" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C317" s="31" t="inlineStr">
+      <c r="C320" s="31" t="inlineStr">
         <is>
           <t>How do vaccines work, and why do some require boosters?</t>
         </is>
       </c>
-      <c r="D317" s="31" t="inlineStr">
+      <c r="D320" s="31" t="inlineStr">
         <is>
           <t>Vaccine presents antigen (weakened/killed pathogen, subunit protein, or mRNA) without disease, training immune memory.
 **Mechanism:**
@@ -8931,25 +9026,54 @@
 **Why boosters**: antibody titres wane (inactivated/subunit weaker); mutating viruses (flu) change antigens.</t>
         </is>
       </c>
-      <c r="E317" s="30" t="n">
+      <c r="E320" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="318">
-      <c r="A318" s="16" t="n">
+    <row r="321">
+      <c r="A321" s="28" t="n">
+        <v>429</v>
+      </c>
+      <c r="B321" s="29" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="C321" s="29" t="inlineStr">
+        <is>
+          <t>What is a chemical bond and what are the different types?</t>
+        </is>
+      </c>
+      <c r="D321" s="29" t="inlineStr">
+        <is>
+          <t>A chemical bond is an attractive force holding atoms together. Bond type determines substance properties.
+Ionic: electron transfer (metal to non-metal) -&gt; oppositely charged ions. NaCl. High melting point, brittle, conducts when dissolved.
+Covalent: shared electrons. Non-metals bonding. Single/double/triple. Polar covalent: unequal sharing (H2O — O pulls electrons). Lower melting points, poor conductors.
+Metallic: cations in sea of delocalised electrons. Electrons free to move. Conducts electricity and heat; malleable, ductile.
+Hydrogen bonds: not a true bond — electrostatic attraction between H bonded to F/O/N and another F/O/N. Responsible for water's high boiling point, surface tension, ice floating, DNA base pairing, protein folding.
+Van der Waals: temporary dipole-induced dipole. Weakest. Why noble gases liquify; why geckos stick to walls.
+Strength: ionic ≈ covalent &gt; metallic &gt;&gt; hydrogen &gt;&gt; van der Waals.</t>
+        </is>
+      </c>
+      <c r="E321" s="28" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="16" t="n">
         <v>430</v>
       </c>
-      <c r="B318" s="17" t="inlineStr">
+      <c r="B322" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C318" s="17" t="inlineStr">
+      <c r="C322" s="17" t="inlineStr">
         <is>
           <t>What is free will, and does science undermine it?</t>
         </is>
       </c>
-      <c r="D318" s="17" t="inlineStr">
+      <c r="D322" s="17" t="inlineStr">
         <is>
           <t>Are our choices genuinely ours, or determined by prior causes?
 **Three positions:**
@@ -8961,25 +9085,56 @@
 **Does science undermine it?** Depends what you mean. Compatibilist free will survives. Hard determinism mostly fringe.</t>
         </is>
       </c>
-      <c r="E318" s="16" t="n">
+      <c r="E322" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="319">
-      <c r="A319" s="22" t="n">
+    <row r="323">
+      <c r="A323" s="16" t="n">
+        <v>430</v>
+      </c>
+      <c r="B323" s="17" t="inlineStr">
+        <is>
+          <t>Philosophy</t>
+        </is>
+      </c>
+      <c r="C323" s="17" t="inlineStr">
+        <is>
+          <t>What is consciousness and why is it so hard to explain?</t>
+        </is>
+      </c>
+      <c r="D323" s="17" t="inlineStr">
+        <is>
+          <t>Hard problem (Chalmers 1995): why does physical brain activity produce subjective experience — the redness of red, painfulness of pain? Distinct from 'easy problems' (attention, memory, behaviour).
+Why hard: even complete neuroscience of colour processing wouldn't explain why there's something it FEELS like to see red. Philosophical zombie (physically identical, no inner experience) seems conceivable — suggests consciousness isn't logically entailed by physical facts.
+Major positions:
+1. Physicalism/Materialism: consciousness is brain activity; hard problem is confused (Dennett: consciousness is a 'user illusion')
+2. Dualism (Descartes): mind and matter distinct substances. Problem: how do they interact?
+3. Property dualism: one substance with physical and phenomenal properties
+4. Panpsychism: consciousness fundamental and ubiquitous; combination problem: how do micro-experiences unify?
+5. Illusionism (Frankish): phenomenal consciousness is an introspective illusion
+Scientific approaches: Global Workspace Theory (Baars), Integrated Information Theory (Tononi IIT), Higher Order Theories. None solves the hard problem.</t>
+        </is>
+      </c>
+      <c r="E323" s="16" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="22" t="n">
         <v>431</v>
       </c>
-      <c r="B319" s="23" t="inlineStr">
+      <c r="B324" s="23" t="inlineStr">
         <is>
           <t>Astronomy</t>
         </is>
       </c>
-      <c r="C319" s="23" t="inlineStr">
+      <c r="C324" s="23" t="inlineStr">
         <is>
           <t>What are neutron stars and how do they form?</t>
         </is>
       </c>
-      <c r="D319" s="23" t="inlineStr">
+      <c r="D324" s="23" t="inlineStr">
         <is>
           <t>Massive star (8-20 solar masses) core collapses. If core mass 1.4-3 solar masses, electron degeneracy fails. Protons + electrons merge (inverse beta decay) -&gt; neutron star.
 **Properties:**
@@ -8992,25 +9147,25 @@
 **Neutron star mergers (GW170817, 2017)**: first gravitational wave + electromagnetic detection. Kilonova: r-process nucleosynthesis produces gold, platinum, uranium. Primary source of heavy elements.</t>
         </is>
       </c>
-      <c r="E319" s="22" t="n">
+      <c r="E324" s="22" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="320">
-      <c r="A320" s="24" t="n">
+    <row r="325">
+      <c r="A325" s="24" t="n">
         <v>432</v>
       </c>
-      <c r="B320" s="25" t="inlineStr">
+      <c r="B325" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C320" s="25" t="inlineStr">
+      <c r="C325" s="25" t="inlineStr">
         <is>
           <t>What is the Dunning-Kruger effect, and is it as universal as people think?</t>
         </is>
       </c>
-      <c r="D320" s="25" t="inlineStr">
+      <c r="D325" s="25" t="inlineStr">
         <is>
           <t>Kruger &amp; Dunning (1999): people with limited knowledge overestimate competence; experts underestimate relative ability (task seems easy to them too).
 **Original study**: bottom quartile performers on logic/grammar/humour overestimated by ~50 percentile points.
@@ -9024,25 +9179,25 @@
 - Domain-specific: expert engineer may still have DK in social skills</t>
         </is>
       </c>
-      <c r="E320" s="24" t="n">
+      <c r="E325" s="24" t="n">
         <v>8.5</v>
       </c>
     </row>
-    <row r="321">
-      <c r="A321" s="12" t="n">
+    <row r="326">
+      <c r="A326" s="12" t="n">
         <v>433</v>
       </c>
-      <c r="B321" s="13" t="inlineStr">
+      <c r="B326" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C321" s="13" t="inlineStr">
+      <c r="C326" s="13" t="inlineStr">
         <is>
           <t>Why did the Roman Empire fall?</t>
         </is>
       </c>
-      <c r="D321" s="13" t="inlineStr">
+      <c r="D326" s="13" t="inlineStr">
         <is>
           <t>Western Empire fell 476 CE (Romulus Augustulus deposed). Eastern Empire (Byzantium) lasted to 1453. No single cause:
 **Military/political:** overextended borders; Germanic foederati with divided loyalty; political instability (50 emperors in 50 years, 235-284 CE); military power to make/unmake emperors.
@@ -9055,25 +9210,25 @@
 **What didn't fall**: Eastern Empire thrived. Fall was primarily western.</t>
         </is>
       </c>
-      <c r="E321" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" s="2" t="n">
+      <c r="E326" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="2" t="n">
         <v>434</v>
       </c>
-      <c r="B322" s="3" t="inlineStr">
+      <c r="B327" s="3" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C322" s="3" t="inlineStr">
+      <c r="C327" s="3" t="inlineStr">
         <is>
           <t>How does GPS actually work?</t>
         </is>
       </c>
-      <c r="D322" s="3" t="inlineStr">
+      <c r="D327" s="3" t="inlineStr">
         <is>
           <t>24-32 satellites at ~20,200km; 6 orbital planes; each completes 2 orbits/day.
 **Core principle: trilateration via time signals.**
@@ -9089,25 +9244,25 @@
 - Net: +38 microseconds/day. Without correction: GPS drifts ~10km/day. Einstein's corrections are in the system.</t>
         </is>
       </c>
-      <c r="E322" s="2" t="n">
+      <c r="E327" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="323">
-      <c r="A323" s="18" t="n">
+    <row r="328">
+      <c r="A328" s="18" t="n">
         <v>435</v>
       </c>
-      <c r="B323" s="19" t="inlineStr">
+      <c r="B328" s="19" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C323" s="19" t="inlineStr">
+      <c r="C328" s="19" t="inlineStr">
         <is>
           <t>What is epigenetics and does it challenge our understanding of inheritance?</t>
         </is>
       </c>
-      <c r="D323" s="19" t="inlineStr">
+      <c r="D328" s="19" t="inlineStr">
         <is>
           <t>Heritable changes in gene expression without DNA sequence changes. Genome = instruction manual; epigenome = which instructions are read.
 **Mechanisms:**
@@ -9119,25 +9274,25 @@
 Does NOT validate Lamarck — mechanisms are different from direct inheritance of acquired characteristics.</t>
         </is>
       </c>
-      <c r="E323" s="18" t="n">
+      <c r="E328" s="18" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="324">
-      <c r="A324" s="14" t="n">
+    <row r="329">
+      <c r="A329" s="14" t="n">
         <v>436</v>
       </c>
-      <c r="B324" s="15" t="inlineStr">
+      <c r="B329" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C324" s="15" t="inlineStr">
+      <c r="C329" s="15" t="inlineStr">
         <is>
           <t>What is a prime number, and what do we know about their distribution?</t>
         </is>
       </c>
-      <c r="D324" s="15" t="inlineStr">
+      <c r="D329" s="15" t="inlineStr">
         <is>
           <t>A prime: natural number &gt; 1 with no divisors other than 1 and itself. Euclid (~300 BCE): infinitely many.
 Fundamental Theorem of Arithmetic: every integer &gt; 1 is prime or unique product of primes.
@@ -9149,25 +9304,25 @@
 **Practical importance**: RSA encryption relies on difficulty of factoring large numbers.</t>
         </is>
       </c>
-      <c r="E324" s="14" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" s="24" t="n">
+      <c r="E329" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="24" t="n">
         <v>437</v>
       </c>
-      <c r="B325" s="25" t="inlineStr">
+      <c r="B330" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C325" s="25" t="inlineStr">
+      <c r="C330" s="25" t="inlineStr">
         <is>
           <t>How reliable is eyewitness testimony, and what does the research say?</t>
         </is>
       </c>
-      <c r="D325" s="25" t="inlineStr">
+      <c r="D330" s="25" t="inlineStr">
         <is>
           <t>Memory is reconstructive, not reproductive (Loftus). We rebuild memories each time, subject to suggestion.
 **Key experiments:**
@@ -9178,25 +9333,25 @@
 **What helps**: sequential lineups, blind administration, record initial statement, open questions first.</t>
         </is>
       </c>
-      <c r="E325" s="24" t="n">
+      <c r="E330" s="24" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="326">
-      <c r="A326" s="6" t="n">
+    <row r="331">
+      <c r="A331" s="6" t="n">
         <v>438</v>
       </c>
-      <c r="B326" s="7" t="inlineStr">
+      <c r="B331" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C326" s="7" t="inlineStr">
+      <c r="C331" s="7" t="inlineStr">
         <is>
           <t>What is the difference between heat and temperature?</t>
         </is>
       </c>
-      <c r="D326" s="7" t="inlineStr">
+      <c r="D331" s="7" t="inlineStr">
         <is>
           <t>**Temperature**: average kinetic energy per molecule. Measured in Kelvin/Celsius/Fahrenheit.
 **Heat**: *transfer* of thermal energy between objects due to temperature difference. Heat is a process, not a property. Pool at same temperature as coffee mug: pool contains far more thermal energy.
@@ -9206,25 +9361,25 @@
 **Water vs air at 100C**: water burns much more — higher thermal mass + latent heat of condensation deliver more energy per contact.</t>
         </is>
       </c>
-      <c r="E326" s="6" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" s="2" t="n">
+      <c r="E331" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="n">
         <v>439</v>
       </c>
-      <c r="B327" s="3" t="inlineStr">
+      <c r="B332" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C327" s="3" t="inlineStr">
+      <c r="C332" s="3" t="inlineStr">
         <is>
           <t>What is structural racism, and how does it differ from individual racism?</t>
         </is>
       </c>
-      <c r="D327" s="3" t="inlineStr">
+      <c r="D332" s="3" t="inlineStr">
         <is>
           <t>**Individual racism**: prejudice and discriminatory acts by identifiable individuals. Overt bias.
 **Structural racism**: racial disparities from systems, policies, norms — even without individual racist intent.
@@ -9236,25 +9391,25 @@
 **Evidence**: audit studies (identical CVs with Black vs white names) consistently find measurable hiring discrimination.</t>
         </is>
       </c>
-      <c r="E327" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" s="26" t="n">
+      <c r="E332" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="26" t="n">
         <v>440</v>
       </c>
-      <c r="B328" s="27" t="inlineStr">
+      <c r="B333" s="27" t="inlineStr">
         <is>
           <t>Ecology</t>
         </is>
       </c>
-      <c r="C328" s="27" t="inlineStr">
+      <c r="C333" s="27" t="inlineStr">
         <is>
           <t>What is the nitrogen cycle and why is it essential for life?</t>
         </is>
       </c>
-      <c r="D328" s="27" t="inlineStr">
+      <c r="D333" s="27" t="inlineStr">
         <is>
           <t>N2 = 78% of atmosphere, but most organisms can't use N2 (triple bond N=N, 945 kJ/mol). Life needs reactive N (NH3, NO3-, organic N).
 **Nitrogen cycle:**
@@ -9266,25 +9421,25 @@
 **Limiting nutrient**: N limits most ecosystems. Excess (fertilisers) -&gt; eutrophication -&gt; algal blooms -&gt; oxygen depletion -&gt; dead zones (Gulf of Mexico). Haber also weaponised N (chlorine, phosgene).</t>
         </is>
       </c>
-      <c r="E328" s="26" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" s="30" t="n">
+      <c r="E333" s="26" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="30" t="n">
         <v>441</v>
       </c>
-      <c r="B329" s="31" t="inlineStr">
+      <c r="B334" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C329" s="31" t="inlineStr">
+      <c r="C334" s="31" t="inlineStr">
         <is>
           <t>What is antibiotic resistance and how does it develop?</t>
         </is>
       </c>
-      <c r="D329" s="31" t="inlineStr">
+      <c r="D334" s="31" t="inlineStr">
         <is>
           <t>Antibiotics target cell wall (penicillin), protein synthesis (tetracycline), DNA replication (fluoroquinolones), or membranes. Resistance = survival.
 **Darwinian mechanism:**
@@ -9298,25 +9453,25 @@
 **Why few new antibiotics**: 10-15yr development; brief low-cost use = poor financial incentive vs lifelong drugs.</t>
         </is>
       </c>
-      <c r="E329" s="30" t="n">
+      <c r="E334" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="330">
-      <c r="A330" s="12" t="n">
+    <row r="335">
+      <c r="A335" s="12" t="n">
         <v>442</v>
       </c>
-      <c r="B330" s="13" t="inlineStr">
+      <c r="B335" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C330" s="13" t="inlineStr">
+      <c r="C335" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the Magna Carta?</t>
         </is>
       </c>
-      <c r="D330" s="13" t="inlineStr">
+      <c r="D335" s="13" t="inlineStr">
         <is>
           <t>June 1215: English barons forced King John to sign. Originally limited royal power in narrow feudal ways — mostly barons' rights, not ordinary people.
 **Key clauses**: Cl. 39 — no free man imprisoned without lawful judgment of peers ('due process'); Cl. 40 — no selling/denying justice.
@@ -9326,25 +9481,25 @@
 **Lasting principle**: rule of law over arbitrary power -&gt; constitutional government, habeas corpus, human rights.</t>
         </is>
       </c>
-      <c r="E330" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="331">
-      <c r="A331" s="20" t="n">
+      <c r="E335" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="20" t="n">
         <v>443</v>
       </c>
-      <c r="B331" s="21" t="inlineStr">
+      <c r="B336" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C331" s="21" t="inlineStr">
+      <c r="C336" s="21" t="inlineStr">
         <is>
           <t>What is machine learning and how is it different from traditional programming?</t>
         </is>
       </c>
-      <c r="D331" s="21" t="inlineStr">
+      <c r="D336" s="21" t="inlineStr">
         <is>
           <t>**Traditional programming**: programmer writes explicit rules. Input + rules -&gt; output. Brittle; can't generalise.
 **Machine learning**: provide data + correct answers; algorithm finds the rules. Input + labels -&gt; model -&gt; generalises to new data.
@@ -9357,25 +9512,25 @@
 **Scale**: LLMs (GPT, Claude) = transformers on trillions of tokens; emergent capabilities at scale.</t>
         </is>
       </c>
-      <c r="E331" s="20" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" s="16" t="n">
+      <c r="E336" s="20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="16" t="n">
         <v>444</v>
       </c>
-      <c r="B332" s="17" t="inlineStr">
+      <c r="B337" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C332" s="17" t="inlineStr">
+      <c r="C337" s="17" t="inlineStr">
         <is>
           <t>What is the ship of Theseus paradox, and what is it really asking?</t>
         </is>
       </c>
-      <c r="D332" s="17" t="inlineStr">
+      <c r="D337" s="17" t="inlineStr">
         <is>
           <t>Plutarch (~100 CE): every plank of Theseus's ship replaced over time. Still the same ship?
 **Hobbes extension**: original planks collected and reassembled. Two ships claim to be the original. Which is it?
@@ -9389,25 +9544,25 @@
 **Parfit** (*Reasons and Persons*): personal identity is not what matters — psychological continuity is what matters; 'same' may be an empty question.</t>
         </is>
       </c>
-      <c r="E332" s="16" t="n">
+      <c r="E337" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="333">
-      <c r="A333" s="2" t="n">
+    <row r="338">
+      <c r="A338" s="2" t="n">
         <v>445</v>
       </c>
-      <c r="B333" s="3" t="inlineStr">
+      <c r="B338" s="3" t="inlineStr">
         <is>
           <t>Music</t>
         </is>
       </c>
-      <c r="C333" s="3" t="inlineStr">
+      <c r="C338" s="3" t="inlineStr">
         <is>
           <t>Why does music make us emotional?</t>
         </is>
       </c>
-      <c r="D333" s="3" t="inlineStr">
+      <c r="D338" s="3" t="inlineStr">
         <is>
           <t>Multiple converging mechanisms:
 1. **Expectation/violation** (Meyer 1956, Huron 2006): music is temporal prediction. Correct resolution = dopaminergic reward. Surprise + resolution = stronger reward. Chills = surprising resolution.
@@ -9419,25 +9574,25 @@
 **Mystery of sad music pleasure**: safe simulation, hormonal empathy reward, artistic resolution — distinct emotion from actual grief.</t>
         </is>
       </c>
-      <c r="E333" s="2" t="n">
+      <c r="E338" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="334">
-      <c r="A334" s="4" t="n">
+    <row r="339">
+      <c r="A339" s="4" t="n">
         <v>446</v>
       </c>
-      <c r="B334" s="5" t="inlineStr">
+      <c r="B339" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="C334" s="5" t="inlineStr">
+      <c r="C339" s="5" t="inlineStr">
         <is>
           <t>How do children acquire language so rapidly?</t>
         </is>
       </c>
-      <c r="D334" s="5" t="inlineStr">
+      <c r="D339" s="5" t="inlineStr">
         <is>
           <t>First words ~12 months, two-word phrases ~18-24 months, complex sentences by 3-4 years — from imperfect, fragmented input.
 **Poverty of the stimulus**: children overgeneralise rules ('goed', 'mouses') but never make wrong rule errors. Acquire structure-dependent rules without examples of errors.
@@ -9449,25 +9604,25 @@
 **Mechanisms**: statistical learning (8-month-olds track syllable transition probabilities), joint attention, motherese (simplified grammar + exaggerated prosody).</t>
         </is>
       </c>
-      <c r="E334" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="335">
-      <c r="A335" s="6" t="n">
+      <c r="E339" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="6" t="n">
         <v>447</v>
       </c>
-      <c r="B335" s="7" t="inlineStr">
+      <c r="B340" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C335" s="7" t="inlineStr">
+      <c r="C340" s="7" t="inlineStr">
         <is>
           <t>What is the photoelectric effect, and why did it matter for quantum mechanics?</t>
         </is>
       </c>
-      <c r="D335" s="7" t="inlineStr">
+      <c r="D340" s="7" t="inlineStr">
         <is>
           <t>Light hits metal -&gt; electrons ejected, BUT only above a threshold frequency. Below threshold: no electrons regardless of intensity.
 **Classical prediction**: intensity drives ejection. WRONG.
@@ -9480,25 +9635,25 @@
 4. Technology: photovoltaics, CCDs, photomultipliers</t>
         </is>
       </c>
-      <c r="E335" s="6" t="n">
+      <c r="E340" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="336">
-      <c r="A336" s="2" t="n">
+    <row r="341">
+      <c r="A341" s="2" t="n">
         <v>448</v>
       </c>
-      <c r="B336" s="3" t="inlineStr">
+      <c r="B341" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C336" s="3" t="inlineStr">
+      <c r="C341" s="3" t="inlineStr">
         <is>
           <t>What is social mobility and what actually predicts it?</t>
         </is>
       </c>
-      <c r="D336" s="3" t="inlineStr">
+      <c r="D341" s="3" t="inlineStr">
         <is>
           <t>Movement between socioeconomic strata. Intergenerational (parent to child) vs intragenerational (within lifetime).
 **Great Gatsby Curve** (Miles Corak): more income inequality -&gt; LOWER intergenerational mobility. Denmark (low inequality) = high mobility; US, UK = lower.
@@ -9511,25 +9666,25 @@
 Absolute mobility (exceeding parents in absolute terms) has historically been high; relative mobility much more constrained.</t>
         </is>
       </c>
-      <c r="E336" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" s="28" t="n">
+      <c r="E341" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="28" t="n">
         <v>449</v>
       </c>
-      <c r="B337" s="29" t="inlineStr">
+      <c r="B342" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C337" s="29" t="inlineStr">
+      <c r="C342" s="29" t="inlineStr">
         <is>
           <t>How do batteries work chemically, and what limits their energy density?</t>
         </is>
       </c>
-      <c r="D337" s="29" t="inlineStr">
+      <c r="D342" s="29" t="inlineStr">
         <is>
           <t>Battery = chemical -&gt; electrical energy via spatially separated redox reactions.
 Anode: oxidation (loses electrons). Cathode: reduction (gains electrons). Electrons flow externally (current); ions flow internally through electrolyte.
@@ -9546,25 +9701,25 @@
 **Theoretical limits**: Li-ion ~265 Wh/kg practical; Li-sulfur 2,600 Wh/kg; Li-air 11,680 Wh/kg (comparable to gasoline).</t>
         </is>
       </c>
-      <c r="E337" s="28" t="n">
+      <c r="E342" s="28" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="338">
-      <c r="A338" s="2" t="n">
+    <row r="343">
+      <c r="A343" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="B338" s="3" t="inlineStr">
+      <c r="B343" s="3" t="inlineStr">
         <is>
           <t>General Knowledge</t>
         </is>
       </c>
-      <c r="C338" s="3" t="inlineStr">
+      <c r="C343" s="3" t="inlineStr">
         <is>
           <t>What is the most important invention in human history, and why?</t>
         </is>
       </c>
-      <c r="D338" s="3" t="inlineStr">
+      <c r="D343" s="3" t="inlineStr">
         <is>
           <t>Depends on dimension valued. Four strong candidates:
 **Language**: meta-invention enabling all others to accumulate. But may have evolved rather than been invented.
@@ -9576,7 +9731,7 @@
 **Meta-point**: no invention stands alone. Cumulative innovation is humanity's real superpower.</t>
         </is>
       </c>
-      <c r="E338" s="2" t="n">
+      <c r="E343" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9701,14 +9856,14 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>9.57</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>158, 173, 219, 240, 259, 278, 292, 309, 357, 375, 389, 406, 408, 431</t>
+          <t>158, 173, 219, 240, 259, 278, 292, 309, 357, 375, 389, 406, 408, 427, 431</t>
         </is>
       </c>
     </row>
@@ -9809,14 +9964,14 @@
         </is>
       </c>
       <c r="B12" s="29" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" s="29" t="n">
-        <v>9.09</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>212, 233, 245, 274, 334, 365, 391, 406, 408, 424, 449</t>
+          <t>212, 233, 245, 274, 334, 365, 391, 406, 408, 424, 429, 449</t>
         </is>
       </c>
     </row>
@@ -9899,14 +10054,14 @@
         </is>
       </c>
       <c r="B17" s="21" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C17" s="21" t="n">
-        <v>9.289999999999999</v>
+        <v>9.31</v>
       </c>
       <c r="D17" s="21" t="inlineStr">
         <is>
-          <t>157, 184, 252, 258, 352, 377, 388, 398, 398, 409, 428, 443</t>
+          <t>157, 184, 252, 258, 352, 377, 388, 398, 398, 409, 426, 428, 443</t>
         </is>
       </c>
     </row>
@@ -10655,14 +10810,14 @@
         </is>
       </c>
       <c r="B59" s="17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C59" s="17" t="n">
-        <v>9.43</v>
+        <v>9.44</v>
       </c>
       <c r="D59" s="17" t="inlineStr">
         <is>
-          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 444</t>
+          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 444</t>
         </is>
       </c>
     </row>
@@ -10907,14 +11062,14 @@
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C73" s="3" t="n">
-        <v>9.029999999999999</v>
+        <v>9.06</v>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 413, 439, 448</t>
+          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 413, 428, 439, 448</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q431-Q435, update Excel (347 entries)
Q431 Biology: epigenetics — DNA methylation, Dutch Hunger Winter
Q432 Economics: game theory — Nash equilibrium, Prisoner's Dilemma
Q433 Physics: nuclear fission — E=mc2, chain reaction, reactor vs bomb
Q434 Literature: what makes great literature — intersubjective standard
Q435 Neuroscience: sleep — glymphatic clearance, memory consolidation

Also: recovered stalled training, restarted with unbuffered output

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E343"/>
+  <dimension ref="A1:E348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9152,20 +9152,53 @@
       </c>
     </row>
     <row r="325">
-      <c r="A325" s="24" t="n">
+      <c r="A325" s="18" t="n">
+        <v>431</v>
+      </c>
+      <c r="B325" s="19" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C325" s="19" t="inlineStr">
+        <is>
+          <t>What is epigenetics and how does environment affect gene expression?</t>
+        </is>
+      </c>
+      <c r="D325" s="19" t="inlineStr">
+        <is>
+          <t>Epigenetics: heritable changes in gene expression without DNA sequence changes. The genome is fixed; the epigenome is dynamic.
+Core mechanisms:
+- DNA methylation: methyl groups silence genes (CpG sites). Passed through cell division.
+- Histone modification: acetylation/methylation of histone tails changes DNA packing — loose=expressed, tight=silenced
+- Non-coding RNA: microRNAs regulate transcription/translation
+Environmental effects:
+- Diet: folate/B12 donate methyl groups. Dutch Hunger Winter (1944-45): starved mothers' children had altered methylation decades later — higher obesity and heart disease rates
+- Stress: glucocorticoids alter HPA axis methylation — lifelong altered stress reactivity
+- Toxins: BPA, tobacco, air pollution alter methylation
+- Exercise: induces epigenetic changes in muscle metabolism genes
+Transgenerational inheritance: some marks survive reprogramming (Overkalix cohort — grandfather food supply predicts grandson mortality). Mechanistically controversial.</t>
+        </is>
+      </c>
+      <c r="E325" s="18" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="24" t="n">
         <v>432</v>
       </c>
-      <c r="B325" s="25" t="inlineStr">
+      <c r="B326" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C325" s="25" t="inlineStr">
+      <c r="C326" s="25" t="inlineStr">
         <is>
           <t>What is the Dunning-Kruger effect, and is it as universal as people think?</t>
         </is>
       </c>
-      <c r="D325" s="25" t="inlineStr">
+      <c r="D326" s="25" t="inlineStr">
         <is>
           <t>Kruger &amp; Dunning (1999): people with limited knowledge overestimate competence; experts underestimate relative ability (task seems easy to them too).
 **Original study**: bottom quartile performers on logic/grammar/humour overestimated by ~50 percentile points.
@@ -9179,25 +9212,56 @@
 - Domain-specific: expert engineer may still have DK in social skills</t>
         </is>
       </c>
-      <c r="E325" s="24" t="n">
+      <c r="E326" s="24" t="n">
         <v>8.5</v>
       </c>
     </row>
-    <row r="326">
-      <c r="A326" s="12" t="n">
+    <row r="327">
+      <c r="A327" s="8" t="n">
+        <v>432</v>
+      </c>
+      <c r="B327" s="9" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="C327" s="9" t="inlineStr">
+        <is>
+          <t>What is game theory and what has it explained?</t>
+        </is>
+      </c>
+      <c r="D327" s="9" t="inlineStr">
+        <is>
+          <t>Game theory: mathematical study of strategic interaction among rational agents. Von Neumann &amp; Morgenstern (1944); Nash equilibrium (1950).
+Nash Equilibrium: no player can improve outcome by unilaterally changing strategy. Not necessarily the best collective outcome.
+Prisoner's Dilemma: both defecting is Nash equilibrium even though mutual cooperation is better — individually rational choices produce collectively bad outcomes.
+What it explains:
+- Arms races (defect-defect equilibrium)
+- Auction design: Vickrey auctions, spectrum auctions (Nobel 2020, Milgrom &amp; Wilson)
+- Evolutionary biology: hawk-dove game, evolutionarily stable strategies (Maynard Smith)
+- Voting theory, trade negotiations, antibiotic resistance (each patient defects by demanding antibiotics)
+Limits: assumes rationality; people reject unfair offers even at personal cost (ultimatum game); tit-for-tat wins in repeated games (Axelrod tournaments).</t>
+        </is>
+      </c>
+      <c r="E327" s="8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="12" t="n">
         <v>433</v>
       </c>
-      <c r="B326" s="13" t="inlineStr">
+      <c r="B328" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C326" s="13" t="inlineStr">
+      <c r="C328" s="13" t="inlineStr">
         <is>
           <t>Why did the Roman Empire fall?</t>
         </is>
       </c>
-      <c r="D326" s="13" t="inlineStr">
+      <c r="D328" s="13" t="inlineStr">
         <is>
           <t>Western Empire fell 476 CE (Romulus Augustulus deposed). Eastern Empire (Byzantium) lasted to 1453. No single cause:
 **Military/political:** overextended borders; Germanic foederati with divided loyalty; political instability (50 emperors in 50 years, 235-284 CE); military power to make/unmake emperors.
@@ -9210,25 +9274,54 @@
 **What didn't fall**: Eastern Empire thrived. Fall was primarily western.</t>
         </is>
       </c>
-      <c r="E326" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" s="2" t="n">
+      <c r="E328" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="6" t="n">
+        <v>433</v>
+      </c>
+      <c r="B329" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="C329" s="7" t="inlineStr">
+        <is>
+          <t>How does nuclear fission work and why does it release so much energy?</t>
+        </is>
+      </c>
+      <c r="D329" s="7" t="inlineStr">
+        <is>
+          <t>Nuclear fission: heavy nucleus (U-235 or Pu-239) splits into two smaller nuclei + 2-3 neutrons + energy.
+Why so much energy: products weigh LESS than original (mass defect ~0.1%). Missing mass converted to energy via E=mc^2. U-235 releases ~200 MeV per fission vs few eV for coal — ~50 million times more energy per reaction.
+Chain reaction: neutron strikes U-235 -&gt; unstable U-236 -&gt; splits -&gt; 200 MeV + 2-3 neutrons -&gt; each strikes another U-235. If each fission produces &gt;= 1 subsequent: reaction sustains. Critical mass for pure U-235: ~52 kg sphere.
+Reactor vs bomb:
+- Reactor: controlled (k≈1), control rods absorb neutrons, moderator slows them
+- Bomb: supercritical (k&gt;&gt;1), exponential chain reaction in microseconds
+Binding energy curve: iron-56 has highest binding energy per nucleon. Heavier nuclei release energy by fission; lighter by fusion.</t>
+        </is>
+      </c>
+      <c r="E329" s="6" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="n">
         <v>434</v>
       </c>
-      <c r="B327" s="3" t="inlineStr">
+      <c r="B330" s="3" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="C327" s="3" t="inlineStr">
+      <c r="C330" s="3" t="inlineStr">
         <is>
           <t>How does GPS actually work?</t>
         </is>
       </c>
-      <c r="D327" s="3" t="inlineStr">
+      <c r="D330" s="3" t="inlineStr">
         <is>
           <t>24-32 satellites at ~20,200km; 6 orbital planes; each completes 2 orbits/day.
 **Core principle: trilateration via time signals.**
@@ -9244,25 +9337,58 @@
 - Net: +38 microseconds/day. Without correction: GPS drifts ~10km/day. Einstein's corrections are in the system.</t>
         </is>
       </c>
-      <c r="E327" s="2" t="n">
+      <c r="E330" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="328">
-      <c r="A328" s="18" t="n">
+    <row r="331">
+      <c r="A331" s="2" t="n">
+        <v>434</v>
+      </c>
+      <c r="B331" s="3" t="inlineStr">
+        <is>
+          <t>Literature</t>
+        </is>
+      </c>
+      <c r="C331" s="3" t="inlineStr">
+        <is>
+          <t>What makes great literature great — is there an objective standard?</t>
+        </is>
+      </c>
+      <c r="D331" s="3" t="inlineStr">
+        <is>
+          <t>Contested but not without structure.
+Arguments for objective standards:
+- Longevity: works surviving centuries across cultures generate inexhaustible new interpretations
+- Formal complexity: density of language, structural sophistication, earned ambiguity
+- Cognitive depth: literary fiction readers score higher on theory of mind tasks (Mar &amp; Oatley research)
+- Bloom's aesthetic value: surprise that becomes inevitable; strong misreading
+Arguments against:
+- Canons excluded women and non-Western voices — 'greatness' tracked power
+- Reader response (Iser, Fish): meaning is relational, completed by the reader
+- Bourdieu: literary taste is class distinction, not intrinsic merit
+Middle ground: quality judgments are intersubjective — built through critical conversation over time. Some texts reward rereading across centuries; that persistence is evidence of something, if not proof of absolute value.</t>
+        </is>
+      </c>
+      <c r="E331" s="2" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="18" t="n">
         <v>435</v>
       </c>
-      <c r="B328" s="19" t="inlineStr">
+      <c r="B332" s="19" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="C328" s="19" t="inlineStr">
+      <c r="C332" s="19" t="inlineStr">
         <is>
           <t>What is epigenetics and does it challenge our understanding of inheritance?</t>
         </is>
       </c>
-      <c r="D328" s="19" t="inlineStr">
+      <c r="D332" s="19" t="inlineStr">
         <is>
           <t>Heritable changes in gene expression without DNA sequence changes. Genome = instruction manual; epigenome = which instructions are read.
 **Mechanisms:**
@@ -9274,25 +9400,60 @@
 Does NOT validate Lamarck — mechanisms are different from direct inheritance of acquired characteristics.</t>
         </is>
       </c>
-      <c r="E328" s="18" t="n">
+      <c r="E332" s="18" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="329">
-      <c r="A329" s="14" t="n">
+    <row r="333">
+      <c r="A333" s="10" t="n">
+        <v>435</v>
+      </c>
+      <c r="B333" s="11" t="inlineStr">
+        <is>
+          <t>Neuroscience</t>
+        </is>
+      </c>
+      <c r="C333" s="11" t="inlineStr">
+        <is>
+          <t>How does sleep work and why do we need it?</t>
+        </is>
+      </c>
+      <c r="D333" s="11" t="inlineStr">
+        <is>
+          <t>Sleep is active and essential — rats deprived die in ~3 weeks.
+Architecture (90-min cycles, 4-6/night):
+- NREM 1/2: light sleep, sleep spindles
+- NREM 3 (slow-wave): delta waves, most restorative
+- REM: dreaming, brain nearly as active as waking, muscle atonia
+Early cycles: more deep sleep. Later cycles: more REM.
+Why we need it:
+- Memory consolidation: hippocampus replays experiences -&gt; transfers to neocortex for long-term storage
+- Glymphatic clearance (Nedergaard 2013): brain cells shrink 60%, CSF flushes amyloid-beta and other metabolic waste
+- Immune function: cytokine production, immune suppression without sleep
+- Synaptic homeostasis (Tononi/Cirelli): waking strengthens synapses; sleep downscales them
+- Metabolic: deprivation increases ghrelin (hunger), decreases leptin (satiety)
+Sleep debt not infinitely recoverable. Caffeine masks impairment without restoring function.</t>
+        </is>
+      </c>
+      <c r="E333" s="10" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="14" t="n">
         <v>436</v>
       </c>
-      <c r="B329" s="15" t="inlineStr">
+      <c r="B334" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="C329" s="15" t="inlineStr">
+      <c r="C334" s="15" t="inlineStr">
         <is>
           <t>What is a prime number, and what do we know about their distribution?</t>
         </is>
       </c>
-      <c r="D329" s="15" t="inlineStr">
+      <c r="D334" s="15" t="inlineStr">
         <is>
           <t>A prime: natural number &gt; 1 with no divisors other than 1 and itself. Euclid (~300 BCE): infinitely many.
 Fundamental Theorem of Arithmetic: every integer &gt; 1 is prime or unique product of primes.
@@ -9304,25 +9465,25 @@
 **Practical importance**: RSA encryption relies on difficulty of factoring large numbers.</t>
         </is>
       </c>
-      <c r="E329" s="14" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" s="24" t="n">
+      <c r="E334" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="24" t="n">
         <v>437</v>
       </c>
-      <c r="B330" s="25" t="inlineStr">
+      <c r="B335" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C330" s="25" t="inlineStr">
+      <c r="C335" s="25" t="inlineStr">
         <is>
           <t>How reliable is eyewitness testimony, and what does the research say?</t>
         </is>
       </c>
-      <c r="D330" s="25" t="inlineStr">
+      <c r="D335" s="25" t="inlineStr">
         <is>
           <t>Memory is reconstructive, not reproductive (Loftus). We rebuild memories each time, subject to suggestion.
 **Key experiments:**
@@ -9333,25 +9494,25 @@
 **What helps**: sequential lineups, blind administration, record initial statement, open questions first.</t>
         </is>
       </c>
-      <c r="E330" s="24" t="n">
+      <c r="E335" s="24" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="331">
-      <c r="A331" s="6" t="n">
+    <row r="336">
+      <c r="A336" s="6" t="n">
         <v>438</v>
       </c>
-      <c r="B331" s="7" t="inlineStr">
+      <c r="B336" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C331" s="7" t="inlineStr">
+      <c r="C336" s="7" t="inlineStr">
         <is>
           <t>What is the difference between heat and temperature?</t>
         </is>
       </c>
-      <c r="D331" s="7" t="inlineStr">
+      <c r="D336" s="7" t="inlineStr">
         <is>
           <t>**Temperature**: average kinetic energy per molecule. Measured in Kelvin/Celsius/Fahrenheit.
 **Heat**: *transfer* of thermal energy between objects due to temperature difference. Heat is a process, not a property. Pool at same temperature as coffee mug: pool contains far more thermal energy.
@@ -9361,25 +9522,25 @@
 **Water vs air at 100C**: water burns much more — higher thermal mass + latent heat of condensation deliver more energy per contact.</t>
         </is>
       </c>
-      <c r="E331" s="6" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" s="2" t="n">
+      <c r="E336" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="n">
         <v>439</v>
       </c>
-      <c r="B332" s="3" t="inlineStr">
+      <c r="B337" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C332" s="3" t="inlineStr">
+      <c r="C337" s="3" t="inlineStr">
         <is>
           <t>What is structural racism, and how does it differ from individual racism?</t>
         </is>
       </c>
-      <c r="D332" s="3" t="inlineStr">
+      <c r="D337" s="3" t="inlineStr">
         <is>
           <t>**Individual racism**: prejudice and discriminatory acts by identifiable individuals. Overt bias.
 **Structural racism**: racial disparities from systems, policies, norms — even without individual racist intent.
@@ -9391,25 +9552,25 @@
 **Evidence**: audit studies (identical CVs with Black vs white names) consistently find measurable hiring discrimination.</t>
         </is>
       </c>
-      <c r="E332" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="333">
-      <c r="A333" s="26" t="n">
+      <c r="E337" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="26" t="n">
         <v>440</v>
       </c>
-      <c r="B333" s="27" t="inlineStr">
+      <c r="B338" s="27" t="inlineStr">
         <is>
           <t>Ecology</t>
         </is>
       </c>
-      <c r="C333" s="27" t="inlineStr">
+      <c r="C338" s="27" t="inlineStr">
         <is>
           <t>What is the nitrogen cycle and why is it essential for life?</t>
         </is>
       </c>
-      <c r="D333" s="27" t="inlineStr">
+      <c r="D338" s="27" t="inlineStr">
         <is>
           <t>N2 = 78% of atmosphere, but most organisms can't use N2 (triple bond N=N, 945 kJ/mol). Life needs reactive N (NH3, NO3-, organic N).
 **Nitrogen cycle:**
@@ -9421,25 +9582,25 @@
 **Limiting nutrient**: N limits most ecosystems. Excess (fertilisers) -&gt; eutrophication -&gt; algal blooms -&gt; oxygen depletion -&gt; dead zones (Gulf of Mexico). Haber also weaponised N (chlorine, phosgene).</t>
         </is>
       </c>
-      <c r="E333" s="26" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="334">
-      <c r="A334" s="30" t="n">
+      <c r="E338" s="26" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="30" t="n">
         <v>441</v>
       </c>
-      <c r="B334" s="31" t="inlineStr">
+      <c r="B339" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C334" s="31" t="inlineStr">
+      <c r="C339" s="31" t="inlineStr">
         <is>
           <t>What is antibiotic resistance and how does it develop?</t>
         </is>
       </c>
-      <c r="D334" s="31" t="inlineStr">
+      <c r="D339" s="31" t="inlineStr">
         <is>
           <t>Antibiotics target cell wall (penicillin), protein synthesis (tetracycline), DNA replication (fluoroquinolones), or membranes. Resistance = survival.
 **Darwinian mechanism:**
@@ -9453,25 +9614,25 @@
 **Why few new antibiotics**: 10-15yr development; brief low-cost use = poor financial incentive vs lifelong drugs.</t>
         </is>
       </c>
-      <c r="E334" s="30" t="n">
+      <c r="E339" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="335">
-      <c r="A335" s="12" t="n">
+    <row r="340">
+      <c r="A340" s="12" t="n">
         <v>442</v>
       </c>
-      <c r="B335" s="13" t="inlineStr">
+      <c r="B340" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C335" s="13" t="inlineStr">
+      <c r="C340" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the Magna Carta?</t>
         </is>
       </c>
-      <c r="D335" s="13" t="inlineStr">
+      <c r="D340" s="13" t="inlineStr">
         <is>
           <t>June 1215: English barons forced King John to sign. Originally limited royal power in narrow feudal ways — mostly barons' rights, not ordinary people.
 **Key clauses**: Cl. 39 — no free man imprisoned without lawful judgment of peers ('due process'); Cl. 40 — no selling/denying justice.
@@ -9481,25 +9642,25 @@
 **Lasting principle**: rule of law over arbitrary power -&gt; constitutional government, habeas corpus, human rights.</t>
         </is>
       </c>
-      <c r="E335" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="336">
-      <c r="A336" s="20" t="n">
+      <c r="E340" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="20" t="n">
         <v>443</v>
       </c>
-      <c r="B336" s="21" t="inlineStr">
+      <c r="B341" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C336" s="21" t="inlineStr">
+      <c r="C341" s="21" t="inlineStr">
         <is>
           <t>What is machine learning and how is it different from traditional programming?</t>
         </is>
       </c>
-      <c r="D336" s="21" t="inlineStr">
+      <c r="D341" s="21" t="inlineStr">
         <is>
           <t>**Traditional programming**: programmer writes explicit rules. Input + rules -&gt; output. Brittle; can't generalise.
 **Machine learning**: provide data + correct answers; algorithm finds the rules. Input + labels -&gt; model -&gt; generalises to new data.
@@ -9512,25 +9673,25 @@
 **Scale**: LLMs (GPT, Claude) = transformers on trillions of tokens; emergent capabilities at scale.</t>
         </is>
       </c>
-      <c r="E336" s="20" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" s="16" t="n">
+      <c r="E341" s="20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="16" t="n">
         <v>444</v>
       </c>
-      <c r="B337" s="17" t="inlineStr">
+      <c r="B342" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C337" s="17" t="inlineStr">
+      <c r="C342" s="17" t="inlineStr">
         <is>
           <t>What is the ship of Theseus paradox, and what is it really asking?</t>
         </is>
       </c>
-      <c r="D337" s="17" t="inlineStr">
+      <c r="D342" s="17" t="inlineStr">
         <is>
           <t>Plutarch (~100 CE): every plank of Theseus's ship replaced over time. Still the same ship?
 **Hobbes extension**: original planks collected and reassembled. Two ships claim to be the original. Which is it?
@@ -9544,25 +9705,25 @@
 **Parfit** (*Reasons and Persons*): personal identity is not what matters — psychological continuity is what matters; 'same' may be an empty question.</t>
         </is>
       </c>
-      <c r="E337" s="16" t="n">
+      <c r="E342" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="338">
-      <c r="A338" s="2" t="n">
+    <row r="343">
+      <c r="A343" s="2" t="n">
         <v>445</v>
       </c>
-      <c r="B338" s="3" t="inlineStr">
+      <c r="B343" s="3" t="inlineStr">
         <is>
           <t>Music</t>
         </is>
       </c>
-      <c r="C338" s="3" t="inlineStr">
+      <c r="C343" s="3" t="inlineStr">
         <is>
           <t>Why does music make us emotional?</t>
         </is>
       </c>
-      <c r="D338" s="3" t="inlineStr">
+      <c r="D343" s="3" t="inlineStr">
         <is>
           <t>Multiple converging mechanisms:
 1. **Expectation/violation** (Meyer 1956, Huron 2006): music is temporal prediction. Correct resolution = dopaminergic reward. Surprise + resolution = stronger reward. Chills = surprising resolution.
@@ -9574,25 +9735,25 @@
 **Mystery of sad music pleasure**: safe simulation, hormonal empathy reward, artistic resolution — distinct emotion from actual grief.</t>
         </is>
       </c>
-      <c r="E338" s="2" t="n">
+      <c r="E343" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="339">
-      <c r="A339" s="4" t="n">
+    <row r="344">
+      <c r="A344" s="4" t="n">
         <v>446</v>
       </c>
-      <c r="B339" s="5" t="inlineStr">
+      <c r="B344" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="C339" s="5" t="inlineStr">
+      <c r="C344" s="5" t="inlineStr">
         <is>
           <t>How do children acquire language so rapidly?</t>
         </is>
       </c>
-      <c r="D339" s="5" t="inlineStr">
+      <c r="D344" s="5" t="inlineStr">
         <is>
           <t>First words ~12 months, two-word phrases ~18-24 months, complex sentences by 3-4 years — from imperfect, fragmented input.
 **Poverty of the stimulus**: children overgeneralise rules ('goed', 'mouses') but never make wrong rule errors. Acquire structure-dependent rules without examples of errors.
@@ -9604,25 +9765,25 @@
 **Mechanisms**: statistical learning (8-month-olds track syllable transition probabilities), joint attention, motherese (simplified grammar + exaggerated prosody).</t>
         </is>
       </c>
-      <c r="E339" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" s="6" t="n">
+      <c r="E344" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="6" t="n">
         <v>447</v>
       </c>
-      <c r="B340" s="7" t="inlineStr">
+      <c r="B345" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C340" s="7" t="inlineStr">
+      <c r="C345" s="7" t="inlineStr">
         <is>
           <t>What is the photoelectric effect, and why did it matter for quantum mechanics?</t>
         </is>
       </c>
-      <c r="D340" s="7" t="inlineStr">
+      <c r="D345" s="7" t="inlineStr">
         <is>
           <t>Light hits metal -&gt; electrons ejected, BUT only above a threshold frequency. Below threshold: no electrons regardless of intensity.
 **Classical prediction**: intensity drives ejection. WRONG.
@@ -9635,25 +9796,25 @@
 4. Technology: photovoltaics, CCDs, photomultipliers</t>
         </is>
       </c>
-      <c r="E340" s="6" t="n">
+      <c r="E345" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="341">
-      <c r="A341" s="2" t="n">
+    <row r="346">
+      <c r="A346" s="2" t="n">
         <v>448</v>
       </c>
-      <c r="B341" s="3" t="inlineStr">
+      <c r="B346" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C341" s="3" t="inlineStr">
+      <c r="C346" s="3" t="inlineStr">
         <is>
           <t>What is social mobility and what actually predicts it?</t>
         </is>
       </c>
-      <c r="D341" s="3" t="inlineStr">
+      <c r="D346" s="3" t="inlineStr">
         <is>
           <t>Movement between socioeconomic strata. Intergenerational (parent to child) vs intragenerational (within lifetime).
 **Great Gatsby Curve** (Miles Corak): more income inequality -&gt; LOWER intergenerational mobility. Denmark (low inequality) = high mobility; US, UK = lower.
@@ -9666,25 +9827,25 @@
 Absolute mobility (exceeding parents in absolute terms) has historically been high; relative mobility much more constrained.</t>
         </is>
       </c>
-      <c r="E341" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" s="28" t="n">
+      <c r="E346" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="28" t="n">
         <v>449</v>
       </c>
-      <c r="B342" s="29" t="inlineStr">
+      <c r="B347" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C342" s="29" t="inlineStr">
+      <c r="C347" s="29" t="inlineStr">
         <is>
           <t>How do batteries work chemically, and what limits their energy density?</t>
         </is>
       </c>
-      <c r="D342" s="29" t="inlineStr">
+      <c r="D347" s="29" t="inlineStr">
         <is>
           <t>Battery = chemical -&gt; electrical energy via spatially separated redox reactions.
 Anode: oxidation (loses electrons). Cathode: reduction (gains electrons). Electrons flow externally (current); ions flow internally through electrolyte.
@@ -9701,25 +9862,25 @@
 **Theoretical limits**: Li-ion ~265 Wh/kg practical; Li-sulfur 2,600 Wh/kg; Li-air 11,680 Wh/kg (comparable to gasoline).</t>
         </is>
       </c>
-      <c r="E342" s="28" t="n">
+      <c r="E347" s="28" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="343">
-      <c r="A343" s="2" t="n">
+    <row r="348">
+      <c r="A348" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="B343" s="3" t="inlineStr">
+      <c r="B348" s="3" t="inlineStr">
         <is>
           <t>General Knowledge</t>
         </is>
       </c>
-      <c r="C343" s="3" t="inlineStr">
+      <c r="C348" s="3" t="inlineStr">
         <is>
           <t>What is the most important invention in human history, and why?</t>
         </is>
       </c>
-      <c r="D343" s="3" t="inlineStr">
+      <c r="D348" s="3" t="inlineStr">
         <is>
           <t>Depends on dimension valued. Four strong candidates:
 **Language**: meta-invention enabling all others to accumulate. But may have evolved rather than been invented.
@@ -9731,7 +9892,7 @@
 **Meta-point**: no invention stands alone. Cumulative innovation is humanity's real superpower.</t>
         </is>
       </c>
-      <c r="E343" s="2" t="n">
+      <c r="E348" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -9910,14 +10071,14 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>9.32</v>
+        <v>9.31</v>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>156, 171, 181, 222, 243, 266, 282, 287, 297, 304, 313, 383, 400, 400, 417, 421, 435</t>
+          <t>156, 171, 181, 222, 243, 266, 282, 287, 297, 304, 313, 383, 400, 400, 417, 421, 431, 435</t>
         </is>
       </c>
     </row>
@@ -10144,14 +10305,14 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C22" s="9" t="n">
         <v>9.119999999999999</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425</t>
+          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425, 432</t>
         </is>
       </c>
     </row>
@@ -10504,14 +10665,14 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>8.9</v>
+        <v>8.83</v>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>164, 253, 355, 382, 427</t>
+          <t>164, 253, 355, 382, 427, 434</t>
         </is>
       </c>
     </row>
@@ -10666,14 +10827,14 @@
         </is>
       </c>
       <c r="B51" s="11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C51" s="11" t="n">
-        <v>9.4</v>
+        <v>9.41</v>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>152, 217, 238, 241, 254, 269, 289, 299, 302, 332, 362, 385, 403, 403, 423</t>
+          <t>152, 217, 238, 241, 254, 269, 289, 299, 302, 332, 362, 385, 403, 403, 423, 435</t>
         </is>
       </c>
     </row>
@@ -10936,14 +11097,14 @@
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>9.59</v>
+        <v>9.58</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 438, 447</t>
+          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 447</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q436-Q440, fix OOM crash, update Excel (352 entries)
Training fixes: batch 4->2, grad_accum 1->2, gradient_checkpointing=true,
save_steps 5000->2000. Prevents Windows OOM kill at ~step 18k with seq=384.
Speed: 518 tok/s -> 3123 tok/s after fix.

Q436 History: Cold War — Cuban crisis, Berlin Wall, Gorbachev
Q437 CS: how the internet works — IP/TCP/DNS/BGP
Q438 Biology: microbiome — SCFAs, gut-brain axis, FMT
Q439 Philosophy: free will vs determinism — compatibilism
Q440 Mathematics: infinity sizes — Cantor, diagonal argument

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E348"/>
+  <dimension ref="A1:E353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9470,20 +9470,51 @@
       </c>
     </row>
     <row r="335">
-      <c r="A335" s="24" t="n">
+      <c r="A335" s="12" t="n">
+        <v>436</v>
+      </c>
+      <c r="B335" s="13" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="C335" s="13" t="inlineStr">
+        <is>
+          <t>What was the Cold War and why did it end?</t>
+        </is>
+      </c>
+      <c r="D335" s="13" t="inlineStr">
+        <is>
+          <t>Cold War (1947-1991): ideological and geopolitical standoff between US (liberal capitalism) and USSR (Marxist-Leninism). No direct military conflict between superpowers.
+Key crises: Cuban Missile Crisis (1962) — 13-day standoff, closest to nuclear war; Vietnam (US defeat 1975); Afghanistan 1979-89 (Soviet Vietnam).
+Why it ended:
+1. Economic exhaustion: Soviet command economy couldn't match US military spending; consumer shortages, oil revenue collapse after 1985
+2. Gorbachev's reforms: glasnost + perestroika — intended to save the system, released forces he couldn't control
+3. 1989 revolutions: Poland, Hungary, Czechoslovakia, East Germany, Romania — dominoes in months; Berlin Wall fell Nov 9 1989
+4. Nationalist movements: Baltic states, Ukraine, Soviet republics pushed independence
+5. Reagan's military pressure (contested): defence buildup may have accelerated Soviet economic strain
+USSR dissolved December 25 1991. Gorbachev resigned.</t>
+        </is>
+      </c>
+      <c r="E335" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="24" t="n">
         <v>437</v>
       </c>
-      <c r="B335" s="25" t="inlineStr">
+      <c r="B336" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="C335" s="25" t="inlineStr">
+      <c r="C336" s="25" t="inlineStr">
         <is>
           <t>How reliable is eyewitness testimony, and what does the research say?</t>
         </is>
       </c>
-      <c r="D335" s="25" t="inlineStr">
+      <c r="D336" s="25" t="inlineStr">
         <is>
           <t>Memory is reconstructive, not reproductive (Loftus). We rebuild memories each time, subject to suggestion.
 **Key experiments:**
@@ -9494,25 +9525,57 @@
 **What helps**: sequential lineups, blind administration, record initial statement, open questions first.</t>
         </is>
       </c>
-      <c r="E335" s="24" t="n">
+      <c r="E336" s="24" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="336">
-      <c r="A336" s="6" t="n">
+    <row r="337">
+      <c r="A337" s="20" t="n">
+        <v>437</v>
+      </c>
+      <c r="B337" s="21" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="C337" s="21" t="inlineStr">
+        <is>
+          <t>How does the internet actually work?</t>
+        </is>
+      </c>
+      <c r="D337" s="21" t="inlineStr">
+        <is>
+          <t>The internet is a global network of networks connected by agreed-upon protocols — not a single thing but a set of standards.
+Physical: fibre optic cables (~400 submarine cables carry ~99% of intercontinental traffic), copper, wireless, data centres, routers, ISPs.
+Key protocols:
+- IP: every device has an address; breaks data into packets routed independently; reassembled at destination
+- TCP: reliable delivery over IP — acknowledges packets, requests retransmission, reorders out-of-sequence
+- UDP: fast, no delivery guarantee — video streaming, gaming
+- DNS: translates domain names to IP addresses; hierarchical distributed database
+- HTTP/HTTPS: web pages; HTTPS adds TLS encryption
+Routing: BGP (Border Gateway Protocol) lets autonomous systems (ISPs, companies) exchange routing info. Packets hop router to router.
+The cloud: other people's computers (data centres) running your software.</t>
+        </is>
+      </c>
+      <c r="E337" s="20" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="6" t="n">
         <v>438</v>
       </c>
-      <c r="B336" s="7" t="inlineStr">
+      <c r="B338" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C336" s="7" t="inlineStr">
+      <c r="C338" s="7" t="inlineStr">
         <is>
           <t>What is the difference between heat and temperature?</t>
         </is>
       </c>
-      <c r="D336" s="7" t="inlineStr">
+      <c r="D338" s="7" t="inlineStr">
         <is>
           <t>**Temperature**: average kinetic energy per molecule. Measured in Kelvin/Celsius/Fahrenheit.
 **Heat**: *transfer* of thermal energy between objects due to temperature difference. Heat is a process, not a property. Pool at same temperature as coffee mug: pool contains far more thermal energy.
@@ -9522,25 +9585,57 @@
 **Water vs air at 100C**: water burns much more — higher thermal mass + latent heat of condensation deliver more energy per contact.</t>
         </is>
       </c>
-      <c r="E336" s="6" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" s="2" t="n">
+      <c r="E338" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="18" t="n">
+        <v>438</v>
+      </c>
+      <c r="B339" s="19" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C339" s="19" t="inlineStr">
+        <is>
+          <t>What is the microbiome and how does it affect health?</t>
+        </is>
+      </c>
+      <c r="D339" s="19" t="inlineStr">
+        <is>
+          <t>Human microbiome: ~38 trillion microorganisms (bacteria/archaea/fungi/viruses) — roughly equal to human cell count. Gut microbiome (~1.5 kg, mostly colon) is most studied.
+What it does:
+- Ferments dietary fibre into short-chain fatty acids (butyrate/propionate/acetate) — primary fuel for colon cells, anti-inflammatory
+- Trains immune system: early colonisation shapes immune development; germ-free mice have underdeveloped immunity
+- Produces vitamins: B12, K2, B vitamins
+- Gut-brain axis: vagus nerve + metabolites + immune signals link gut to brain
+- Colonisation resistance: outcompetes pathogens
+Dysbiosis: antibiotics -&gt; C. difficile overgrowth; associated with IBD, obesity, T2D, depression (correlational).
+FMT (faecal microbiota transplant): &gt;90% cure rate for recurrent C. difficile. Experimental for other conditions.
+Caution: most probiotic products have weak evidence for healthy individuals.</t>
+        </is>
+      </c>
+      <c r="E339" s="18" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="n">
         <v>439</v>
       </c>
-      <c r="B337" s="3" t="inlineStr">
+      <c r="B340" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C337" s="3" t="inlineStr">
+      <c r="C340" s="3" t="inlineStr">
         <is>
           <t>What is structural racism, and how does it differ from individual racism?</t>
         </is>
       </c>
-      <c r="D337" s="3" t="inlineStr">
+      <c r="D340" s="3" t="inlineStr">
         <is>
           <t>**Individual racism**: prejudice and discriminatory acts by identifiable individuals. Overt bias.
 **Structural racism**: racial disparities from systems, policies, norms — even without individual racist intent.
@@ -9552,25 +9647,54 @@
 **Evidence**: audit studies (identical CVs with Black vs white names) consistently find measurable hiring discrimination.</t>
         </is>
       </c>
-      <c r="E337" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" s="26" t="n">
+      <c r="E340" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="16" t="n">
+        <v>439</v>
+      </c>
+      <c r="B341" s="17" t="inlineStr">
+        <is>
+          <t>Philosophy</t>
+        </is>
+      </c>
+      <c r="C341" s="17" t="inlineStr">
+        <is>
+          <t>What is free will and is it compatible with determinism?</t>
+        </is>
+      </c>
+      <c r="D341" s="17" t="inlineStr">
+        <is>
+          <t>Determinism: every event including decisions is the inevitable result of prior causes + physical laws.
+Three positions:
+1. Hard determinism: determinism true AND free will is an illusion. Retributive punishment incoherent. (Pereboom)
+2. Libertarian free will: genuine free will exists outside determinism. Quantum indeterminacy invoked — but randomness ≠ agency.
+3. Compatibilism (majority view): free will = acting according to own desires/reasoning, free from coercion. Doesn't require 'could have done otherwise.' Frankfurt cases: moral responsibility doesn't require alternative possibilities. (Hume, Frankfurt, Dennett)
+Neuroscience: Libet (1983) — readiness potential precedes conscious decision by ~350ms. Suggests decision before 'we' decide. Critiqued: measured simple wrist flick, not complex decisions.
+Practical: compatibilism preserves moral responsibility; hard determinism supports rehabilitation over retribution.</t>
+        </is>
+      </c>
+      <c r="E341" s="16" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="26" t="n">
         <v>440</v>
       </c>
-      <c r="B338" s="27" t="inlineStr">
+      <c r="B342" s="27" t="inlineStr">
         <is>
           <t>Ecology</t>
         </is>
       </c>
-      <c r="C338" s="27" t="inlineStr">
+      <c r="C342" s="27" t="inlineStr">
         <is>
           <t>What is the nitrogen cycle and why is it essential for life?</t>
         </is>
       </c>
-      <c r="D338" s="27" t="inlineStr">
+      <c r="D342" s="27" t="inlineStr">
         <is>
           <t>N2 = 78% of atmosphere, but most organisms can't use N2 (triple bond N=N, 945 kJ/mol). Life needs reactive N (NH3, NO3-, organic N).
 **Nitrogen cycle:**
@@ -9582,25 +9706,53 @@
 **Limiting nutrient**: N limits most ecosystems. Excess (fertilisers) -&gt; eutrophication -&gt; algal blooms -&gt; oxygen depletion -&gt; dead zones (Gulf of Mexico). Haber also weaponised N (chlorine, phosgene).</t>
         </is>
       </c>
-      <c r="E338" s="26" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="339">
-      <c r="A339" s="30" t="n">
+      <c r="E342" s="26" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="14" t="n">
+        <v>440</v>
+      </c>
+      <c r="B343" s="15" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="C343" s="15" t="inlineStr">
+        <is>
+          <t>What is infinity and are there different sizes of it?</t>
+        </is>
+      </c>
+      <c r="D343" s="15" t="inlineStr">
+        <is>
+          <t>Yes — Cantor (1873) proved some infinities are strictly larger than others.
+Countable infinity (aleph-0): integers are infinite. Rational numbers are ALSO countably infinite — Cantor showed a bijection with integers by diagonal enumeration. Surprising: as many rationals as integers.
+Uncountable infinity: real numbers are strictly larger. Cantor's diagonal argument: assume a complete list of reals between 0 and 1. Construct a number differing from the nth number at the nth digit. This new number isn't in the list — no complete list exists. Reals are uncountably infinite, aleph-1 &gt; aleph-0.
+Hierarchy: 2^(aleph-0) &gt; aleph-0. Power set of any infinite set is strictly larger. Infinitely many distinct infinities.
+Continuum Hypothesis: is there an infinity between aleph-0 and the reals? Godel (1940) + Cohen (1963) proved it's INDEPENDENT of ZFC — can't be proved or disproved from standard axioms.
+Practical: most functions are uncomputable (countably many programs, uncountably many functions).</t>
+        </is>
+      </c>
+      <c r="E343" s="14" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="30" t="n">
         <v>441</v>
       </c>
-      <c r="B339" s="31" t="inlineStr">
+      <c r="B344" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="C339" s="31" t="inlineStr">
+      <c r="C344" s="31" t="inlineStr">
         <is>
           <t>What is antibiotic resistance and how does it develop?</t>
         </is>
       </c>
-      <c r="D339" s="31" t="inlineStr">
+      <c r="D344" s="31" t="inlineStr">
         <is>
           <t>Antibiotics target cell wall (penicillin), protein synthesis (tetracycline), DNA replication (fluoroquinolones), or membranes. Resistance = survival.
 **Darwinian mechanism:**
@@ -9614,25 +9766,25 @@
 **Why few new antibiotics**: 10-15yr development; brief low-cost use = poor financial incentive vs lifelong drugs.</t>
         </is>
       </c>
-      <c r="E339" s="30" t="n">
+      <c r="E344" s="30" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="340">
-      <c r="A340" s="12" t="n">
+    <row r="345">
+      <c r="A345" s="12" t="n">
         <v>442</v>
       </c>
-      <c r="B340" s="13" t="inlineStr">
+      <c r="B345" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C340" s="13" t="inlineStr">
+      <c r="C345" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the Magna Carta?</t>
         </is>
       </c>
-      <c r="D340" s="13" t="inlineStr">
+      <c r="D345" s="13" t="inlineStr">
         <is>
           <t>June 1215: English barons forced King John to sign. Originally limited royal power in narrow feudal ways — mostly barons' rights, not ordinary people.
 **Key clauses**: Cl. 39 — no free man imprisoned without lawful judgment of peers ('due process'); Cl. 40 — no selling/denying justice.
@@ -9642,25 +9794,25 @@
 **Lasting principle**: rule of law over arbitrary power -&gt; constitutional government, habeas corpus, human rights.</t>
         </is>
       </c>
-      <c r="E340" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="341">
-      <c r="A341" s="20" t="n">
+      <c r="E345" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="20" t="n">
         <v>443</v>
       </c>
-      <c r="B341" s="21" t="inlineStr">
+      <c r="B346" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C341" s="21" t="inlineStr">
+      <c r="C346" s="21" t="inlineStr">
         <is>
           <t>What is machine learning and how is it different from traditional programming?</t>
         </is>
       </c>
-      <c r="D341" s="21" t="inlineStr">
+      <c r="D346" s="21" t="inlineStr">
         <is>
           <t>**Traditional programming**: programmer writes explicit rules. Input + rules -&gt; output. Brittle; can't generalise.
 **Machine learning**: provide data + correct answers; algorithm finds the rules. Input + labels -&gt; model -&gt; generalises to new data.
@@ -9673,25 +9825,25 @@
 **Scale**: LLMs (GPT, Claude) = transformers on trillions of tokens; emergent capabilities at scale.</t>
         </is>
       </c>
-      <c r="E341" s="20" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" s="16" t="n">
+      <c r="E346" s="20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="16" t="n">
         <v>444</v>
       </c>
-      <c r="B342" s="17" t="inlineStr">
+      <c r="B347" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C342" s="17" t="inlineStr">
+      <c r="C347" s="17" t="inlineStr">
         <is>
           <t>What is the ship of Theseus paradox, and what is it really asking?</t>
         </is>
       </c>
-      <c r="D342" s="17" t="inlineStr">
+      <c r="D347" s="17" t="inlineStr">
         <is>
           <t>Plutarch (~100 CE): every plank of Theseus's ship replaced over time. Still the same ship?
 **Hobbes extension**: original planks collected and reassembled. Two ships claim to be the original. Which is it?
@@ -9705,25 +9857,25 @@
 **Parfit** (*Reasons and Persons*): personal identity is not what matters — psychological continuity is what matters; 'same' may be an empty question.</t>
         </is>
       </c>
-      <c r="E342" s="16" t="n">
+      <c r="E347" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="343">
-      <c r="A343" s="2" t="n">
+    <row r="348">
+      <c r="A348" s="2" t="n">
         <v>445</v>
       </c>
-      <c r="B343" s="3" t="inlineStr">
+      <c r="B348" s="3" t="inlineStr">
         <is>
           <t>Music</t>
         </is>
       </c>
-      <c r="C343" s="3" t="inlineStr">
+      <c r="C348" s="3" t="inlineStr">
         <is>
           <t>Why does music make us emotional?</t>
         </is>
       </c>
-      <c r="D343" s="3" t="inlineStr">
+      <c r="D348" s="3" t="inlineStr">
         <is>
           <t>Multiple converging mechanisms:
 1. **Expectation/violation** (Meyer 1956, Huron 2006): music is temporal prediction. Correct resolution = dopaminergic reward. Surprise + resolution = stronger reward. Chills = surprising resolution.
@@ -9735,25 +9887,25 @@
 **Mystery of sad music pleasure**: safe simulation, hormonal empathy reward, artistic resolution — distinct emotion from actual grief.</t>
         </is>
       </c>
-      <c r="E343" s="2" t="n">
+      <c r="E348" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="344">
-      <c r="A344" s="4" t="n">
+    <row r="349">
+      <c r="A349" s="4" t="n">
         <v>446</v>
       </c>
-      <c r="B344" s="5" t="inlineStr">
+      <c r="B349" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="C344" s="5" t="inlineStr">
+      <c r="C349" s="5" t="inlineStr">
         <is>
           <t>How do children acquire language so rapidly?</t>
         </is>
       </c>
-      <c r="D344" s="5" t="inlineStr">
+      <c r="D349" s="5" t="inlineStr">
         <is>
           <t>First words ~12 months, two-word phrases ~18-24 months, complex sentences by 3-4 years — from imperfect, fragmented input.
 **Poverty of the stimulus**: children overgeneralise rules ('goed', 'mouses') but never make wrong rule errors. Acquire structure-dependent rules without examples of errors.
@@ -9765,25 +9917,25 @@
 **Mechanisms**: statistical learning (8-month-olds track syllable transition probabilities), joint attention, motherese (simplified grammar + exaggerated prosody).</t>
         </is>
       </c>
-      <c r="E344" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="345">
-      <c r="A345" s="6" t="n">
+      <c r="E349" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="6" t="n">
         <v>447</v>
       </c>
-      <c r="B345" s="7" t="inlineStr">
+      <c r="B350" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C345" s="7" t="inlineStr">
+      <c r="C350" s="7" t="inlineStr">
         <is>
           <t>What is the photoelectric effect, and why did it matter for quantum mechanics?</t>
         </is>
       </c>
-      <c r="D345" s="7" t="inlineStr">
+      <c r="D350" s="7" t="inlineStr">
         <is>
           <t>Light hits metal -&gt; electrons ejected, BUT only above a threshold frequency. Below threshold: no electrons regardless of intensity.
 **Classical prediction**: intensity drives ejection. WRONG.
@@ -9796,25 +9948,25 @@
 4. Technology: photovoltaics, CCDs, photomultipliers</t>
         </is>
       </c>
-      <c r="E345" s="6" t="n">
+      <c r="E350" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="346">
-      <c r="A346" s="2" t="n">
+    <row r="351">
+      <c r="A351" s="2" t="n">
         <v>448</v>
       </c>
-      <c r="B346" s="3" t="inlineStr">
+      <c r="B351" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C346" s="3" t="inlineStr">
+      <c r="C351" s="3" t="inlineStr">
         <is>
           <t>What is social mobility and what actually predicts it?</t>
         </is>
       </c>
-      <c r="D346" s="3" t="inlineStr">
+      <c r="D351" s="3" t="inlineStr">
         <is>
           <t>Movement between socioeconomic strata. Intergenerational (parent to child) vs intragenerational (within lifetime).
 **Great Gatsby Curve** (Miles Corak): more income inequality -&gt; LOWER intergenerational mobility. Denmark (low inequality) = high mobility; US, UK = lower.
@@ -9827,25 +9979,25 @@
 Absolute mobility (exceeding parents in absolute terms) has historically been high; relative mobility much more constrained.</t>
         </is>
       </c>
-      <c r="E346" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" s="28" t="n">
+      <c r="E351" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="28" t="n">
         <v>449</v>
       </c>
-      <c r="B347" s="29" t="inlineStr">
+      <c r="B352" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C347" s="29" t="inlineStr">
+      <c r="C352" s="29" t="inlineStr">
         <is>
           <t>How do batteries work chemically, and what limits their energy density?</t>
         </is>
       </c>
-      <c r="D347" s="29" t="inlineStr">
+      <c r="D352" s="29" t="inlineStr">
         <is>
           <t>Battery = chemical -&gt; electrical energy via spatially separated redox reactions.
 Anode: oxidation (loses electrons). Cathode: reduction (gains electrons). Electrons flow externally (current); ions flow internally through electrolyte.
@@ -9862,25 +10014,25 @@
 **Theoretical limits**: Li-ion ~265 Wh/kg practical; Li-sulfur 2,600 Wh/kg; Li-air 11,680 Wh/kg (comparable to gasoline).</t>
         </is>
       </c>
-      <c r="E347" s="28" t="n">
+      <c r="E352" s="28" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="348">
-      <c r="A348" s="2" t="n">
+    <row r="353">
+      <c r="A353" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="B348" s="3" t="inlineStr">
+      <c r="B353" s="3" t="inlineStr">
         <is>
           <t>General Knowledge</t>
         </is>
       </c>
-      <c r="C348" s="3" t="inlineStr">
+      <c r="C353" s="3" t="inlineStr">
         <is>
           <t>What is the most important invention in human history, and why?</t>
         </is>
       </c>
-      <c r="D348" s="3" t="inlineStr">
+      <c r="D353" s="3" t="inlineStr">
         <is>
           <t>Depends on dimension valued. Four strong candidates:
 **Language**: meta-invention enabling all others to accumulate. But may have evolved rather than been invented.
@@ -9892,7 +10044,7 @@
 **Meta-point**: no invention stands alone. Cumulative innovation is humanity's real superpower.</t>
         </is>
       </c>
-      <c r="E348" s="2" t="n">
+      <c r="E353" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10071,14 +10223,14 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>9.31</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>156, 171, 181, 222, 243, 266, 282, 287, 297, 304, 313, 383, 400, 400, 417, 421, 431, 435</t>
+          <t>156, 171, 181, 222, 243, 266, 282, 287, 297, 304, 313, 383, 400, 400, 417, 421, 431, 435, 438</t>
         </is>
       </c>
     </row>
@@ -10215,14 +10367,14 @@
         </is>
       </c>
       <c r="B17" s="21" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C17" s="21" t="n">
-        <v>9.31</v>
+        <v>9.25</v>
       </c>
       <c r="D17" s="21" t="inlineStr">
         <is>
-          <t>157, 184, 252, 258, 352, 377, 388, 398, 398, 409, 426, 428, 443</t>
+          <t>157, 184, 252, 258, 352, 377, 388, 398, 398, 409, 426, 428, 437, 443</t>
         </is>
       </c>
     </row>
@@ -10521,14 +10673,14 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>9.119999999999999</v>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 442</t>
+          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 436, 442</t>
         </is>
       </c>
     </row>
@@ -10719,14 +10871,14 @@
         </is>
       </c>
       <c r="B45" s="15" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C45" s="15" t="n">
         <v>9.56</v>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436</t>
+          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436, 440</t>
         </is>
       </c>
     </row>
@@ -10971,14 +11123,14 @@
         </is>
       </c>
       <c r="B59" s="17" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C59" s="17" t="n">
         <v>9.44</v>
       </c>
       <c r="D59" s="17" t="inlineStr">
         <is>
-          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 444</t>
+          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 439, 444</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q441-Q445, update Excel (357 entries)
Q441 Neuroscience: default mode network — rumination, meditation, Alzheimer's
Q442 Physics: double-slit experiment — wave-particle duality, Feynman
Q443 Economics: inflation — demand-pull, Friedman, Phillips Curve
Q444 History: Scientific Revolution — Copernicus to Newton, Kuhn
Q445 Psychology: attachment theory — Bowlby, Ainsworth, Strange Situation

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E353"/>
+  <dimension ref="A1:E358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9771,20 +9771,50 @@
       </c>
     </row>
     <row r="345">
-      <c r="A345" s="12" t="n">
+      <c r="A345" s="10" t="n">
+        <v>441</v>
+      </c>
+      <c r="B345" s="11" t="inlineStr">
+        <is>
+          <t>Neuroscience</t>
+        </is>
+      </c>
+      <c r="C345" s="11" t="inlineStr">
+        <is>
+          <t>What is the default mode network and what does it do?</t>
+        </is>
+      </c>
+      <c r="D345" s="11" t="inlineStr">
+        <is>
+          <t>Default mode network (DMN): brain regions MORE active during rest than focused tasks — identified when PET/fMRI researchers noticed consistent deactivations during tasks.
+Key regions: medial prefrontal cortex, posterior cingulate cortex, precuneus, angular gyrus, hippocampus.
+What it does: mind-wandering/daydreaming; self-referential processing; theory of mind (mentalising); autobiographical memory retrieval; prospection (simulating future).
+Why it matters:
+- Depression: DMN hyperactive — rumination = excessive medial PFC activity
+- Meditation: experienced meditators show reduced DMN activity; stronger disengagement
+- Alzheimer's: amyloid-beta deposits preferentially in DMN hubs
+Anticorrelation: DMN and task-positive (dorsal attention) network are anticorrelated — one active, the other suppressed.</t>
+        </is>
+      </c>
+      <c r="E345" s="10" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="12" t="n">
         <v>442</v>
       </c>
-      <c r="B345" s="13" t="inlineStr">
+      <c r="B346" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="C345" s="13" t="inlineStr">
+      <c r="C346" s="13" t="inlineStr">
         <is>
           <t>What was the significance of the Magna Carta?</t>
         </is>
       </c>
-      <c r="D345" s="13" t="inlineStr">
+      <c r="D346" s="13" t="inlineStr">
         <is>
           <t>June 1215: English barons forced King John to sign. Originally limited royal power in narrow feudal ways — mostly barons' rights, not ordinary people.
 **Key clauses**: Cl. 39 — no free man imprisoned without lawful judgment of peers ('due process'); Cl. 40 — no selling/denying justice.
@@ -9794,25 +9824,56 @@
 **Lasting principle**: rule of law over arbitrary power -&gt; constitutional government, habeas corpus, human rights.</t>
         </is>
       </c>
-      <c r="E345" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" s="20" t="n">
+      <c r="E346" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="6" t="n">
+        <v>442</v>
+      </c>
+      <c r="B347" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="C347" s="7" t="inlineStr">
+        <is>
+          <t>What is the double-slit experiment and what does it prove?</t>
+        </is>
+      </c>
+      <c r="D347" s="7" t="inlineStr">
+        <is>
+          <t>Feynman: the double-slit experiment contains 'the only mystery' of quantum mechanics.
+Quantum version: fire electrons one at a time at two slits -&gt; over time, interference pattern builds (alternating bands) — as if each electron passes through BOTH slits simultaneously.
+Measurement paradox: place detector at slits to observe which slit -&gt; interference pattern DISAPPEARS. Electrons behave like classical particles.
+What it proves:
+1. Wave-particle duality: quantum objects show both wave (interference) and particle (individual detection) properties
+2. Superposition: unobserved electron is in superposition of both paths
+3. Observation collapses wavefunction: interaction with macroscopic system forces definite outcome
+4. Non-locality: quantum state spread across both slits simultaneously
+Interpretation problem: Copenhagen (don't ask), Many-Worlds (universe branches), Pilot Wave (hidden variable). Still contested.</t>
+        </is>
+      </c>
+      <c r="E347" s="6" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="20" t="n">
         <v>443</v>
       </c>
-      <c r="B346" s="21" t="inlineStr">
+      <c r="B348" s="21" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="C346" s="21" t="inlineStr">
+      <c r="C348" s="21" t="inlineStr">
         <is>
           <t>What is machine learning and how is it different from traditional programming?</t>
         </is>
       </c>
-      <c r="D346" s="21" t="inlineStr">
+      <c r="D348" s="21" t="inlineStr">
         <is>
           <t>**Traditional programming**: programmer writes explicit rules. Input + rules -&gt; output. Brittle; can't generalise.
 **Machine learning**: provide data + correct answers; algorithm finds the rules. Input + labels -&gt; model -&gt; generalises to new data.
@@ -9825,25 +9886,57 @@
 **Scale**: LLMs (GPT, Claude) = transformers on trillions of tokens; emergent capabilities at scale.</t>
         </is>
       </c>
-      <c r="E346" s="20" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" s="16" t="n">
+      <c r="E348" s="20" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="8" t="n">
+        <v>443</v>
+      </c>
+      <c r="B349" s="9" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="C349" s="9" t="inlineStr">
+        <is>
+          <t>What is inflation and what causes it?</t>
+        </is>
+      </c>
+      <c r="D349" s="9" t="inlineStr">
+        <is>
+          <t>Inflation: sustained increase in general price level / decline in purchasing power of money.
+Measured by: CPI (consumer basket), PCE (Fed's preferred), PPI (producer prices). Core excludes food/energy.
+Causes:
+1. Demand-pull: too much money chasing too few goods (2021-22 stimulus + supply constraints)
+2. Cost-push: supply shocks raise production costs (1973 oil embargo -&gt; stagflation)
+3. Wage-price spiral: expected inflation -&gt; wage demands -&gt; price rises -&gt; validates expectations (1970s)
+4. Monetary (Friedman): inflation is always and everywhere a monetary phenomenon — excess money growth. Hyperinflations (Weimar 1923, Zimbabwe 2008) always monetary.
+Expectations crucial: if 5% expected, 5% negotiated, 5% occurs. Anchoring expectations is central banking's core job.
+Why 2% target: deflation worse — Fisher debt deflation spiral; 2% buffer lets central banks cut real rates.
+Phillips Curve: inflation-unemployment tradeoff; stagflation showed it can break down.</t>
+        </is>
+      </c>
+      <c r="E349" s="8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="16" t="n">
         <v>444</v>
       </c>
-      <c r="B347" s="17" t="inlineStr">
+      <c r="B350" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="C347" s="17" t="inlineStr">
+      <c r="C350" s="17" t="inlineStr">
         <is>
           <t>What is the ship of Theseus paradox, and what is it really asking?</t>
         </is>
       </c>
-      <c r="D347" s="17" t="inlineStr">
+      <c r="D350" s="17" t="inlineStr">
         <is>
           <t>Plutarch (~100 CE): every plank of Theseus's ship replaced over time. Still the same ship?
 **Hobbes extension**: original planks collected and reassembled. Two ships claim to be the original. Which is it?
@@ -9857,25 +9950,58 @@
 **Parfit** (*Reasons and Persons*): personal identity is not what matters — psychological continuity is what matters; 'same' may be an empty question.</t>
         </is>
       </c>
-      <c r="E347" s="16" t="n">
+      <c r="E350" s="16" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="348">
-      <c r="A348" s="2" t="n">
+    <row r="351">
+      <c r="A351" s="12" t="n">
+        <v>444</v>
+      </c>
+      <c r="B351" s="13" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="C351" s="13" t="inlineStr">
+        <is>
+          <t>What was the Scientific Revolution and who drove it?</t>
+        </is>
+      </c>
+      <c r="D351" s="13" t="inlineStr">
+        <is>
+          <t>Scientific Revolution (~1543-1687): replaced Aristotelian authority with empirical observation and mathematical description.
+Key figures:
+- Copernicus (1543): heliocentric model, removed Earth from centre
+- Tycho Brahe: 20 years of precise naked-eye astronomical data
+- Kepler: used Brahe's data -&gt; three laws of planetary motion (elliptical orbits)
+- Galileo: telescope (Jupiter's moons, Venus phases), mathematical motion, inertia; Church conflict
+- Vesalius (1543): dissection-based human anatomy, overturned Galen
+- Harvey (1628): circulation of blood — experimental proof
+- Newton (1687): Principia — universal gravitation, three laws of motion, unified terrestrial and celestial mechanics. The capstone.
+What changed: empirical + mathematical over ancient authority; geocentric -&gt; heliocentric infinite universe; observer is authoritative.
+Kuhn (Structure of Scientific Revolutions): paradigm shifts are discontinuous. Others argue continuity with medieval and Islamic science.</t>
+        </is>
+      </c>
+      <c r="E351" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="n">
         <v>445</v>
       </c>
-      <c r="B348" s="3" t="inlineStr">
+      <c r="B352" s="3" t="inlineStr">
         <is>
           <t>Music</t>
         </is>
       </c>
-      <c r="C348" s="3" t="inlineStr">
+      <c r="C352" s="3" t="inlineStr">
         <is>
           <t>Why does music make us emotional?</t>
         </is>
       </c>
-      <c r="D348" s="3" t="inlineStr">
+      <c r="D352" s="3" t="inlineStr">
         <is>
           <t>Multiple converging mechanisms:
 1. **Expectation/violation** (Meyer 1956, Huron 2006): music is temporal prediction. Correct resolution = dopaminergic reward. Surprise + resolution = stronger reward. Chills = surprising resolution.
@@ -9887,25 +10013,55 @@
 **Mystery of sad music pleasure**: safe simulation, hormonal empathy reward, artistic resolution — distinct emotion from actual grief.</t>
         </is>
       </c>
-      <c r="E348" s="2" t="n">
+      <c r="E352" s="2" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="349">
-      <c r="A349" s="4" t="n">
+    <row r="353">
+      <c r="A353" s="24" t="n">
+        <v>445</v>
+      </c>
+      <c r="B353" s="25" t="inlineStr">
+        <is>
+          <t>Psychology</t>
+        </is>
+      </c>
+      <c r="C353" s="25" t="inlineStr">
+        <is>
+          <t>What is attachment theory and how does early bonding shape adult life?</t>
+        </is>
+      </c>
+      <c r="D353" s="25" t="inlineStr">
+        <is>
+          <t>Bowlby (1950s-70s): evolved attachment system — innate need for close bonds with caregivers, critical for survival and development.
+Ainsworth's Strange Situation (1970s): separate 12-month-olds briefly, observe reunion:
+1. Secure (~65%): distressed on separation, comforted on return. Reliably responsive caregiver. -&gt; Adults: comfortable with intimacy, good emotion regulation.
+2. Anxious/Ambivalent (~15%): intensely distressed, not easily comforted (clingy/angry). Inconsistent caregiver. -&gt; Adults: preoccupied with relationships, fear abandonment.
+3. Avoidant (~20%): appear unconcerned but physiologically stressed (suppress expression). Consistently rejecting caregiver. -&gt; Adults: uncomfortable with closeness, dismissive.
+4. Disorganised: contradictory approach/avoid. Frightened/frightening caregiver (abuse/trauma). Strongest predictor of psychopathology.
+Internal working models: mental representations of self/others formed from early experience — shape all future relationships.
+Continuity vs change: moderately stable but not fixed. Therapy and new relationships can shift patterns. Earned security is real.</t>
+        </is>
+      </c>
+      <c r="E353" s="24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="4" t="n">
         <v>446</v>
       </c>
-      <c r="B349" s="5" t="inlineStr">
+      <c r="B354" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="C349" s="5" t="inlineStr">
+      <c r="C354" s="5" t="inlineStr">
         <is>
           <t>How do children acquire language so rapidly?</t>
         </is>
       </c>
-      <c r="D349" s="5" t="inlineStr">
+      <c r="D354" s="5" t="inlineStr">
         <is>
           <t>First words ~12 months, two-word phrases ~18-24 months, complex sentences by 3-4 years — from imperfect, fragmented input.
 **Poverty of the stimulus**: children overgeneralise rules ('goed', 'mouses') but never make wrong rule errors. Acquire structure-dependent rules without examples of errors.
@@ -9917,25 +10073,25 @@
 **Mechanisms**: statistical learning (8-month-olds track syllable transition probabilities), joint attention, motherese (simplified grammar + exaggerated prosody).</t>
         </is>
       </c>
-      <c r="E349" s="4" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" s="6" t="n">
+      <c r="E354" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="6" t="n">
         <v>447</v>
       </c>
-      <c r="B350" s="7" t="inlineStr">
+      <c r="B355" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C350" s="7" t="inlineStr">
+      <c r="C355" s="7" t="inlineStr">
         <is>
           <t>What is the photoelectric effect, and why did it matter for quantum mechanics?</t>
         </is>
       </c>
-      <c r="D350" s="7" t="inlineStr">
+      <c r="D355" s="7" t="inlineStr">
         <is>
           <t>Light hits metal -&gt; electrons ejected, BUT only above a threshold frequency. Below threshold: no electrons regardless of intensity.
 **Classical prediction**: intensity drives ejection. WRONG.
@@ -9948,25 +10104,25 @@
 4. Technology: photovoltaics, CCDs, photomultipliers</t>
         </is>
       </c>
-      <c r="E350" s="6" t="n">
+      <c r="E355" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="351">
-      <c r="A351" s="2" t="n">
+    <row r="356">
+      <c r="A356" s="2" t="n">
         <v>448</v>
       </c>
-      <c r="B351" s="3" t="inlineStr">
+      <c r="B356" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C351" s="3" t="inlineStr">
+      <c r="C356" s="3" t="inlineStr">
         <is>
           <t>What is social mobility and what actually predicts it?</t>
         </is>
       </c>
-      <c r="D351" s="3" t="inlineStr">
+      <c r="D356" s="3" t="inlineStr">
         <is>
           <t>Movement between socioeconomic strata. Intergenerational (parent to child) vs intragenerational (within lifetime).
 **Great Gatsby Curve** (Miles Corak): more income inequality -&gt; LOWER intergenerational mobility. Denmark (low inequality) = high mobility; US, UK = lower.
@@ -9979,25 +10135,25 @@
 Absolute mobility (exceeding parents in absolute terms) has historically been high; relative mobility much more constrained.</t>
         </is>
       </c>
-      <c r="E351" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="352">
-      <c r="A352" s="28" t="n">
+      <c r="E356" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="28" t="n">
         <v>449</v>
       </c>
-      <c r="B352" s="29" t="inlineStr">
+      <c r="B357" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C352" s="29" t="inlineStr">
+      <c r="C357" s="29" t="inlineStr">
         <is>
           <t>How do batteries work chemically, and what limits their energy density?</t>
         </is>
       </c>
-      <c r="D352" s="29" t="inlineStr">
+      <c r="D357" s="29" t="inlineStr">
         <is>
           <t>Battery = chemical -&gt; electrical energy via spatially separated redox reactions.
 Anode: oxidation (loses electrons). Cathode: reduction (gains electrons). Electrons flow externally (current); ions flow internally through electrolyte.
@@ -10014,25 +10170,25 @@
 **Theoretical limits**: Li-ion ~265 Wh/kg practical; Li-sulfur 2,600 Wh/kg; Li-air 11,680 Wh/kg (comparable to gasoline).</t>
         </is>
       </c>
-      <c r="E352" s="28" t="n">
+      <c r="E357" s="28" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="353">
-      <c r="A353" s="2" t="n">
+    <row r="358">
+      <c r="A358" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="B353" s="3" t="inlineStr">
+      <c r="B358" s="3" t="inlineStr">
         <is>
           <t>General Knowledge</t>
         </is>
       </c>
-      <c r="C353" s="3" t="inlineStr">
+      <c r="C358" s="3" t="inlineStr">
         <is>
           <t>What is the most important invention in human history, and why?</t>
         </is>
       </c>
-      <c r="D353" s="3" t="inlineStr">
+      <c r="D358" s="3" t="inlineStr">
         <is>
           <t>Depends on dimension valued. Four strong candidates:
 **Language**: meta-invention enabling all others to accumulate. But may have evolved rather than been invented.
@@ -10044,7 +10200,7 @@
 **Meta-point**: no invention stands alone. Cumulative innovation is humanity's real superpower.</t>
         </is>
       </c>
-      <c r="E353" s="2" t="n">
+      <c r="E358" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10457,14 +10613,14 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>9.119999999999999</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425, 432</t>
+          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425, 432, 443</t>
         </is>
       </c>
     </row>
@@ -10673,14 +10829,14 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C34" s="13" t="n">
-        <v>9.119999999999999</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 436, 442</t>
+          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 436, 442, 444</t>
         </is>
       </c>
     </row>
@@ -10979,14 +11135,14 @@
         </is>
       </c>
       <c r="B51" s="11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C51" s="11" t="n">
-        <v>9.41</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>152, 217, 238, 241, 254, 269, 289, 299, 302, 332, 362, 385, 403, 403, 423, 435</t>
+          <t>152, 217, 238, 241, 254, 269, 289, 299, 302, 332, 362, 385, 403, 403, 423, 435, 441</t>
         </is>
       </c>
     </row>
@@ -11249,14 +11405,14 @@
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>9.58</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 447</t>
+          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447</t>
         </is>
       </c>
     </row>
@@ -11321,14 +11477,14 @@
         </is>
       </c>
       <c r="B70" s="25" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C70" s="25" t="n">
         <v>9.109999999999999</v>
       </c>
       <c r="D70" s="25" t="inlineStr">
         <is>
-          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 424, 432, 437</t>
+          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 424, 432, 437, 445</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q446-Q450, update Excel (362 entries)
Q446 Ecology: climate change — IPCC AR6, greenhouse physics, 97% consensus
Q447 Mathematics: derivatives — gradient descent, backpropagation, marginal cost
Q448 Sociology: structural racism — redlining, audit studies, without intent
Q449 Physics: relativity — time dilation, GPS, E=mc2, LIGO
Q450 Literature: magical realism — Garcia Marquez, Latin America origins

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E358"/>
+  <dimension ref="A1:E363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10078,20 +10078,48 @@
       </c>
     </row>
     <row r="355">
-      <c r="A355" s="6" t="n">
+      <c r="A355" s="26" t="n">
+        <v>446</v>
+      </c>
+      <c r="B355" s="27" t="inlineStr">
+        <is>
+          <t>Ecology</t>
+        </is>
+      </c>
+      <c r="C355" s="27" t="inlineStr">
+        <is>
+          <t>What is climate change and how confident are scientists?</t>
+        </is>
+      </c>
+      <c r="D355" s="27" t="inlineStr">
+        <is>
+          <t>Climate change: long-term shift in global temperatures primarily driven by human GHG emissions since ~1750.
+IPCC AR6 (2021): +1.1C above pre-industrial; human causation 'unequivocal'; CO2 at 420ppm (highest in 3M years); warming rate fastest in 65M years.
+Mechanism: CO2/CH4/N2O absorb outgoing infrared, re-emit in all directions -&gt; more energy trapped. Physics: Fourier (1824), Tyndall (1859), Arrhenius (1896) calculated ~5C per CO2 doubling.
+Evidence (independent, all consistent): surface temperature records; ocean heat rising; sea level +20cm since 1900; Arctic ice declining; glaciers retreating; species range shifts; isotope fingerprinting proves fossil fuel origin.
+Projections: each 0.5C matters — coral reefs, extreme heat, food security scale nonlinearly.
+Consensus: 97%+ of climate scientists; every national academy of science worldwide.</t>
+        </is>
+      </c>
+      <c r="E355" s="26" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="6" t="n">
         <v>447</v>
       </c>
-      <c r="B355" s="7" t="inlineStr">
+      <c r="B356" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="C355" s="7" t="inlineStr">
+      <c r="C356" s="7" t="inlineStr">
         <is>
           <t>What is the photoelectric effect, and why did it matter for quantum mechanics?</t>
         </is>
       </c>
-      <c r="D355" s="7" t="inlineStr">
+      <c r="D356" s="7" t="inlineStr">
         <is>
           <t>Light hits metal -&gt; electrons ejected, BUT only above a threshold frequency. Below threshold: no electrons regardless of intensity.
 **Classical prediction**: intensity drives ejection. WRONG.
@@ -10104,25 +10132,56 @@
 4. Technology: photovoltaics, CCDs, photomultipliers</t>
         </is>
       </c>
-      <c r="E355" s="6" t="n">
+      <c r="E356" s="6" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="356">
-      <c r="A356" s="2" t="n">
+    <row r="357">
+      <c r="A357" s="14" t="n">
+        <v>447</v>
+      </c>
+      <c r="B357" s="15" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="C357" s="15" t="inlineStr">
+        <is>
+          <t>What is a derivative intuitively, and what are its real-world uses?</t>
+        </is>
+      </c>
+      <c r="D357" s="15" t="inlineStr">
+        <is>
+          <t>Derivative: instantaneous rate of change — slope of the tangent line at a point. f'(x) = lim[h-&gt;0] (f(x+h)-f(x))/h.
+Physically: position -&gt; velocity -&gt; acceleration (each a derivative of the prior).
+Real-world uses:
+- Physics: Maxwell's equations, Schrodinger equation, Newton's laws — all differential equations
+- Optimisation: f'(x)=0 at maxima/minima — profit, efficiency, aerodynamics
+- Machine learning: gradient descent trains neural networks by computing derivative of loss with respect to weights; backpropagation uses chain rule
+- Economics: marginal cost/revenue = derivatives; optimal production where they're equal
+- Medicine: drug concentration rates, disease spread (dN/dt = rN)
+Chain rule: derivative of f(g(x)) = f'(g(x)) * g'(x). Foundation of backpropagation.</t>
+        </is>
+      </c>
+      <c r="E357" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="n">
         <v>448</v>
       </c>
-      <c r="B356" s="3" t="inlineStr">
+      <c r="B358" s="3" t="inlineStr">
         <is>
           <t>Sociology</t>
         </is>
       </c>
-      <c r="C356" s="3" t="inlineStr">
+      <c r="C358" s="3" t="inlineStr">
         <is>
           <t>What is social mobility and what actually predicts it?</t>
         </is>
       </c>
-      <c r="D356" s="3" t="inlineStr">
+      <c r="D358" s="3" t="inlineStr">
         <is>
           <t>Movement between socioeconomic strata. Intergenerational (parent to child) vs intragenerational (within lifetime).
 **Great Gatsby Curve** (Miles Corak): more income inequality -&gt; LOWER intergenerational mobility. Denmark (low inequality) = high mobility; US, UK = lower.
@@ -10135,25 +10194,57 @@
 Absolute mobility (exceeding parents in absolute terms) has historically been high; relative mobility much more constrained.</t>
         </is>
       </c>
-      <c r="E356" s="2" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="357">
-      <c r="A357" s="28" t="n">
+      <c r="E358" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="n">
+        <v>448</v>
+      </c>
+      <c r="B359" s="3" t="inlineStr">
+        <is>
+          <t>Sociology</t>
+        </is>
+      </c>
+      <c r="C359" s="3" t="inlineStr">
+        <is>
+          <t>What is structural racism and how does it differ from individual prejudice?</t>
+        </is>
+      </c>
+      <c r="D359" s="3" t="inlineStr">
+        <is>
+          <t>Individual racism: personal prejudiced beliefs or biased actions.
+Structural racism: racial inequality embedded in laws, institutions, policies producing racially disparate outcomes WITHOUT requiring individual racist intent.
+Examples:
+- Redlining (US 1930s-60s): federal maps denied mortgages in Black neighbourhoods -&gt; no homeownership -&gt; no wealth accumulation -&gt; compounding wealth gap for generations
+- Employment: audit studies (identical CVs, different names) — 'Black-sounding' names get 50% fewer callbacks (Bertrand &amp; Mullainathan 2004)
+- Criminal justice: same offences produce harsher sentences for Black defendants
+- Healthcare: Black patients systematically undertreated for pain
+- Intergenerational: neighbourhood/school/wealth partly determined by prior generations' access to biased systems
+Why 'without intent' matters: property-tax school funding isn't individually racist, but if property values were shaped by redlining, outcomes are racially unequal.
+Controversy: critics argue it blurs causation and removes individual agency.</t>
+        </is>
+      </c>
+      <c r="E359" s="2" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="28" t="n">
         <v>449</v>
       </c>
-      <c r="B357" s="29" t="inlineStr">
+      <c r="B360" s="29" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="C357" s="29" t="inlineStr">
+      <c r="C360" s="29" t="inlineStr">
         <is>
           <t>How do batteries work chemically, and what limits their energy density?</t>
         </is>
       </c>
-      <c r="D357" s="29" t="inlineStr">
+      <c r="D360" s="29" t="inlineStr">
         <is>
           <t>Battery = chemical -&gt; electrical energy via spatially separated redox reactions.
 Anode: oxidation (loses electrons). Cathode: reduction (gains electrons). Electrons flow externally (current); ions flow internally through electrolyte.
@@ -10170,25 +10261,56 @@
 **Theoretical limits**: Li-ion ~265 Wh/kg practical; Li-sulfur 2,600 Wh/kg; Li-air 11,680 Wh/kg (comparable to gasoline).</t>
         </is>
       </c>
-      <c r="E357" s="28" t="n">
+      <c r="E360" s="28" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="358">
-      <c r="A358" s="2" t="n">
+    <row r="361">
+      <c r="A361" s="6" t="n">
+        <v>449</v>
+      </c>
+      <c r="B361" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="C361" s="7" t="inlineStr">
+        <is>
+          <t>What is relativity and what does it actually say?</t>
+        </is>
+      </c>
+      <c r="D361" s="7" t="inlineStr">
+        <is>
+          <t>Special Relativity (Einstein 1905): two postulates: (1) laws of physics identical in all inertial frames; (2) speed of light c constant for all observers.
+Consequences (all verified):
+- Time dilation: moving clocks run slow. GPS must correct 38 microseconds/day or errors reach 10km/day
+- Length contraction: objects moving relative to you are shorter
+- Relativity of simultaneity: simultaneous in one frame may not be in another
+- E=mc^2: mass-energy equivalence; tiny mass = enormous energy; foundation of nuclear power
+- Speed limit: nothing with mass can reach c
+General Relativity (1915): mass-energy curves spacetime; objects follow geodesics through curved spacetime — what we observe as gravity.
+Verified: gravitational lensing (Eddington 1919), gravitational waves (LIGO 2015), black holes, GPS corrections, perihelion of Mercury.</t>
+        </is>
+      </c>
+      <c r="E361" s="6" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="B358" s="3" t="inlineStr">
+      <c r="B362" s="3" t="inlineStr">
         <is>
           <t>General Knowledge</t>
         </is>
       </c>
-      <c r="C358" s="3" t="inlineStr">
+      <c r="C362" s="3" t="inlineStr">
         <is>
           <t>What is the most important invention in human history, and why?</t>
         </is>
       </c>
-      <c r="D358" s="3" t="inlineStr">
+      <c r="D362" s="3" t="inlineStr">
         <is>
           <t>Depends on dimension valued. Four strong candidates:
 **Language**: meta-invention enabling all others to accumulate. But may have evolved rather than been invented.
@@ -10200,7 +10322,39 @@
 **Meta-point**: no invention stands alone. Cumulative innovation is humanity's real superpower.</t>
         </is>
       </c>
-      <c r="E358" s="2" t="n">
+      <c r="E362" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="B363" s="3" t="inlineStr">
+        <is>
+          <t>Literature</t>
+        </is>
+      </c>
+      <c r="C363" s="3" t="inlineStr">
+        <is>
+          <t>What is magical realism and why did it emerge from Latin America?</t>
+        </is>
+      </c>
+      <c r="D363" s="3" t="inlineStr">
+        <is>
+          <t>Magical realism: magical elements presented matter-of-factly in realistic narrative — no explanation, no surprise. A character ascends to heaven while doing laundry; recorded as unremarkably as weather.
+Features: magical accepted without question; realistic political/historical context; circular time; permeable line between dream/myth/reality.
+Key authors:
+- Garcia Marquez: One Hundred Years of Solitude (1967) — defining text; Buendia family; insomnia plague; yellow butterflies; Macondo
+- Isabel Allende: House of the Spirits — Chile, political violence, clairvoyance
+- Toni Morrison: Beloved — slavery's trauma; ghost literal and metaphorical
+- Salman Rushdie: Midnight's Children — India's partition
+- Borges: labyrinths, infinite libraries — proto-magical realism
+Why Latin America: oral traditions blend myth and fact; Indigenous cosmologies where spirits coexist with humans; political repression made direct critique dangerous — magical displacement allowed critique of dictatorship; hybrid Indigenous/African/European cultures produced hybrid epistemologies.
+Garcia Marquez on grandmother: 'She told the most atrocious things without batting an eyelid.'</t>
+        </is>
+      </c>
+      <c r="E363" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -10595,14 +10749,14 @@
         </is>
       </c>
       <c r="B21" s="27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>9.06</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="D21" s="27" t="inlineStr">
         <is>
-          <t>169, 210, 236, 255, 349, 393, 415, 440</t>
+          <t>169, 210, 236, 255, 349, 393, 415, 440, 446</t>
         </is>
       </c>
     </row>
@@ -10973,14 +11127,14 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>8.83</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>164, 253, 355, 382, 427, 434</t>
+          <t>164, 253, 355, 382, 427, 434, 450</t>
         </is>
       </c>
     </row>
@@ -11027,14 +11181,14 @@
         </is>
       </c>
       <c r="B45" s="15" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C45" s="15" t="n">
-        <v>9.56</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436, 440</t>
+          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436, 440, 447</t>
         </is>
       </c>
     </row>
@@ -11405,14 +11559,14 @@
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>9.58</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447</t>
+          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447, 449</t>
         </is>
       </c>
     </row>
@@ -11531,14 +11685,14 @@
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C73" s="3" t="n">
-        <v>9.06</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 413, 428, 439, 448</t>
+          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 413, 428, 439, 448, 448</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q451-Q455: Geology, Medicine, Psychology, Astronomy, Literature (367 total)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E363"/>
+  <dimension ref="A1:E368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10358,6 +10358,173 @@
         <v>9</v>
       </c>
     </row>
+    <row r="364">
+      <c r="A364" s="2" t="n">
+        <v>451</v>
+      </c>
+      <c r="B364" s="3" t="inlineStr">
+        <is>
+          <t>Geology</t>
+        </is>
+      </c>
+      <c r="C364" s="3" t="inlineStr">
+        <is>
+          <t>How do earthquakes happen, and what determines their destructiveness?</t>
+        </is>
+      </c>
+      <c r="D364" s="3" t="inlineStr">
+        <is>
+          <t>Earthquakes occur when stress accumulated along fault lines releases suddenly, sending seismic waves through the Earth.
+**Plate tectonics basis**: Earth's lithosphere is divided into ~15 major plates. At boundaries, plates converge, diverge, or slide past each other. Friction locks faults -- stress builds for decades, centuries. When friction is overcome, fault slips -- earthquake.
+**Types of faults**: Strike-slip (San Andreas -- horizontal motion); thrust/reverse (Himalayas -- compression); normal (Basin and Range -- extension). Subduction zones (oceanic plate under continental) produce megathrust quakes -- the largest type (Tohoku 2011, Mw 9.0; Valdivia 1960, Mw 9.5).
+**Magnitude**: Moment magnitude (Mw) measures total energy released. Log scale -- Mw 7 releases ~32x more energy than Mw 6. Mw 9 is approx. 1000x Mw 7.
+**Destructiveness factors**:
+1. Depth: shallow (&lt;70km) = more damage at surface
+2. Distance from epicentre
+3. Soil type: soft sediment amplifies shaking (Mexico City 1985)
+4. Building quality: 2010 Haiti (Mw 7.0) killed 200k; 2011 Christchurch (Mw 6.3) killed 185 -- same magnitude, opposite building standards
+5. Tsunami potential: submarine earthquakes displace water
+**Prediction**: no reliable short-term prediction exists. Long-term probabilistic forecasts (UCERF for California) estimate 63% chance of Mw 6.7+ in Bay Area within 30 years.</t>
+        </is>
+      </c>
+      <c r="E364" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="30" t="n">
+        <v>452</v>
+      </c>
+      <c r="B365" s="31" t="inlineStr">
+        <is>
+          <t>Medicine</t>
+        </is>
+      </c>
+      <c r="C365" s="31" t="inlineStr">
+        <is>
+          <t>What is antibiotic resistance and how serious is the threat?</t>
+        </is>
+      </c>
+      <c r="D365" s="31" t="inlineStr">
+        <is>
+          <t>Antibiotic resistance occurs when bacteria evolve mechanisms to survive drugs that once killed them.
+**Mechanisms**:
+1. Enzyme production: beta-lactamases destroy penicillin ring
+2. Efflux pumps: bacteria actively expel antibiotics
+3. Target modification: MRSA alters penicillin-binding proteins
+4. Reduced permeability: gram-negatives limit drug entry
+**How resistance spreads**: horizontal gene transfer -- bacteria share resistance genes via plasmids (not just vertical inheritance). One resistant bacterium can share its resistance with unrelated species rapidly.
+**Scale of the problem**: WHO labels AMR a top-10 global health threat. 2019: ~1.27 million deaths directly attributable to AMR (Lancet). By 2050: projections of 10 million deaths/year (O'Neill Review 2016) if unchecked -- exceeding cancer.
+**Key culprits**: ESKAPE pathogens (Enterococcus, Staph aureus, Klebsiella, Acinetobacter, Pseudomonas, Enterobacter). CRE (carbapenem-resistant Enterobacteriaceae) resistant to last-resort antibiotics.
+**Drivers**: overprescribing in humans; massive agricultural use (70% of all antibiotics); incomplete courses; poor infection control.
+**Solutions**: new antibiotic development (dry pipeline -- low profit); phage therapy; antibiotic stewardship; vaccines reducing infection rates; rapid diagnostics.</t>
+        </is>
+      </c>
+      <c r="E365" s="30" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="24" t="n">
+        <v>453</v>
+      </c>
+      <c r="B366" s="25" t="inlineStr">
+        <is>
+          <t>Psychology</t>
+        </is>
+      </c>
+      <c r="C366" s="25" t="inlineStr">
+        <is>
+          <t>What is the bystander effect and why does it happen?</t>
+        </is>
+      </c>
+      <c r="D366" s="25" t="inlineStr">
+        <is>
+          <t>The bystander effect: people are less likely to help in an emergency when others are present.
+**Origin**: Kitty Genovese (1964) -- stabbed outside her Queens apartment; 38 witnesses reportedly did nothing. Motivated Darley &amp; Latane's classic experiments.
+**Experiment (1968)**: subject alone or with confederates hears someone having a seizure via intercom. Alone: 85% helped within 52 seconds. With 4 others: only 31% helped within 3 minutes.
+**Mechanisms**:
+1. **Diffusion of responsibility**: 'someone else will help' -- responsibility divided among observers
+2. **Pluralistic ignorance**: everyone looks calm so everyone assumes it's not an emergency so nobody acts
+3. **Evaluation apprehension**: fear of looking foolish if wrong about emergency
+4. **Ambiguity reduction**: unclear situations -- look to others -- see inaction -- assume no problem
+**Reversals**: bystander effect weakens when:
+- Emergency is unambiguous (blood, fire)
+- Bystander has relevant expertise
+- Victim is similar to helper
+- Direct eye contact with victim
+- You point at specific person: 'You in the red -- call 911'
+**Genovese note**: the '38 witnesses saw everything' story was exaggerated by media. Few had full view. Mechanism still real, origin story partly myth.</t>
+        </is>
+      </c>
+      <c r="E366" s="24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="22" t="n">
+        <v>454</v>
+      </c>
+      <c r="B367" s="23" t="inlineStr">
+        <is>
+          <t>Astronomy</t>
+        </is>
+      </c>
+      <c r="C367" s="23" t="inlineStr">
+        <is>
+          <t>What is dark matter and what is the evidence for it?</t>
+        </is>
+      </c>
+      <c r="D367" s="23" t="inlineStr">
+        <is>
+          <t>Dark matter: non-luminous mass that does not interact electromagnetically but does exert gravity. Makes up ~27% of universe's energy budget (ordinary matter ~5%, dark energy ~68%).
+**Evidence**:
+1. **Galaxy rotation curves** (Rubin 1970s): stars at galaxy edges orbit faster than Newtonian gravity from visible matter predicts. Flat rotation curve implies invisible mass halo
+2. **Galaxy clusters**: cluster mass from gravitational lensing far exceeds visible mass. Bullet Cluster (2006): collision of two clusters -- hot gas (visible) slowed by interaction; dark matter (lensing map) passed straight through
+3. **CMB**: acoustic peaks in cosmic microwave background fit perfectly only with ~27% dark matter component
+4. **Large-scale structure**: galaxies form along filaments consistent with cold dark matter simulations (LCDM)
+**What it might be**:
+- WIMPs (weakly interacting massive particles) -- theoretically motivated, null results at LHC and direct detection experiments (LUX, XENONnT)
+- Axions -- very light, QCD-motivated; ALP experiments ongoing
+- Primordial black holes -- LIGO constraints limit contribution
+- Sterile neutrinos
+**Alternative**: MOND (modified Newtonian dynamics) -- adjust gravity instead. Explains rotation curves but fails at cluster scales.
+**Status**: dark matter existence extremely well-supported; its particle nature unknown. A top unsolved problem in physics.</t>
+        </is>
+      </c>
+      <c r="E367" s="22" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="n">
+        <v>455</v>
+      </c>
+      <c r="B368" s="3" t="inlineStr">
+        <is>
+          <t>Literature</t>
+        </is>
+      </c>
+      <c r="C368" s="3" t="inlineStr">
+        <is>
+          <t>What makes Shakespeare's work so enduringly significant?</t>
+        </is>
+      </c>
+      <c r="D368" s="3" t="inlineStr">
+        <is>
+          <t>Shakespeare (1564-1616) wrote 37 plays, 154 sonnets, and long poems across comedy, tragedy, history, and romance -- in 20 years of active writing.
+**Language**: coined or first-recorded ~1,700 words (bedroom, lonely, generous, obscene, swagger). Blank verse (iambic pentameter) flexible enough for noble and colloquial speech alike. Puns, wordplay, metaphor density unprecedented.
+**Psychological depth**: characters reason, contradict themselves, change. Hamlet contemplates inaction; Macbeth understands his own corruption; Iago is evil and self-aware about it; Lear learns through suffering. Predates psychology as field by 300 years but maps inner life precisely.
+**Universality**: tragedies turn on jealousy (Othello), ambition (Macbeth), indecision (Hamlet), family (Lear) -- universal drives. No setting-specific politics that date the work.
+**Influence**: largest influence on English language after King James Bible. Freud used Hamlet to develop Oedipal theory. Harold Bloom argued Shakespeare 'invented the human' -- modern Western self-conception.
+**Survival bias note**: we have ~3,000 plays from Elizabethan era; most lost. Shakespeare's survived partly due to the First Folio (1623), compiled by actors who preserved 18 plays that would otherwise be lost.
+**Ongoing relevance**: performed in every country; adapted across cultures (Kurosawa's Ran = King Lear; 10 Things I Hate About You = Taming of the Shrew). The plays scale across contexts because they're about humans, not Tudor politics.</t>
+        </is>
+      </c>
+      <c r="E368" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10479,14 +10646,14 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>9.529999999999999</v>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>158, 173, 219, 240, 259, 278, 292, 309, 357, 375, 389, 406, 408, 427, 431</t>
+          <t>158, 173, 219, 240, 259, 278, 292, 309, 357, 375, 389, 406, 408, 427, 431, 454</t>
         </is>
       </c>
     </row>
@@ -10947,14 +11114,14 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>9.140000000000001</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>147, 208, 281, 312, 322, 359, 417</t>
+          <t>147, 208, 281, 312, 322, 359, 417, 451</t>
         </is>
       </c>
     </row>
@@ -11127,14 +11294,14 @@
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>8.859999999999999</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>164, 253, 355, 382, 427, 434, 450</t>
+          <t>164, 253, 355, 382, 427, 434, 450, 455</t>
         </is>
       </c>
     </row>
@@ -11217,14 +11384,14 @@
         </is>
       </c>
       <c r="B47" s="31" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C47" s="31" t="n">
-        <v>9.18</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="D47" s="31" t="inlineStr">
         <is>
-          <t>230, 279, 294, 344, 379, 395, 411, 411, 422, 429, 441</t>
+          <t>230, 279, 294, 344, 379, 395, 411, 411, 422, 429, 441, 452</t>
         </is>
       </c>
     </row>
@@ -11631,14 +11798,14 @@
         </is>
       </c>
       <c r="B70" s="25" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C70" s="25" t="n">
-        <v>9.109999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="D70" s="25" t="inlineStr">
         <is>
-          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 424, 432, 437, 445</t>
+          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 424, 432, 437, 445, 453</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q456-Q460: Chemistry, Politics, Nutrition, Math, Anthropology (372 total)
Also fix learning check: correct system prompt is training JSONL's prompt,
not hardcoded 'helpful AI assistant created by Aliyu Yusuf'. 236-entry model
confirmed 4/4 with correct SYS prompt. Previous checks were broken.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E368"/>
+  <dimension ref="A1:E373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10525,6 +10525,174 @@
         <v>9</v>
       </c>
     </row>
+    <row r="369">
+      <c r="A369" s="28" t="n">
+        <v>456</v>
+      </c>
+      <c r="B369" s="29" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="C369" s="29" t="inlineStr">
+        <is>
+          <t>What is entropy, and why does it always increase?</t>
+        </is>
+      </c>
+      <c r="D369" s="29" t="inlineStr">
+        <is>
+          <t>Entropy (S) measures the number of microscopic arrangements (microstates) compatible with a macroscopic state. More arrangements = higher entropy.
+**Second Law of Thermodynamics**: in an isolated system, entropy never decreases. It increases or stays the same.
+**Why it increases**: probability. A gas released into a vacuum spreads out because the disordered states vastly outnumber the ordered ones -- not because of any force, but because disorder is overwhelmingly more likely. Boltzmann: S = k ln(W), where W is the number of microstates.
+**Examples**:
+- Ice melting: liquid water has more microstates than crystal ice
+- Perfume spreading: molecules explore all available space
+- Stars forming: locally decreases entropy (order from gas) but radiates far more entropy as heat
+**Arrow of time**: entropy gives time its direction. The laws of physics are symmetric -- they work the same forward and backward -- but entropy breaks that symmetry. The past is defined as lower entropy.
+**Maxwell's Demon**: thought experiment of a demon sorting fast/slow molecules to decrease entropy. Resolved by Szilard (1929) and Landauer (1961): the demon must erase memory, which costs entropy -- so the second law holds.
+**Heat death**: eventual equilibrium state of universe -- maximum entropy, no temperature differences, no useful work possible.</t>
+        </is>
+      </c>
+      <c r="E369" s="28" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="2" t="n">
+        <v>457</v>
+      </c>
+      <c r="B370" s="3" t="inlineStr">
+        <is>
+          <t>Political Science</t>
+        </is>
+      </c>
+      <c r="C370" s="3" t="inlineStr">
+        <is>
+          <t>What is democracy and why do some democracies fail?</t>
+        </is>
+      </c>
+      <c r="D370" s="3" t="inlineStr">
+        <is>
+          <t>Democracy: a system where political power derives from the governed, expressed through free elections, rule of law, and protection of rights.
+**Types**:
+- Direct (Athens): citizens vote on every decision. Impractical at scale.
+- Representative: elect representatives who govern. Most modern democracies.
+- Liberal democracy: adds constraints on majority power -- minority rights, press freedom, independent judiciary.
+**Why democracies fail (Levitsky &amp; Ziblatt, How Democracies Die, 2018)**:
+1. **Executive aggrandisement**: elected leaders gradually grab power -- filling courts, weakening press, harassing opponents. Legal but antidemocratic.
+2. **Polarisation**: when parties see each other as existential enemies, norms of mutual toleration break down -- 'anything goes to win.'
+3. **Weak institutions**: democracies require strong courts, free press, civil society. Without them, leaders face no check.
+4. **Economic crisis**: Weimar Germany, Venezuela -- economic collapse drives voters to authoritarians promising order.
+**Historical record**: Freedom House 2023 -- 17th consecutive year of democratic decline globally. Hungary and Turkey went from democracy to competitive authoritarianism under elected leaders.
+**What sustains it**: independent judiciary, civilian control of military, strong civic culture, two-party or multi-party competition, peaceful transfers of power as norm.</t>
+        </is>
+      </c>
+      <c r="E370" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="2" t="n">
+        <v>458</v>
+      </c>
+      <c r="B371" s="3" t="inlineStr">
+        <is>
+          <t>Nutrition</t>
+        </is>
+      </c>
+      <c r="C371" s="3" t="inlineStr">
+        <is>
+          <t>What does the science actually say about diet and health?</t>
+        </is>
+      </c>
+      <c r="D371" s="3" t="inlineStr">
+        <is>
+          <t>Nutrition science is hard: humans can't be randomised to diets for decades, self-reporting is unreliable, and food is chemically complex.
+**What the evidence actually supports**:
+1. **Mediterranean diet**: highest quality evidence (PREDIMED RCT, 2013) -- reduces cardiovascular events ~30%. Olive oil, vegetables, fish, nuts, moderate wine.
+2. **Ultra-processed foods (UPF)**: Nova classification. UPFs linked to obesity, T2 diabetes, depression, all-cause mortality in cohort studies. Mechanisms unclear -- could be additives, processing, or displacement of whole foods.
+3. **Fibre**: consistently beneficial -- gut microbiome, colorectal cancer risk, satiety, blood glucose control.
+4. **Added sugar**: strong evidence for metabolic harm at high doses (T2 diabetes, NAFLD).
+5. **Saturated fat**: more complicated than '70s advice -- butter vs processed meat differ. Total fat less important than fat type.
+**Contested**:
+- Red meat: processed clearly harmful; unprocessed uncertain
+- Eggs: probably fine for most people
+- Dairy: no clear harm in most evidence
+- Low-carb vs low-fat: similar outcomes at 1-2 years; adherence is the main driver
+**What we don't know**: optimal macronutrient ratio, individual variation (gut microbiome, genetics), whether associations are causal.
+**Consensus**: varied whole foods, mostly plants, minimal processing, limited added sugar. Almost no controversy about that.</t>
+        </is>
+      </c>
+      <c r="E371" s="2" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="14" t="n">
+        <v>459</v>
+      </c>
+      <c r="B372" s="15" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="C372" s="15" t="inlineStr">
+        <is>
+          <t>What is Godel's incompleteness theorem and why does it matter?</t>
+        </is>
+      </c>
+      <c r="D372" s="15" t="inlineStr">
+        <is>
+          <t>Godel (1931): any consistent formal system powerful enough to describe basic arithmetic contains true statements that cannot be proved within that system.
+**Two theorems**:
+1. **First incompleteness**: for any consistent, sufficiently powerful formal system F, there exists a statement G ('I am not provable in F') that is true but unprovable in F.
+2. **Second incompleteness**: F cannot prove its own consistency.
+**How he did it**: Godel numbering -- encode every formula and proof as a number. Then construct a self-referential formula G that says 'the formula with Godel number X is not provable' where X is the Godel number of G itself. If F is consistent, G can't be proved; if F proves G, F is inconsistent.
+**Why it matters**:
+- Killed Hilbert's programme: math cannot be fully formalised into one complete, consistent system
+- Not 'math is broken' -- it means no single formal system captures all mathematical truth
+- Human mathematicians vs computers: some argue Godel implies human intuition transcends formal systems (Penrose). Contested.
+**Common misconceptions**:
+- Doesn't mean 'everything is unprovable' -- most math is provable
+- Doesn't mean truth is relative
+- Doesn't apply to every formal system -- only those that include arithmetic
+**Impact**: foundations of mathematics, computer science (Turing's halting problem is equivalent), philosophy of mind.</t>
+        </is>
+      </c>
+      <c r="E372" s="14" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="2" t="n">
+        <v>460</v>
+      </c>
+      <c r="B373" s="3" t="inlineStr">
+        <is>
+          <t>Anthropology</t>
+        </is>
+      </c>
+      <c r="C373" s="3" t="inlineStr">
+        <is>
+          <t>What is culture and how does it shape human behaviour?</t>
+        </is>
+      </c>
+      <c r="D373" s="3" t="inlineStr">
+        <is>
+          <t>Culture: the shared beliefs, practices, symbols, values, and norms transmitted across generations within a group. Humans are uniquely cultural animals -- we inherit not just genes but accumulated knowledge.
+**Cultural universals** (Brown 1991): every human culture has language, music, kinship systems, rituals, tools, religion/supernatural beliefs, taboos. But the specific forms vary enormously.
+**How culture shapes behaviour**:
+1. **Cognition**: WEIRD (Western, Educated, Industrial, Rich, Democratic) samples dominate psychology research. Cross-cultural tests show different: perception (Muller-Lyer illusion less effective in non-WEIRD populations), reasoning (analytic vs holistic), self-concept (independent vs interdependent).
+2. **Emotion**: Ekman's 6 basic emotions (fear, anger, joy, sadness, disgust, surprise) show universal facial expressions, but emotional display rules and experience vary. Inuit have many words for snow-related emotional states; some cultures lack a concept of 'depression.'
+3. **Morality**: Haidt's moral foundations (care, fairness, loyalty, authority, purity) -- cultures weight them differently. Individualist cultures emphasise care/fairness; collectivist add loyalty/authority.
+**Nature vs culture**: not a binary. Gene-culture coevolution -- lactase persistence spread where cattle herding developed. Culture shapes which genes are selected.
+**Cultural change**: cultures aren't static. Contact, trade, media, migration all accelerate change. Globalisation homogenises some aspects (English, jeans, smartphones) while local cultures resist and adapt.</t>
+        </is>
+      </c>
+      <c r="E373" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10592,14 +10760,14 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>191, 261, 341, 378</t>
+          <t>191, 261, 341, 378, 460</t>
         </is>
       </c>
     </row>
@@ -10754,14 +10922,14 @@
         </is>
       </c>
       <c r="B12" s="29" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" s="29" t="n">
         <v>9.039999999999999</v>
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>212, 233, 245, 274, 334, 365, 391, 406, 408, 424, 429, 449</t>
+          <t>212, 233, 245, 274, 334, 365, 391, 406, 408, 424, 429, 449, 456</t>
         </is>
       </c>
     </row>
@@ -11348,14 +11516,14 @@
         </is>
       </c>
       <c r="B45" s="15" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C45" s="15" t="n">
-        <v>9.529999999999999</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436, 440, 447</t>
+          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436, 440, 447, 459</t>
         </is>
       </c>
     </row>
@@ -11546,14 +11714,14 @@
         </is>
       </c>
       <c r="B56" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>9</v>
+        <v>8.75</v>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>354, 458</t>
         </is>
       </c>
     </row>
@@ -11780,14 +11948,14 @@
         </is>
       </c>
       <c r="B69" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C69" s="3" t="n">
-        <v>8.75</v>
+        <v>8.83</v>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>197, 415</t>
+          <t>197, 415, 457</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q461-Q465: GPS, Consciousness, 2008 Crisis, Language Acquisition, Cold War (377 total)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E373"/>
+  <dimension ref="A1:E378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10693,6 +10693,172 @@
         <v>9</v>
       </c>
     </row>
+    <row r="374">
+      <c r="A374" s="2" t="n">
+        <v>461</v>
+      </c>
+      <c r="B374" s="3" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C374" s="3" t="inlineStr">
+        <is>
+          <t>How does GPS work, and how accurate can it get?</t>
+        </is>
+      </c>
+      <c r="D374" s="3" t="inlineStr">
+        <is>
+          <t>GPS (Global Positioning System): 31 satellites in medium Earth orbit (~20,200 km), each broadcasting its position and a precise timestamp from atomic clocks.
+**How it works**:
+1. Your receiver picks up signals from at least 4 satellites
+2. Signal travel time x speed of light = distance to each satellite
+3. 3 satellites give a 3D position (trilateration); 4th corrects receiver clock error
+4. Result: latitude, longitude, altitude, time
+**Accuracy**:
+- Standard civilian GPS: 3-5 metres horizontal
+- Differential GPS (DGPS): ground stations correct atmospheric error -- sub-metre
+- RTK (Real-Time Kinematic): carrier phase corrections -- centimetre accuracy. Used in surveying, autonomous vehicles
+- PPP (Precise Point Positioning): ~10cm without base station
+**Sources of error**:
+- Ionospheric delay: charged particles slow signals (~5m error; dual-frequency receivers compensate)
+- Tropospheric delay: water vapour (~1m)
+- Multipath: signals bouncing off buildings
+- Satellite geometry (GDOP): poorly positioned satellites amplify errors
+**Relativistic corrections**: both special relativity (satellites move fast -- clocks slow) and general relativity (gravity weaker at altitude -- clocks fast) must be corrected. Without it: 10km/day position error.
+**Other systems**: GLONASS (Russia), Galileo (EU), BeiDou (China) -- together called GNSS. Multi-constellation receivers are more accurate.</t>
+        </is>
+      </c>
+      <c r="E374" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="2" t="n">
+        <v>462</v>
+      </c>
+      <c r="B375" s="3" t="inlineStr">
+        <is>
+          <t>Cognitive Science</t>
+        </is>
+      </c>
+      <c r="C375" s="3" t="inlineStr">
+        <is>
+          <t>What is consciousness and why is it so hard to explain?</t>
+        </is>
+      </c>
+      <c r="D375" s="3" t="inlineStr">
+        <is>
+          <t>Consciousness is subjective experience -- 'what it is like' to be you. The hardest problem in science.
+**The Hard Problem** (Chalmers 1995): why does physical brain activity give rise to subjective experience (qualia)? We can explain attention, memory, behaviour (easy problems) -- but not why there is 'something it is like' to see red.
+**Major theories**:
+1. **Global Workspace Theory** (Baars, Dehaene): consciousness = information broadcast globally across brain. Explains reportability and access. Doesn't explain why broadcasting feels like anything.
+2. **Integrated Information Theory** (Tononi): consciousness = phi (integrated information). Any system with high phi is conscious. Implies possible consciousness in simple networks; disputed.
+3. **Higher-Order Theories**: you're conscious of X only when you have a thought about X. Explains metacognition.
+4. **Predictive Processing** (Clark, Friston): brain is a prediction machine; consciousness = models of the world and self.
+**Neural correlates**: fMRI shows prefrontal-parietal network active during conscious perception; thalamus as gating mechanism; gamma oscillations at 40Hz correlate with awareness.
+**Disorders of consciousness**: vegetative state patients sometimes show fMRI activity in response to commands -- covert awareness. Raises legal/ethical questions.
+**The mystery remains**: no theory explains why information processing feels like anything. Penrose/Hameroff: quantum effects in microtubules (mostly rejected). Panpsychism: consciousness is fundamental like mass or charge. Most neuroscientists remain physicalists but admit the explanation is missing.</t>
+        </is>
+      </c>
+      <c r="E375" s="2" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="8" t="n">
+        <v>463</v>
+      </c>
+      <c r="B376" s="9" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="C376" s="9" t="inlineStr">
+        <is>
+          <t>What caused the 2008 financial crisis, and did we fix it?</t>
+        </is>
+      </c>
+      <c r="D376" s="9" t="inlineStr">
+        <is>
+          <t>Cascade of interconnected failures -- system designed to fail.
+Housing bubble: 2000-2006, US prices rose ~124%; fueled by low interest rates post-dotcom and predatory subprime lending. Banks lent to borrowers with no income, no assets (NINJA loans).
+**Securitisation machine**: banks packaged mortgages into MBS (mortgage-backed securities), sold to investors. Then CDOs (collateralised debt obligations) -- slices of MBS. Rating agencies stamped AAA on toxic tranches. No one held the risk.
+**Leverage**: banks leveraged 30:1+. Lehman Brothers: $30 of assets per $1 equity. 3% decline = insolvent.
+**Trigger**: 2006 peak, 2007 subprime defaults rise. Bear Stearns hedge funds collapse Aug 2007. Lehman Brothers bankrupt Sep 2008 -- $600B failure, largest in history. Money market funds 'broke the buck.' Credit seized globally.
+**Contagion**: derivatives (especially CDS -- credit default swaps) linked every major institution. AIG wrote $400B in CDS with no capital. Government bailed it out ($182B).
+**Response**: TARP ($700B bank bailout); QE ($3.5T asset purchases); Dodd-Frank 2010 (stress tests, Volcker rule, consumer protection).
+**Fixed?**: Banks are better capitalised (Basel III). But: shadow banking still large; leverage moved to private equity; systemic risk harder to see; political will to regulate fades in good times.</t>
+        </is>
+      </c>
+      <c r="E376" s="8" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="4" t="n">
+        <v>464</v>
+      </c>
+      <c r="B377" s="5" t="inlineStr">
+        <is>
+          <t>Linguistics</t>
+        </is>
+      </c>
+      <c r="C377" s="5" t="inlineStr">
+        <is>
+          <t>How do children learn language so quickly -- and what does it tell us about the mind?</t>
+        </is>
+      </c>
+      <c r="D377" s="5" t="inlineStr">
+        <is>
+          <t>Children go from babbling at 6 months to grammatical sentences at 3 years, mastering a system adults take years to learn deliberately. How?
+**Milestones**: cooing (2m) -&gt; babbling (6m) -&gt; first words (12m) -&gt; two-word phrases (18-24m) -&gt; sentences with grammar (36m). Critical period for native accent acquisition: before ~12 years.
+**Behaviorist view** (Skinner): imitation and reinforcement. Demolished by Chomsky (1959): children produce sentences they've never heard; they overgeneralise rules ('goed', 'mouses'); no amount of reinforcement explains this creativity.
+**Nativist view** (Chomsky): Language Acquisition Device (LAD) -- innate universal grammar. Children are pre-wired for language structure. Evidence: all languages share deep structural properties; deaf children invent grammar spontaneously; creoles have grammar.
+**Social-interactionist view** (Tomasello): children learn by joint attention and intention reading. They map words to what adults intend, not just what they point at. Very social species-specific.
+**Statistical learning** (Saffran): 8-month-olds can segment words from speech by tracking transitional probabilities between syllables -- no explicit teaching.
+**Poverty of stimulus** (Chomsky): input is too impoverished and noisy to explain what children learn. Some grammar must be innate.
+**Current consensus**: probably an interaction -- innate capacities (not full grammar, but learning biases and social cognition) + rich statistical learning + social scaffolding.</t>
+        </is>
+      </c>
+      <c r="E377" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="12" t="n">
+        <v>465</v>
+      </c>
+      <c r="B378" s="13" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="C378" s="13" t="inlineStr">
+        <is>
+          <t>What was the Cold War and how did it shape the modern world?</t>
+        </is>
+      </c>
+      <c r="D378" s="13" t="inlineStr">
+        <is>
+          <t>The Cold War (1947-1991): ideological, geopolitical, and military competition between the US-led West and Soviet-led East -- never direct war between superpowers, but constant proxy conflicts.
+**Origins**: post-WWII power vacuum. USSR occupied Eastern Europe; Truman Doctrine (1947) committed US to containing Soviet expansion; Marshall Plan ($13B) rebuilt Western Europe; NATO founded 1949; Soviets test A-bomb 1949.
+**Key crises**:
+- Korean War 1950-53: first proxy war; 3M dead
+- Berlin crises 1948, 1961 (Wall built)
+- Cuban Missile Crisis 1962: 13 days -- closest to nuclear war; Khrushchev/Kennedy back-channel deal
+- Vietnam 1955-75: US loses first war; 58k American, 2M+ Vietnamese dead
+- Soviet-Afghan War 1979-89: USSR's Vietnam
+**Arms race**: US/USSR built 70,000 nuclear warheads combined. MAD (Mutually Assured Destruction) -- deterrence through guaranteed annihilation. Accidentally stabilising.
+**Space race**: Sputnik 1957, Gagarin 1961, Apollo 11 1969. Drove technology (internet = ARPANET, GPS, microchips).
+**End**: Gorbachev's glasnost and perestroika; economic collapse of USSR; Berlin Wall falls Nov 1989; Soviet dissolution Dec 1991.
+**Legacy**: NATO expansion; US global hegemony; nuclear proliferation; Middle East interventions; China's rise; Russia's revanchism; authoritarian-democracy ideological divide persisting today.</t>
+        </is>
+      </c>
+      <c r="E378" s="12" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10976,14 +11142,14 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>8.94</v>
+        <v>9</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>174, 207, 221, 246, 277, 295, 311, 321, 366</t>
+          <t>174, 207, 221, 246, 277, 295, 311, 321, 366, 462</t>
         </is>
       </c>
     </row>
@@ -11102,14 +11268,14 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>9.109999999999999</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425, 432, 443</t>
+          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425, 432, 443, 463</t>
         </is>
       </c>
     </row>
@@ -11318,14 +11484,14 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C34" s="13" t="n">
-        <v>9.109999999999999</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 436, 442, 444</t>
+          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 436, 442, 444, 465</t>
         </is>
       </c>
     </row>
@@ -11444,14 +11610,14 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>8.85</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>148, 216, 268, 326, 364, 396, 396, 419, 420, 446</t>
+          <t>148, 216, 268, 326, 364, 396, 396, 419, 420, 446, 464</t>
         </is>
       </c>
     </row>
@@ -12056,14 +12222,14 @@
         </is>
       </c>
       <c r="B75" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>9.119999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>283, 314, 410, 434</t>
+          <t>283, 314, 410, 434, 461</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q466-Q470: Epigenetics, Standard Model, Cancer, Free Will, Biodiversity (382 total)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E378"/>
+  <dimension ref="A1:E383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10859,6 +10859,186 @@
         <v>9.5</v>
       </c>
     </row>
+    <row r="379">
+      <c r="A379" s="18" t="n">
+        <v>466</v>
+      </c>
+      <c r="B379" s="19" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C379" s="19" t="inlineStr">
+        <is>
+          <t>What is epigenetics and can you inherit your parents' experiences?</t>
+        </is>
+      </c>
+      <c r="D379" s="19" t="inlineStr">
+        <is>
+          <t>Epigenetics: changes in gene expression that do not involve changes to the DNA sequence itself. The genome is the hardware; the epigenome is the software that determines which genes are active.
+**Mechanisms**:
+1. **DNA methylation**: methyl groups attach to cytosine, typically silencing genes. Inherited through cell division.
+2. **Histone modification**: DNA wraps around histone proteins. Acetylation (relaxes, activates); methylation (condenses, silences). Marks can be heritable.
+3. **Non-coding RNA**: miRNA and lncRNA regulate gene expression post-transcriptionally.
+**Transgenerational inheritance -- what the evidence shows**:
+- Dutch Hunger Winter (1944-45): children and grandchildren of famine-exposed women showed metabolic differences -- higher obesity, cardiovascular disease rates decades later.
+- Swedish Overkalix study: grandfathers' food availability in prepubertal period correlated with grandsons' lifespan.
+- Mouse studies: stressed/obese parents pass epigenetic marks in sperm/eggs that affect offspring behaviour and metabolism.
+**What it does NOT mean**: you cannot pass on skills or memories (Lamarck was still wrong about that). The effects are statistical tendencies, not deterministic programming.
+**Cancer**: epigenetic dysregulation is a hallmark of cancer. Hypermethylation silences tumour suppressors; hypomethylation activates oncogenes. Epigenetic drugs (HDAC inhibitors) are cancer therapeutics.
+**Reversibility**: unlike genetic mutations, epigenetic marks can be reversed -- by environment, diet, drugs. This is both the hope and complexity of epigenetics.</t>
+        </is>
+      </c>
+      <c r="E379" s="18" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="6" t="n">
+        <v>467</v>
+      </c>
+      <c r="B380" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="C380" s="7" t="inlineStr">
+        <is>
+          <t>What is the Standard Model of particle physics and what does it leave out?</t>
+        </is>
+      </c>
+      <c r="D380" s="7" t="inlineStr">
+        <is>
+          <t>The Standard Model (SM): our best description of the fundamental particles and forces of nature. Developed 1960s-1970s, confirmed by decades of experiment.
+**Particles**:
+- Fermions (matter): 6 quarks (up, down, strange, charm, bottom, top) + 6 leptons (electron, muon, tau + their neutrinos)
+- Bosons (force carriers): photon (EM), W+/W- and Z (weak), gluons x8 (strong), Higgs (mass)
+**Forces in SM** (3 of 4):
+- Electromagnetic (QED): photons; infinite range; binds atoms
+- Weak nuclear: W/Z bosons; very short range; radioactive decay, neutrinos
+- Strong nuclear (QCD): gluons; binds quarks inside protons; confinement
+**Higgs mechanism**: gives mass to W/Z bosons and fermions. Higgs boson confirmed at LHC 2012 (Englert and Higgs, Nobel 2013).
+**What SM leaves out**:
+1. **Gravity**: no quantum theory of gravity. General relativity breaks at Planck scale. This is the deepest problem in physics.
+2. **Dark matter**: SM has no candidate particle (WIMPs, axions not in SM)
+3. **Dark energy**: unexplained
+4. **Matter-antimatter asymmetry**: SM predicts equal amounts; we're made of matter
+5. **Neutrino mass**: SM assumes massless; oscillations prove they have mass
+6. **Hierarchy problem**: why is the Higgs so much lighter than Planck mass?
+**Extensions**: Supersymmetry (no evidence at LHC), string theory (not testable yet), extra dimensions. SM accurate to 1 in 10^12 -- most precise theory ever -- but clearly incomplete.</t>
+        </is>
+      </c>
+      <c r="E380" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="30" t="n">
+        <v>468</v>
+      </c>
+      <c r="B381" s="31" t="inlineStr">
+        <is>
+          <t>Medicine</t>
+        </is>
+      </c>
+      <c r="C381" s="31" t="inlineStr">
+        <is>
+          <t>How does cancer develop, and why is it so hard to cure?</t>
+        </is>
+      </c>
+      <c r="D381" s="31" t="inlineStr">
+        <is>
+          <t>Cancer: uncontrolled cell division resulting from accumulated mutations that disable normal growth controls.
+**Hallmarks of cancer** (Hanahan &amp; Weinberg 2000, updated 2011):
+1. Sustaining proliferative signalling
+2. Evading growth suppressors (p53, Rb)
+3. Resisting cell death (apoptosis evasion -- Bcl-2 overexpression)
+4. Enabling replicative immortality (telomerase reactivation)
+5. Inducing angiogenesis (VEGF -- tumour grows blood supply)
+6. Activating invasion and metastasis
+7. Reprogramming energy metabolism (Warburg effect: aerobic glycolysis)
+8. Evading immune destruction
+**Why mutations accumulate**: DNA replication errors (~1 per 10^9 bp per division); environmental mutagens (UV, tobacco, HPV, aflatoxin); repair system failures (BRCA1/2 = defective double-strand break repair).
+**Why it's hard to cure**:
+- **Tumour heterogeneity**: one tumour contains millions of genetically distinct cells. Kill most -&gt; survivors resistant.
+- **Evolution within tumour**: cancer is Darwinian selection under treatment pressure.
+- **Metastasis**: 90% of cancer deaths from metastases, not primary tumour. Micro-metastases invisible at diagnosis.
+- **Normal cell similarity**: hard to target cancer without harming normal rapidly dividing cells.
+**Modern advances**: targeted therapy (imatinib for CML -- BCR-ABL inhibitor; remarkable results); immunotherapy (checkpoint inhibitors -- PD-1/CTLA-4 -- 20% of advanced melanoma achieve durable remission); CAR-T for blood cancers; early detection via liquid biopsy.</t>
+        </is>
+      </c>
+      <c r="E381" s="30" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="16" t="n">
+        <v>469</v>
+      </c>
+      <c r="B382" s="17" t="inlineStr">
+        <is>
+          <t>Philosophy</t>
+        </is>
+      </c>
+      <c r="C382" s="17" t="inlineStr">
+        <is>
+          <t>What is free will and does it exist?</t>
+        </is>
+      </c>
+      <c r="D382" s="17" t="inlineStr">
+        <is>
+          <t>Free will: the capacity to make choices that are genuinely 'up to you' -- not determined by prior causes.
+**Three positions**:
+1. **Hard determinism**: every event, including every thought and choice, is causally determined by prior events + laws of physics. Free will is an illusion. (Laplace's demon: perfect knowledge of physics = predict all future.)
+2. **Libertarian free will** (not political): some choices are genuinely undetermined -- quantum indeterminacy, agent causation, or substance dualism. But random quantum events don't help -- randomness isn't control.
+3. **Compatibilism** (most philosophers): free will and determinism are compatible. 'Free' means acting from your own desires, values, and reasoning -- not external compulsion. Hume, Frankfurt, Dennett.
+**Neuroscience**: Libet (1983) -- readiness potential precedes conscious awareness of intention by ~500ms. Suggests brain 'decides' before you're aware. Replicated but debated: later studies show you can still 'veto'; timing of awareness measurement disputed.
+**Why it matters**:
+- **Moral responsibility**: if no free will, can we blame criminals? Compatibilists: yes -- punishment works; people respond to incentives; it's about shaping future behaviour.
+- **Criminal justice**: some neuroscientists argue we should shift from retributive to rehabilitative justice.
+- **Psychology**: believing in free will correlates with less cheating, more effort, better outcomes (Baumeister 2008).
+**Consensus**: most philosophers are compatibilists. Hard determinism gains ground in neuroscience. The debate is partly definitional -- what counts as 'free'?</t>
+        </is>
+      </c>
+      <c r="E382" s="16" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="n">
+        <v>470</v>
+      </c>
+      <c r="B383" s="3" t="inlineStr">
+        <is>
+          <t>Environmental Science</t>
+        </is>
+      </c>
+      <c r="C383" s="3" t="inlineStr">
+        <is>
+          <t>What is biodiversity and why does losing it matter?</t>
+        </is>
+      </c>
+      <c r="D383" s="3" t="inlineStr">
+        <is>
+          <t>Biodiversity: the variety of life at three levels -- genetic diversity within species, species diversity within ecosystems, ecosystem diversity across the planet.
+**Current scale**: ~8.7 million eukaryotic species estimated (Mora 2011); only ~2 million described. 1 million threatened with extinction (IPBES 2019). Current extinction rate: 100-1000x background rate -- Earth's 6th mass extinction.
+**Why it matters -- ecosystem services**:
+1. **Pollination**: 75% of food crops depend on pollinators. Bee decline threatens food security.
+2. **Pest control**: natural predators suppress agricultural pests. Loss increases pesticide need.
+3. **Carbon sequestration**: forests, wetlands, soils store carbon. Biodiversity sustains these ecosystems.
+4. **Water purification**: wetland plants filter pollutants. Mangroves protect coasts from storms.
+5. **Soil formation**: decomposers, earthworms, mycorrhizae make soil that grows food.
+6. **Medicine**: 50% of drugs derived from natural compounds. Undiscovered species may hold cures.
+**Stability argument**: diverse ecosystems are more resilient to disturbance. Monocultures collapse easily (Irish Potato Famine: single variety wiped out by single pathogen).
+**Drivers of loss** (HIPPO): Habitat loss (primary), Invasive species, Pollution, Population growth, Overharvesting.
+**Intrinsic value**: many argue species have value independent of human use. The last Northern White Rhino is irreplaceable regardless of economic utility.
+**Solutions**: protected areas (30x30 target); wildlife corridors; rewilding; reducing meat consumption (70% of agricultural land for livestock); international agreements (Kunming-Montreal 2022).</t>
+        </is>
+      </c>
+      <c r="E383" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11034,14 +11214,14 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>9.289999999999999</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>156, 171, 181, 222, 243, 266, 282, 287, 297, 304, 313, 383, 400, 400, 417, 421, 431, 435, 438</t>
+          <t>156, 171, 181, 222, 243, 266, 282, 287, 297, 304, 313, 383, 400, 400, 417, 421, 431, 435, 438, 466</t>
         </is>
       </c>
     </row>
@@ -11286,14 +11466,14 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>9.25</v>
+        <v>9.17</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>335, 413</t>
+          <t>335, 413, 470</t>
         </is>
       </c>
     </row>
@@ -11718,14 +11898,14 @@
         </is>
       </c>
       <c r="B47" s="31" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C47" s="31" t="n">
-        <v>9.210000000000001</v>
+        <v>9.23</v>
       </c>
       <c r="D47" s="31" t="inlineStr">
         <is>
-          <t>230, 279, 294, 344, 379, 395, 411, 411, 422, 429, 441, 452</t>
+          <t>230, 279, 294, 344, 379, 395, 411, 411, 422, 429, 441, 452, 468</t>
         </is>
       </c>
     </row>
@@ -11934,14 +12114,14 @@
         </is>
       </c>
       <c r="B59" s="17" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C59" s="17" t="n">
         <v>9.44</v>
       </c>
       <c r="D59" s="17" t="inlineStr">
         <is>
-          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 439, 444</t>
+          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 439, 444, 469</t>
         </is>
       </c>
     </row>
@@ -12060,14 +12240,14 @@
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>9.58</v>
+        <v>9.59</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447, 449</t>
+          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447, 449, 467</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q471-Q475: Addiction, Primes, Trauma, Inflation, Meaning of Life (387 total)
Training restarted after crash at ~step 17800 (no checkpoint lost, resume from 16000).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E383"/>
+  <dimension ref="A1:E388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11039,6 +11039,183 @@
         <v>9</v>
       </c>
     </row>
+    <row r="384">
+      <c r="A384" s="10" t="n">
+        <v>471</v>
+      </c>
+      <c r="B384" s="11" t="inlineStr">
+        <is>
+          <t>Neuroscience</t>
+        </is>
+      </c>
+      <c r="C384" s="11" t="inlineStr">
+        <is>
+          <t>How does addiction work in the brain, and why is it so hard to quit?</t>
+        </is>
+      </c>
+      <c r="D384" s="11" t="inlineStr">
+        <is>
+          <t>Addiction: compulsive substance use or behaviour despite harmful consequences. A brain disease, not a moral failing.
+**The dopamine system**: the mesolimbic pathway (VTA to nucleus accumbens) is the core reward circuit. Normally releases dopamine in response to natural rewards (food, sex, social connection). Drugs hijack this system -- cocaine blocks dopamine reuptake (10x normal spike); heroin mimics endorphins; alcohol enhances GABA and suppresses glutamate.
+**Neuroadaptation**:
+1. **Tolerance**: repeated stimulation downregulates dopamine receptors -- need more drug for same effect
+2. **Withdrawal**: baseline dopamine drops below normal -- dysphoria, craving, physical symptoms
+3. **Sensitisation**: drug cues (environment, paraphernalia) trigger dopamine release even without drug -- Pavlovian conditioning. This persists for years.
+**Prefrontal cortex damage**: addiction impairs the PFC, which controls impulse suppression. Less top-down control over limbic drives. Decision-making becomes biased toward immediate reward.
+**Why quitting is hard**:
+- Withdrawal is acutely miserable
+- Cue-triggered cravings persist for years (rat park experiments: environment matters enormously)
+- Social networks often revolve around substance
+- Underlying trauma/mental illness driving use
+**Treatment**: best evidence for opioid addiction -- methadone and buprenorphine (harm reduction). Naltrexone for alcohol/opioids. CBT, motivational interviewing. Peer support (AA: mixed evidence but social component powerful). No magic cure -- relapse rates ~40-60%.</t>
+        </is>
+      </c>
+      <c r="E384" s="10" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="14" t="n">
+        <v>472</v>
+      </c>
+      <c r="B385" s="15" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="C385" s="15" t="inlineStr">
+        <is>
+          <t>What is a prime number and why do mathematicians care so deeply about them?</t>
+        </is>
+      </c>
+      <c r="D385" s="15" t="inlineStr">
+        <is>
+          <t>A prime number is a natural number greater than 1 with no positive divisors other than 1 and itself. First primes: 2, 3, 5, 7, 11, 13...
+**Fundamental Theorem of Arithmetic**: every integer &gt; 1 is either prime or uniquely factorisable into primes. Primes are the atoms of number theory.
+**Distribution**: primes become sparser as numbers grow, but never stop (Euclid's proof: assume finitely many, multiply them all and add 1 -- the result is divisible by none of them, contradiction). Prime Number Theorem: primes near N appear with density approximately 1/ln(N).
+**Twin primes**: pairs differing by 2 (3,5; 11,13; 17,19). Conjectured to be infinite -- unproven. Zhang 2013: proved gaps &lt; 70 million infinitely often (later reduced to 246 by Maynard).
+**Why mathematicians care**:
+1. **RSA cryptography**: security rests on the difficulty of factoring large semiprimes (p x q). Factor a 2048-bit number and you break internet encryption.
+2. **Riemann Hypothesis**: zeros of the zeta function control prime distribution. Still unproven.
+3. **Addbach's conjecture**: every even integer &gt; 2 is the sum of two primes (e.g. 4=2+2, 28=5+23). Verified to 4x10^18. Unproven.
+4. **Mersenne primes**: of form 2^p - 1. Used in computing, random number generation. Only 51 known.
+**Largest known prime** (as of 2024): 2^136,279,841 - 1 (over 41 million digits). Found by GIMPS distributed computing project.
+**Practical**: AES, RSA, HTTPS, Bitcoin -- all depend on prime-based mathematics.</t>
+        </is>
+      </c>
+      <c r="E385" s="14" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="24" t="n">
+        <v>473</v>
+      </c>
+      <c r="B386" s="25" t="inlineStr">
+        <is>
+          <t>Psychology</t>
+        </is>
+      </c>
+      <c r="C386" s="25" t="inlineStr">
+        <is>
+          <t>What is trauma and how does it rewire the brain?</t>
+        </is>
+      </c>
+      <c r="D386" s="25" t="inlineStr">
+        <is>
+          <t>Trauma: an overwhelming experience that exceeds the capacity to cope, leaving lasting psychological and neurobiological changes.
+**PTSD neurobiology**:
+1. **Amygdala** (fear centre): hyperactivated in PTSD -- threat detection system stuck on high alert. Responds to cues associated with trauma even in safety.
+2. **Hippocampus** (memory): volume reduced in PTSD (~8% smaller on average). Impairs contextualisation of fear memories -- trauma feels present, not past.
+3. **Prefrontal cortex** (regulation): hypoactivated -- reduced capacity to 'talk down' the amygdala. Explains intrusive thoughts, hypervigilance.
+4. **HPA axis**: stress hormone system (cortisol) dysregulated -- either chronically elevated or blunted (as seen in combat veterans).
+**Polyvagal theory** (Porges): trauma hijacks the autonomic nervous system -- freeze, fight, flight. Ventral vagal (social engagement) offline; dorsal vagal (shutdown) engaged.
+**Developmental trauma**: ACEs (Adverse Childhood Experiences) study (Felitti 1998) -- 10 categories of childhood adversity. 4+ ACEs dramatically increase rates of depression, addiction, obesity, heart disease, early death. Dose-response relationship.
+**Treatment**:
+- EMDR (Eye Movement Desensitisation and Reprocessing): evidence-based, possibly reconsolidates traumatic memories
+- Prolonged Exposure: gradual desensitisation
+- CPT (Cognitive Processing Therapy): restructures trauma-related beliefs
+- Ketamine and MDMA-assisted therapy: promising Phase 3 trials for PTSD
+**Resilience**: most people exposed to trauma do NOT develop PTSD. Social support is the strongest protective factor.</t>
+        </is>
+      </c>
+      <c r="E386" s="24" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="8" t="n">
+        <v>474</v>
+      </c>
+      <c r="B387" s="9" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="C387" s="9" t="inlineStr">
+        <is>
+          <t>What is inflation, what causes it, and how is it controlled?</t>
+        </is>
+      </c>
+      <c r="D387" s="9" t="inlineStr">
+        <is>
+          <t>Inflation: a general, sustained rise in the price level -- equivalently, a decline in purchasing power of money.
+**Measurement**: CPI (Consumer Price Index) -- basket of goods/services; PCE (Personal Consumption Expenditures) -- Fed's preferred measure; Core (excludes food and energy -- more stable).
+**Causes**:
+1. **Demand-pull**: too much money chasing too few goods. Economy overheating; spending exceeds productive capacity.
+2. **Cost-push**: supply shocks raise production costs (oil crises 1973, 2022 energy shock) -- firms pass costs to consumers.
+3. **Built-in (wage-price spiral)**: workers demand higher wages to compensate for inflation; firms raise prices to cover wage costs; repeat.
+4. **Monetary**: Milton Friedman: 'Inflation is always and everywhere a monetary phenomenon.' Excessive money supply growth (printing money) devalues currency.
+**Hyperinflation examples**: Weimar Germany 1923 (paper money as wallpaper); Zimbabwe 2008 (100 trillion dollar note); Venezuela 2018 (1,000,000% annual rate).
+**Control -- central bank tools**:
+- **Interest rates**: raise rates -&gt; credit more expensive -&gt; less borrowing/spending -&gt; demand falls -&gt; prices stabilise. 2022-2023: Fed raised rates from 0.25% to 5.25% to fight post-COVID inflation.
+- **Quantitative tightening**: reduce money supply by selling assets.
+- **Reserve requirements**: how much banks must hold vs lend.
+**Trade-off**: fighting inflation slows growth, raises unemployment (Phillips Curve -- inverse relationship, though contested post-1970s stagflation).
+**Target**: most central banks target 2% inflation -- enough to avoid deflation, small enough to not distort decisions.</t>
+        </is>
+      </c>
+      <c r="E387" s="8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="16" t="n">
+        <v>475</v>
+      </c>
+      <c r="B388" s="17" t="inlineStr">
+        <is>
+          <t>Philosophy</t>
+        </is>
+      </c>
+      <c r="C388" s="17" t="inlineStr">
+        <is>
+          <t>What is the meaning of life -- and is it even a well-formed question?</t>
+        </is>
+      </c>
+      <c r="D388" s="17" t="inlineStr">
+        <is>
+          <t>Possibly the oldest philosophical question. The answer depends on what 'meaning' means.
+**Three sub-questions** (Susan Wolf):
+1. What is the meaning of life? (cosmic purpose)
+2. What is a meaningful life? (personal significance)
+3. What makes life worth living? (value, wellbeing)
+**Major answers**:
+**Religious**: life has meaning given by a creator. Purpose is to fulfil divine will, achieve salvation, or realise dharma. Meaning is objective and given, not constructed.
+**Nihilism** (Nietzsche's diagnosis, not prescription): God is dead; with Him, objective meaning is gone. The universe is indifferent. Nothing matters inherently.
+**Existentialism** (Sartre, Camus): existence precedes essence -- we have no preset purpose. We create meaning through authentic choices. Camus: life is absurd (we crave meaning in an indifferent universe); the response is rebellion, not despair.
+**Analytic approaches**:
+- **Desire satisfaction**: life is meaningful when you get what you want. Problem: you can want trivial or harmful things.
+- **Objective list** (Parfit): knowledge, friendship, achievement, aesthetic experience. Meaningful regardless of whether desired.
+- **Engagement theory** (Wolf): meaning arises from active engagement with objectively worthwhile projects.
+**Is it well-formed?** Wittgenstein: 'The solution to the problem of life is seen in the vanishing of the problem.' The question may dissolve under analysis -- not answerable because it's not asking for a specific fact.
+**Working answer** most find satisfying: meaning is constructed, not found. Deep relationships, purposeful work, growth, contribution to something beyond yourself. Consistent across cultures and secular/religious traditions.</t>
+        </is>
+      </c>
+      <c r="E388" s="16" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11448,14 +11625,14 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>9.130000000000001</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425, 432, 443, 463</t>
+          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425, 432, 443, 463, 474</t>
         </is>
       </c>
     </row>
@@ -11862,14 +12039,14 @@
         </is>
       </c>
       <c r="B45" s="15" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C45" s="15" t="n">
-        <v>9.550000000000001</v>
+        <v>9.52</v>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436, 440, 447, 459</t>
+          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436, 440, 447, 459, 472</t>
         </is>
       </c>
     </row>
@@ -11970,14 +12147,14 @@
         </is>
       </c>
       <c r="B51" s="11" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C51" s="11" t="n">
-        <v>9.380000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>152, 217, 238, 241, 254, 269, 289, 299, 302, 332, 362, 385, 403, 403, 423, 435, 441</t>
+          <t>152, 217, 238, 241, 254, 269, 289, 299, 302, 332, 362, 385, 403, 403, 423, 435, 441, 471</t>
         </is>
       </c>
     </row>
@@ -12114,14 +12291,14 @@
         </is>
       </c>
       <c r="B59" s="17" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C59" s="17" t="n">
-        <v>9.44</v>
+        <v>9.42</v>
       </c>
       <c r="D59" s="17" t="inlineStr">
         <is>
-          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 439, 444, 469</t>
+          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 439, 444, 469, 475</t>
         </is>
       </c>
     </row>
@@ -12312,14 +12489,14 @@
         </is>
       </c>
       <c r="B70" s="25" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C70" s="25" t="n">
-        <v>9.1</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="D70" s="25" t="inlineStr">
         <is>
-          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 424, 432, 437, 445, 453</t>
+          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 424, 432, 437, 445, 453, 473</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q476-Q480: Light/PE Effect, Renaissance, Neuroplasticity, Ship of Theseus, Stratification (392 total)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E388"/>
+  <dimension ref="A1:E393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11216,6 +11216,182 @@
         <v>9</v>
       </c>
     </row>
+    <row r="389">
+      <c r="A389" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="B389" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="C389" s="7" t="inlineStr">
+        <is>
+          <t>What is light and what is the photoelectric effect?</t>
+        </is>
+      </c>
+      <c r="D389" s="7" t="inlineStr">
+        <is>
+          <t>Light is electromagnetic radiation -- oscillating electric and magnetic fields propagating through space at c (299,792,458 m/s in vacuum). It behaves as both wave and particle depending on how you measure it.
+**Wave properties**: wavelength determines colour (400nm violet to 700nm red); frequency determines energy (E=hf). Interference, diffraction, polarisation -- all wave behaviour.
+**Particle (photon) properties**: light comes in discrete packets (quanta). Each photon carries energy E=hf where h is Planck's constant.
+**Photoelectric effect**: when light hits a metal surface, electrons are ejected -- but only if frequency exceeds a threshold, regardless of intensity. Low-frequency bright light ejects no electrons; dim high-frequency light does.
+**Classical prediction**: higher intensity should always eject electrons by dumping more energy. This failed.
+**Einstein's explanation (1905, Nobel 1921)**: light comes in photons of energy E=hf. A single photon must have enough energy (high enough frequency) to overcome the electron's binding energy (work function). More photons (intensity) just eject more electrons -- they don't make each ejection easier.
+**Why it matters**:
+- Proved quantisation of light -- established quantum mechanics
+- Solar cells: photons knock electrons free in semiconductor, generating current (same principle)
+- Digital cameras: CCD sensors use photoelectric effect to convert light to electrical signal
+- Night vision, medical X-ray detectors, photomultiplier tubes
+**Wave-particle duality**: light is neither purely wave nor purely particle. It is a quantum object that exhibits both properties depending on experimental setup (double-slit: wave; photodetector: particle).</t>
+        </is>
+      </c>
+      <c r="E389" s="6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="12" t="n">
+        <v>477</v>
+      </c>
+      <c r="B390" s="13" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="C390" s="13" t="inlineStr">
+        <is>
+          <t>What was the Renaissance and why did it happen in Italy?</t>
+        </is>
+      </c>
+      <c r="D390" s="13" t="inlineStr">
+        <is>
+          <t>Renaissance (French: 'rebirth'): European cultural, artistic, and intellectual revival from roughly 1300-1600, centred first in Italian city-states.
+**What it was**: revival of classical Greek and Roman learning; explosion of art, architecture, literature, science, philosophy. Shift from medieval theological focus to humanist celebration of human potential.
+**Key figures**: Leonardo da Vinci (art, engineering, anatomy, everything); Michelangelo (Sistine Chapel, David, Pieta); Raphael; Botticelli; Machiavelli (The Prince -- realpolitik); Petrarch (considered first humanist); Galileo (astronomy, scientific method).
+**Why Italy first?**
+1. **Wealth**: Italian city-states (Florence, Venice, Milan, Rome) were Europe's commercial centres. Banks (Medici), trade, textiles generated surplus for patronage.
+2. **City-state competition**: Medici vs Sforza vs Doge -- rival patrons competing through art and architecture. Florence alone had extraordinary concentration of talent.
+3. **Classical proximity**: Italy sat on Roman ruins. Greek manuscripts flooded in after fall of Constantinople 1453 -- Byzantine scholars fled west with texts.
+4. **Weak feudal system**: merchants, not hereditary nobility, dominated. More social mobility, more secular outlook.
+5. **Church patronage**: popes commissioned art (Sistine Chapel, St Peter's Basilica) -- enormous funding for artists.
+**Spread**: printing press (Gutenberg 1440) spread Renaissance ideas across Europe. Northern Renaissance: Erasmus, More, Shakespeare, Durer.
+**Legacy**: scientific revolution, Reformation, humanism -- the Renaissance ended the Middle Ages and began modernity.</t>
+        </is>
+      </c>
+      <c r="E390" s="12" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="10" t="n">
+        <v>478</v>
+      </c>
+      <c r="B391" s="11" t="inlineStr">
+        <is>
+          <t>Neuroscience</t>
+        </is>
+      </c>
+      <c r="C391" s="11" t="inlineStr">
+        <is>
+          <t>What is neuroplasticity and can the adult brain really change?</t>
+        </is>
+      </c>
+      <c r="D391" s="11" t="inlineStr">
+        <is>
+          <t>Neuroplasticity: the brain's ability to reorganise itself by forming new neural connections throughout life. The old view -- brain fixed after childhood -- is wrong.
+**Types of plasticity**:
+1. **Synaptic plasticity**: individual synapse strength changes. Long-term potentiation (LTP) -- repeated firing strengthens connection ('neurons that fire together wire together', Hebb 1949). Basis of learning and memory.
+2. **Structural plasticity**: physical growth of new dendrites, synapses. Occurs in response to learning and experience.
+3. **Neurogenesis**: new neurons generated in adult brain -- primarily in hippocampus (dentate gyrus) and olfactory bulb. Controversial in humans but confirmed in rodents; human evidence growing.
+4. **Cortical remapping**: brain regions reassign to new functions after injury or deprivation.
+**Evidence**:
+- London taxi drivers: hippocampus posterior enlarged vs controls; size correlated with years of experience (Maguire 2000)
+- Blind individuals: visual cortex repurposed for tactile and auditory processing
+- Stroke recovery: neighbouring regions take over damaged functions with rehabilitation
+- Musicians: enlarged motor cortex representation for fingers; auditory cortex differences
+- Phantom limb: amputated limb representation invaded by face area (Ramachandran) -- explains why touching face triggers phantom sensation
+**Limits**: plasticity declines with age but never stops. Critical periods (language accent, binocular vision) close in childhood. Adult plasticity requires effort, attention, and repetition -- passive exposure doesn't rewire the brain.
+**Implications**: learning is physical change. Sleep consolidates plastic changes. Cognitive reserve from education delays dementia symptoms.</t>
+        </is>
+      </c>
+      <c r="E391" s="10" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="16" t="n">
+        <v>479</v>
+      </c>
+      <c r="B392" s="17" t="inlineStr">
+        <is>
+          <t>Philosophy</t>
+        </is>
+      </c>
+      <c r="C392" s="17" t="inlineStr">
+        <is>
+          <t>What is the Ship of Theseus problem and why does it matter for identity?</t>
+        </is>
+      </c>
+      <c r="D392" s="17" t="inlineStr">
+        <is>
+          <t>The Ship of Theseus: a ship's planks are replaced one by one over time. Eventually every original plank is replaced. Is it still the same ship?
+**Extended version** (Hobbes): if you collected all the original planks and reassembled them, which ship is the 'real' Ship of Theseus?
+**The problem**: it tests intuitions about identity, continuity, and what makes something the same thing over time.
+**Candidate criteria for identity**:
+1. **Material continuity**: same matter = same object. Fails -- our bodies replace most atoms every few years, yet we persist.
+2. **Structural continuity**: same form/structure = same object. Works better but: gradual vs sudden replacement matters?
+3. **Causal continuity**: the right kind of causal chain links past and present. The replacement ship descends causally from the original.
+4. **Functional continuity**: same function, same identity. The sailing ship is the same ship.
+5. **Psychological continuity** (for persons): Locke -- memory links personal identity. Derek Parfit: identity may not be what matters; what matters is psychological continuity and connectedness, even if identity is vague.
+**Real-world stakes**:
+- Personal identity: are you the same person as your 5-year-old self? (almost no shared neurons or memories)
+- Corporations: is Apple the same company that Steve Jobs founded?
+- Nations: is modern Greece the same as ancient Greece?
+- Medical: when does a patient in persistent vegetative state cease to be the same person?
+- AI: if an AI's weights are updated, is it the same system?
+**Parfit's conclusion**: personal identity is not what matters. What matters is psychological connectedness -- and that can hold to varying degrees. This undermines the moral importance we place on strict identity.</t>
+        </is>
+      </c>
+      <c r="E392" s="16" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="2" t="n">
+        <v>480</v>
+      </c>
+      <c r="B393" s="3" t="inlineStr">
+        <is>
+          <t>Sociology</t>
+        </is>
+      </c>
+      <c r="C393" s="3" t="inlineStr">
+        <is>
+          <t>What is social stratification and why do inequalities persist?</t>
+        </is>
+      </c>
+      <c r="D393" s="3" t="inlineStr">
+        <is>
+          <t>Social stratification: the hierarchical arrangement of individuals and groups in society based on wealth, power, prestige, and other resources.
+**Three dimensions** (Weber): class (economic), status (social honour/prestige), party (political power). These often align but can diverge (a respected professor may earn less than a plumber).
+**Major theoretical frameworks**:
+1. **Functionalism** (Davis &amp; Moore 1945): inequality is functional -- it motivates talented people to fill important, demanding roles. Controversial and widely critiqued (ignores structural barriers; assumes meritocracy).
+2. **Conflict theory** (Marx): classes defined by relationship to means of production. Bourgeoisie exploit proletariat. Inequality is maintained by power, ideology, and force -- not merit.
+3. **Bourdieu**: multiple forms of capital -- economic, cultural (education, taste, credentials), social (networks), symbolic (prestige). Elite groups convert one into another, reproducing advantage across generations.
+**Why inequalities persist**:
+- **Intergenerational transmission**: wealth, education, networks, social capital inherited. Estate tax avoidance, legacy admissions, nepotism.
+- **Structural barriers**: neighbourhood schools reflect local tax base; zip code predicts life outcomes.
+- **Cultural reproduction** (Bourdieu): cultural capital (how you speak, what you know, tastes) signals class membership and gatekeeps elite institutions.
+- **Cumulative advantage**: Matthew effect -- 'to those who have, more will be given.' Small early advantages compound (head start in reading -&gt; better school -&gt; better job).
+- **Ideology**: belief in meritocracy legitimises inequality. People blame poverty on individual failure, not structure.
+**Mobility**: US has lower intergenerational mobility than most Western European countries despite 'American Dream' ideology (Chetty et al. 2014). Scandinavia has highest mobility.</t>
+        </is>
+      </c>
+      <c r="E393" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11841,14 +12017,14 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C34" s="13" t="n">
-        <v>9.130000000000001</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 436, 442, 444, 465</t>
+          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 436, 442, 444, 465, 477</t>
         </is>
       </c>
     </row>
@@ -12147,14 +12323,14 @@
         </is>
       </c>
       <c r="B51" s="11" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C51" s="11" t="n">
         <v>9.390000000000001</v>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>152, 217, 238, 241, 254, 269, 289, 299, 302, 332, 362, 385, 403, 403, 423, 435, 441, 471</t>
+          <t>152, 217, 238, 241, 254, 269, 289, 299, 302, 332, 362, 385, 403, 403, 423, 435, 441, 471, 478</t>
         </is>
       </c>
     </row>
@@ -12291,14 +12467,14 @@
         </is>
       </c>
       <c r="B59" s="17" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C59" s="17" t="n">
-        <v>9.42</v>
+        <v>9.4</v>
       </c>
       <c r="D59" s="17" t="inlineStr">
         <is>
-          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 439, 444, 469, 475</t>
+          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 439, 444, 469, 475, 479</t>
         </is>
       </c>
     </row>
@@ -12417,14 +12593,14 @@
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>9.59</v>
+        <v>9.57</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447, 449, 467</t>
+          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447, 449, 467, 476</t>
         </is>
       </c>
     </row>
@@ -12543,14 +12719,14 @@
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C73" s="3" t="n">
         <v>9.029999999999999</v>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 413, 428, 439, 448, 448</t>
+          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 413, 428, 439, 448, 448, 480</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q481-Q485: ML/Neural Nets, Effective Altruism, Batteries, Big Bang, Cognitive Dissonance (397 total)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E393"/>
+  <dimension ref="A1:E398"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11392,6 +11392,191 @@
         <v>9</v>
       </c>
     </row>
+    <row r="394">
+      <c r="A394" s="20" t="n">
+        <v>481</v>
+      </c>
+      <c r="B394" s="21" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="C394" s="21" t="inlineStr">
+        <is>
+          <t>What is machine learning and how does a neural network actually learn?</t>
+        </is>
+      </c>
+      <c r="D394" s="21" t="inlineStr">
+        <is>
+          <t>Machine learning: systems that improve their performance on a task through experience, without being explicitly programmed with rules.
+**Three paradigms**:
+1. **Supervised**: learn from labelled examples (input -&gt; correct output). Classification, regression.
+2. **Unsupervised**: find patterns in unlabelled data. Clustering, dimensionality reduction.
+3. **Reinforcement**: agent takes actions, receives rewards, learns policy maximising cumulative reward.
+**How a neural network learns**:
+1. **Forward pass**: input flows through layers of neurons. Each neuron: weighted sum of inputs + bias, passed through activation function (ReLU, sigmoid). Output is a prediction.
+2. **Loss**: compare prediction to ground truth using a loss function (cross-entropy for classification, MSE for regression).
+3. **Backpropagation**: compute gradient of loss with respect to every weight -- using chain rule of calculus. How much did each weight contribute to the error?
+4. **Gradient descent**: update each weight in the direction that reduces loss: w = w - lr * gradient. Learning rate controls step size.
+5. **Repeat**: billions of times over the training data (stochastic gradient descent: mini-batches).
+**What networks learn**: not rules. Distributed representations. Early layers detect edges/colours; middle layers detect shapes; later layers detect objects. Hierarchy of features, emergent from optimisation.
+**Key innovations**: ReLU (avoids vanishing gradient), dropout (prevents overfitting), batch normalisation (stabilises training), attention mechanism (transformers -- learns which parts of input to focus on).
+**Scale matters**: more parameters + more data + more compute = better performance. GPT-4 has ~1 trillion parameters; trained on internet-scale text.</t>
+        </is>
+      </c>
+      <c r="E394" s="20" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="2" t="n">
+        <v>482</v>
+      </c>
+      <c r="B395" s="3" t="inlineStr">
+        <is>
+          <t>Ethics</t>
+        </is>
+      </c>
+      <c r="C395" s="3" t="inlineStr">
+        <is>
+          <t>What is effective altruism and what are the strongest criticisms of it?</t>
+        </is>
+      </c>
+      <c r="D395" s="3" t="inlineStr">
+        <is>
+          <t>Effective altruism (EA): a philosophical and social movement using evidence and reason to determine the most effective ways to benefit others.
+**Core ideas** (Peter Singer, William MacAskill):
+- Cause neutrality: don't assume your local community or country matters more
+- Impartiality: future people and distant strangers count equally
+- Evidence-based: measure impact rigorously (GiveWell: cost per life saved)
+- Earning to give: high-salary career + donating effectively can do more good than low-pay NGO work
+- Longtermism: existential risks (AI, pandemics, nuclear) affect vastly more future people -- may outweigh all present suffering
+**Top EA causes**: global health (malaria nets, deworming -- GiveDirectly, Against Malaria Foundation); animal welfare (factory farming causes immense suffering at scale); AI safety (preventing catastrophic AI risk).
+**Strongest criticisms**:
+1. **Systemic change neglect**: EA focuses on charity, not structural causes of poverty. Fixes symptoms, not systems (Amia Srinivasan).
+2. **Legibility bias**: only measurable impacts count. Hard-to-measure things (art, culture, community, dignity) get ignored.
+3. **Longtermism hubris**: speculative future trillions outweigh present suffering -- used to justify ignoring current needs for uncertain future benefits.
+4. **Demandingness**: Singer's argument (drowning child) implies most people should give until marginal utility of their money equals marginal utility of recipient -- radical implication most reject.
+5. **FTX scandal** (2022): Sam Bankman-Fried, prominent EA figure, committed massive fraud 'for the greater good' -- exposed utilitarian ends-justify-means risk.
+**Response from EA**: criticisms taken seriously; movement has evolved. Systemic change and policy increasingly included.</t>
+        </is>
+      </c>
+      <c r="E395" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="28" t="n">
+        <v>483</v>
+      </c>
+      <c r="B396" s="29" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="C396" s="29" t="inlineStr">
+        <is>
+          <t>How do batteries work, and what are the limits of lithium-ion?</t>
+        </is>
+      </c>
+      <c r="D396" s="29" t="inlineStr">
+        <is>
+          <t>A battery converts chemical energy to electrical energy through controlled redox (reduction-oxidation) reactions.
+**Basic principle**: two electrodes (anode and cathode) separated by electrolyte. At anode: oxidation -- atoms lose electrons. At cathode: reduction -- atoms gain electrons. Electrons flow through external circuit (that's the current). Ions flow through electrolyte to balance charge.
+**Lithium-ion (dominant technology)**:
+- Anode: graphite (lithium ions intercalate between carbon layers during charging)
+- Cathode: lithium metal oxide (LiCoO2, LiFePO4, NMC variants)
+- Electrolyte: lithium salt in organic solvent
+- Charging: external current forces Li+ from cathode to anode; discharging reverses
+- Energy density: ~250 Wh/kg (much better than lead-acid at 35 Wh/kg)
+**Why lithium?**: lightest metal, high electrochemical potential, small ion fits in electrode lattices.
+**Limits of lithium-ion**:
+1. **Energy density ceiling**: theoretical max ~350 Wh/kg -- approaching it. Not enough for long-haul aviation or shipping.
+2. **Dendrite growth**: lithium metal anodes (better density) form needle-like dendrites that pierce separator -- short circuit, fire.
+3. **Thermal runaway**: puncture, overcharge, or manufacturing defect can cascade to fire. Aviation bans bulk Li shipment.
+4. **Cycle degradation**: capacity fades after 500-1000 charge cycles. SEI (solid electrolyte interphase) layer grows.
+5. **Supply chain**: cobalt (DRC, ethical concerns), lithium (Chile/Australia), nickel -- geopolitically concentrated.
+**Next generation**: solid-state batteries (solid electrolyte -- no fire risk, higher density, faster charge); lithium-sulphur (theoretical 2600 Wh/kg); sodium-ion (cheaper, abundant). All face commercialisation challenges.</t>
+        </is>
+      </c>
+      <c r="E396" s="28" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="22" t="n">
+        <v>484</v>
+      </c>
+      <c r="B397" s="23" t="inlineStr">
+        <is>
+          <t>Astronomy</t>
+        </is>
+      </c>
+      <c r="C397" s="23" t="inlineStr">
+        <is>
+          <t>How did the universe begin, and what happened in the first seconds?</t>
+        </is>
+      </c>
+      <c r="D397" s="23" t="inlineStr">
+        <is>
+          <t>The Big Bang: the universe began ~13.8 billion years ago from an extremely hot, dense state. Not an explosion in space -- an expansion of space itself.
+**Evidence**:
+1. **Hubble expansion** (1929): galaxies receding -- further away, faster recession. Run time backward: convergence.
+2. **CMB** (Cosmic Microwave Background): Penzias &amp; Wilson 1965 -- faint 2.7K microwave radiation in every direction. Predicted by Big Bang theory as afterglow of recombination.
+3. **Light element abundances**: Big Bang nucleosynthesis predicts ~75% hydrogen, ~25% helium, trace lithium. Observed match is precise.
+**First seconds** (timeline):
+- t=10^-43s (Planck time): physics breaks down. Quantum gravity needed.
+- t=10^-36s: inflation -- exponential expansion (10^26 in 10^-33s). Explains flatness and horizon problems.
+- t=10^-12s: electroweak phase transition -- weak and electromagnetic forces separate.
+- t=10^-6s: quarks confine into protons and neutrons (quark-hadron transition).
+- t=1s: neutrinos decouple; electron-positron annihilation heats photons.
+- t=3min: nucleosynthesis -- protons and neutrons fuse into helium nuclei. Stops when universe cools too much.
+- t=380,000 years: recombination -- electrons combine with nuclei; universe becomes transparent. CMB emitted.
+- t=400M years: first stars ignite (Population III stars -- pure hydrogen/helium, massive, short-lived).
+**What came before?**: unknown. Hawking: the question may be meaningless -- 'before' requires time, which began with the Big Bang. Some models: eternal inflation, cyclic universes, quantum fluctuation from nothing.</t>
+        </is>
+      </c>
+      <c r="E397" s="22" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="24" t="n">
+        <v>485</v>
+      </c>
+      <c r="B398" s="25" t="inlineStr">
+        <is>
+          <t>Psychology</t>
+        </is>
+      </c>
+      <c r="C398" s="25" t="inlineStr">
+        <is>
+          <t>What is cognitive dissonance and how do people resolve it?</t>
+        </is>
+      </c>
+      <c r="D398" s="25" t="inlineStr">
+        <is>
+          <t>Cognitive dissonance (Festinger 1957): the mental discomfort that arises when a person holds two or more contradictory beliefs, values, or when their actions contradict their beliefs.
+**Classic experiment** (Festinger &amp; Carlsmith 1959): subjects did a boring task, then told the next participant it was interesting -- for $1 or $20. Those paid $1 rated the task as more enjoyable. Why? $20 justified the lie; $1 didn't -- so the $1 group changed their belief to reduce dissonance.
+**How people resolve dissonance**:
+1. **Change the belief**: smoker learns smoking causes cancer -&gt; quits. Ideal but hardest.
+2. **Change the behaviour**: actually quits. Also ideal.
+3. **Add consonant cognitions**: 'I know smokers who lived to 100'; 'Stress kills too'; 'I'll quit eventually.' Easier but doesn't solve the problem.
+4. **Reduce importance**: 'Health isn't everything.' Minimise the dissonant element.
+5. **Denial**: ignore or reject the contradictory evidence. Most common under threat.
+**Real-world examples**:
+- Cult members whose prophecy fails: often double down rather than leave (Festinger's 'When Prophecy Fails' 1956)
+- Hazing: 'I suffered to join, so this group must be valuable' (justification of effort)
+- Consumer psychology: post-purchase rationalisation -- we believe we made a good choice to reduce doubt
+- Political beliefs: voters ignore evidence contradicting their candidate
+**Self-perception theory** (Bem): alternative explanation -- we infer our beliefs from observing our behaviour, not necessarily from resolving discomfort. Both theories explain some results better.
+**Why it matters**: understanding dissonance explains why people are resistant to changing minds even with evidence. The threat model: contradicting a core belief is perceived as an attack on the self.</t>
+        </is>
+      </c>
+      <c r="E398" s="24" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11513,14 +11698,14 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>9.529999999999999</v>
+        <v>9.56</v>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>158, 173, 219, 240, 259, 278, 292, 309, 357, 375, 389, 406, 408, 427, 431, 454</t>
+          <t>158, 173, 219, 240, 259, 278, 292, 309, 357, 375, 389, 406, 408, 427, 431, 454, 484</t>
         </is>
       </c>
     </row>
@@ -11621,14 +11806,14 @@
         </is>
       </c>
       <c r="B12" s="29" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C12" s="29" t="n">
         <v>9.039999999999999</v>
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>212, 233, 245, 274, 334, 365, 391, 406, 408, 424, 429, 449, 456</t>
+          <t>212, 233, 245, 274, 334, 365, 391, 406, 408, 424, 429, 449, 456, 483</t>
         </is>
       </c>
     </row>
@@ -11711,14 +11896,14 @@
         </is>
       </c>
       <c r="B17" s="21" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C17" s="21" t="n">
-        <v>9.25</v>
+        <v>9.27</v>
       </c>
       <c r="D17" s="21" t="inlineStr">
         <is>
-          <t>157, 184, 252, 258, 352, 377, 388, 398, 398, 409, 426, 428, 437, 443</t>
+          <t>157, 184, 252, 258, 352, 377, 388, 398, 398, 409, 426, 428, 437, 443, 481</t>
         </is>
       </c>
     </row>
@@ -11855,14 +12040,14 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>9.119999999999999</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>160, 225, 260, 285, 310, 338, 369, 419</t>
+          <t>160, 225, 260, 285, 310, 338, 369, 419, 482</t>
         </is>
       </c>
     </row>
@@ -12665,14 +12850,14 @@
         </is>
       </c>
       <c r="B70" s="25" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C70" s="25" t="n">
-        <v>9.119999999999999</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="D70" s="25" t="inlineStr">
         <is>
-          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 424, 432, 437, 445, 453, 473</t>
+          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 424, 432, 437, 445, 453, 473, 485</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q486-Q490: Immune System, Relativity, Game Theory, French Revolution, Evolution (402 total)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E398"/>
+  <dimension ref="A1:E403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11577,6 +11577,195 @@
         <v>9</v>
       </c>
     </row>
+    <row r="399">
+      <c r="A399" s="30" t="n">
+        <v>486</v>
+      </c>
+      <c r="B399" s="31" t="inlineStr">
+        <is>
+          <t>Medicine</t>
+        </is>
+      </c>
+      <c r="C399" s="31" t="inlineStr">
+        <is>
+          <t>How does the immune system actually work?</t>
+        </is>
+      </c>
+      <c r="D399" s="31" t="inlineStr">
+        <is>
+          <t>The immune system: a layered defence network that distinguishes self from non-self and eliminates pathogens.
+**Two branches**:
+1. **Innate immunity** (fast, non-specific): first responders. Physical barriers (skin, mucus); phagocytes (neutrophils, macrophages) engulf invaders; natural killer cells destroy infected cells; complement proteins puncture bacteria; inflammation signals danger.
+2. **Adaptive immunity** (slow, specific, memory): tailored to each threat.
+   - **B cells**: produce antibodies -- Y-shaped proteins that bind antigens on pathogens. IgG (blood), IgA (gut/lungs), IgE (allergies).
+   - **T cells**: helper T cells (CD4+) coordinate immune response; cytotoxic T cells (CD8+) kill infected cells directly.
+   - **Memory cells**: persist after infection -- next exposure triggers faster, stronger response. Basis of vaccination.
+**How it recognises threats**: pattern recognition receptors (Toll-like receptors) detect molecular patterns shared by pathogens (bacterial LPS, viral RNA) -- absent in healthy human cells.
+**MHC (Major Histocompatibility Complex)**: every cell displays peptide fragments on MHC molecules. T cells check these. Foreign peptide = kill. Self peptide = leave alone. MHC mismatch is why transplants are rejected.
+**How it avoids attacking self**: thymic education -- T cells that react to self-antigens are deleted in the thymus. Failures cause autoimmune disease (Type 1 diabetes, lupus, MS, rheumatoid arthritis).
+**Vaccines**: show the immune system a harmless version of a pathogen (live attenuated, killed, subunit, or mRNA-encoded antigen). Memory cells form. Real infection triggers rapid recall response before disease establishes.</t>
+        </is>
+      </c>
+      <c r="E399" s="30" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="6" t="n">
+        <v>487</v>
+      </c>
+      <c r="B400" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="C400" s="7" t="inlineStr">
+        <is>
+          <t>What is relativity and why does it matter for everyday technology?</t>
+        </is>
+      </c>
+      <c r="D400" s="7" t="inlineStr">
+        <is>
+          <t>Einstein's two theories of relativity reshaped our understanding of space, time, mass, and energy.
+**Special Relativity (1905)**:
+- **Two postulates**: (1) laws of physics are the same in all inertial frames; (2) speed of light c is the same for all observers regardless of motion.
+- **Consequences**: time dilation (moving clocks run slow -- gamma factor = 1/sqrt(1-v^2/c^2)); length contraction; mass-energy equivalence E=mc^2.
+- **Simultaneity is relative**: two events simultaneous in one frame are not in another moving frame.
+**General Relativity (1915)**:
+- **Equivalence principle**: gravity and acceleration are locally indistinguishable. A person in a rocket accelerating at g feels identical to standing on Earth.
+- **Space-time curvature**: mass-energy curves space-time. Objects follow geodesics (straightest paths) in curved space-time -- this IS gravity.
+- **Predictions**: gravitational time dilation (clocks run slower in stronger gravity); gravitational lensing (light bends around mass); black holes; gravitational waves (confirmed LIGO 2015).
+**Why it matters for everyday technology**:
+- **GPS**: satellites move fast (SR: clocks slow by 7 microseconds/day) and are farther from Earth's gravity (GR: clocks fast by 45 microseconds/day). Net: +38 microseconds/day. Uncorrected: GPS drifts 10 km/day. Corrected in software -- every GPS device applies relativity.
+- **Particle accelerators**: relativistic mass increase accounted for in LHC design.
+- **Nuclear energy**: E=mc^2 -- small mass loss in fission/fusion releases enormous energy.
+- **PET scans**: positron-electron annihilation produces gamma rays analysed using relativistic kinematics.</t>
+        </is>
+      </c>
+      <c r="E400" s="6" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="8" t="n">
+        <v>488</v>
+      </c>
+      <c r="B401" s="9" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="C401" s="9" t="inlineStr">
+        <is>
+          <t>What is game theory and where does it actually apply?</t>
+        </is>
+      </c>
+      <c r="D401" s="9" t="inlineStr">
+        <is>
+          <t>Game theory: the mathematical study of strategic interactions -- situations where each player's outcome depends on others' choices.
+**Core concepts**:
+- **Players**: decision-makers with defined strategies and payoffs
+- **Strategies**: complete plans for every contingency
+- **Payoffs**: outcomes for each combination of strategies
+- **Nash Equilibrium**: no player can improve by unilaterally deviating
+**Key games**:
+- **Prisoner's Dilemma**: individual rationality leads to collectively worse outcome (defect/defect worse than cooperate/cooperate). Explains arms races, overfishing, climate action failure.
+- **Chicken**: both players prefer to swerve, but each wants the other to swerve. Nuclear deterrence modelled this way.
+- **Stag Hunt**: cooperation gives best outcome but requires trust. Explains why societies get stuck in low-trust equilibria.
+- **Repeated games**: folk theorem -- cooperation can emerge if players interact repeatedly and value the future (tit-for-tat in iterated Prisoner's Dilemma).
+**Real applications**:
+1. **Auctions**: Vickrey auction (second-price sealed bid) makes truthful bidding dominant strategy. FCC spectrum auctions designed using game theory.
+2. **Nuclear strategy**: MAD -- mutually assured destruction is a Nash equilibrium (neither side benefits from first strike if retaliation guaranteed).
+3. **Economics**: oligopoly pricing (OPEC), labour bargaining, trade policy.
+4. **Biology**: evolutionarily stable strategies (Maynard Smith) -- hawk-dove game explains animal conflict.
+5. **Platform economics**: two-sided markets (Uber, Airbnb) designed using mechanism design.
+**Limits**: assumes rationality; real humans cooperate more than theory predicts (ultimatum game -- people reject unfair offers even at cost to themselves). Behavioural game theory adds psychology.</t>
+        </is>
+      </c>
+      <c r="E401" s="8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="12" t="n">
+        <v>489</v>
+      </c>
+      <c r="B402" s="13" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="C402" s="13" t="inlineStr">
+        <is>
+          <t>What was the French Revolution and why did it matter?</t>
+        </is>
+      </c>
+      <c r="D402" s="13" t="inlineStr">
+        <is>
+          <t>The French Revolution (1789-1799): the most consequential political upheaval in modern history, dismantling the old order and establishing principles that still define democratic governance.
+**Causes**:
+1. **Fiscal crisis**: France bankrupt after supporting American Revolution; Louis XVI unable to tax nobility.
+2. **Enlightenment ideas**: Rousseau, Voltaire, Locke -- popular sovereignty, natural rights, critique of absolute monarchy.
+3. **Food crisis**: 1788 harvest failure; bread prices soaring; common people starving while aristocracy was exempt from taxes.
+4. **Social structure**: three estates -- clergy (1st), nobility (2nd), everyone else (3rd, 97% of population). Third Estate paid all taxes, had no political power.
+**Key events**:
+- 1789: Estates-General convened; Third Estate forms National Assembly; Bastille stormed (July 14); Declaration of Rights of Man
+- 1791: Constitutional monarchy established
+- 1792: War with Austria/Prussia; monarchy abolished; First Republic
+- 1793-94: Reign of Terror (Robespierre, Committee of Public Safety) -- 17,000 executed; 40,000 died in custody
+- 1795: Thermidorian Reaction -- moderates take power
+- 1799: Napoleon's coup (18 Brumaire) ends the Revolution
+**Why it mattered**:
+- Established that sovereignty belongs to the people, not God or kings
+- Liberty, Equality, Fraternity became template for democratic movements worldwide
+- Abolished feudalism and privileges of birth overnight
+- Triggered waves of revolution across Europe (1830, 1848)
+- Napoleon spread revolutionary legal codes (Code Napoleon) across Europe
+- Showed revolutions can consume their own children (Robespierre guillotined)</t>
+        </is>
+      </c>
+      <c r="E402" s="12" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="18" t="n">
+        <v>490</v>
+      </c>
+      <c r="B403" s="19" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C403" s="19" t="inlineStr">
+        <is>
+          <t>What is evolution by natural selection and what are the most common misconceptions?</t>
+        </is>
+      </c>
+      <c r="D403" s="19" t="inlineStr">
+        <is>
+          <t>Evolution by natural selection (Darwin 1859, Wallace co-discovery): populations of organisms change over generations because individuals with heritable traits better suited to their environment survive and reproduce more.
+**Four requirements**:
+1. **Variation**: individuals in population differ
+2. **Heritability**: variation is passed to offspring
+3. **Differential reproduction**: some variants reproduce more
+4. **Time**: accumulate over generations
+**Mechanisms**: natural selection (environment filters); sexual selection (mate choice); genetic drift (random changes, important in small populations); gene flow (migration); mutation (source of new variation).
+**Evidence**: fossil record (transitional forms); comparative anatomy (homologous structures -- bat wing/human hand/whale flipper share bones); molecular evidence (shared DNA, endogenous retroviruses); observed evolution (antibiotic resistance; peppered moths; Galapagos finches beak changes in real time, Grant 1973).
+**Most common misconceptions**:
+1. 'Evolution is just a theory' -- in science, theory means well-supported explanatory framework (gravity is also 'just a theory')
+2. 'Organisms evolve on purpose' -- selection has no goal; it is blind. Giraffes didn't try to grow long necks.
+3. 'Humans evolved from chimps' -- humans and chimps share a common ancestor ~6-7 million years ago.
+4. 'Evolution means progress' -- no direction or improvement, just fit to current environment. A bacterium is as evolved as a human.
+5. 'Missing link' -- all fossils are transitional. Tiktaalik (fish with limb-like fins) is one famous example.
+6. 'It's random' -- mutation is random; selection is not. Selection is the non-random part.
+**Modern synthesis**: Darwinian selection + Mendelian genetics + molecular biology. Supplemented now by evo-devo (development), epigenetics, niche construction.</t>
+        </is>
+      </c>
+      <c r="E403" s="18" t="n">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11752,14 +11941,14 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>9.279999999999999</v>
+        <v>9.31</v>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>156, 171, 181, 222, 243, 266, 282, 287, 297, 304, 313, 383, 400, 400, 417, 421, 431, 435, 438, 466</t>
+          <t>156, 171, 181, 222, 243, 266, 282, 287, 297, 304, 313, 383, 400, 400, 417, 421, 431, 435, 438, 466, 490</t>
         </is>
       </c>
     </row>
@@ -11986,14 +12175,14 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C22" s="9" t="n">
         <v>9.119999999999999</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425, 432, 443, 463, 474</t>
+          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425, 432, 443, 463, 474, 488</t>
         </is>
       </c>
     </row>
@@ -12202,14 +12391,14 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C34" s="13" t="n">
-        <v>9.119999999999999</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 436, 442, 444, 465, 477</t>
+          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 436, 442, 444, 465, 477, 489</t>
         </is>
       </c>
     </row>
@@ -12436,14 +12625,14 @@
         </is>
       </c>
       <c r="B47" s="31" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C47" s="31" t="n">
-        <v>9.23</v>
+        <v>9.25</v>
       </c>
       <c r="D47" s="31" t="inlineStr">
         <is>
-          <t>230, 279, 294, 344, 379, 395, 411, 411, 422, 429, 441, 452, 468</t>
+          <t>230, 279, 294, 344, 379, 395, 411, 411, 422, 429, 441, 452, 468, 486</t>
         </is>
       </c>
     </row>
@@ -12778,14 +12967,14 @@
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C66" s="7" t="n">
         <v>9.57</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447, 449, 467, 476</t>
+          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447, 449, 467, 476, 487</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q491-Q495: Microbiome, Black Holes, Crime, Internet, Calculus (407 total)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E403"/>
+  <dimension ref="A1:E408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11766,6 +11766,167 @@
         <v>10</v>
       </c>
     </row>
+    <row r="404">
+      <c r="A404" s="30" t="n">
+        <v>491</v>
+      </c>
+      <c r="B404" s="31" t="inlineStr">
+        <is>
+          <t>Medicine</t>
+        </is>
+      </c>
+      <c r="C404" s="31" t="inlineStr">
+        <is>
+          <t>What is the microbiome and how does it affect health?</t>
+        </is>
+      </c>
+      <c r="D404" s="31" t="inlineStr">
+        <is>
+          <t>The microbiome: the ~38 trillion microorganisms (bacteria, fungi, archaea, viruses) living in and on the human body -- roughly equal to the number of human cells. The gut microbiome is the most studied.
+**What it does**:
+1. **Digestion**: breaks down complex carbohydrates, fibres, produces short-chain fatty acids (SCFAs -- butyrate, propionate, acetate) that feed colonocytes and regulate inflammation.
+2. **Immune training**: ~70% of immune system is gut-associated. Microbiome educates immune cells to distinguish friend from foe. Germ-free mice have severely underdeveloped immune systems.
+3. **Neurotransmitters**: gut produces ~90% of body's serotonin. Gut-brain axis -- vagus nerve carries signals bidirectionally. Dysbiosis linked to depression, anxiety.
+4. **Vitamin synthesis**: B12, K2, some B vitamins.
+5. **Pathogen resistance**: competitive exclusion -- colonised gut harder for pathogens to invade (C. diff flourishes when antibiotics wipe out competition).
+**Dysbiosis and disease**: disrupted microbiome linked to IBD, IBS, obesity, Type 2 diabetes, colorectal cancer, autism (correlation, causation unclear), depression. Antibiotic overuse = major disruptor.
+**Faecal microbiota transplant (FMT)**: transfer of donor stool to recipient. 90% cure rate for recurrent C. diff infection -- best evidence of microbiome causation. Clinical trials ongoing for IBD, obesity, cancer.
+**What builds a healthy microbiome**: fibre diversity (30 different plants per week -- Tim Spector research); fermented foods (yogurt, kefir, kimchi -- Sonnenburg 2021 RCT shows increased microbiome diversity); avoid unnecessary antibiotics; vaginal birth and breastfeeding inoculate infant microbiome.
+**Caveats**: most microbiome research is correlational. Probiotic supplements have weak evidence for healthy adults. The field is young -- many claims outpace evidence.</t>
+        </is>
+      </c>
+      <c r="E404" s="30" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="6" t="n">
+        <v>492</v>
+      </c>
+      <c r="B405" s="7" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="C405" s="7" t="inlineStr">
+        <is>
+          <t>What is a black hole and what happens at the singularity?</t>
+        </is>
+      </c>
+      <c r="D405" s="7" t="inlineStr">
+        <is>
+          <t>A black hole: a region of space-time where gravity is so strong that nothing -- not even light -- can escape once past the event horizon.
+**Formation**: massive stars (&gt;20 solar masses) exhaust nuclear fuel, core collapses under gravity. If remaining mass exceeds ~3 solar masses (Tolman-Oppenheimer-Volkoff limit), nothing stops the collapse -- black hole. Also: supermassive black holes (millions to billions of solar masses) at galaxy centres (Sagittarius A* = 4 million solar masses at Milky Way centre).
+**Event horizon**: the point of no return. Not a physical surface -- you'd feel nothing crossing it (locally). But your future light cone points only inward. Radius = Schwarzschild radius: r = 2GM/c^2. For Earth's mass: ~9mm.
+**Hawking radiation** (1974): quantum effects near event horizon cause black holes to emit thermal radiation and slowly evaporate. Temperature inversely proportional to mass -- stellar black holes are colder than CMB and essentially don't evaporate on cosmic timescales. Micro black holes would evaporate instantly.
+**The singularity**: general relativity predicts infinite density, infinite curvature at the centre. This is a breakdown of the theory, not a physical reality. Singularity = where GR stops working. Quantum gravity (string theory, loop quantum gravity) should resolve it -- but we don't have the theory yet.
+**Information paradox**: Hawking radiation is thermal (random). If black hole evaporates completely, information about what fell in is destroyed -- violating quantum mechanics. Still unresolved. Possible resolution: information is encoded in Hawking radiation (subtle correlations), or in a 'remnant.'</t>
+        </is>
+      </c>
+      <c r="E405" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="2" t="n">
+        <v>493</v>
+      </c>
+      <c r="B406" s="3" t="inlineStr">
+        <is>
+          <t>Sociology</t>
+        </is>
+      </c>
+      <c r="C406" s="3" t="inlineStr">
+        <is>
+          <t>What causes crime, and does punishment actually reduce it?</t>
+        </is>
+      </c>
+      <c r="D406" s="3" t="inlineStr">
+        <is>
+          <t>Crime is not caused by a single factor -- it emerges from interaction of individual, social, and structural variables.
+**Individual-level factors**: low self-control (Gottfredson &amp; Hirschi), antisocial personality, substance abuse, mental illness (small effect -- most mentally ill are not violent; most violent are not mentally ill).
+**Social/environmental factors**:
+1. **Social disorganisation theory** (Shaw &amp; McKay 1942): crime concentrates in neighbourhoods with weak social ties, high turnover, poverty -- not in people.
+2. **Strain theory** (Merton): crime results from gap between culturally valued goals (wealth, success) and legitimate means to achieve them. Innovate (crime) when blocked.
+3. **Social learning**: crime learned in peer groups (differential association -- Sutherland).
+4. **Routine activity theory**: crime occurs when motivated offender + suitable target + absent guardian converge.
+**Structural factors**: poverty, inequality (Gini coefficient predicts crime better than poverty alone), unemployment, housing instability, childhood adversity (ACEs), neighbourhood disinvestment.
+**Does punishment reduce crime?**
+- **Certainty &gt; severity**: research consistently shows certainty of being caught deters more than harshness of punishment. Most offenders don't think they'll be caught.
+- **Death penalty**: no reliable deterrent effect (states with/without have similar homicide rates).
+- **Mass incarceration**: US incarcerates 2M people (highest per capita globally). Criminologists broadly agree: past a threshold, more imprisonment increases crime (family disruption, stigma, criminal networks). Returns to prison are close to zero after ~1980s.
+- **What works**: early childhood intervention (Perry Preschool -- ROI 7-12x), drug treatment, cognitive-behavioural therapy, community policing, environmental design (crime decreases with more streetlights).</t>
+        </is>
+      </c>
+      <c r="E406" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="2" t="n">
+        <v>494</v>
+      </c>
+      <c r="B407" s="3" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C407" s="3" t="inlineStr">
+        <is>
+          <t>How does the internet actually work?</t>
+        </is>
+      </c>
+      <c r="D407" s="3" t="inlineStr">
+        <is>
+          <t>The internet: a global network of interconnected networks using standardised protocols to route and deliver data.
+**Physical layer**: fibre optic cables (light pulses -- transatlantic cables carry terabits/second); copper (DSL, coaxial); wireless (WiFi, 4G/5G -- radio waves). Everything is ultimately photons or electrons.
+**IP (Internet Protocol)**: every device has an IP address (IPv4: 32-bit = ~4 billion addresses, nearly exhausted; IPv6: 128-bit = 340 undecillion addresses). Data broken into packets (~1,500 bytes each), each labelled with source and destination IP.
+**Routing**: packets travel through routers -- each router has a routing table and forwards the packet toward the destination using BGP (Border Gateway Protocol). Packets may take different paths and reassemble at destination.
+**TCP (Transmission Control Protocol)**: guarantees delivery and order. Three-way handshake (SYN, SYN-ACK, ACK). Receiver acknowledges packets; sender retransmits lost ones. Slower but reliable. Used for web, email.
+**UDP**: no handshake, no acknowledgement. Fast but lossy. Used for video streaming, gaming, VoIP -- better to drop a frame than freeze.
+**DNS (Domain Name System)**: translates human-readable names (google.com) to IP addresses. Hierarchical: root servers -&gt; TLD servers (.com, .org) -&gt; authoritative servers. Your browser caches results.
+**HTTPS**: HTTP + TLS encryption. TLS handshake: server sends certificate (signed by trusted CA); client verifies; they negotiate encryption keys using asymmetric cryptography (RSA/ECDH); subsequent traffic encrypted with symmetric key (AES). The padlock in your browser.
+**What you actually see**: when you type a URL, browser does DNS lookup, opens TCP connection, sends HTTP request, server sends back HTML/CSS/JS, browser renders. The whole process in ~100 milliseconds.</t>
+        </is>
+      </c>
+      <c r="E407" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="14" t="n">
+        <v>495</v>
+      </c>
+      <c r="B408" s="15" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="C408" s="15" t="inlineStr">
+        <is>
+          <t>What is calculus and why was it such a revolutionary invention?</t>
+        </is>
+      </c>
+      <c r="D408" s="15" t="inlineStr">
+        <is>
+          <t>Calculus: the mathematics of continuous change. Two branches -- differential calculus (rates of change) and integral calculus (accumulation) -- linked by the Fundamental Theorem of Calculus.
+**Differential calculus**: the derivative. If f(x) describes position, f'(x) = velocity, f''(x) = acceleration. Formally: the limit of (f(x+h)-f(x))/h as h-&gt;0. The slope of the tangent line at a point.
+**Integral calculus**: the integral. Area under a curve, total accumulation. If you know velocity, integrate to get distance. Antiderivative of f'(x) is f(x) + C.
+**Fundamental Theorem of Calculus**: differentiation and integration are inverse operations. Revolutionary -- linked two seemingly unrelated problems.
+**History**: Newton and Leibniz independently invented calculus (1660s-1680s). Bitter priority dispute (Newton claimed first, published later; Leibniz published first). Modern notation (dy/dx, integral sign) is Leibniz's. Newton's dot notation still used in physics.
+**Why it was revolutionary**:
+1. **Physics**: Newton's laws of motion use derivatives (F=ma = F=m*d^2x/dt^2). Without calculus, no mechanics, no orbital calculation, no space travel.
+2. **Engineering**: stress in beams, fluid flow, heat transfer -- all calculus.
+3. **Electricity and magnetism**: Maxwell's equations (calculus) predicted radio waves before Hertz discovered them experimentally.
+4. **Economics**: marginal utility, marginal cost, optimisation -- economics runs on calculus.
+5. **Machine learning**: backpropagation is just calculus (chain rule for partial derivatives).
+**Limits and rigor**: Newton and Leibniz used 'infinitesimals' intuitively. Cauchy and Weierstrass (1800s) put it on rigorous footing with epsilon-delta definition of limits -- removing the 'ghost of departed quantities' that Berkeley mocked.</t>
+        </is>
+      </c>
+      <c r="E408" s="14" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12589,14 +12750,14 @@
         </is>
       </c>
       <c r="B45" s="15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C45" s="15" t="n">
         <v>9.52</v>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436, 440, 447, 459, 472</t>
+          <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436, 440, 447, 459, 472, 495</t>
         </is>
       </c>
     </row>
@@ -12625,14 +12786,14 @@
         </is>
       </c>
       <c r="B47" s="31" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C47" s="31" t="n">
-        <v>9.25</v>
+        <v>9.23</v>
       </c>
       <c r="D47" s="31" t="inlineStr">
         <is>
-          <t>230, 279, 294, 344, 379, 395, 411, 411, 422, 429, 441, 452, 468, 486</t>
+          <t>230, 279, 294, 344, 379, 395, 411, 411, 422, 429, 441, 452, 468, 486, 491</t>
         </is>
       </c>
     </row>
@@ -12967,14 +13128,14 @@
         </is>
       </c>
       <c r="B66" s="7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>9.57</v>
+        <v>9.58</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447, 449, 467, 476, 487</t>
+          <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447, 449, 467, 476, 487, 492</t>
         </is>
       </c>
     </row>
@@ -13093,14 +13254,14 @@
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C73" s="3" t="n">
         <v>9.029999999999999</v>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 413, 428, 439, 448, 448, 480</t>
+          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 413, 428, 439, 448, 448, 480, 493</t>
         </is>
       </c>
     </row>
@@ -13129,14 +13290,14 @@
         </is>
       </c>
       <c r="B75" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>9.1</v>
+        <v>9.08</v>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>283, 314, 410, 434, 461</t>
+          <t>283, 314, 410, 434, 461, 494</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q496-Q500: Sleep, Philosophy of Science, Industrial Revolution, Placebo, Camus Absurd (412 total)
Milestone: Q500 reached. 412 entries across 79 domains.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E408"/>
+  <dimension ref="A1:E413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11927,6 +11927,189 @@
         <v>9.5</v>
       </c>
     </row>
+    <row r="409">
+      <c r="A409" s="10" t="n">
+        <v>496</v>
+      </c>
+      <c r="B409" s="11" t="inlineStr">
+        <is>
+          <t>Neuroscience</t>
+        </is>
+      </c>
+      <c r="C409" s="11" t="inlineStr">
+        <is>
+          <t>How does sleep work and why do we need it?</t>
+        </is>
+      </c>
+      <c r="D409" s="11" t="inlineStr">
+        <is>
+          <t>Sleep: a reversible state of reduced consciousness and metabolic activity occupying roughly a third of human life. Not passive rest -- an active, essential biological process.
+**Architecture**: sleep cycles ~90 minutes, repeating 4-6 times per night.
+- NREM Stage 1 (N1): light sleep, hypnic jerks, theta waves
+- NREM Stage 2 (N2): sleep spindles, K-complexes; bulk of sleep
+- NREM Stage 3 (N3): slow-wave sleep (SWS); delta waves; deepest; hardest to wake from
+- REM: rapid eye movement; dreaming; body paralysed (atonia); brain active as waking
+Earlier cycles: more SWS. Later cycles: more REM.
+**What sleep does**:
+1. **Memory consolidation**: hippocampus replays waking experiences during SWS; transfers to cortex. REM strengthens emotional memories and creative associations.
+2. **Glymphatic clearance**: during SWS, cerebrospinal fluid flushes through brain, clearing metabolic waste including amyloid-beta (Alzheimer's protein). Brain shrinks ~20% during sleep to allow flow.
+3. **Immune function**: cytokine production peaks during sleep; sleep deprivation impairs vaccine response by 50%.
+4. **Metabolic regulation**: leptin/ghrelin balance disrupted by poor sleep -- increases hunger, reduces satiety.
+5. **Cellular repair**: growth hormone released during SWS; protein synthesis, tissue repair.
+**Sleep deprivation effects**: 24h awake = legally drunk (0.10% BAC equivalent performance). 17 days of restricted sleep: cognitive performance equivalent to 48h total deprivation. Chronic restriction not fully recoverable with one night.
+**Why we dream (REM)**: uncertain. Theories: memory consolidation; threat simulation (Revonsuo); emotional processing (Walker); random activation (Hobson's activation-synthesis). No consensus.
+**Circadian rhythm**: SCN (suprachiasmatic nucleus) in hypothalamus is master clock; light resets it via retinal ganglion cells (ipRGCs). Melatonin signals darkness. Blue light at night delays melatonin by up to 3 hours.</t>
+        </is>
+      </c>
+      <c r="E409" s="10" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="16" t="n">
+        <v>497</v>
+      </c>
+      <c r="B410" s="17" t="inlineStr">
+        <is>
+          <t>Philosophy</t>
+        </is>
+      </c>
+      <c r="C410" s="17" t="inlineStr">
+        <is>
+          <t>What is the philosophy of science — what makes something scientific?</t>
+        </is>
+      </c>
+      <c r="D410" s="17" t="inlineStr">
+        <is>
+          <t>Philosophy of science: the study of the methods, foundations, and implications of science. Its central question: what distinguishes science from non-science?
+**Logical positivism** (Vienna Circle, 1920s): only statements verifiable by experience are meaningful. 'God exists' is meaningless; '2+2=4' is analytic; 'water boils at 100C' is verifiable. Problem: the verification principle itself is not verifiable.
+**Falsificationism** (Popper 1934): science cannot verify theories -- only falsify them. A theory is scientific iff it makes predictions that could in principle be proven wrong. 'All swans are white' is falsifiable; 'God works in mysterious ways' is not. Good science actively tries to disprove itself.
+Problem: the Duhem-Quine thesis -- any observation can be 'saved' by adjusting auxiliary hypotheses. No single test definitively refutes a theory.
+**Paradigm shifts** (Kuhn 1962): science proceeds through normal science (puzzle-solving within a paradigm) punctuated by revolutions (paradigm shifts). Scientists resist anomalies; eventually accumulate until a new framework wins. Implication: science is a social activity, not purely logical.
+**Lakatos**: research programmes have a hard core (unfalsifiable assumptions) protected by a belt of auxiliary hypotheses. Progressive programmes make novel predictions; degenerative ones just patch anomalies.
+**Feyerabend**: 'anything goes' -- no universal scientific method. History of science shows successful violations of every proposed rule.
+**Demarcation problem**: what marks the line? Astrology makes predictions but fails them. Psychoanalysis is unfalsifiable. Creation science mimics scientific form. No single criterion suffices.
+**Modern consensus**: science is characterised by: testable predictions, peer review, replication, willingness to revise, cumulative progress. It is a method, not a body of facts.</t>
+        </is>
+      </c>
+      <c r="E410" s="16" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="12" t="n">
+        <v>498</v>
+      </c>
+      <c r="B411" s="13" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="C411" s="13" t="inlineStr">
+        <is>
+          <t>What was the Industrial Revolution and how did it change human life?</t>
+        </is>
+      </c>
+      <c r="D411" s="13" t="inlineStr">
+        <is>
+          <t>The Industrial Revolution (Britain ~1760-1840, spreading globally to 1900): the transition from agrarian, handicraft economies to manufacturing, machine production, and urban society. The most fundamental transformation of human material life since agriculture.
+**Key technologies**:
+- Steam engine (Watt 1769, improved 1782): applied to textile mills, mines, railways, ships
+- Spinning jenny (Hargreaves 1764), water frame (Arkwright 1769): mechanised textile production
+- Puddling process (Cort 1784): mass production of wrought iron
+- Steam locomotive (Stephenson's Rocket 1829): railways transformed movement of goods and people
+**Why Britain first?**
+1. Coal and iron geographically co-located
+2. Secure property rights, patent system
+3. Empire provided raw materials and markets
+4. Agricultural revolution freed labour for factories
+5. Canal system already existed for bulk transport
+**How it changed human life**:
+- Urbanisation: Britain 20% urban in 1800, 70% by 1900. Manchester grew from 25,000 to 350,000 in 100 years.
+- Living standards: initially fell for factory workers (child labour, 14-hour days, dangerous conditions). Rose substantially by late 19th century -- real wages doubled 1820-1870.
+- Life expectancy: urban death rates initially ROSE (cholera, typhoid, overcrowding). Sanitation reforms from 1850s reversed this.
+- Family structure: nuclear family; women and children entered workforce; later withdrew to 'separate spheres.'
+- Time discipline: factory clock replaced natural rhythms; punctuality became a virtue.
+**Long-run effect**: GDP per capita roughly flat for millennia; hockey-stick growth from 1800. Humans today live 40+ years longer than in 1800, with health and material comfort unimaginable to predecessors.</t>
+        </is>
+      </c>
+      <c r="E411" s="12" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="24" t="n">
+        <v>499</v>
+      </c>
+      <c r="B412" s="25" t="inlineStr">
+        <is>
+          <t>Psychology</t>
+        </is>
+      </c>
+      <c r="C412" s="25" t="inlineStr">
+        <is>
+          <t>What is the placebo effect and how powerful is it really?</t>
+        </is>
+      </c>
+      <c r="D412" s="25" t="inlineStr">
+        <is>
+          <t>Placebo effect: measurable, real physiological or psychological improvement resulting from inert treatment -- driven by expectation, conditioning, and the therapeutic relationship.
+**How real it is**: not 'just in your head' -- measurable biological changes:
+- Parkinson's patients given saline injections show dopamine release in striatum (de la Fuente-Fernandez 2001)
+- Placebo painkillers activate endogenous opioid system (naloxone blocks placebo analgesia)
+- Placebo asthma inhalers improve subjective breathing (though not lung function)
+- Sham surgery for knee osteoarthritis (Moseley 2002) performed as well as real surgery for pain and function over 2 years
+**Nocebo**: the reverse -- inert treatment causing harm through negative expectation. Patients told a drug causes nausea develop nausea.
+**Factors that increase placebo effect**:
+- Warm, empathic clinician
+- Expensive-seeming treatment
+- More invasive procedure (injection &gt; pill; sham surgery &gt; injection)
+- Confident delivery ('this will definitely help')
+- Conditioning (prior positive experience with medication)
+**Open-label placebos**: Kaptchuk (2010) -- patients told explicitly 'these are sugar pills with no active ingredient, but placebos can be powerful.' Significant improvement in IBS. The ritual may be as important as belief.
+**Drug trials**: most psychiatric drugs have placebo response rates of 30-50%. Antidepressant effect sizes over placebo are modest (Kirsch 2008 meta-analysis: ~2 points on Hamilton scale for severe depression). Effect is real but smaller than marketing suggests for mild-moderate cases.
+**Ethical dimension**: deliberately deceiving patients to leverage placebo is ethically fraught. Open-label placebos suggest deception may not even be required.</t>
+        </is>
+      </c>
+      <c r="E412" s="24" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="B413" s="3" t="inlineStr">
+        <is>
+          <t>Existentialism</t>
+        </is>
+      </c>
+      <c r="C413" s="3" t="inlineStr">
+        <is>
+          <t>What did Albert Camus mean by the Absurd, and how should we respond to it?</t>
+        </is>
+      </c>
+      <c r="D413" s="3" t="inlineStr">
+        <is>
+          <t>Camus (1913-1960): one of the 20th century's most important philosophers, though he rejected the label. His central idea: the Absurd.
+**The Absurd**: the conflict between two facts:
+1. Human beings have an insatiable need for meaning, clarity, and purpose
+2. The universe offers none -- it is silent, indifferent, chaotic
+The Absurd is not in humans or the world alone, but in the confrontation between them.
+**The Myth of Sisyphus (1942)**: Sisyphus condemned to roll a boulder up a hill forever, watch it roll back, repeat. Camus: this is the human condition. We work toward goals that ultimately mean nothing.
+**Three responses Camus considered**:
+1. **Physical suicide**: killing yourself because life is meaningless. Camus rejects this -- it avoids the Absurd rather than confronting it.
+2. **Philosophical suicide** (Kierkegaard's leap of faith): inventing a god or transcendent meaning to escape the Absurd. Camus calls this intellectual dishonesty -- a 'leap' that denies what reason shows us.
+3. **Revolt**: Camus's answer. Acknowledge the Absurd fully. Refuse to be crushed by it. Live defiantly in spite of it. Create your own meaning through passionate engagement with life.
+**The conclusion**: 'One must imagine Sisyphus happy.' He owns his fate. The struggle itself toward the heights is enough. Meaning is not found -- it is made, moment by moment, in full knowledge of the Absurd.
+**Camus vs Sartre**: both rejected God, but Sartre found radical freedom empowering; Camus found the silence oppressive but liveable. Camus also rejected Marxist 'leap' -- replacing God with History as a transcendent guarantee.
+**Legacy**: Camus remains the philosopher most read for actually living, not just analysing. The Absurd resonates with modern secular anxiety.</t>
+        </is>
+      </c>
+      <c r="E413" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11938,7 +12121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D79"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12422,205 +12605,205 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Folklore</t>
+          <t>Existentialism</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>317</t>
+          <t>500</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Game Theory</t>
+          <t>Folklore</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C28" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>195, 318</t>
+          <t>317</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>General Knowledge</t>
+          <t>Game Theory</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>450</t>
+          <t>195, 318</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
+          <t>General Knowledge</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>450</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
           <t>Genetics</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B31" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C31" s="3" t="n">
         <v>9.119999999999999</v>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>163, 228, 251, 276</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="33" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="33" t="inlineStr">
         <is>
           <t>Geography</t>
         </is>
       </c>
-      <c r="B31" s="33" t="n">
+      <c r="B32" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="C31" s="33" t="n">
+      <c r="C32" s="33" t="n">
         <v>8.5</v>
       </c>
-      <c r="D31" s="33" t="inlineStr">
+      <c r="D32" s="33" t="inlineStr">
         <is>
           <t>405</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>Geology</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>9.119999999999999</v>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>147, 208, 281, 312, 322, 359, 417, 451</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
+          <t>Geology</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>147, 208, 281, 312, 322, 359, 417, 451</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
           <t>Geology / Biology</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B34" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="C34" s="3" t="n">
         <v>9.5</v>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>183</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="B34" s="13" t="n">
-        <v>25</v>
-      </c>
-      <c r="C34" s="13" t="n">
-        <v>9.140000000000001</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
-        <is>
-          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 436, 442, 444, 465, 477, 489</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>History of Philosophy</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>288</t>
+      <c r="B35" s="13" t="n">
+        <v>26</v>
+      </c>
+      <c r="C35" s="13" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>153, 166, 177, 223, 237, 247, 265, 275, 298, 305, 353, 386, 397, 397, 410, 420, 422, 425, 433, 436, 442, 444, 465, 477, 489, 498</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>History of Science</t>
+          <t>History of Philosophy</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>213, 368</t>
+          <t>288</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>History of Technology</t>
+          <t>History of Science</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>9</v>
+        <v>9.5</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>213, 368</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Immunology</t>
+          <t>History of Technology</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
@@ -12631,266 +12814,266 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>333</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Information Theory</t>
+          <t>Immunology</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>205, 350</t>
+          <t>329</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Law</t>
+          <t>Information Theory</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
         <v>2</v>
       </c>
       <c r="C40" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>205, 350</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Law</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" s="3" t="n">
         <v>8.75</v>
       </c>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>348, 409</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="B41" s="5" t="n">
+      <c r="B42" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="C41" s="5" t="n">
+      <c r="C42" s="5" t="n">
         <v>8.859999999999999</v>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>148, 216, 268, 326, 364, 396, 396, 419, 420, 446, 464</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>Literature</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="C42" s="3" t="n">
-        <v>8.880000000000001</v>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>164, 253, 355, 382, 427, 434, 450, 455</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Marine Biology</t>
+          <t>Literature</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>9</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>337</t>
+          <t>164, 253, 355, 382, 427, 434, 450, 455</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
+          <t>Marine Biology</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>337</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
           <t>Materials Science</t>
         </is>
       </c>
-      <c r="B44" s="3" t="n">
+      <c r="B45" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C44" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="C45" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>200, 319, 370</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="15" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="B45" s="15" t="n">
+      <c r="B46" s="15" t="n">
         <v>22</v>
       </c>
-      <c r="C45" s="15" t="n">
+      <c r="C46" s="15" t="n">
         <v>9.52</v>
       </c>
-      <c r="D45" s="15" t="inlineStr">
+      <c r="D46" s="15" t="inlineStr">
         <is>
           <t>154, 168, 215, 229, 242, 264, 290, 340, 380, 394, 404, 404, 412, 414, 418, 423, 436, 440, 447, 459, 472, 495</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>Mathematics / Economics</t>
         </is>
       </c>
-      <c r="B46" s="3" t="n">
+      <c r="B47" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C46" s="3" t="n">
+      <c r="C47" s="3" t="n">
         <v>9.5</v>
       </c>
-      <c r="D46" s="3" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>180</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="31" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="31" t="inlineStr">
         <is>
           <t>Medicine</t>
         </is>
       </c>
-      <c r="B47" s="31" t="n">
+      <c r="B48" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="C47" s="31" t="n">
+      <c r="C48" s="31" t="n">
         <v>9.23</v>
       </c>
-      <c r="D47" s="31" t="inlineStr">
+      <c r="D48" s="31" t="inlineStr">
         <is>
           <t>230, 279, 294, 344, 379, 395, 411, 411, 422, 429, 441, 452, 468, 486, 491</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>Meteorology</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>204</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Meteorology</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C49" s="3" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>445</t>
+          <t>204</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
+          <t>Music</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>445</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
           <t>Music Theory</t>
         </is>
       </c>
-      <c r="B50" s="3" t="n">
+      <c r="B51" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C50" s="3" t="n">
+      <c r="C51" s="3" t="n">
         <v>8.67</v>
       </c>
-      <c r="D50" s="3" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>198, 328, 414</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="11" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t>Neuroscience</t>
         </is>
       </c>
-      <c r="B51" s="11" t="n">
-        <v>19</v>
-      </c>
-      <c r="C51" s="11" t="n">
-        <v>9.390000000000001</v>
-      </c>
-      <c r="D51" s="11" t="inlineStr">
-        <is>
-          <t>152, 217, 238, 241, 254, 269, 289, 299, 302, 332, 362, 385, 403, 403, 423, 435, 441, 471, 478</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>Neuroscience / Linguistics</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C52" s="3" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>186</t>
+      <c r="B52" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="C52" s="11" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>152, 217, 238, 241, 254, 269, 289, 299, 302, 332, 362, 385, 403, 403, 423, 435, 441, 471, 478, 496</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Neuroscience / Philosophy</t>
+          <t>Neuroscience / Linguistics</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
@@ -12901,14 +13084,14 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>176</t>
+          <t>186</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Neuroscience / Psychology</t>
+          <t>Neuroscience / Philosophy</t>
         </is>
       </c>
       <c r="B54" s="3" t="n">
@@ -12919,140 +13102,140 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>176</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Number Theory</t>
+          <t>Neuroscience / Psychology</t>
         </is>
       </c>
       <c r="B55" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C55" s="3" t="n">
-        <v>10</v>
+        <v>9.5</v>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>165</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Nutrition</t>
+          <t>Number Theory</t>
         </is>
       </c>
       <c r="B56" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>8.75</v>
+        <v>10</v>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>354, 458</t>
+          <t>206</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Nutrition Science</t>
+          <t>Nutrition</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C57" s="3" t="n">
-        <v>8</v>
+        <v>8.75</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>354, 458</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nutrition Science</t>
         </is>
       </c>
       <c r="B58" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
+          <t>196</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Oceanography</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
           <t>199</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="17" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="17" t="inlineStr">
         <is>
           <t>Philosophy</t>
         </is>
       </c>
-      <c r="B59" s="17" t="n">
-        <v>20</v>
-      </c>
-      <c r="C59" s="17" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="D59" s="17" t="inlineStr">
-        <is>
-          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 439, 444, 469, 475, 479</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>Philosophy / History</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C60" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>185</t>
+      <c r="B60" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="C60" s="17" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="D60" s="17" t="inlineStr">
+        <is>
+          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 439, 444, 469, 475, 479, 497</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Philosophy / Neuroscience</t>
+          <t>Philosophy / History</t>
         </is>
       </c>
       <c r="B61" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C61" s="3" t="n">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>185</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Philosophy / Physics</t>
+          <t>Philosophy / Neuroscience</t>
         </is>
       </c>
       <c r="B62" s="3" t="n">
@@ -13063,266 +13246,266 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>146</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Philosophy of Language</t>
+          <t>Philosophy / Physics</t>
         </is>
       </c>
       <c r="B63" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C63" s="3" t="n">
         <v>9.5</v>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>250, 374</t>
+          <t>190</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Philosophy of Mind</t>
+          <t>Philosophy of Language</t>
         </is>
       </c>
       <c r="B64" s="3" t="n">
         <v>2</v>
       </c>
       <c r="C64" s="3" t="n">
-        <v>10</v>
+        <v>9.5</v>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>209, 345</t>
+          <t>250, 374</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Philosophy of Science</t>
+          <t>Philosophy of Mind</t>
         </is>
       </c>
       <c r="B65" s="3" t="n">
         <v>2</v>
       </c>
       <c r="C65" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>209, 345</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Philosophy of Science</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" s="3" t="n">
         <v>9.5</v>
       </c>
-      <c r="D65" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>301, 330</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="7" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="B66" s="7" t="n">
+      <c r="B67" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="C66" s="7" t="n">
+      <c r="C67" s="7" t="n">
         <v>9.58</v>
       </c>
-      <c r="D66" s="7" t="inlineStr">
+      <c r="D67" s="7" t="inlineStr">
         <is>
           <t>149, 161, 170, 187, 224, 235, 248, 256, 262, 272, 286, 296, 307, 342, 367, 381, 401, 401, 412, 421, 426, 433, 438, 442, 447, 449, 467, 476, 487, 492</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>Physiology</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C67" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>192</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Political Philosophy</t>
+          <t>Physiology</t>
         </is>
       </c>
       <c r="B68" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C68" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>325</t>
+          <t>192</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
+          <t>Political Philosophy</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
           <t>Political Science</t>
         </is>
       </c>
-      <c r="B69" s="3" t="n">
+      <c r="B70" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C69" s="3" t="n">
+      <c r="C70" s="3" t="n">
         <v>8.83</v>
       </c>
-      <c r="D69" s="3" t="inlineStr">
+      <c r="D70" s="3" t="inlineStr">
         <is>
           <t>197, 415, 457</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="25" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="25" t="inlineStr">
         <is>
           <t>Psychology</t>
         </is>
       </c>
-      <c r="B70" s="25" t="n">
-        <v>22</v>
-      </c>
-      <c r="C70" s="25" t="n">
+      <c r="B71" s="25" t="n">
+        <v>23</v>
+      </c>
+      <c r="C71" s="25" t="n">
         <v>9.109999999999999</v>
       </c>
-      <c r="D70" s="25" t="inlineStr">
-        <is>
-          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 424, 432, 437, 445, 453, 473, 485</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>Quantum Computing</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C71" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>194</t>
+      <c r="D71" s="25" t="inlineStr">
+        <is>
+          <t>159, 179, 214, 232, 249, 263, 284, 306, 336, 360, 376, 392, 407, 407, 416, 424, 432, 437, 445, 453, 473, 485, 499</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Robotics</t>
+          <t>Quantum Computing</t>
         </is>
       </c>
       <c r="B72" s="3" t="n">
         <v>1</v>
       </c>
       <c r="C72" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>194</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Sociology</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C73" s="3" t="n">
-        <v>9.029999999999999</v>
+        <v>8</v>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 413, 428, 439, 448, 448, 480, 493</t>
+          <t>211</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Statistics</t>
+          <t>Sociology</t>
         </is>
       </c>
       <c r="B74" s="3" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="C74" s="3" t="n">
-        <v>10</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>162, 188, 226, 234, 257, 273, 293, 308, 343, 371, 390, 405, 413, 428, 439, 448, 448, 480, 493</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Statistics</t>
         </is>
       </c>
       <c r="B75" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C75" s="3" t="n">
-        <v>9.08</v>
+        <v>10</v>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>283, 314, 410, 434, 461, 494</t>
+          <t>356</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="B76" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C76" s="3" t="n">
-        <v>9</v>
+        <v>9.08</v>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>283, 314, 410, 434, 461, 494</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Thermodynamics</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="B77" s="3" t="n">
@@ -13333,14 +13516,14 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>193</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Urban Planning</t>
+          <t>Thermodynamics</t>
         </is>
       </c>
       <c r="B78" s="3" t="n">
@@ -13351,12 +13534,30 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>193</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Urban Planning</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C79" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>323</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
         <is>
           <t>What is e
 e ≈ 2.71828. Unique number where eˣ is its own derivative — rate of change equals value at every point. Discovered by Jacob Bernoulli 1683 via compound interest ($1 at 100% continuous = $e after 1 year). Appears in: population growth, normal distribution, Poisson processes, entropy. Euler's identity: e^(iπ) + 1 = 0. Describes processes that grow by feeding on themselves. Emerges from structure of continuous change itself. Transcendental number.
@@ -13542,13 +13743,13 @@
 Q107 First Cell Membrane: amphiphilic fatty acids spontaneously self-assemble into vesicles to minimize free energy — no enzymes needed; fatty acids in meteorites (Murchison) and hydrothermal vents; Szo</t>
         </is>
       </c>
-      <c r="B79" s="3" t="n">
+      <c r="B80" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C79" s="3" t="n">
+      <c r="C80" s="3" t="n">
         <v>9.5</v>
       </c>
-      <c r="D79" s="3" t="inlineStr">
+      <c r="D80" s="3" t="inlineStr">
         <is>
           <t>37</t>
         </is>

</xml_diff>

<commit_message>
Add Q501-Q505: Inflation, CRISPR, Self/Identity, Black Holes, Linguistic Relativity (417 total)
</commit_message>
<xml_diff>
--- a/yaya-ai/data/yaya_qa_export.xlsx
+++ b/yaya-ai/data/yaya_qa_export.xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E413"/>
+  <dimension ref="A1:E418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12110,6 +12110,186 @@
         <v>10</v>
       </c>
     </row>
+    <row r="414">
+      <c r="A414" s="8" t="n">
+        <v>501</v>
+      </c>
+      <c r="B414" s="9" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="C414" s="9" t="inlineStr">
+        <is>
+          <t>What is inflation, and why is it so hard to control?</t>
+        </is>
+      </c>
+      <c r="D414" s="9" t="inlineStr">
+        <is>
+          <t>Inflation: sustained rise in the general price level — or equivalently, fall in purchasing power of money. If prices rise 7%, your salary buys 7% less.
+**What causes it**:
+1. **Demand-pull**: too much money chasing too few goods. Wartime economies; massive stimulus.
+2. **Cost-push**: supply costs rise (oil shock 1973; COVID supply chains). Costs passed to prices.
+3. **Built-in (wage-price spiral)**: workers expect inflation → demand higher wages → firms raise prices to compensate → repeat.
+4. **Monetary**: Milton Friedman: 'Inflation is always and everywhere a monetary phenomenon.' Print more money than output grows → prices rise. Weimar Germany 1923; Zimbabwe 2008 (100 trillion dollar note).
+**The Fisher Equation**: MV = PQ. Money supply × velocity = price level × real output. Hold V and Q constant: doubling M doubles P.
+**Why hard to control**:
+- Central banks use interest rates (raise rates → borrowing costly → demand falls → prices stabilise). But:
+- Rate rises hurt debtors, raise unemployment, can trigger recessions.
+- Supply-side inflation (energy, food) doesn't respond to rate hikes — you're crushing demand to fight a supply problem.
+- Expectations are self-fulfilling: if people believe 10% inflation is coming, they demand 10% wage rises, making it happen.
+- Political pressure: governments don't want high rates near elections.
+**The 2% target**: most central banks target 2% — low enough to preserve purchasing power; high enough to avoid deflation (falling prices → consumers defer spending → recession death spiral; Japan's 'lost decades').
+**2021-2023 inflation**: COVID stimulus + supply chain disruption + energy shock (Ukraine war) combined all three causes simultaneously. Fed raised rates 500bps in 18 months — fastest since Volcker 1980.</t>
+        </is>
+      </c>
+      <c r="E414" s="8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="2" t="n">
+        <v>502</v>
+      </c>
+      <c r="B415" s="3" t="inlineStr">
+        <is>
+          <t>Genetics</t>
+        </is>
+      </c>
+      <c r="C415" s="3" t="inlineStr">
+        <is>
+          <t>What is CRISPR-Cas9 and how does gene editing work?</t>
+        </is>
+      </c>
+      <c r="D415" s="3" t="inlineStr">
+        <is>
+          <t>CRISPR-Cas9: a molecular tool that lets scientists edit DNA with unprecedented precision. Nobel Prize 2020 (Doudna and Charpentier). Derived from a bacterial immune system.
+**How bacteria use CRISPR**: when a virus infects a bacterium, the bacterium can store fragments of viral DNA in its genome (CRISPR arrays). If the same virus attacks again, the bacterium transcribes these into guide RNA, which directs the Cas9 protein to cut the viral DNA. It is a biological immune memory.
+**How scientists repurposed it**:
+1. Design a guide RNA (gRNA) that matches any target DNA sequence (20 bases)
+2. Load it into Cas9 protein
+3. Deliver to cells (virus vector, lipid nanoparticle, electroporation)
+4. Cas9 scans DNA, finds the matching sequence + PAM motif (NGG), cuts both strands
+5. Cell's repair machinery kicks in:
+   - **NHEJ** (non-homologous end joining): error-prone repair → insertions/deletions → gene knockout
+   - **HDR** (homology-directed repair): provide a template → precise edit or gene insertion
+**Applications**:
+- **Medicine**: sickle cell disease and beta-thalassemia cured in trials (2023) — edit stem cells to reactivate fetal haemoglobin. Cancer immunotherapy (edit T cells). Inherited blindness.
+- **Agriculture**: disease-resistant crops; hornless cattle; non-browning mushrooms.
+- **Research**: knock out any gene to study its function.
+**Ethical concerns**:
+- **Germline editing**: He Jiankui (2018) edited human embryos to resist HIV — twins born, scientist jailed. Heritable changes affect all descendants — irreversible.
+- **Off-target cuts**: Cas9 occasionally cuts wrong sites.
+- **Enhancement vs therapy**: where is the line?
+**Next generation**: base editors (change one nucleotide without cutting); prime editors ('find and replace' for DNA). More precise, fewer off-targets.</t>
+        </is>
+      </c>
+      <c r="E415" s="2" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="16" t="n">
+        <v>503</v>
+      </c>
+      <c r="B416" s="17" t="inlineStr">
+        <is>
+          <t>Philosophy</t>
+        </is>
+      </c>
+      <c r="C416" s="17" t="inlineStr">
+        <is>
+          <t>Does the self exist — or is personal identity an illusion?</t>
+        </is>
+      </c>
+      <c r="D416" s="17" t="inlineStr">
+        <is>
+          <t>The self: the sense of being a continuous, unified 'I' persisting through time. One of philosophy's hardest questions — and neuroscience is making it harder.
+**The bundle theory (Hume 1739)**: look inward for a 'self' — you find only a stream of perceptions: thoughts, feelings, sensations, memories. No observer behind them. The self is a bundle of experiences, not a separate thing. Like a nation: many components, no single 'nationhood' beyond them.
+**The narrative self (Dennett, Ricoeur)**: the self is a story the brain tells — a coherent narrative constructed from experience. Not a fixed entity but an ongoing fiction. Useful fiction, but fiction nonetheless. The brain's 'press secretary' rationalising decisions already made.
+**Personal identity over time (Locke vs Parfit)**:
+- Locke: identity = psychological continuity — memory connects your past self to present self.
+- Problem: if teleporter destroys you and recreates an identical person on Mars, is that you?
+- Parfit (1984): personal identity is not what matters. What matters is psychological continuity and connectedness. If the Mars copy has all your memories and character, the question 'is it really you?' may be empty. Identity is not a deep fact.
+**The neuroscience view**: no single 'self centre' in the brain. Default mode network generates self-referential processing but is distributed. Split-brain patients (corpus callosum severed) show two semi-independent streams of consciousness — one 'self' or two?
+**Buddhist philosophy**: anatta (no-self) — the sense of a permanent, unified self is a cognitive illusion that causes suffering. Meditation reveals the constructed nature of self.
+**The paradox**: whatever asks 'does the self exist?' is itself the self. The question may be self-refuting — or self-illuminating.</t>
+        </is>
+      </c>
+      <c r="E416" s="16" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="2" t="n">
+        <v>504</v>
+      </c>
+      <c r="B417" s="3" t="inlineStr">
+        <is>
+          <t>Astrophysics</t>
+        </is>
+      </c>
+      <c r="C417" s="3" t="inlineStr">
+        <is>
+          <t>What is a black hole — and what actually happens inside one?</t>
+        </is>
+      </c>
+      <c r="D417" s="3" t="inlineStr">
+        <is>
+          <t>Black hole: a region of spacetime where gravity is so extreme that nothing — not even light — can escape past the event horizon. Not a hole; a massive, collapsed object.
+**Formation**: when a massive star (&gt;20 solar masses) exhausts its nuclear fuel, radiation pressure fails, core collapses under gravity, rebounds in supernova, leaving behind a singularity. Supermassive black holes (millions-billions of solar masses) at galactic centres: formation unclear — primordial? Grown by accretion and mergers?
+**Key features**:
+- **Event horizon**: the point of no return. Radius = Schwarzschild radius: r = 2GM/c². For Sun: ~3km. For Earth: ~9mm.
+- **Singularity**: at the centre, density infinite, spacetime curvature infinite. GR breaks down here — quantum gravity needed.
+- **Hawking radiation** (1974): quantum effects near event horizon cause black holes to slowly emit thermal radiation and eventually evaporate. Temperature inversely proportional to mass. Stellar-mass BH: evaporation time &gt;&gt; age of universe.
+**What happens if you fall in** (from your perspective):
+- For a large BH: cross event horizon without drama — tidal forces modest at r_s.
+- No local 'wall' — you feel nothing special at the horizon.
+- Tidal forces (spaghettification) kill you as you approach singularity.
+- Light from outside universe appears increasingly blueshifted.
+**From outside observer's perspective**:
+- You appear to slow down, freeze, redshift to invisibility at horizon.
+- You never appear to cross — time dilation becomes infinite at event horizon.
+**The information paradox**: Hawking radiation is thermal (random) — so when a BH evaporates, all information about what fell in is destroyed. But quantum mechanics says information cannot be destroyed. Unresolved. Possible resolution: holographic principle — information encoded on event horizon surface.
+**Confirmed observations**: EHT imaged M87* (2019) and SgrA* (2022) — first direct images. Gravitational waves from BH mergers detected by LIGO (2015).</t>
+        </is>
+      </c>
+      <c r="E417" s="2" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="4" t="n">
+        <v>505</v>
+      </c>
+      <c r="B418" s="5" t="inlineStr">
+        <is>
+          <t>Linguistics</t>
+        </is>
+      </c>
+      <c r="C418" s="5" t="inlineStr">
+        <is>
+          <t>How does language shape thought — does your language change how you think?</t>
+        </is>
+      </c>
+      <c r="D418" s="5" t="inlineStr">
+        <is>
+          <t>Linguistic relativity (Sapir-Whorf hypothesis): the language you speak influences how you perceive and think about the world. Two versions: strong (language determines thought — now rejected) and weak (language influences thought — supported by evidence).
+**The strong hypothesis (Whorf 1940s)**: argued Hopi Indians had no tense — therefore thought about time differently. Later debunked: Hopi does have temporal concepts; Whorf's analysis was flawed.
+**Modern evidence for weak version** (Boroditsky et al.):
+- **Colour perception**: Russian has distinct words for light blue (goluboy) and dark blue (siniy). Russian speakers discriminate shades of blue faster than English speakers in the blue-boundary range. Language primes categorical perception.
+- **Spatial orientation**: Guugu Yimithirr (Australia) uses cardinal directions (north/south/east/west) not relative (left/right/behind). Speakers maintain perfect orientation at all times, even indoors. Language shapes navigation.
+- **Number**: Piraha (Amazon) has no exact number words above 2. Speakers cannot reliably perform exact numerical tasks.
+- **Gender**: Spanish/French nouns have gender. Speakers describe gendered objects using attributes matching grammatical gender (bridge = masculine in German, feminine in Spanish → described differently).
+- **Time direction**: Mandarin speakers more naturally think of time vertically (earlier above, later below). English speakers think horizontally.
+**What language doesn't determine**: pre-linguistic infants and great apes have numerical, spatial, and causal concepts without language. Thought precedes language developmentally; language is not the sole medium of thought.
+**Practical implication**: multilingual people report feeling 'different' in different languages — different emotional tone, different social identity, different association networks. Language is not a cage but a lens.</t>
+        </is>
+      </c>
+      <c r="E418" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12249,14 +12429,14 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>9.5</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>231, 327</t>
+          <t>231, 327, 504</t>
         </is>
       </c>
     </row>
@@ -12519,14 +12699,14 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>9.119999999999999</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425, 432, 443, 463, 474, 488</t>
+          <t>151, 175, 218, 244, 271, 291, 303, 331, 358, 363, 373, 384, 402, 402, 418, 425, 432, 443, 463, 474, 488, 501</t>
         </is>
       </c>
     </row>
@@ -12681,14 +12861,14 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>9.119999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>163, 228, 251, 276</t>
+          <t>163, 228, 251, 276, 502</t>
         </is>
       </c>
     </row>
@@ -12879,14 +13059,14 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>8.859999999999999</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>148, 216, 268, 326, 364, 396, 396, 419, 420, 446, 464</t>
+          <t>148, 216, 268, 326, 364, 396, 396, 419, 420, 446, 464, 505</t>
         </is>
       </c>
     </row>
@@ -13203,14 +13383,14 @@
         </is>
       </c>
       <c r="B60" s="17" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C60" s="17" t="n">
-        <v>9.380000000000001</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="D60" s="17" t="inlineStr">
         <is>
-          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 439, 444, 469, 475, 479, 497</t>
+          <t>155, 172, 182, 220, 239, 270, 280, 315, 361, 387, 399, 399, 416, 430, 430, 439, 444, 469, 475, 479, 497, 503</t>
         </is>
       </c>
     </row>

</xml_diff>